<commit_message>
Relatório de compras 05/10/2026 10:16
</commit_message>
<xml_diff>
--- a/data/relatorio.xlsx
+++ b/data/relatorio.xlsx
@@ -1735,10 +1735,10 @@
         <v>1</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>59.9</v>
+        <v>18.5</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>59.9</v>
+        <v>18.5</v>
       </c>
       <c r="H33" s="2" t="n">
         <v>1398686</v>
@@ -1782,10 +1782,10 @@
         <v>1</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>18.5</v>
+        <v>9.3</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>18.5</v>
+        <v>9.3</v>
       </c>
       <c r="H34" s="2" t="n">
         <v>1398686</v>
@@ -1829,10 +1829,10 @@
         <v>1</v>
       </c>
       <c r="F35" s="5" t="n">
-        <v>9.3</v>
+        <v>59.9</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>9.3</v>
+        <v>59.9</v>
       </c>
       <c r="H35" s="2" t="n">
         <v>1398686</v>
@@ -4414,10 +4414,10 @@
         <v>1</v>
       </c>
       <c r="F90" s="5" t="n">
-        <v>200</v>
+        <v>67</v>
       </c>
       <c r="G90" s="4" t="n">
-        <v>200</v>
+        <v>67</v>
       </c>
       <c r="H90" s="2" t="n">
         <v>1402331</v>
@@ -4461,10 +4461,10 @@
         <v>1</v>
       </c>
       <c r="F91" s="5" t="n">
-        <v>67</v>
+        <v>200</v>
       </c>
       <c r="G91" s="4" t="n">
-        <v>67</v>
+        <v>200</v>
       </c>
       <c r="H91" s="2" t="n">
         <v>1402331</v>
@@ -4884,10 +4884,10 @@
         <v>30</v>
       </c>
       <c r="F100" s="5" t="n">
-        <v>1.85</v>
+        <v>0.6</v>
       </c>
       <c r="G100" s="4" t="n">
-        <v>55.5</v>
+        <v>18</v>
       </c>
       <c r="H100" s="2" t="n">
         <v>1402783</v>
@@ -4928,13 +4928,13 @@
         </is>
       </c>
       <c r="E101" s="4" t="n">
-        <v>200</v>
+        <v>268</v>
       </c>
       <c r="F101" s="5" t="n">
-        <v>0.17</v>
+        <v>0.22</v>
       </c>
       <c r="G101" s="4" t="n">
-        <v>34</v>
+        <v>58.96</v>
       </c>
       <c r="H101" s="2" t="n">
         <v>1402783</v>
@@ -4975,13 +4975,13 @@
         </is>
       </c>
       <c r="E102" s="4" t="n">
-        <v>268</v>
+        <v>60</v>
       </c>
       <c r="F102" s="5" t="n">
         <v>0.22</v>
       </c>
       <c r="G102" s="4" t="n">
-        <v>58.96</v>
+        <v>13.2</v>
       </c>
       <c r="H102" s="2" t="n">
         <v>1402783</v>
@@ -5022,13 +5022,13 @@
         </is>
       </c>
       <c r="E103" s="4" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F103" s="5" t="n">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="G103" s="4" t="n">
-        <v>13.2</v>
+        <v>3</v>
       </c>
       <c r="H103" s="2" t="n">
         <v>1402783</v>
@@ -5072,10 +5072,10 @@
         <v>30</v>
       </c>
       <c r="F104" s="5" t="n">
-        <v>0.1</v>
+        <v>0.42</v>
       </c>
       <c r="G104" s="4" t="n">
-        <v>3</v>
+        <v>12.6</v>
       </c>
       <c r="H104" s="2" t="n">
         <v>1402783</v>
@@ -5119,10 +5119,10 @@
         <v>30</v>
       </c>
       <c r="F105" s="5" t="n">
-        <v>0.42</v>
+        <v>0.12</v>
       </c>
       <c r="G105" s="4" t="n">
-        <v>12.6</v>
+        <v>3.6</v>
       </c>
       <c r="H105" s="2" t="n">
         <v>1402783</v>
@@ -5163,13 +5163,13 @@
         </is>
       </c>
       <c r="E106" s="4" t="n">
-        <v>30</v>
+        <v>200</v>
       </c>
       <c r="F106" s="5" t="n">
-        <v>0.6</v>
+        <v>0.17</v>
       </c>
       <c r="G106" s="4" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="H106" s="2" t="n">
         <v>1402783</v>
@@ -5213,10 +5213,10 @@
         <v>30</v>
       </c>
       <c r="F107" s="5" t="n">
-        <v>0.12</v>
+        <v>1.85</v>
       </c>
       <c r="G107" s="4" t="n">
-        <v>3.6</v>
+        <v>55.5</v>
       </c>
       <c r="H107" s="2" t="n">
         <v>1402783</v>
@@ -5257,13 +5257,13 @@
         </is>
       </c>
       <c r="E108" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F108" s="5" t="n">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="G108" s="4" t="n">
-        <v>324</v>
+        <v>890</v>
       </c>
       <c r="H108" s="2" t="n">
         <v>1402788</v>
@@ -5398,13 +5398,13 @@
         </is>
       </c>
       <c r="E111" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F111" s="5" t="n">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="G111" s="4" t="n">
-        <v>890</v>
+        <v>324</v>
       </c>
       <c r="H111" s="2" t="n">
         <v>1402788</v>
@@ -7607,13 +7607,13 @@
         </is>
       </c>
       <c r="E158" s="4" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F158" s="5" t="n">
-        <v>0.54</v>
+        <v>19.32</v>
       </c>
       <c r="G158" s="4" t="n">
-        <v>10.8</v>
+        <v>19.32</v>
       </c>
       <c r="H158" s="2" t="n">
         <v>1405673</v>
@@ -7657,10 +7657,10 @@
         <v>1</v>
       </c>
       <c r="F159" s="5" t="n">
-        <v>19.32</v>
+        <v>17.43</v>
       </c>
       <c r="G159" s="4" t="n">
-        <v>19.32</v>
+        <v>17.43</v>
       </c>
       <c r="H159" s="2" t="n">
         <v>1405673</v>
@@ -7704,10 +7704,10 @@
         <v>1</v>
       </c>
       <c r="F160" s="5" t="n">
-        <v>18.91</v>
+        <v>17.43</v>
       </c>
       <c r="G160" s="4" t="n">
-        <v>18.91</v>
+        <v>17.43</v>
       </c>
       <c r="H160" s="2" t="n">
         <v>1405673</v>
@@ -7751,10 +7751,10 @@
         <v>1</v>
       </c>
       <c r="F161" s="5" t="n">
-        <v>19.32</v>
+        <v>18.91</v>
       </c>
       <c r="G161" s="4" t="n">
-        <v>19.32</v>
+        <v>18.91</v>
       </c>
       <c r="H161" s="2" t="n">
         <v>1405673</v>
@@ -7795,13 +7795,13 @@
         </is>
       </c>
       <c r="E162" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F162" s="5" t="n">
-        <v>17.43</v>
+        <v>13.17</v>
       </c>
       <c r="G162" s="4" t="n">
-        <v>17.43</v>
+        <v>26.34</v>
       </c>
       <c r="H162" s="2" t="n">
         <v>1405673</v>
@@ -7936,13 +7936,13 @@
         </is>
       </c>
       <c r="E165" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F165" s="5" t="n">
-        <v>5.67</v>
+        <v>19.71</v>
       </c>
       <c r="G165" s="4" t="n">
-        <v>28.35</v>
+        <v>19.71</v>
       </c>
       <c r="H165" s="2" t="n">
         <v>1405673</v>
@@ -7986,10 +7986,10 @@
         <v>1</v>
       </c>
       <c r="F166" s="5" t="n">
-        <v>19.71</v>
+        <v>19.32</v>
       </c>
       <c r="G166" s="4" t="n">
-        <v>19.71</v>
+        <v>19.32</v>
       </c>
       <c r="H166" s="2" t="n">
         <v>1405673</v>
@@ -8030,13 +8030,13 @@
         </is>
       </c>
       <c r="E167" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F167" s="5" t="n">
-        <v>13.17</v>
+        <v>18.91</v>
       </c>
       <c r="G167" s="4" t="n">
-        <v>26.34</v>
+        <v>18.91</v>
       </c>
       <c r="H167" s="2" t="n">
         <v>1405673</v>
@@ -8077,13 +8077,13 @@
         </is>
       </c>
       <c r="E168" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F168" s="5" t="n">
-        <v>18.91</v>
+        <v>5.67</v>
       </c>
       <c r="G168" s="4" t="n">
-        <v>18.91</v>
+        <v>28.35</v>
       </c>
       <c r="H168" s="2" t="n">
         <v>1405673</v>
@@ -8124,13 +8124,13 @@
         </is>
       </c>
       <c r="E169" s="4" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F169" s="5" t="n">
-        <v>17.43</v>
+        <v>0.54</v>
       </c>
       <c r="G169" s="4" t="n">
-        <v>17.43</v>
+        <v>10.8</v>
       </c>
       <c r="H169" s="2" t="n">
         <v>1405673</v>
@@ -10947,10 +10947,10 @@
         <v>2</v>
       </c>
       <c r="F229" s="5" t="n">
-        <v>4451.305</v>
+        <v>593.505</v>
       </c>
       <c r="G229" s="4" t="n">
-        <v>8902.61</v>
+        <v>1187.01</v>
       </c>
       <c r="H229" s="2" t="n">
         <v>1410106</v>
@@ -10994,10 +10994,10 @@
         <v>2</v>
       </c>
       <c r="F230" s="5" t="n">
-        <v>2374.03</v>
+        <v>4451.305</v>
       </c>
       <c r="G230" s="4" t="n">
-        <v>4748.06</v>
+        <v>8902.61</v>
       </c>
       <c r="H230" s="2" t="n">
         <v>1410106</v>
@@ -11041,10 +11041,10 @@
         <v>2</v>
       </c>
       <c r="F231" s="5" t="n">
-        <v>593.505</v>
+        <v>2374.03</v>
       </c>
       <c r="G231" s="4" t="n">
-        <v>1187.01</v>
+        <v>4748.06</v>
       </c>
       <c r="H231" s="2" t="n">
         <v>1410106</v>
@@ -13999,13 +13999,13 @@
         </is>
       </c>
       <c r="E294" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F294" s="5" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="G294" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H294" s="2" t="n">
         <v>1423209</v>
@@ -14046,13 +14046,13 @@
         </is>
       </c>
       <c r="E295" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F295" s="5" t="n">
-        <v>19</v>
+        <v>3.5</v>
       </c>
       <c r="G295" s="4" t="n">
-        <v>228</v>
+        <v>14</v>
       </c>
       <c r="H295" s="2" t="n">
         <v>1423209</v>
@@ -14093,13 +14093,13 @@
         </is>
       </c>
       <c r="E296" s="4" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F296" s="5" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="G296" s="4" t="n">
-        <v>16</v>
+        <v>228</v>
       </c>
       <c r="H296" s="2" t="n">
         <v>1423209</v>
@@ -14140,10 +14140,10 @@
         </is>
       </c>
       <c r="E297" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F297" s="5" t="n">
-        <v>3.5</v>
+        <v>14</v>
       </c>
       <c r="G297" s="4" t="n">
         <v>14</v>
@@ -14610,13 +14610,13 @@
         </is>
       </c>
       <c r="E307" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F307" s="5" t="n">
-        <v>6.5</v>
+        <v>4.65</v>
       </c>
       <c r="G307" s="4" t="n">
-        <v>6.5</v>
+        <v>18.6</v>
       </c>
       <c r="H307" s="2" t="n">
         <v>1423662</v>
@@ -14657,13 +14657,13 @@
         </is>
       </c>
       <c r="E308" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F308" s="5" t="n">
-        <v>4.65</v>
+        <v>6.5</v>
       </c>
       <c r="G308" s="4" t="n">
-        <v>18.6</v>
+        <v>6.5</v>
       </c>
       <c r="H308" s="2" t="n">
         <v>1423662</v>
@@ -15503,13 +15503,13 @@
         </is>
       </c>
       <c r="E326" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F326" s="5" t="n">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="G326" s="4" t="n">
-        <v>1170</v>
+        <v>115</v>
       </c>
       <c r="H326" s="2" t="n">
         <v>1429513</v>
@@ -15647,10 +15647,10 @@
         <v>9</v>
       </c>
       <c r="F329" s="5" t="n">
-        <v>189</v>
+        <v>130</v>
       </c>
       <c r="G329" s="4" t="n">
-        <v>1701</v>
+        <v>1170</v>
       </c>
       <c r="H329" s="2" t="n">
         <v>1429513</v>
@@ -15691,13 +15691,13 @@
         </is>
       </c>
       <c r="E330" s="4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F330" s="5" t="n">
-        <v>115</v>
+        <v>189</v>
       </c>
       <c r="G330" s="4" t="n">
-        <v>115</v>
+        <v>1701</v>
       </c>
       <c r="H330" s="2" t="n">
         <v>1429513</v>
@@ -16020,13 +16020,13 @@
         </is>
       </c>
       <c r="E337" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F337" s="5" t="n">
-        <v>17.32</v>
+        <v>39</v>
       </c>
       <c r="G337" s="4" t="n">
-        <v>69.28</v>
+        <v>234</v>
       </c>
       <c r="H337" s="2" t="n">
         <v>1431621</v>
@@ -16161,13 +16161,13 @@
         </is>
       </c>
       <c r="E340" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F340" s="5" t="n">
-        <v>39</v>
+        <v>17.32</v>
       </c>
       <c r="G340" s="4" t="n">
-        <v>234</v>
+        <v>69.28</v>
       </c>
       <c r="H340" s="2" t="n">
         <v>1431621</v>
@@ -16302,13 +16302,13 @@
         </is>
       </c>
       <c r="E343" s="4" t="n">
-        <v>2.7</v>
+        <v>1</v>
       </c>
       <c r="F343" s="5" t="n">
-        <v>80</v>
+        <v>1900</v>
       </c>
       <c r="G343" s="4" t="n">
-        <v>216</v>
+        <v>1900</v>
       </c>
       <c r="H343" s="2" t="n">
         <v>1431836</v>
@@ -16349,13 +16349,13 @@
         </is>
       </c>
       <c r="E344" s="4" t="n">
-        <v>1</v>
+        <v>2.7</v>
       </c>
       <c r="F344" s="5" t="n">
-        <v>1900</v>
+        <v>80</v>
       </c>
       <c r="G344" s="4" t="n">
-        <v>1900</v>
+        <v>216</v>
       </c>
       <c r="H344" s="2" t="n">
         <v>1431836</v>
@@ -16819,13 +16819,13 @@
         </is>
       </c>
       <c r="E354" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F354" s="5" t="n">
-        <v>3.45</v>
+        <v>28.9</v>
       </c>
       <c r="G354" s="4" t="n">
-        <v>6.9</v>
+        <v>115.6</v>
       </c>
       <c r="H354" s="2" t="n">
         <v>1432029</v>
@@ -16866,13 +16866,13 @@
         </is>
       </c>
       <c r="E355" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F355" s="5" t="n">
-        <v>28.9</v>
+        <v>3.45</v>
       </c>
       <c r="G355" s="4" t="n">
-        <v>115.6</v>
+        <v>6.9</v>
       </c>
       <c r="H355" s="2" t="n">
         <v>1432029</v>
@@ -16916,10 +16916,10 @@
         <v>15</v>
       </c>
       <c r="F356" s="5" t="n">
-        <v>3.99</v>
+        <v>1.5</v>
       </c>
       <c r="G356" s="4" t="n">
-        <v>59.85</v>
+        <v>22.5</v>
       </c>
       <c r="H356" s="2" t="n">
         <v>1432046</v>
@@ -16963,10 +16963,10 @@
         <v>15</v>
       </c>
       <c r="F357" s="5" t="n">
-        <v>1.5</v>
+        <v>3.99</v>
       </c>
       <c r="G357" s="4" t="n">
-        <v>22.5</v>
+        <v>59.85</v>
       </c>
       <c r="H357" s="2" t="n">
         <v>1432046</v>
@@ -17903,10 +17903,10 @@
         <v>1</v>
       </c>
       <c r="F377" s="5" t="n">
-        <v>5.28</v>
+        <v>6.63</v>
       </c>
       <c r="G377" s="4" t="n">
-        <v>5.28</v>
+        <v>6.63</v>
       </c>
       <c r="H377" s="2" t="n">
         <v>1437076</v>
@@ -17947,13 +17947,13 @@
         </is>
       </c>
       <c r="E378" s="4" t="n">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="F378" s="5" t="n">
-        <v>0.63</v>
+        <v>2.95</v>
       </c>
       <c r="G378" s="4" t="n">
-        <v>50.4</v>
+        <v>5.9</v>
       </c>
       <c r="H378" s="2" t="n">
         <v>1437076</v>
@@ -17994,13 +17994,13 @@
         </is>
       </c>
       <c r="E379" s="4" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="F379" s="5" t="n">
-        <v>4.12</v>
+        <v>1.95</v>
       </c>
       <c r="G379" s="4" t="n">
-        <v>8.24</v>
+        <v>58.5</v>
       </c>
       <c r="H379" s="2" t="n">
         <v>1437076</v>
@@ -18044,10 +18044,10 @@
         <v>1</v>
       </c>
       <c r="F380" s="5" t="n">
-        <v>5.62</v>
+        <v>5.28</v>
       </c>
       <c r="G380" s="4" t="n">
-        <v>5.62</v>
+        <v>5.28</v>
       </c>
       <c r="H380" s="2" t="n">
         <v>1437076</v>
@@ -18088,13 +18088,13 @@
         </is>
       </c>
       <c r="E381" s="4" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="F381" s="5" t="n">
-        <v>1.29</v>
+        <v>0.63</v>
       </c>
       <c r="G381" s="4" t="n">
-        <v>12.9</v>
+        <v>50.4</v>
       </c>
       <c r="H381" s="2" t="n">
         <v>1437076</v>
@@ -18135,13 +18135,13 @@
         </is>
       </c>
       <c r="E382" s="4" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="F382" s="5" t="n">
-        <v>2.53</v>
+        <v>4.12</v>
       </c>
       <c r="G382" s="4" t="n">
-        <v>253</v>
+        <v>8.24</v>
       </c>
       <c r="H382" s="2" t="n">
         <v>1437076</v>
@@ -18182,13 +18182,13 @@
         </is>
       </c>
       <c r="E383" s="4" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F383" s="5" t="n">
-        <v>2.53</v>
+        <v>5.62</v>
       </c>
       <c r="G383" s="4" t="n">
-        <v>253</v>
+        <v>5.62</v>
       </c>
       <c r="H383" s="2" t="n">
         <v>1437076</v>
@@ -18229,13 +18229,13 @@
         </is>
       </c>
       <c r="E384" s="4" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="F384" s="5" t="n">
-        <v>2.53</v>
+        <v>27.7</v>
       </c>
       <c r="G384" s="4" t="n">
-        <v>253</v>
+        <v>55.4</v>
       </c>
       <c r="H384" s="2" t="n">
         <v>1437076</v>
@@ -18276,13 +18276,13 @@
         </is>
       </c>
       <c r="E385" s="4" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="F385" s="5" t="n">
-        <v>4.16</v>
+        <v>1.29</v>
       </c>
       <c r="G385" s="4" t="n">
-        <v>416</v>
+        <v>12.9</v>
       </c>
       <c r="H385" s="2" t="n">
         <v>1437076</v>
@@ -18323,13 +18323,13 @@
         </is>
       </c>
       <c r="E386" s="4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F386" s="5" t="n">
-        <v>6.28</v>
+        <v>2.53</v>
       </c>
       <c r="G386" s="4" t="n">
-        <v>314</v>
+        <v>253</v>
       </c>
       <c r="H386" s="2" t="n">
         <v>1437076</v>
@@ -18370,13 +18370,13 @@
         </is>
       </c>
       <c r="E387" s="4" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F387" s="5" t="n">
-        <v>6.63</v>
+        <v>2.53</v>
       </c>
       <c r="G387" s="4" t="n">
-        <v>6.63</v>
+        <v>253</v>
       </c>
       <c r="H387" s="2" t="n">
         <v>1437076</v>
@@ -18417,13 +18417,13 @@
         </is>
       </c>
       <c r="E388" s="4" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="F388" s="5" t="n">
-        <v>8.81</v>
+        <v>2.53</v>
       </c>
       <c r="G388" s="4" t="n">
-        <v>17.62</v>
+        <v>253</v>
       </c>
       <c r="H388" s="2" t="n">
         <v>1437076</v>
@@ -18464,13 +18464,13 @@
         </is>
       </c>
       <c r="E389" s="4" t="n">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="F389" s="5" t="n">
-        <v>3.6</v>
+        <v>4.16</v>
       </c>
       <c r="G389" s="4" t="n">
-        <v>14.4</v>
+        <v>416</v>
       </c>
       <c r="H389" s="2" t="n">
         <v>1437076</v>
@@ -18511,13 +18511,13 @@
         </is>
       </c>
       <c r="E390" s="4" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F390" s="5" t="n">
-        <v>30.25</v>
+        <v>6.28</v>
       </c>
       <c r="G390" s="4" t="n">
-        <v>30.25</v>
+        <v>314</v>
       </c>
       <c r="H390" s="2" t="n">
         <v>1437076</v>
@@ -18558,13 +18558,13 @@
         </is>
       </c>
       <c r="E391" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F391" s="5" t="n">
-        <v>30.25</v>
+        <v>8.81</v>
       </c>
       <c r="G391" s="4" t="n">
-        <v>90.75</v>
+        <v>17.62</v>
       </c>
       <c r="H391" s="2" t="n">
         <v>1437076</v>
@@ -18605,13 +18605,13 @@
         </is>
       </c>
       <c r="E392" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F392" s="5" t="n">
-        <v>15.27</v>
+        <v>3.6</v>
       </c>
       <c r="G392" s="4" t="n">
-        <v>30.54</v>
+        <v>14.4</v>
       </c>
       <c r="H392" s="2" t="n">
         <v>1437076</v>
@@ -18652,13 +18652,13 @@
         </is>
       </c>
       <c r="E393" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F393" s="5" t="n">
-        <v>27.7</v>
+        <v>30.25</v>
       </c>
       <c r="G393" s="4" t="n">
-        <v>55.4</v>
+        <v>30.25</v>
       </c>
       <c r="H393" s="2" t="n">
         <v>1437076</v>
@@ -18699,13 +18699,13 @@
         </is>
       </c>
       <c r="E394" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F394" s="5" t="n">
-        <v>2.95</v>
+        <v>30.25</v>
       </c>
       <c r="G394" s="4" t="n">
-        <v>5.9</v>
+        <v>90.75</v>
       </c>
       <c r="H394" s="2" t="n">
         <v>1437076</v>
@@ -18746,13 +18746,13 @@
         </is>
       </c>
       <c r="E395" s="4" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="F395" s="5" t="n">
-        <v>1.95</v>
+        <v>15.27</v>
       </c>
       <c r="G395" s="4" t="n">
-        <v>58.5</v>
+        <v>30.54</v>
       </c>
       <c r="H395" s="2" t="n">
         <v>1437076</v>
@@ -18796,10 +18796,10 @@
         <v>80</v>
       </c>
       <c r="F396" s="5" t="n">
-        <v>0.19</v>
+        <v>0.86</v>
       </c>
       <c r="G396" s="4" t="n">
-        <v>15.2</v>
+        <v>68.8</v>
       </c>
       <c r="H396" s="2" t="n">
         <v>1437076</v>
@@ -18843,10 +18843,10 @@
         <v>80</v>
       </c>
       <c r="F397" s="5" t="n">
-        <v>0.86</v>
+        <v>0.19</v>
       </c>
       <c r="G397" s="4" t="n">
-        <v>68.8</v>
+        <v>15.2</v>
       </c>
       <c r="H397" s="2" t="n">
         <v>1437076</v>
@@ -19028,13 +19028,13 @@
         </is>
       </c>
       <c r="E401" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F401" s="5" t="n">
-        <v>6.75</v>
+        <v>8.5</v>
       </c>
       <c r="G401" s="4" t="n">
-        <v>27</v>
+        <v>25.5</v>
       </c>
       <c r="H401" s="2" t="n">
         <v>1437082</v>
@@ -19075,13 +19075,13 @@
         </is>
       </c>
       <c r="E402" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F402" s="5" t="n">
-        <v>8.5</v>
+        <v>6.75</v>
       </c>
       <c r="G402" s="4" t="n">
-        <v>25.5</v>
+        <v>27</v>
       </c>
       <c r="H402" s="2" t="n">
         <v>1437082</v>
@@ -19592,13 +19592,13 @@
         </is>
       </c>
       <c r="E413" s="4" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F413" s="5" t="n">
-        <v>0.37</v>
+        <v>2</v>
       </c>
       <c r="G413" s="4" t="n">
-        <v>9.25</v>
+        <v>100</v>
       </c>
       <c r="H413" s="2" t="n">
         <v>1442011</v>
@@ -19639,13 +19639,13 @@
         </is>
       </c>
       <c r="E414" s="4" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F414" s="5" t="n">
-        <v>0.3</v>
+        <v>0.49</v>
       </c>
       <c r="G414" s="4" t="n">
-        <v>30</v>
+        <v>24.5</v>
       </c>
       <c r="H414" s="2" t="n">
         <v>1442011</v>
@@ -19689,10 +19689,10 @@
         <v>50</v>
       </c>
       <c r="F415" s="5" t="n">
-        <v>0.3</v>
+        <v>0.22</v>
       </c>
       <c r="G415" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="H415" s="2" t="n">
         <v>1442011</v>
@@ -19736,10 +19736,10 @@
         <v>50</v>
       </c>
       <c r="F416" s="5" t="n">
-        <v>0.49</v>
+        <v>0.3</v>
       </c>
       <c r="G416" s="4" t="n">
-        <v>24.5</v>
+        <v>15</v>
       </c>
       <c r="H416" s="2" t="n">
         <v>1442011</v>
@@ -19780,13 +19780,13 @@
         </is>
       </c>
       <c r="E417" s="4" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="F417" s="5" t="n">
-        <v>2</v>
+        <v>0.37</v>
       </c>
       <c r="G417" s="4" t="n">
-        <v>100</v>
+        <v>9.25</v>
       </c>
       <c r="H417" s="2" t="n">
         <v>1442011</v>
@@ -19827,13 +19827,13 @@
         </is>
       </c>
       <c r="E418" s="4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F418" s="5" t="n">
-        <v>0.22</v>
+        <v>0.3</v>
       </c>
       <c r="G418" s="4" t="n">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="H418" s="2" t="n">
         <v>1442011</v>
@@ -19924,10 +19924,10 @@
         <v>1</v>
       </c>
       <c r="F420" s="5" t="n">
-        <v>23.36</v>
+        <v>32.64</v>
       </c>
       <c r="G420" s="4" t="n">
-        <v>23.36</v>
+        <v>32.64</v>
       </c>
       <c r="H420" s="2" t="n">
         <v>1442024</v>
@@ -20018,10 +20018,10 @@
         <v>1</v>
       </c>
       <c r="F422" s="5" t="n">
-        <v>32.64</v>
+        <v>23.36</v>
       </c>
       <c r="G422" s="4" t="n">
-        <v>32.64</v>
+        <v>23.36</v>
       </c>
       <c r="H422" s="2" t="n">
         <v>1442024</v>
@@ -20159,10 +20159,10 @@
         <v>0.05</v>
       </c>
       <c r="F425" s="5" t="n">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="G425" s="4" t="n">
-        <v>5</v>
+        <v>2.25</v>
       </c>
       <c r="H425" s="2" t="n">
         <v>1442618</v>
@@ -20206,10 +20206,10 @@
         <v>0.05</v>
       </c>
       <c r="F426" s="5" t="n">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="G426" s="4" t="n">
-        <v>2.25</v>
+        <v>5</v>
       </c>
       <c r="H426" s="2" t="n">
         <v>1442618</v>
@@ -20485,13 +20485,13 @@
         </is>
       </c>
       <c r="E432" s="4" t="n">
-        <v>0.2</v>
+        <v>0.06</v>
       </c>
       <c r="F432" s="5" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="G432" s="4" t="n">
-        <v>6</v>
+        <v>5.4</v>
       </c>
       <c r="H432" s="2" t="n">
         <v>1442618</v>
@@ -20535,10 +20535,10 @@
         <v>0.08</v>
       </c>
       <c r="F433" s="5" t="n">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="G433" s="4" t="n">
-        <v>2.8</v>
+        <v>7.2</v>
       </c>
       <c r="H433" s="2" t="n">
         <v>1442618</v>
@@ -20579,13 +20579,13 @@
         </is>
       </c>
       <c r="E434" s="4" t="n">
-        <v>0.08</v>
+        <v>0.25</v>
       </c>
       <c r="F434" s="5" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G434" s="4" t="n">
-        <v>1.6</v>
+        <v>5.5</v>
       </c>
       <c r="H434" s="2" t="n">
         <v>1442618</v>
@@ -20626,13 +20626,13 @@
         </is>
       </c>
       <c r="E435" s="4" t="n">
-        <v>0.08</v>
+        <v>0.25</v>
       </c>
       <c r="F435" s="5" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G435" s="4" t="n">
-        <v>0.48</v>
+        <v>2.5</v>
       </c>
       <c r="H435" s="2" t="n">
         <v>1442618</v>
@@ -20673,13 +20673,13 @@
         </is>
       </c>
       <c r="E436" s="4" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="F436" s="5" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="G436" s="4" t="n">
-        <v>1.8</v>
+        <v>5.6</v>
       </c>
       <c r="H436" s="2" t="n">
         <v>1442618</v>
@@ -20720,13 +20720,13 @@
         </is>
       </c>
       <c r="E437" s="4" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="F437" s="5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G437" s="4" t="n">
-        <v>8</v>
+        <v>5.6</v>
       </c>
       <c r="H437" s="2" t="n">
         <v>1442618</v>
@@ -20767,13 +20767,13 @@
         </is>
       </c>
       <c r="E438" s="4" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="F438" s="5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="G438" s="4" t="n">
-        <v>5.6</v>
+        <v>8</v>
       </c>
       <c r="H438" s="2" t="n">
         <v>1442618</v>
@@ -20814,13 +20814,13 @@
         </is>
       </c>
       <c r="E439" s="4" t="n">
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
       <c r="F439" s="5" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="G439" s="4" t="n">
-        <v>5.6</v>
+        <v>6</v>
       </c>
       <c r="H439" s="2" t="n">
         <v>1442618</v>
@@ -20861,13 +20861,13 @@
         </is>
       </c>
       <c r="E440" s="4" t="n">
-        <v>0.25</v>
+        <v>0.08</v>
       </c>
       <c r="F440" s="5" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="G440" s="4" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="H440" s="2" t="n">
         <v>1442618</v>
@@ -20908,13 +20908,13 @@
         </is>
       </c>
       <c r="E441" s="4" t="n">
-        <v>0.25</v>
+        <v>0.08</v>
       </c>
       <c r="F441" s="5" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G441" s="4" t="n">
-        <v>5.5</v>
+        <v>1.6</v>
       </c>
       <c r="H441" s="2" t="n">
         <v>1442618</v>
@@ -20955,13 +20955,13 @@
         </is>
       </c>
       <c r="E442" s="4" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="F442" s="5" t="n">
-        <v>90</v>
+        <v>6</v>
       </c>
       <c r="G442" s="4" t="n">
-        <v>5.4</v>
+        <v>0.48</v>
       </c>
       <c r="H442" s="2" t="n">
         <v>1442618</v>
@@ -21002,13 +21002,13 @@
         </is>
       </c>
       <c r="E443" s="4" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="F443" s="5" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="G443" s="4" t="n">
-        <v>7.2</v>
+        <v>1.8</v>
       </c>
       <c r="H443" s="2" t="n">
         <v>1442618</v>
@@ -22788,13 +22788,13 @@
         </is>
       </c>
       <c r="E481" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F481" s="5" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G481" s="4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H481" s="2" t="n">
         <v>1461456</v>
@@ -22835,13 +22835,13 @@
         </is>
       </c>
       <c r="E482" s="4" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="F482" s="5" t="n">
-        <v>2.5</v>
+        <v>11</v>
       </c>
       <c r="G482" s="4" t="n">
-        <v>47.5</v>
+        <v>11</v>
       </c>
       <c r="H482" s="2" t="n">
         <v>1461456</v>
@@ -22882,13 +22882,13 @@
         </is>
       </c>
       <c r="E483" s="4" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="F483" s="5" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="G483" s="4" t="n">
-        <v>14</v>
+        <v>47.5</v>
       </c>
       <c r="H483" s="2" t="n">
         <v>1461456</v>
@@ -25984,13 +25984,13 @@
         </is>
       </c>
       <c r="E549" s="4" t="n">
-        <v>0.8</v>
+        <v>2</v>
       </c>
       <c r="F549" s="5" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G549" s="4" t="n">
-        <v>12.8</v>
+        <v>28</v>
       </c>
       <c r="H549" s="2" t="n">
         <v>1480786</v>
@@ -26031,13 +26031,13 @@
         </is>
       </c>
       <c r="E550" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F550" s="5" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="G550" s="4" t="n">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H550" s="2" t="n">
         <v>1480786</v>
@@ -26125,13 +26125,13 @@
         </is>
       </c>
       <c r="E552" s="4" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="F552" s="5" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="G552" s="4" t="n">
-        <v>12</v>
+        <v>6.25</v>
       </c>
       <c r="H552" s="2" t="n">
         <v>1480786</v>
@@ -26172,13 +26172,13 @@
         </is>
       </c>
       <c r="E553" s="4" t="n">
-        <v>2</v>
+        <v>0.8</v>
       </c>
       <c r="F553" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G553" s="4" t="n">
-        <v>30</v>
+        <v>12.8</v>
       </c>
       <c r="H553" s="2" t="n">
         <v>1480786</v>
@@ -26219,13 +26219,13 @@
         </is>
       </c>
       <c r="E554" s="4" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="F554" s="5" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G554" s="4" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H554" s="2" t="n">
         <v>1480786</v>
@@ -26266,13 +26266,13 @@
         </is>
       </c>
       <c r="E555" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F555" s="5" t="n">
         <v>15</v>
       </c>
       <c r="G555" s="4" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H555" s="2" t="n">
         <v>1480786</v>
@@ -26313,13 +26313,13 @@
         </is>
       </c>
       <c r="E556" s="4" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F556" s="5" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G556" s="4" t="n">
-        <v>6.25</v>
+        <v>15</v>
       </c>
       <c r="H556" s="2" t="n">
         <v>1480786</v>
@@ -26360,13 +26360,13 @@
         </is>
       </c>
       <c r="E557" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F557" s="5" t="n">
-        <v>8.81</v>
+        <v>0.33</v>
       </c>
       <c r="G557" s="4" t="n">
-        <v>17.62</v>
+        <v>2.64</v>
       </c>
       <c r="H557" s="2" t="n">
         <v>1480796</v>
@@ -26407,13 +26407,13 @@
         </is>
       </c>
       <c r="E558" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F558" s="5" t="n">
-        <v>0.33</v>
+        <v>8.81</v>
       </c>
       <c r="G558" s="4" t="n">
-        <v>2.64</v>
+        <v>17.62</v>
       </c>
       <c r="H558" s="2" t="n">
         <v>1480796</v>
@@ -26454,13 +26454,13 @@
         </is>
       </c>
       <c r="E559" s="4" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F559" s="5" t="n">
-        <v>14.06</v>
+        <v>1.89</v>
       </c>
       <c r="G559" s="4" t="n">
-        <v>14.06</v>
+        <v>37.8</v>
       </c>
       <c r="H559" s="2" t="n">
         <v>1480796</v>
@@ -26501,13 +26501,13 @@
         </is>
       </c>
       <c r="E560" s="4" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="F560" s="5" t="n">
-        <v>1.89</v>
+        <v>2.95</v>
       </c>
       <c r="G560" s="4" t="n">
-        <v>37.8</v>
+        <v>5.9</v>
       </c>
       <c r="H560" s="2" t="n">
         <v>1480796</v>
@@ -26548,13 +26548,13 @@
         </is>
       </c>
       <c r="E561" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F561" s="5" t="n">
-        <v>2.95</v>
+        <v>14.06</v>
       </c>
       <c r="G561" s="4" t="n">
-        <v>5.9</v>
+        <v>14.06</v>
       </c>
       <c r="H561" s="2" t="n">
         <v>1480796</v>
@@ -26974,10 +26974,10 @@
         <v>1</v>
       </c>
       <c r="F570" s="5" t="n">
-        <v>6.08</v>
+        <v>5.74</v>
       </c>
       <c r="G570" s="4" t="n">
-        <v>6.08</v>
+        <v>5.74</v>
       </c>
       <c r="H570" s="2" t="n">
         <v>1482331</v>
@@ -27021,10 +27021,10 @@
         <v>1</v>
       </c>
       <c r="F571" s="5" t="n">
-        <v>5.74</v>
+        <v>6.08</v>
       </c>
       <c r="G571" s="4" t="n">
-        <v>5.74</v>
+        <v>6.08</v>
       </c>
       <c r="H571" s="2" t="n">
         <v>1482331</v>
@@ -27068,10 +27068,10 @@
         <v>1</v>
       </c>
       <c r="F572" s="5" t="n">
-        <v>31.33</v>
+        <v>117.18</v>
       </c>
       <c r="G572" s="4" t="n">
-        <v>31.33</v>
+        <v>117.18</v>
       </c>
       <c r="H572" s="2" t="n">
         <v>1482331</v>
@@ -27115,10 +27115,10 @@
         <v>1</v>
       </c>
       <c r="F573" s="5" t="n">
-        <v>6.16</v>
+        <v>55.88</v>
       </c>
       <c r="G573" s="4" t="n">
-        <v>6.16</v>
+        <v>55.88</v>
       </c>
       <c r="H573" s="2" t="n">
         <v>1482331</v>
@@ -27209,10 +27209,10 @@
         <v>1</v>
       </c>
       <c r="F575" s="5" t="n">
-        <v>55.88</v>
+        <v>6.16</v>
       </c>
       <c r="G575" s="4" t="n">
-        <v>55.88</v>
+        <v>6.16</v>
       </c>
       <c r="H575" s="2" t="n">
         <v>1482331</v>
@@ -27256,10 +27256,10 @@
         <v>1</v>
       </c>
       <c r="F576" s="5" t="n">
-        <v>117.18</v>
+        <v>31.33</v>
       </c>
       <c r="G576" s="4" t="n">
-        <v>117.18</v>
+        <v>31.33</v>
       </c>
       <c r="H576" s="2" t="n">
         <v>1482331</v>
@@ -27394,13 +27394,13 @@
         </is>
       </c>
       <c r="E579" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F579" s="5" t="n">
-        <v>2.6</v>
+        <v>7</v>
       </c>
       <c r="G579" s="4" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="H579" s="2" t="n">
         <v>1482337</v>
@@ -27441,13 +27441,13 @@
         </is>
       </c>
       <c r="E580" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F580" s="5" t="n">
-        <v>2.6</v>
+        <v>9</v>
       </c>
       <c r="G580" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="H580" s="2" t="n">
         <v>1482337</v>
@@ -27535,13 +27535,13 @@
         </is>
       </c>
       <c r="E582" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F582" s="5" t="n">
-        <v>9</v>
+        <v>2.6</v>
       </c>
       <c r="G582" s="4" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H582" s="2" t="n">
         <v>1482337</v>
@@ -27582,13 +27582,13 @@
         </is>
       </c>
       <c r="E583" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F583" s="5" t="n">
-        <v>7</v>
+        <v>2.6</v>
       </c>
       <c r="G583" s="4" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="H583" s="2" t="n">
         <v>1482337</v>
@@ -28619,10 +28619,10 @@
         <v>1</v>
       </c>
       <c r="F605" s="5" t="n">
-        <v>165</v>
+        <v>195</v>
       </c>
       <c r="G605" s="4" t="n">
-        <v>165</v>
+        <v>195</v>
       </c>
       <c r="H605" s="2" t="n">
         <v>1490619</v>
@@ -28666,10 +28666,10 @@
         <v>1</v>
       </c>
       <c r="F606" s="5" t="n">
-        <v>195</v>
+        <v>230</v>
       </c>
       <c r="G606" s="4" t="n">
-        <v>195</v>
+        <v>230</v>
       </c>
       <c r="H606" s="2" t="n">
         <v>1490619</v>
@@ -28713,10 +28713,10 @@
         <v>1</v>
       </c>
       <c r="F607" s="5" t="n">
-        <v>230</v>
+        <v>165</v>
       </c>
       <c r="G607" s="4" t="n">
-        <v>230</v>
+        <v>165</v>
       </c>
       <c r="H607" s="2" t="n">
         <v>1490619</v>
@@ -28851,13 +28851,13 @@
         </is>
       </c>
       <c r="E610" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F610" s="5" t="n">
-        <v>41.71</v>
+        <v>6.6</v>
       </c>
       <c r="G610" s="4" t="n">
-        <v>83.42</v>
+        <v>19.8</v>
       </c>
       <c r="H610" s="2" t="n">
         <v>1490652</v>
@@ -28898,13 +28898,13 @@
         </is>
       </c>
       <c r="E611" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F611" s="5" t="n">
-        <v>49.9</v>
+        <v>55.99</v>
       </c>
       <c r="G611" s="4" t="n">
-        <v>49.9</v>
+        <v>167.97</v>
       </c>
       <c r="H611" s="2" t="n">
         <v>1490652</v>
@@ -28948,10 +28948,10 @@
         <v>10</v>
       </c>
       <c r="F612" s="5" t="n">
-        <v>0.86</v>
+        <v>0.48</v>
       </c>
       <c r="G612" s="4" t="n">
-        <v>8.6</v>
+        <v>4.8</v>
       </c>
       <c r="H612" s="2" t="n">
         <v>1490652</v>
@@ -28992,13 +28992,13 @@
         </is>
       </c>
       <c r="E613" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F613" s="5" t="n">
-        <v>55.99</v>
+        <v>0.86</v>
       </c>
       <c r="G613" s="4" t="n">
-        <v>167.97</v>
+        <v>8.6</v>
       </c>
       <c r="H613" s="2" t="n">
         <v>1490652</v>
@@ -29039,13 +29039,13 @@
         </is>
       </c>
       <c r="E614" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F614" s="5" t="n">
-        <v>6.6</v>
+        <v>17.52</v>
       </c>
       <c r="G614" s="4" t="n">
-        <v>19.8</v>
+        <v>70.08</v>
       </c>
       <c r="H614" s="2" t="n">
         <v>1490652</v>
@@ -29086,13 +29086,13 @@
         </is>
       </c>
       <c r="E615" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F615" s="5" t="n">
-        <v>17.52</v>
+        <v>41.71</v>
       </c>
       <c r="G615" s="4" t="n">
-        <v>70.08</v>
+        <v>83.42</v>
       </c>
       <c r="H615" s="2" t="n">
         <v>1490652</v>
@@ -29133,13 +29133,13 @@
         </is>
       </c>
       <c r="E616" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F616" s="5" t="n">
-        <v>0.48</v>
+        <v>49.9</v>
       </c>
       <c r="G616" s="4" t="n">
-        <v>4.8</v>
+        <v>49.9</v>
       </c>
       <c r="H616" s="2" t="n">
         <v>1490652</v>
@@ -29180,13 +29180,13 @@
         </is>
       </c>
       <c r="E617" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F617" s="5" t="n">
-        <v>34.82</v>
+        <v>2.84</v>
       </c>
       <c r="G617" s="4" t="n">
-        <v>34.82</v>
+        <v>28.4</v>
       </c>
       <c r="H617" s="2" t="n">
         <v>1490652</v>
@@ -29227,13 +29227,13 @@
         </is>
       </c>
       <c r="E618" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F618" s="5" t="n">
-        <v>2.84</v>
+        <v>34.82</v>
       </c>
       <c r="G618" s="4" t="n">
-        <v>28.4</v>
+        <v>34.82</v>
       </c>
       <c r="H618" s="2" t="n">
         <v>1490652</v>
@@ -29368,13 +29368,13 @@
         </is>
       </c>
       <c r="E621" s="4" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="F621" s="5" t="n">
-        <v>26.31</v>
+        <v>3.76</v>
       </c>
       <c r="G621" s="4" t="n">
-        <v>52.62</v>
+        <v>75.2</v>
       </c>
       <c r="H621" s="2" t="n">
         <v>1492428</v>
@@ -29509,13 +29509,13 @@
         </is>
       </c>
       <c r="E624" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F624" s="5" t="n">
-        <v>4.18</v>
+        <v>26.31</v>
       </c>
       <c r="G624" s="4" t="n">
-        <v>50.16</v>
+        <v>52.62</v>
       </c>
       <c r="H624" s="2" t="n">
         <v>1492428</v>
@@ -29556,13 +29556,13 @@
         </is>
       </c>
       <c r="E625" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F625" s="5" t="n">
-        <v>5.62</v>
+        <v>4.18</v>
       </c>
       <c r="G625" s="4" t="n">
-        <v>11.24</v>
+        <v>50.16</v>
       </c>
       <c r="H625" s="2" t="n">
         <v>1492428</v>
@@ -29603,13 +29603,13 @@
         </is>
       </c>
       <c r="E626" s="4" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="F626" s="5" t="n">
-        <v>3.76</v>
+        <v>5.62</v>
       </c>
       <c r="G626" s="4" t="n">
-        <v>75.2</v>
+        <v>11.24</v>
       </c>
       <c r="H626" s="2" t="n">
         <v>1492428</v>
@@ -29885,13 +29885,13 @@
         </is>
       </c>
       <c r="E632" s="4" t="n">
-        <v>0.1</v>
+        <v>2</v>
       </c>
       <c r="F632" s="5" t="n">
-        <v>75</v>
+        <v>22</v>
       </c>
       <c r="G632" s="4" t="n">
-        <v>7.5</v>
+        <v>44</v>
       </c>
       <c r="H632" s="2" t="n">
         <v>1493814</v>
@@ -29932,13 +29932,13 @@
         </is>
       </c>
       <c r="E633" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F633" s="5" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="G633" s="4" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="H633" s="2" t="n">
         <v>1493814</v>
@@ -29979,13 +29979,13 @@
         </is>
       </c>
       <c r="E634" s="4" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="F634" s="5" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="G634" s="4" t="n">
-        <v>40</v>
+        <v>7.5</v>
       </c>
       <c r="H634" s="2" t="n">
         <v>1493814</v>
@@ -30308,13 +30308,13 @@
         </is>
       </c>
       <c r="E641" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F641" s="5" t="n">
-        <v>1</v>
+        <v>23.95</v>
       </c>
       <c r="G641" s="4" t="n">
-        <v>10</v>
+        <v>23.95</v>
       </c>
       <c r="H641" s="2" t="n">
         <v>1497640</v>
@@ -30449,13 +30449,13 @@
         </is>
       </c>
       <c r="E644" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F644" s="5" t="n">
-        <v>23.95</v>
+        <v>1</v>
       </c>
       <c r="G644" s="4" t="n">
-        <v>23.95</v>
+        <v>10</v>
       </c>
       <c r="H644" s="2" t="n">
         <v>1497640</v>
@@ -31721,10 +31721,10 @@
         <v>2</v>
       </c>
       <c r="F671" s="5" t="n">
-        <v>1.01</v>
+        <v>30</v>
       </c>
       <c r="G671" s="4" t="n">
-        <v>2.02</v>
+        <v>60</v>
       </c>
       <c r="H671" s="2" t="n">
         <v>1503029</v>
@@ -31815,10 +31815,10 @@
         <v>2</v>
       </c>
       <c r="F673" s="5" t="n">
-        <v>30</v>
+        <v>2.03</v>
       </c>
       <c r="G673" s="4" t="n">
-        <v>60</v>
+        <v>4.06</v>
       </c>
       <c r="H673" s="2" t="n">
         <v>1503029</v>
@@ -31859,13 +31859,13 @@
         </is>
       </c>
       <c r="E674" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F674" s="5" t="n">
-        <v>2.03</v>
+        <v>5.39</v>
       </c>
       <c r="G674" s="4" t="n">
-        <v>4.06</v>
+        <v>5.39</v>
       </c>
       <c r="H674" s="2" t="n">
         <v>1503029</v>
@@ -31906,13 +31906,13 @@
         </is>
       </c>
       <c r="E675" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F675" s="5" t="n">
-        <v>30.63</v>
+        <v>1.01</v>
       </c>
       <c r="G675" s="4" t="n">
-        <v>30.63</v>
+        <v>2.02</v>
       </c>
       <c r="H675" s="2" t="n">
         <v>1503029</v>
@@ -31956,10 +31956,10 @@
         <v>1</v>
       </c>
       <c r="F676" s="5" t="n">
-        <v>5.39</v>
+        <v>30.63</v>
       </c>
       <c r="G676" s="4" t="n">
-        <v>5.39</v>
+        <v>30.63</v>
       </c>
       <c r="H676" s="2" t="n">
         <v>1503029</v>
@@ -32188,13 +32188,13 @@
         </is>
       </c>
       <c r="E681" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F681" s="5" t="n">
-        <v>6.01</v>
+        <v>2.1</v>
       </c>
       <c r="G681" s="4" t="n">
-        <v>12.02</v>
+        <v>8.4</v>
       </c>
       <c r="H681" s="2" t="n">
         <v>1503353</v>
@@ -32235,13 +32235,13 @@
         </is>
       </c>
       <c r="E682" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F682" s="5" t="n">
-        <v>2.1</v>
+        <v>6.01</v>
       </c>
       <c r="G682" s="4" t="n">
-        <v>8.4</v>
+        <v>12.02</v>
       </c>
       <c r="H682" s="2" t="n">
         <v>1503353</v>
@@ -32379,10 +32379,10 @@
         <v>1</v>
       </c>
       <c r="F685" s="5" t="n">
-        <v>14.02</v>
+        <v>13.6</v>
       </c>
       <c r="G685" s="4" t="n">
-        <v>14.02</v>
+        <v>13.6</v>
       </c>
       <c r="H685" s="2" t="n">
         <v>1503440</v>
@@ -32473,10 +32473,10 @@
         <v>1</v>
       </c>
       <c r="F687" s="5" t="n">
-        <v>13.6</v>
+        <v>14.02</v>
       </c>
       <c r="G687" s="4" t="n">
-        <v>13.6</v>
+        <v>14.02</v>
       </c>
       <c r="H687" s="2" t="n">
         <v>1503440</v>
@@ -33222,13 +33222,13 @@
         </is>
       </c>
       <c r="E703" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F703" s="5" t="n">
-        <v>27.65</v>
+        <v>2.29</v>
       </c>
       <c r="G703" s="4" t="n">
-        <v>27.65</v>
+        <v>4.58</v>
       </c>
       <c r="H703" s="2" t="n">
         <v>1512391</v>
@@ -33272,10 +33272,10 @@
         <v>2</v>
       </c>
       <c r="F704" s="5" t="n">
-        <v>2.88</v>
+        <v>2.38</v>
       </c>
       <c r="G704" s="4" t="n">
-        <v>5.76</v>
+        <v>4.76</v>
       </c>
       <c r="H704" s="2" t="n">
         <v>1512391</v>
@@ -33316,13 +33316,13 @@
         </is>
       </c>
       <c r="E705" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F705" s="5" t="n">
-        <v>2.29</v>
+        <v>27.65</v>
       </c>
       <c r="G705" s="4" t="n">
-        <v>4.58</v>
+        <v>27.65</v>
       </c>
       <c r="H705" s="2" t="n">
         <v>1512391</v>
@@ -33366,10 +33366,10 @@
         <v>2</v>
       </c>
       <c r="F706" s="5" t="n">
-        <v>2.38</v>
+        <v>2.88</v>
       </c>
       <c r="G706" s="4" t="n">
-        <v>4.76</v>
+        <v>5.76</v>
       </c>
       <c r="H706" s="2" t="n">
         <v>1512391</v>
@@ -33413,10 +33413,10 @@
         <v>1</v>
       </c>
       <c r="F707" s="5" t="n">
-        <v>15.25</v>
+        <v>12.25</v>
       </c>
       <c r="G707" s="4" t="n">
-        <v>15.25</v>
+        <v>12.25</v>
       </c>
       <c r="H707" s="2" t="n">
         <v>1512391</v>
@@ -33507,10 +33507,10 @@
         <v>1</v>
       </c>
       <c r="F709" s="5" t="n">
-        <v>12.25</v>
+        <v>15.25</v>
       </c>
       <c r="G709" s="4" t="n">
-        <v>12.25</v>
+        <v>15.25</v>
       </c>
       <c r="H709" s="2" t="n">
         <v>1512391</v>
@@ -33601,10 +33601,10 @@
         <v>15</v>
       </c>
       <c r="F711" s="5" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="G711" s="4" t="n">
-        <v>12</v>
+        <v>4.5</v>
       </c>
       <c r="H711" s="2" t="n">
         <v>1512750</v>
@@ -33648,10 +33648,10 @@
         <v>15</v>
       </c>
       <c r="F712" s="5" t="n">
-        <v>0.3</v>
+        <v>0.17</v>
       </c>
       <c r="G712" s="4" t="n">
-        <v>4.5</v>
+        <v>2.55</v>
       </c>
       <c r="H712" s="2" t="n">
         <v>1512750</v>
@@ -33692,13 +33692,13 @@
         </is>
       </c>
       <c r="E713" s="4" t="n">
-        <v>15</v>
+        <v>300</v>
       </c>
       <c r="F713" s="5" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="G713" s="4" t="n">
-        <v>2.55</v>
+        <v>45</v>
       </c>
       <c r="H713" s="2" t="n">
         <v>1512750</v>
@@ -33739,13 +33739,13 @@
         </is>
       </c>
       <c r="E714" s="4" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F714" s="5" t="n">
         <v>0.15</v>
       </c>
       <c r="G714" s="4" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="H714" s="2" t="n">
         <v>1512750</v>
@@ -33786,13 +33786,13 @@
         </is>
       </c>
       <c r="E715" s="4" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="F715" s="5" t="n">
-        <v>0.15</v>
+        <v>0.8</v>
       </c>
       <c r="G715" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="H715" s="2" t="n">
         <v>1512750</v>
@@ -33974,13 +33974,13 @@
         </is>
       </c>
       <c r="E719" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F719" s="5" t="n">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="G719" s="4" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="H719" s="2" t="n">
         <v>1513521</v>
@@ -34024,10 +34024,10 @@
         <v>1</v>
       </c>
       <c r="F720" s="5" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="G720" s="4" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="H720" s="2" t="n">
         <v>1513521</v>
@@ -34068,13 +34068,13 @@
         </is>
       </c>
       <c r="E721" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F721" s="5" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G721" s="4" t="n">
-        <v>25</v>
+        <v>170</v>
       </c>
       <c r="H721" s="2" t="n">
         <v>1513521</v>
@@ -34165,10 +34165,10 @@
         <v>1</v>
       </c>
       <c r="F723" s="5" t="n">
-        <v>192.5</v>
+        <v>197.5</v>
       </c>
       <c r="G723" s="4" t="n">
-        <v>192.5</v>
+        <v>197.5</v>
       </c>
       <c r="H723" s="2" t="n">
         <v>1513541</v>
@@ -34212,10 +34212,10 @@
         <v>1</v>
       </c>
       <c r="F724" s="5" t="n">
-        <v>197.5</v>
+        <v>192.5</v>
       </c>
       <c r="G724" s="4" t="n">
-        <v>197.5</v>
+        <v>192.5</v>
       </c>
       <c r="H724" s="2" t="n">
         <v>1513541</v>
@@ -34444,13 +34444,13 @@
         </is>
       </c>
       <c r="E729" s="4" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="F729" s="5" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G729" s="4" t="n">
-        <v>750</v>
+        <v>2000</v>
       </c>
       <c r="H729" s="2" t="n">
         <v>1513779</v>
@@ -34491,13 +34491,13 @@
         </is>
       </c>
       <c r="E730" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F730" s="5" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="G730" s="4" t="n">
-        <v>1000</v>
+        <v>750</v>
       </c>
       <c r="H730" s="2" t="n">
         <v>1513779</v>
@@ -34585,13 +34585,13 @@
         </is>
       </c>
       <c r="E732" s="4" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F732" s="5" t="n">
         <v>100</v>
       </c>
       <c r="G732" s="4" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="H732" s="2" t="n">
         <v>1513779</v>
@@ -34679,13 +34679,13 @@
         </is>
       </c>
       <c r="E734" s="4" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F734" s="5" t="n">
-        <v>5.57</v>
+        <v>4.05</v>
       </c>
       <c r="G734" s="4" t="n">
-        <v>66.84</v>
+        <v>4.05</v>
       </c>
       <c r="H734" s="2" t="n">
         <v>1513837</v>
@@ -34773,13 +34773,13 @@
         </is>
       </c>
       <c r="E736" s="4" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F736" s="5" t="n">
-        <v>4.05</v>
+        <v>5.57</v>
       </c>
       <c r="G736" s="4" t="n">
-        <v>4.05</v>
+        <v>66.84</v>
       </c>
       <c r="H736" s="2" t="n">
         <v>1513837</v>
@@ -35481,10 +35481,10 @@
         <v>0.04</v>
       </c>
       <c r="F751" s="5" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="G751" s="4" t="n">
-        <v>1.4</v>
+        <v>2.4</v>
       </c>
       <c r="H751" s="2" t="n">
         <v>1517956</v>
@@ -35572,13 +35572,13 @@
         </is>
       </c>
       <c r="E753" s="4" t="n">
-        <v>4</v>
+        <v>0.04</v>
       </c>
       <c r="F753" s="5" t="n">
-        <v>95</v>
+        <v>5</v>
       </c>
       <c r="G753" s="4" t="n">
-        <v>380</v>
+        <v>0.2</v>
       </c>
       <c r="H753" s="2" t="n">
         <v>1517956</v>
@@ -35619,13 +35619,13 @@
         </is>
       </c>
       <c r="E754" s="4" t="n">
-        <v>0.04</v>
+        <v>4</v>
       </c>
       <c r="F754" s="5" t="n">
-        <v>60</v>
+        <v>95</v>
       </c>
       <c r="G754" s="4" t="n">
-        <v>2.4</v>
+        <v>380</v>
       </c>
       <c r="H754" s="2" t="n">
         <v>1517956</v>
@@ -35666,13 +35666,13 @@
         </is>
       </c>
       <c r="E755" s="4" t="n">
-        <v>4</v>
+        <v>0.04</v>
       </c>
       <c r="F755" s="5" t="n">
-        <v>0.75</v>
+        <v>35</v>
       </c>
       <c r="G755" s="4" t="n">
-        <v>3</v>
+        <v>1.4</v>
       </c>
       <c r="H755" s="2" t="n">
         <v>1517956</v>
@@ -35713,13 +35713,13 @@
         </is>
       </c>
       <c r="E756" s="4" t="n">
-        <v>0.04</v>
+        <v>4</v>
       </c>
       <c r="F756" s="5" t="n">
-        <v>25</v>
+        <v>0.75</v>
       </c>
       <c r="G756" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H756" s="2" t="n">
         <v>1517956</v>
@@ -35763,10 +35763,10 @@
         <v>0.04</v>
       </c>
       <c r="F757" s="5" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="G757" s="4" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="H757" s="2" t="n">
         <v>1517956</v>
@@ -36280,10 +36280,10 @@
         <v>1</v>
       </c>
       <c r="F768" s="5" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G768" s="4" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H768" s="2" t="n">
         <v>1518833</v>
@@ -36327,10 +36327,10 @@
         <v>1</v>
       </c>
       <c r="F769" s="5" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G769" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H769" s="2" t="n">
         <v>1518833</v>
@@ -36374,10 +36374,10 @@
         <v>1</v>
       </c>
       <c r="F770" s="5" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G770" s="4" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H770" s="2" t="n">
         <v>1518833</v>
@@ -36421,10 +36421,10 @@
         <v>1</v>
       </c>
       <c r="F771" s="5" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G771" s="4" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H771" s="2" t="n">
         <v>1518833</v>
@@ -36559,13 +36559,13 @@
         </is>
       </c>
       <c r="E774" s="4" t="n">
-        <v>1.5</v>
+        <v>0.08</v>
       </c>
       <c r="F774" s="5" t="n">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="G774" s="4" t="n">
-        <v>87</v>
+        <v>1.6</v>
       </c>
       <c r="H774" s="2" t="n">
         <v>1520281</v>
@@ -36606,13 +36606,13 @@
         </is>
       </c>
       <c r="E775" s="4" t="n">
-        <v>0.08</v>
+        <v>2</v>
       </c>
       <c r="F775" s="5" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="G775" s="4" t="n">
-        <v>1.6</v>
+        <v>22</v>
       </c>
       <c r="H775" s="2" t="n">
         <v>1520281</v>
@@ -36653,13 +36653,13 @@
         </is>
       </c>
       <c r="E776" s="4" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="F776" s="5" t="n">
-        <v>11</v>
+        <v>58</v>
       </c>
       <c r="G776" s="4" t="n">
-        <v>33</v>
+        <v>87</v>
       </c>
       <c r="H776" s="2" t="n">
         <v>1520281</v>
@@ -36700,13 +36700,13 @@
         </is>
       </c>
       <c r="E777" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F777" s="5" t="n">
         <v>11</v>
       </c>
       <c r="G777" s="4" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="H777" s="2" t="n">
         <v>1520281</v>
@@ -37076,13 +37076,13 @@
         </is>
       </c>
       <c r="E785" s="4" t="n">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="F785" s="5" t="n">
-        <v>127.6</v>
+        <v>9.1</v>
       </c>
       <c r="G785" s="4" t="n">
-        <v>4593.6</v>
+        <v>127.4</v>
       </c>
       <c r="H785" s="2" t="n">
         <v>1522616</v>
@@ -37123,13 +37123,13 @@
         </is>
       </c>
       <c r="E786" s="4" t="n">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F786" s="5" t="n">
-        <v>9.1</v>
+        <v>54.3</v>
       </c>
       <c r="G786" s="4" t="n">
-        <v>127.4</v>
+        <v>2009.1</v>
       </c>
       <c r="H786" s="2" t="n">
         <v>1522616</v>
@@ -37170,13 +37170,13 @@
         </is>
       </c>
       <c r="E787" s="4" t="n">
-        <v>37</v>
+        <v>69</v>
       </c>
       <c r="F787" s="5" t="n">
         <v>54.3</v>
       </c>
       <c r="G787" s="4" t="n">
-        <v>2009.1</v>
+        <v>3746.7</v>
       </c>
       <c r="H787" s="2" t="n">
         <v>1522616</v>
@@ -37217,13 +37217,13 @@
         </is>
       </c>
       <c r="E788" s="4" t="n">
-        <v>69</v>
+        <v>2</v>
       </c>
       <c r="F788" s="5" t="n">
-        <v>54.3</v>
+        <v>139.6</v>
       </c>
       <c r="G788" s="4" t="n">
-        <v>3746.7</v>
+        <v>279.2</v>
       </c>
       <c r="H788" s="2" t="n">
         <v>1522616</v>
@@ -37264,13 +37264,13 @@
         </is>
       </c>
       <c r="E789" s="4" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F789" s="5" t="n">
-        <v>139.6</v>
+        <v>127.6</v>
       </c>
       <c r="G789" s="4" t="n">
-        <v>279.2</v>
+        <v>1786.4</v>
       </c>
       <c r="H789" s="2" t="n">
         <v>1522616</v>
@@ -37311,13 +37311,13 @@
         </is>
       </c>
       <c r="E790" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F790" s="5" t="n">
-        <v>127.6</v>
+        <v>153.6</v>
       </c>
       <c r="G790" s="4" t="n">
-        <v>1786.4</v>
+        <v>2457.6</v>
       </c>
       <c r="H790" s="2" t="n">
         <v>1522616</v>
@@ -37358,13 +37358,13 @@
         </is>
       </c>
       <c r="E791" s="4" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="F791" s="5" t="n">
-        <v>153.6</v>
+        <v>127.6</v>
       </c>
       <c r="G791" s="4" t="n">
-        <v>2457.6</v>
+        <v>4593.6</v>
       </c>
       <c r="H791" s="2" t="n">
         <v>1522616</v>
@@ -37969,13 +37969,13 @@
         </is>
       </c>
       <c r="E804" s="4" t="n">
-        <v>1</v>
+        <v>1.89</v>
       </c>
       <c r="F804" s="5" t="n">
-        <v>36</v>
+        <v>150</v>
       </c>
       <c r="G804" s="4" t="n">
-        <v>36</v>
+        <v>283.5</v>
       </c>
       <c r="H804" s="2" t="n">
         <v>1524925</v>
@@ -38016,13 +38016,13 @@
         </is>
       </c>
       <c r="E805" s="4" t="n">
-        <v>1.89</v>
+        <v>0.08</v>
       </c>
       <c r="F805" s="5" t="n">
-        <v>150</v>
+        <v>18</v>
       </c>
       <c r="G805" s="4" t="n">
-        <v>283.5</v>
+        <v>1.44</v>
       </c>
       <c r="H805" s="2" t="n">
         <v>1524925</v>
@@ -38063,13 +38063,13 @@
         </is>
       </c>
       <c r="E806" s="4" t="n">
-        <v>0.08</v>
+        <v>1</v>
       </c>
       <c r="F806" s="5" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="G806" s="4" t="n">
-        <v>1.44</v>
+        <v>36</v>
       </c>
       <c r="H806" s="2" t="n">
         <v>1524925</v>
@@ -40319,13 +40319,13 @@
         </is>
       </c>
       <c r="E854" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F854" s="5" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G854" s="4" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="H854" s="2" t="n">
         <v>1532084</v>
@@ -40366,13 +40366,13 @@
         </is>
       </c>
       <c r="E855" s="4" t="n">
-        <v>0.1</v>
+        <v>1.5</v>
       </c>
       <c r="F855" s="5" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G855" s="4" t="n">
-        <v>2.5</v>
+        <v>21</v>
       </c>
       <c r="H855" s="2" t="n">
         <v>1532084</v>
@@ -40413,13 +40413,13 @@
         </is>
       </c>
       <c r="E856" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F856" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G856" s="4" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="H856" s="2" t="n">
         <v>1532084</v>
@@ -40460,13 +40460,13 @@
         </is>
       </c>
       <c r="E857" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F857" s="5" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G857" s="4" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="H857" s="2" t="n">
         <v>1532084</v>
@@ -40507,13 +40507,13 @@
         </is>
       </c>
       <c r="E858" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F858" s="5" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="G858" s="4" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="H858" s="2" t="n">
         <v>1532084</v>
@@ -40554,13 +40554,13 @@
         </is>
       </c>
       <c r="E859" s="4" t="n">
-        <v>1.5</v>
+        <v>0.1</v>
       </c>
       <c r="F859" s="5" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G859" s="4" t="n">
-        <v>21</v>
+        <v>2.5</v>
       </c>
       <c r="H859" s="2" t="n">
         <v>1532084</v>
@@ -40604,10 +40604,10 @@
         <v>1</v>
       </c>
       <c r="F860" s="5" t="n">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="G860" s="4" t="n">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="H860" s="2" t="n">
         <v>1532084</v>
@@ -40883,13 +40883,13 @@
         </is>
       </c>
       <c r="E866" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F866" s="5" t="n">
-        <v>39.9</v>
+        <v>4.9</v>
       </c>
       <c r="G866" s="4" t="n">
-        <v>39.9</v>
+        <v>29.4</v>
       </c>
       <c r="H866" s="2" t="n">
         <v>1533181</v>
@@ -40930,13 +40930,13 @@
         </is>
       </c>
       <c r="E867" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F867" s="5" t="n">
-        <v>4.9</v>
+        <v>6.9</v>
       </c>
       <c r="G867" s="4" t="n">
-        <v>29.4</v>
+        <v>13.8</v>
       </c>
       <c r="H867" s="2" t="n">
         <v>1533181</v>
@@ -40977,13 +40977,13 @@
         </is>
       </c>
       <c r="E868" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F868" s="5" t="n">
-        <v>6.9</v>
+        <v>18.9</v>
       </c>
       <c r="G868" s="4" t="n">
-        <v>13.8</v>
+        <v>18.9</v>
       </c>
       <c r="H868" s="2" t="n">
         <v>1533181</v>
@@ -41027,10 +41027,10 @@
         <v>1</v>
       </c>
       <c r="F869" s="5" t="n">
-        <v>18.9</v>
+        <v>39.9</v>
       </c>
       <c r="G869" s="4" t="n">
-        <v>18.9</v>
+        <v>39.9</v>
       </c>
       <c r="H869" s="2" t="n">
         <v>1533181</v>
@@ -41776,13 +41776,13 @@
         </is>
       </c>
       <c r="E885" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F885" s="5" t="n">
-        <v>0.52</v>
+        <v>0.6</v>
       </c>
       <c r="G885" s="4" t="n">
-        <v>4.16</v>
+        <v>2.4</v>
       </c>
       <c r="H885" s="2" t="n">
         <v>1539898</v>
@@ -41823,13 +41823,13 @@
         </is>
       </c>
       <c r="E886" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F886" s="5" t="n">
-        <v>0.08</v>
+        <v>0.6</v>
       </c>
       <c r="G886" s="4" t="n">
-        <v>0.96</v>
+        <v>2.4</v>
       </c>
       <c r="H886" s="2" t="n">
         <v>1539898</v>
@@ -41870,13 +41870,13 @@
         </is>
       </c>
       <c r="E887" s="4" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="F887" s="5" t="n">
-        <v>0.66</v>
+        <v>0.8</v>
       </c>
       <c r="G887" s="4" t="n">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="H887" s="2" t="n">
         <v>1539898</v>
@@ -41917,13 +41917,13 @@
         </is>
       </c>
       <c r="E888" s="4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F888" s="5" t="n">
-        <v>2.3</v>
+        <v>1</v>
       </c>
       <c r="G888" s="4" t="n">
-        <v>13.8</v>
+        <v>12</v>
       </c>
       <c r="H888" s="2" t="n">
         <v>1539898</v>
@@ -41964,13 +41964,13 @@
         </is>
       </c>
       <c r="E889" s="4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F889" s="5" t="n">
-        <v>1</v>
+        <v>2.3</v>
       </c>
       <c r="G889" s="4" t="n">
-        <v>12</v>
+        <v>13.8</v>
       </c>
       <c r="H889" s="2" t="n">
         <v>1539898</v>
@@ -42011,13 +42011,13 @@
         </is>
       </c>
       <c r="E890" s="4" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="F890" s="5" t="n">
-        <v>0.8</v>
+        <v>0.66</v>
       </c>
       <c r="G890" s="4" t="n">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="H890" s="2" t="n">
         <v>1539898</v>
@@ -42058,13 +42058,13 @@
         </is>
       </c>
       <c r="E891" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F891" s="5" t="n">
-        <v>0.6</v>
+        <v>0.52</v>
       </c>
       <c r="G891" s="4" t="n">
-        <v>2.4</v>
+        <v>4.16</v>
       </c>
       <c r="H891" s="2" t="n">
         <v>1539898</v>
@@ -42108,10 +42108,10 @@
         <v>4</v>
       </c>
       <c r="F892" s="5" t="n">
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="G892" s="4" t="n">
-        <v>2.4</v>
+        <v>2.32</v>
       </c>
       <c r="H892" s="2" t="n">
         <v>1539898</v>
@@ -42152,13 +42152,13 @@
         </is>
       </c>
       <c r="E893" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F893" s="5" t="n">
-        <v>0.58</v>
+        <v>0.81</v>
       </c>
       <c r="G893" s="4" t="n">
-        <v>2.32</v>
+        <v>1.62</v>
       </c>
       <c r="H893" s="2" t="n">
         <v>1539898</v>
@@ -42199,13 +42199,13 @@
         </is>
       </c>
       <c r="E894" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F894" s="5" t="n">
-        <v>0.81</v>
+        <v>0.7</v>
       </c>
       <c r="G894" s="4" t="n">
-        <v>1.62</v>
+        <v>2.8</v>
       </c>
       <c r="H894" s="2" t="n">
         <v>1539898</v>
@@ -42246,13 +42246,13 @@
         </is>
       </c>
       <c r="E895" s="4" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="F895" s="5" t="n">
-        <v>0.17</v>
+        <v>1.2</v>
       </c>
       <c r="G895" s="4" t="n">
-        <v>5.1</v>
+        <v>2.4</v>
       </c>
       <c r="H895" s="2" t="n">
         <v>1539898</v>
@@ -42293,13 +42293,13 @@
         </is>
       </c>
       <c r="E896" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F896" s="5" t="n">
-        <v>0.22</v>
+        <v>1.32</v>
       </c>
       <c r="G896" s="4" t="n">
-        <v>1.32</v>
+        <v>5.28</v>
       </c>
       <c r="H896" s="2" t="n">
         <v>1539898</v>
@@ -42343,10 +42343,10 @@
         <v>12</v>
       </c>
       <c r="F897" s="5" t="n">
-        <v>0.15</v>
+        <v>0.45</v>
       </c>
       <c r="G897" s="4" t="n">
-        <v>1.8</v>
+        <v>5.4</v>
       </c>
       <c r="H897" s="2" t="n">
         <v>1539898</v>
@@ -42387,13 +42387,13 @@
         </is>
       </c>
       <c r="E898" s="4" t="n">
-        <v>8</v>
+        <v>100</v>
       </c>
       <c r="F898" s="5" t="n">
-        <v>0.25</v>
+        <v>0.11</v>
       </c>
       <c r="G898" s="4" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H898" s="2" t="n">
         <v>1539898</v>
@@ -42434,13 +42434,13 @@
         </is>
       </c>
       <c r="E899" s="4" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F899" s="5" t="n">
-        <v>53</v>
+        <v>0.12</v>
       </c>
       <c r="G899" s="4" t="n">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="H899" s="2" t="n">
         <v>1539898</v>
@@ -42481,13 +42481,13 @@
         </is>
       </c>
       <c r="E900" s="4" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="F900" s="5" t="n">
-        <v>0.11</v>
+        <v>0.2</v>
       </c>
       <c r="G900" s="4" t="n">
-        <v>0.66</v>
+        <v>4</v>
       </c>
       <c r="H900" s="2" t="n">
         <v>1539898</v>
@@ -42528,13 +42528,13 @@
         </is>
       </c>
       <c r="E901" s="4" t="n">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="F901" s="5" t="n">
-        <v>0.3</v>
+        <v>0.42</v>
       </c>
       <c r="G901" s="4" t="n">
-        <v>30</v>
+        <v>2.52</v>
       </c>
       <c r="H901" s="2" t="n">
         <v>1539898</v>
@@ -42575,13 +42575,13 @@
         </is>
       </c>
       <c r="E902" s="4" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="F902" s="5" t="n">
-        <v>0.19</v>
+        <v>0.3</v>
       </c>
       <c r="G902" s="4" t="n">
-        <v>5.32</v>
+        <v>3</v>
       </c>
       <c r="H902" s="2" t="n">
         <v>1539898</v>
@@ -42622,13 +42622,13 @@
         </is>
       </c>
       <c r="E903" s="4" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="F903" s="5" t="n">
-        <v>0.2</v>
+        <v>0.33</v>
       </c>
       <c r="G903" s="4" t="n">
-        <v>4.8</v>
+        <v>1.98</v>
       </c>
       <c r="H903" s="2" t="n">
         <v>1539898</v>
@@ -42669,13 +42669,13 @@
         </is>
       </c>
       <c r="E904" s="4" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F904" s="5" t="n">
-        <v>0.48</v>
+        <v>0.21</v>
       </c>
       <c r="G904" s="4" t="n">
-        <v>1.92</v>
+        <v>2.52</v>
       </c>
       <c r="H904" s="2" t="n">
         <v>1539898</v>
@@ -42716,13 +42716,13 @@
         </is>
       </c>
       <c r="E905" s="4" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="F905" s="5" t="n">
-        <v>0.35</v>
+        <v>0.29</v>
       </c>
       <c r="G905" s="4" t="n">
-        <v>2.1</v>
+        <v>4.06</v>
       </c>
       <c r="H905" s="2" t="n">
         <v>1539898</v>
@@ -42763,13 +42763,13 @@
         </is>
       </c>
       <c r="E906" s="4" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F906" s="5" t="n">
-        <v>0.29</v>
+        <v>0.35</v>
       </c>
       <c r="G906" s="4" t="n">
-        <v>4.06</v>
+        <v>2.1</v>
       </c>
       <c r="H906" s="2" t="n">
         <v>1539898</v>
@@ -42810,13 +42810,13 @@
         </is>
       </c>
       <c r="E907" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F907" s="5" t="n">
-        <v>0.21</v>
+        <v>0.48</v>
       </c>
       <c r="G907" s="4" t="n">
-        <v>2.52</v>
+        <v>1.92</v>
       </c>
       <c r="H907" s="2" t="n">
         <v>1539898</v>
@@ -42857,13 +42857,13 @@
         </is>
       </c>
       <c r="E908" s="4" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="F908" s="5" t="n">
-        <v>0.33</v>
+        <v>0.2</v>
       </c>
       <c r="G908" s="4" t="n">
-        <v>1.98</v>
+        <v>4.8</v>
       </c>
       <c r="H908" s="2" t="n">
         <v>1539898</v>
@@ -42904,13 +42904,13 @@
         </is>
       </c>
       <c r="E909" s="4" t="n">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F909" s="5" t="n">
-        <v>0.3</v>
+        <v>0.19</v>
       </c>
       <c r="G909" s="4" t="n">
-        <v>3</v>
+        <v>5.32</v>
       </c>
       <c r="H909" s="2" t="n">
         <v>1539898</v>
@@ -42951,13 +42951,13 @@
         </is>
       </c>
       <c r="E910" s="4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F910" s="5" t="n">
-        <v>0.42</v>
+        <v>0.08</v>
       </c>
       <c r="G910" s="4" t="n">
-        <v>2.52</v>
+        <v>0.96</v>
       </c>
       <c r="H910" s="2" t="n">
         <v>1539898</v>
@@ -42998,13 +42998,13 @@
         </is>
       </c>
       <c r="E911" s="4" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F911" s="5" t="n">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="G911" s="4" t="n">
-        <v>4</v>
+        <v>5.1</v>
       </c>
       <c r="H911" s="2" t="n">
         <v>1539898</v>
@@ -43045,13 +43045,13 @@
         </is>
       </c>
       <c r="E912" s="4" t="n">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="F912" s="5" t="n">
-        <v>0.12</v>
+        <v>0.22</v>
       </c>
       <c r="G912" s="4" t="n">
-        <v>12</v>
+        <v>1.32</v>
       </c>
       <c r="H912" s="2" t="n">
         <v>1539898</v>
@@ -43092,13 +43092,13 @@
         </is>
       </c>
       <c r="E913" s="4" t="n">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="F913" s="5" t="n">
-        <v>0.11</v>
+        <v>0.15</v>
       </c>
       <c r="G913" s="4" t="n">
-        <v>11</v>
+        <v>1.8</v>
       </c>
       <c r="H913" s="2" t="n">
         <v>1539898</v>
@@ -43139,13 +43139,13 @@
         </is>
       </c>
       <c r="E914" s="4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F914" s="5" t="n">
-        <v>0.45</v>
+        <v>0.25</v>
       </c>
       <c r="G914" s="4" t="n">
-        <v>5.4</v>
+        <v>2</v>
       </c>
       <c r="H914" s="2" t="n">
         <v>1539898</v>
@@ -43186,13 +43186,13 @@
         </is>
       </c>
       <c r="E915" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F915" s="5" t="n">
-        <v>1.32</v>
+        <v>53</v>
       </c>
       <c r="G915" s="4" t="n">
-        <v>5.28</v>
+        <v>53</v>
       </c>
       <c r="H915" s="2" t="n">
         <v>1539898</v>
@@ -43233,13 +43233,13 @@
         </is>
       </c>
       <c r="E916" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F916" s="5" t="n">
-        <v>1.2</v>
+        <v>0.11</v>
       </c>
       <c r="G916" s="4" t="n">
-        <v>2.4</v>
+        <v>0.66</v>
       </c>
       <c r="H916" s="2" t="n">
         <v>1539898</v>
@@ -43280,13 +43280,13 @@
         </is>
       </c>
       <c r="E917" s="4" t="n">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="F917" s="5" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="G917" s="4" t="n">
-        <v>2.8</v>
+        <v>30</v>
       </c>
       <c r="H917" s="2" t="n">
         <v>1539898</v>
@@ -43844,13 +43844,13 @@
         </is>
       </c>
       <c r="E929" s="4" t="n">
-        <v>0.28</v>
+        <v>0.04</v>
       </c>
       <c r="F929" s="5" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="G929" s="4" t="n">
-        <v>8.4</v>
+        <v>4</v>
       </c>
       <c r="H929" s="2" t="n">
         <v>1546014</v>
@@ -43891,13 +43891,13 @@
         </is>
       </c>
       <c r="E930" s="4" t="n">
-        <v>0.28</v>
+        <v>1</v>
       </c>
       <c r="F930" s="5" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="G930" s="4" t="n">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="H930" s="2" t="n">
         <v>1546014</v>
@@ -43941,10 +43941,10 @@
         <v>0.28</v>
       </c>
       <c r="F931" s="5" t="n">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="G931" s="4" t="n">
-        <v>4.2</v>
+        <v>28</v>
       </c>
       <c r="H931" s="2" t="n">
         <v>1546014</v>
@@ -43985,13 +43985,13 @@
         </is>
       </c>
       <c r="E932" s="4" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="F932" s="5" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="G932" s="4" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="H932" s="2" t="n">
         <v>1546014</v>
@@ -44032,13 +44032,13 @@
         </is>
       </c>
       <c r="E933" s="4" t="n">
-        <v>0.16</v>
+        <v>0.28</v>
       </c>
       <c r="F933" s="5" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G933" s="4" t="n">
-        <v>5.6</v>
+        <v>8.4</v>
       </c>
       <c r="H933" s="2" t="n">
         <v>1546014</v>
@@ -44079,13 +44079,13 @@
         </is>
       </c>
       <c r="E934" s="4" t="n">
-        <v>0.04</v>
+        <v>0.16</v>
       </c>
       <c r="F934" s="5" t="n">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="G934" s="4" t="n">
-        <v>4</v>
+        <v>5.6</v>
       </c>
       <c r="H934" s="2" t="n">
         <v>1546014</v>
@@ -44126,13 +44126,13 @@
         </is>
       </c>
       <c r="E935" s="4" t="n">
-        <v>0.1</v>
+        <v>0.28</v>
       </c>
       <c r="F935" s="5" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="G935" s="4" t="n">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="H935" s="2" t="n">
         <v>1546014</v>
@@ -44317,10 +44317,10 @@
         <v>1</v>
       </c>
       <c r="F939" s="5" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="G939" s="4" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="H939" s="2" t="n">
         <v>1547044</v>
@@ -44364,10 +44364,10 @@
         <v>1</v>
       </c>
       <c r="F940" s="5" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="G940" s="4" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="H940" s="2" t="n">
         <v>1547044</v>
@@ -44458,10 +44458,10 @@
         <v>1</v>
       </c>
       <c r="F942" s="5" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="G942" s="4" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="H942" s="2" t="n">
         <v>1547044</v>
@@ -44505,10 +44505,10 @@
         <v>1</v>
       </c>
       <c r="F943" s="5" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="G943" s="4" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="H943" s="2" t="n">
         <v>1547044</v>
@@ -44552,10 +44552,10 @@
         <v>1</v>
       </c>
       <c r="F944" s="5" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="G944" s="4" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="H944" s="2" t="n">
         <v>1547044</v>
@@ -44599,10 +44599,10 @@
         <v>1</v>
       </c>
       <c r="F945" s="5" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="G945" s="4" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="H945" s="2" t="n">
         <v>1547044</v>
@@ -45254,13 +45254,13 @@
         </is>
       </c>
       <c r="E959" s="4" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="F959" s="5" t="n">
-        <v>20</v>
+        <v>33.5</v>
       </c>
       <c r="G959" s="4" t="n">
-        <v>4</v>
+        <v>33.5</v>
       </c>
       <c r="H959" s="2" t="n">
         <v>1549629</v>
@@ -45301,13 +45301,13 @@
         </is>
       </c>
       <c r="E960" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F960" s="5" t="n">
-        <v>2</v>
+        <v>1.35</v>
       </c>
       <c r="G960" s="4" t="n">
-        <v>20</v>
+        <v>4.05</v>
       </c>
       <c r="H960" s="2" t="n">
         <v>1549629</v>
@@ -45348,13 +45348,13 @@
         </is>
       </c>
       <c r="E961" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F961" s="5" t="n">
-        <v>21</v>
+        <v>6.1</v>
       </c>
       <c r="G961" s="4" t="n">
-        <v>21</v>
+        <v>30.5</v>
       </c>
       <c r="H961" s="2" t="n">
         <v>1549629</v>
@@ -45442,13 +45442,13 @@
         </is>
       </c>
       <c r="E963" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F963" s="5" t="n">
-        <v>33.5</v>
+        <v>2</v>
       </c>
       <c r="G963" s="4" t="n">
-        <v>33.5</v>
+        <v>20</v>
       </c>
       <c r="H963" s="2" t="n">
         <v>1549629</v>
@@ -45489,13 +45489,13 @@
         </is>
       </c>
       <c r="E964" s="4" t="n">
-        <v>5</v>
+        <v>0.2</v>
       </c>
       <c r="F964" s="5" t="n">
-        <v>6.1</v>
+        <v>20</v>
       </c>
       <c r="G964" s="4" t="n">
-        <v>30.5</v>
+        <v>4</v>
       </c>
       <c r="H964" s="2" t="n">
         <v>1549629</v>
@@ -45536,13 +45536,13 @@
         </is>
       </c>
       <c r="E965" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F965" s="5" t="n">
-        <v>1.35</v>
+        <v>21</v>
       </c>
       <c r="G965" s="4" t="n">
-        <v>4.05</v>
+        <v>21</v>
       </c>
       <c r="H965" s="2" t="n">
         <v>1549629</v>
@@ -48027,13 +48027,13 @@
         </is>
       </c>
       <c r="E1018" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1018" s="5" t="n">
-        <v>51.62</v>
+        <v>104.55</v>
       </c>
       <c r="G1018" s="4" t="n">
-        <v>51.62</v>
+        <v>209.1</v>
       </c>
       <c r="H1018" s="2" t="n">
         <v>1561152</v>
@@ -48074,13 +48074,13 @@
         </is>
       </c>
       <c r="E1019" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1019" s="5" t="n">
-        <v>104.55</v>
+        <v>51.62</v>
       </c>
       <c r="G1019" s="4" t="n">
-        <v>209.1</v>
+        <v>51.62</v>
       </c>
       <c r="H1019" s="2" t="n">
         <v>1561152</v>
@@ -48215,13 +48215,13 @@
         </is>
       </c>
       <c r="E1022" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1022" s="5" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="G1022" s="4" t="n">
-        <v>180</v>
+        <v>110</v>
       </c>
       <c r="H1022" s="2" t="n">
         <v>1561209</v>
@@ -48265,10 +48265,10 @@
         <v>1</v>
       </c>
       <c r="F1023" s="5" t="n">
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="G1023" s="4" t="n">
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="H1023" s="2" t="n">
         <v>1561209</v>
@@ -48309,13 +48309,13 @@
         </is>
       </c>
       <c r="E1024" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1024" s="5" t="n">
         <v>90</v>
       </c>
       <c r="G1024" s="4" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
       <c r="H1024" s="2" t="n">
         <v>1561209</v>
@@ -57806,10 +57806,10 @@
         <v>0.5</v>
       </c>
       <c r="F1226" s="5" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="G1226" s="4" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="H1226" s="2" t="n">
         <v>1589380</v>
@@ -57853,10 +57853,10 @@
         <v>1</v>
       </c>
       <c r="F1227" s="5" t="n">
-        <v>120</v>
+        <v>22</v>
       </c>
       <c r="G1227" s="4" t="n">
-        <v>120</v>
+        <v>22</v>
       </c>
       <c r="H1227" s="2" t="n">
         <v>1589380</v>
@@ -57897,10 +57897,10 @@
         </is>
       </c>
       <c r="E1228" s="4" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="F1228" s="5" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="G1228" s="4" t="n">
         <v>9</v>
@@ -57944,13 +57944,13 @@
         </is>
       </c>
       <c r="E1229" s="4" t="n">
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="F1229" s="5" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G1229" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H1229" s="2" t="n">
         <v>1589380</v>
@@ -57991,13 +57991,13 @@
         </is>
       </c>
       <c r="E1230" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1230" s="5" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G1230" s="4" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="H1230" s="2" t="n">
         <v>1589380</v>
@@ -58038,13 +58038,13 @@
         </is>
       </c>
       <c r="E1231" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1231" s="5" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G1231" s="4" t="n">
-        <v>12.5</v>
+        <v>30</v>
       </c>
       <c r="H1231" s="2" t="n">
         <v>1589380</v>
@@ -58085,13 +58085,13 @@
         </is>
       </c>
       <c r="E1232" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1232" s="5" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G1232" s="4" t="n">
-        <v>30</v>
+        <v>12.5</v>
       </c>
       <c r="H1232" s="2" t="n">
         <v>1589380</v>
@@ -58132,13 +58132,13 @@
         </is>
       </c>
       <c r="E1233" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1233" s="5" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G1233" s="4" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H1233" s="2" t="n">
         <v>1589380</v>
@@ -58179,13 +58179,13 @@
         </is>
       </c>
       <c r="E1234" s="4" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="F1234" s="5" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="G1234" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="H1234" s="2" t="n">
         <v>1589380</v>
@@ -58226,13 +58226,13 @@
         </is>
       </c>
       <c r="E1235" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1235" s="5" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G1235" s="4" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="H1235" s="2" t="n">
         <v>1589380</v>
@@ -58273,13 +58273,13 @@
         </is>
       </c>
       <c r="E1236" s="4" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="F1236" s="5" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="G1236" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H1236" s="2" t="n">
         <v>1589380</v>
@@ -58320,13 +58320,13 @@
         </is>
       </c>
       <c r="E1237" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F1237" s="5" t="n">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="G1237" s="4" t="n">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="H1237" s="2" t="n">
         <v>1589380</v>
@@ -58370,10 +58370,10 @@
         <v>1</v>
       </c>
       <c r="F1238" s="5" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G1238" s="4" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="H1238" s="2" t="n">
         <v>1589380</v>
@@ -58414,13 +58414,13 @@
         </is>
       </c>
       <c r="E1239" s="4" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="F1239" s="5" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="G1239" s="4" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H1239" s="2" t="n">
         <v>1589380</v>
@@ -58508,10 +58508,10 @@
         </is>
       </c>
       <c r="E1241" s="4" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F1241" s="5" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="G1241" s="4" t="n">
         <v>15</v>
@@ -59730,13 +59730,13 @@
         </is>
       </c>
       <c r="E1267" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F1267" s="5" t="n">
-        <v>14.23</v>
+        <v>1.29</v>
       </c>
       <c r="G1267" s="4" t="n">
-        <v>14.23</v>
+        <v>5.16</v>
       </c>
       <c r="H1267" s="2" t="n">
         <v>1591999</v>
@@ -59780,10 +59780,10 @@
         <v>2</v>
       </c>
       <c r="F1268" s="5" t="n">
-        <v>3.25</v>
+        <v>13.17</v>
       </c>
       <c r="G1268" s="4" t="n">
-        <v>6.5</v>
+        <v>26.34</v>
       </c>
       <c r="H1268" s="2" t="n">
         <v>1591999</v>
@@ -59827,10 +59827,10 @@
         <v>1</v>
       </c>
       <c r="F1269" s="5" t="n">
-        <v>215.83</v>
+        <v>14.23</v>
       </c>
       <c r="G1269" s="4" t="n">
-        <v>215.83</v>
+        <v>14.23</v>
       </c>
       <c r="H1269" s="2" t="n">
         <v>1591999</v>
@@ -59871,13 +59871,13 @@
         </is>
       </c>
       <c r="E1270" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F1270" s="5" t="n">
-        <v>1.29</v>
+        <v>3.25</v>
       </c>
       <c r="G1270" s="4" t="n">
-        <v>5.16</v>
+        <v>6.5</v>
       </c>
       <c r="H1270" s="2" t="n">
         <v>1591999</v>
@@ -59918,13 +59918,13 @@
         </is>
       </c>
       <c r="E1271" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1271" s="5" t="n">
-        <v>13.17</v>
+        <v>215.83</v>
       </c>
       <c r="G1271" s="4" t="n">
-        <v>26.34</v>
+        <v>215.83</v>
       </c>
       <c r="H1271" s="2" t="n">
         <v>1591999</v>
@@ -60156,10 +60156,10 @@
         <v>25</v>
       </c>
       <c r="F1276" s="5" t="n">
-        <v>0.19</v>
+        <v>0.92</v>
       </c>
       <c r="G1276" s="4" t="n">
-        <v>4.75</v>
+        <v>23</v>
       </c>
       <c r="H1276" s="2" t="n">
         <v>1591999</v>
@@ -60203,10 +60203,10 @@
         <v>25</v>
       </c>
       <c r="F1277" s="5" t="n">
-        <v>0.58</v>
+        <v>0.19</v>
       </c>
       <c r="G1277" s="4" t="n">
-        <v>14.5</v>
+        <v>4.75</v>
       </c>
       <c r="H1277" s="2" t="n">
         <v>1591999</v>
@@ -60250,10 +60250,10 @@
         <v>25</v>
       </c>
       <c r="F1278" s="5" t="n">
-        <v>0.92</v>
+        <v>0.58</v>
       </c>
       <c r="G1278" s="4" t="n">
-        <v>23</v>
+        <v>14.5</v>
       </c>
       <c r="H1278" s="2" t="n">
         <v>1591999</v>
@@ -61845,13 +61845,13 @@
         </is>
       </c>
       <c r="E1312" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1312" s="5" t="n">
-        <v>1.17</v>
+        <v>4.7</v>
       </c>
       <c r="G1312" s="4" t="n">
-        <v>2.34</v>
+        <v>4.7</v>
       </c>
       <c r="H1312" s="2" t="n">
         <v>1595677</v>
@@ -61895,10 +61895,10 @@
         <v>1</v>
       </c>
       <c r="F1313" s="5" t="n">
-        <v>4.7</v>
+        <v>3.09</v>
       </c>
       <c r="G1313" s="4" t="n">
-        <v>4.7</v>
+        <v>3.09</v>
       </c>
       <c r="H1313" s="2" t="n">
         <v>1595677</v>
@@ -61986,13 +61986,13 @@
         </is>
       </c>
       <c r="E1315" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1315" s="5" t="n">
-        <v>3.09</v>
+        <v>1.17</v>
       </c>
       <c r="G1315" s="4" t="n">
-        <v>3.09</v>
+        <v>2.34</v>
       </c>
       <c r="H1315" s="2" t="n">
         <v>1595677</v>
@@ -63349,13 +63349,13 @@
         </is>
       </c>
       <c r="E1344" s="4" t="n">
-        <v>0.39</v>
+        <v>1</v>
       </c>
       <c r="F1344" s="5" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G1344" s="4" t="n">
-        <v>9.75</v>
+        <v>15</v>
       </c>
       <c r="H1344" s="2" t="n">
         <v>1600774</v>
@@ -63396,13 +63396,13 @@
         </is>
       </c>
       <c r="E1345" s="4" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="F1345" s="5" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="G1345" s="4" t="n">
-        <v>18</v>
+        <v>11.2</v>
       </c>
       <c r="H1345" s="2" t="n">
         <v>1600774</v>
@@ -63443,13 +63443,13 @@
         </is>
       </c>
       <c r="E1346" s="4" t="n">
-        <v>0.3</v>
+        <v>100</v>
       </c>
       <c r="F1346" s="5" t="n">
-        <v>60</v>
+        <v>0.75</v>
       </c>
       <c r="G1346" s="4" t="n">
-        <v>18</v>
+        <v>75</v>
       </c>
       <c r="H1346" s="2" t="n">
         <v>1600774</v>
@@ -63493,10 +63493,10 @@
         <v>1</v>
       </c>
       <c r="F1347" s="5" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="G1347" s="4" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="H1347" s="2" t="n">
         <v>1600774</v>
@@ -63537,13 +63537,13 @@
         </is>
       </c>
       <c r="E1348" s="4" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="F1348" s="5" t="n">
-        <v>80</v>
+        <v>18</v>
       </c>
       <c r="G1348" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H1348" s="2" t="n">
         <v>1600774</v>
@@ -63584,13 +63584,13 @@
         </is>
       </c>
       <c r="E1349" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="F1349" s="5" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="G1349" s="4" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H1349" s="2" t="n">
         <v>1600774</v>
@@ -63634,10 +63634,10 @@
         <v>1</v>
       </c>
       <c r="F1350" s="5" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="G1350" s="4" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="H1350" s="2" t="n">
         <v>1600774</v>
@@ -63678,13 +63678,13 @@
         </is>
       </c>
       <c r="E1351" s="4" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F1351" s="5" t="n">
-        <v>28</v>
+        <v>80</v>
       </c>
       <c r="G1351" s="4" t="n">
-        <v>11.2</v>
+        <v>16</v>
       </c>
       <c r="H1351" s="2" t="n">
         <v>1600774</v>
@@ -63725,13 +63725,13 @@
         </is>
       </c>
       <c r="E1352" s="4" t="n">
-        <v>100</v>
+        <v>0.39</v>
       </c>
       <c r="F1352" s="5" t="n">
-        <v>0.75</v>
+        <v>25</v>
       </c>
       <c r="G1352" s="4" t="n">
-        <v>75</v>
+        <v>9.75</v>
       </c>
       <c r="H1352" s="2" t="n">
         <v>1600774</v>
@@ -65746,13 +65746,13 @@
         </is>
       </c>
       <c r="E1395" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1395" s="5" t="n">
-        <v>65.2</v>
+        <v>54.3</v>
       </c>
       <c r="G1395" s="4" t="n">
-        <v>260.8</v>
+        <v>325.8</v>
       </c>
       <c r="H1395" s="2" t="n">
         <v>1603907</v>
@@ -65793,13 +65793,13 @@
         </is>
       </c>
       <c r="E1396" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F1396" s="5" t="n">
         <v>65.2</v>
       </c>
       <c r="G1396" s="4" t="n">
-        <v>130.4</v>
+        <v>260.8</v>
       </c>
       <c r="H1396" s="2" t="n">
         <v>1603907</v>
@@ -65840,13 +65840,13 @@
         </is>
       </c>
       <c r="E1397" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F1397" s="5" t="n">
-        <v>54.3</v>
+        <v>65.2</v>
       </c>
       <c r="G1397" s="4" t="n">
-        <v>325.8</v>
+        <v>130.4</v>
       </c>
       <c r="H1397" s="2" t="n">
         <v>1603907</v>
@@ -66921,13 +66921,13 @@
         </is>
       </c>
       <c r="E1420" s="4" t="n">
-        <v>1.63</v>
+        <v>7.26</v>
       </c>
       <c r="F1420" s="5" t="n">
-        <v>112</v>
+        <v>144</v>
       </c>
       <c r="G1420" s="4" t="n">
-        <v>182.56</v>
+        <v>1045.44</v>
       </c>
       <c r="H1420" s="2" t="n">
         <v>1606285</v>
@@ -66968,13 +66968,13 @@
         </is>
       </c>
       <c r="E1421" s="4" t="n">
-        <v>7.26</v>
+        <v>1.63</v>
       </c>
       <c r="F1421" s="5" t="n">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="G1421" s="4" t="n">
-        <v>1045.44</v>
+        <v>182.56</v>
       </c>
       <c r="H1421" s="2" t="n">
         <v>1606285</v>
@@ -67062,13 +67062,13 @@
         </is>
       </c>
       <c r="E1423" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F1423" s="5" t="n">
-        <v>1.2</v>
+        <v>8.9</v>
       </c>
       <c r="G1423" s="4" t="n">
-        <v>6</v>
+        <v>17.8</v>
       </c>
       <c r="H1423" s="2" t="n">
         <v>1606516</v>
@@ -67250,13 +67250,13 @@
         </is>
       </c>
       <c r="E1427" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F1427" s="5" t="n">
-        <v>43.9</v>
+        <v>1.2</v>
       </c>
       <c r="G1427" s="4" t="n">
-        <v>43.9</v>
+        <v>6</v>
       </c>
       <c r="H1427" s="2" t="n">
         <v>1606516</v>
@@ -67438,13 +67438,13 @@
         </is>
       </c>
       <c r="E1431" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1431" s="5" t="n">
-        <v>8.9</v>
+        <v>43.9</v>
       </c>
       <c r="G1431" s="4" t="n">
-        <v>17.8</v>
+        <v>43.9</v>
       </c>
       <c r="H1431" s="2" t="n">
         <v>1606516</v>
@@ -69227,10 +69227,10 @@
         <v>2</v>
       </c>
       <c r="F1469" s="5" t="n">
-        <v>42.75</v>
+        <v>16.99</v>
       </c>
       <c r="G1469" s="4" t="n">
-        <v>85.5</v>
+        <v>33.98</v>
       </c>
       <c r="H1469" s="2" t="n">
         <v>1608017</v>
@@ -69274,10 +69274,10 @@
         <v>1</v>
       </c>
       <c r="F1470" s="5" t="n">
-        <v>57.99</v>
+        <v>25.9</v>
       </c>
       <c r="G1470" s="4" t="n">
-        <v>57.99</v>
+        <v>25.9</v>
       </c>
       <c r="H1470" s="2" t="n">
         <v>1608017</v>
@@ -69321,10 +69321,10 @@
         <v>1</v>
       </c>
       <c r="F1471" s="5" t="n">
-        <v>25.9</v>
+        <v>57.99</v>
       </c>
       <c r="G1471" s="4" t="n">
-        <v>25.9</v>
+        <v>57.99</v>
       </c>
       <c r="H1471" s="2" t="n">
         <v>1608017</v>
@@ -69368,10 +69368,10 @@
         <v>2</v>
       </c>
       <c r="F1472" s="5" t="n">
-        <v>16.99</v>
+        <v>42.75</v>
       </c>
       <c r="G1472" s="4" t="n">
-        <v>33.98</v>
+        <v>85.5</v>
       </c>
       <c r="H1472" s="2" t="n">
         <v>1608017</v>
@@ -70869,13 +70869,13 @@
         </is>
       </c>
       <c r="E1504" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1504" s="5" t="n">
-        <v>29.24</v>
+        <v>60</v>
       </c>
       <c r="G1504" s="4" t="n">
-        <v>29.24</v>
+        <v>120</v>
       </c>
       <c r="H1504" s="2" t="n">
         <v>1610748</v>
@@ -70963,13 +70963,13 @@
         </is>
       </c>
       <c r="E1506" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1506" s="5" t="n">
-        <v>60</v>
+        <v>29.24</v>
       </c>
       <c r="G1506" s="4" t="n">
-        <v>120</v>
+        <v>29.24</v>
       </c>
       <c r="H1506" s="2" t="n">
         <v>1610748</v>
@@ -71010,13 +71010,13 @@
         </is>
       </c>
       <c r="E1507" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1507" s="5" t="n">
-        <v>6.5</v>
+        <v>3.75</v>
       </c>
       <c r="G1507" s="4" t="n">
-        <v>13</v>
+        <v>3.75</v>
       </c>
       <c r="H1507" s="2" t="n">
         <v>1610784</v>
@@ -71057,13 +71057,13 @@
         </is>
       </c>
       <c r="E1508" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1508" s="5" t="n">
-        <v>3.64</v>
+        <v>6.5</v>
       </c>
       <c r="G1508" s="4" t="n">
-        <v>3.64</v>
+        <v>13</v>
       </c>
       <c r="H1508" s="2" t="n">
         <v>1610784</v>
@@ -71107,10 +71107,10 @@
         <v>1</v>
       </c>
       <c r="F1509" s="5" t="n">
-        <v>3.75</v>
+        <v>3.64</v>
       </c>
       <c r="G1509" s="4" t="n">
-        <v>3.75</v>
+        <v>3.64</v>
       </c>
       <c r="H1509" s="2" t="n">
         <v>1610784</v>

</xml_diff>

<commit_message>
Relatório de compras 08/10/2026 22:01
</commit_message>
<xml_diff>
--- a/data/relatorio.xlsx
+++ b/data/relatorio.xlsx
@@ -372,10 +372,10 @@
         <v>1</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>3.5</v>
+        <v>28.768</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>3.5</v>
+        <v>28.76</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>1397499</v>
@@ -416,13 +416,13 @@
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>4.5</v>
+        <v>23.36</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>4.5</v>
+        <v>70.08</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>1397499</v>
@@ -463,13 +463,13 @@
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>4.675</v>
+        <v>0.63</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>9.35</v>
+        <v>7.56</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>1397499</v>
@@ -510,13 +510,13 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>33.44</v>
+        <v>29.744</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>33.44</v>
+        <v>89.23</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>1397499</v>
@@ -560,10 +560,10 @@
         <v>1</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>28.768</v>
+        <v>4.5</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>28.76</v>
+        <v>4.5</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>1397499</v>
@@ -604,13 +604,13 @@
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>29.744</v>
+        <v>4.675</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>89.23</v>
+        <v>9.35</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>1397499</v>
@@ -651,13 +651,13 @@
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>23.36</v>
+        <v>33.44</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>70.08</v>
+        <v>33.44</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>1397499</v>
@@ -698,13 +698,13 @@
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.63</v>
+        <v>23.36</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>7.56</v>
+        <v>70.08</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>1397499</v>
@@ -745,13 +745,13 @@
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>23.36</v>
+        <v>3.5</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>70.08</v>
+        <v>3.5</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>1397499</v>
@@ -792,13 +792,13 @@
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>200</v>
+        <v>6</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.59</v>
+        <v>0.38</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>118</v>
+        <v>2.28</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>1397500</v>
@@ -839,13 +839,13 @@
         </is>
       </c>
       <c r="E14" s="4" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>29.6</v>
+        <v>0.7</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>1397500</v>
@@ -886,13 +886,13 @@
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.4</v>
+        <v>0.63</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>4</v>
+        <v>1.26</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>1397500</v>
@@ -933,13 +933,13 @@
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.1</v>
+        <v>0.59</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>1397500</v>
@@ -980,13 +980,13 @@
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.38</v>
+        <v>0.74</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>2.28</v>
+        <v>29.6</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>1397500</v>
@@ -1027,13 +1027,13 @@
         </is>
       </c>
       <c r="E18" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.7</v>
+        <v>4</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>1397500</v>
@@ -1074,13 +1074,13 @@
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.63</v>
+        <v>0.1</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>1.26</v>
+        <v>10</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>1397500</v>
@@ -1262,13 +1262,13 @@
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="H23" s="2" t="n">
         <v>1398186</v>
@@ -1356,13 +1356,13 @@
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>40</v>
+        <v>110</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>1398186</v>
@@ -1594,10 +1594,10 @@
         <v>1</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>9.3</v>
+        <v>59.9</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>9.3</v>
+        <v>59.9</v>
       </c>
       <c r="H30" s="2" t="n">
         <v>1398686</v>
@@ -1641,10 +1641,10 @@
         <v>1</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>59.9</v>
+        <v>9.3</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>59.9</v>
+        <v>9.3</v>
       </c>
       <c r="H31" s="2" t="n">
         <v>1398686</v>
@@ -2249,13 +2249,13 @@
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>1.65</v>
+        <v>0.6</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>90.75</v>
+        <v>36</v>
       </c>
       <c r="H44" s="2" t="n">
         <v>1400747</v>
@@ -2343,13 +2343,13 @@
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>0.6</v>
+        <v>1.65</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>36</v>
+        <v>90.75</v>
       </c>
       <c r="H46" s="2" t="n">
         <v>1400747</v>
@@ -3001,13 +3001,13 @@
         </is>
       </c>
       <c r="E60" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>30.25</v>
+        <v>23.65</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>30.25</v>
+        <v>47.3</v>
       </c>
       <c r="H60" s="2" t="n">
         <v>1401617</v>
@@ -3471,13 +3471,13 @@
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="F70" s="5" t="n">
-        <v>23.65</v>
+        <v>3.32</v>
       </c>
       <c r="G70" s="4" t="n">
-        <v>47.3</v>
+        <v>99.6</v>
       </c>
       <c r="H70" s="2" t="n">
         <v>1401617</v>
@@ -3518,13 +3518,13 @@
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="F71" s="5" t="n">
-        <v>3.32</v>
+        <v>30.25</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>99.6</v>
+        <v>30.25</v>
       </c>
       <c r="H71" s="2" t="n">
         <v>1401617</v>
@@ -4367,10 +4367,10 @@
         <v>1</v>
       </c>
       <c r="F89" s="5" t="n">
-        <v>200</v>
+        <v>78</v>
       </c>
       <c r="G89" s="4" t="n">
-        <v>200</v>
+        <v>78</v>
       </c>
       <c r="H89" s="2" t="n">
         <v>1402331</v>
@@ -4414,10 +4414,10 @@
         <v>1</v>
       </c>
       <c r="F90" s="5" t="n">
-        <v>67</v>
+        <v>200</v>
       </c>
       <c r="G90" s="4" t="n">
-        <v>67</v>
+        <v>200</v>
       </c>
       <c r="H90" s="2" t="n">
         <v>1402331</v>
@@ -4461,10 +4461,10 @@
         <v>1</v>
       </c>
       <c r="F91" s="5" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="G91" s="4" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="H91" s="2" t="n">
         <v>1402331</v>
@@ -4881,13 +4881,13 @@
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>200</v>
+        <v>268</v>
       </c>
       <c r="F100" s="5" t="n">
-        <v>0.17</v>
+        <v>0.22</v>
       </c>
       <c r="G100" s="4" t="n">
-        <v>34</v>
+        <v>58.96</v>
       </c>
       <c r="H100" s="2" t="n">
         <v>1402783</v>
@@ -5163,13 +5163,13 @@
         </is>
       </c>
       <c r="E106" s="4" t="n">
-        <v>268</v>
+        <v>200</v>
       </c>
       <c r="F106" s="5" t="n">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="G106" s="4" t="n">
-        <v>58.96</v>
+        <v>34</v>
       </c>
       <c r="H106" s="2" t="n">
         <v>1402783</v>
@@ -5257,13 +5257,13 @@
         </is>
       </c>
       <c r="E108" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F108" s="5" t="n">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="G108" s="4" t="n">
-        <v>890</v>
+        <v>324</v>
       </c>
       <c r="H108" s="2" t="n">
         <v>1402788</v>
@@ -5351,13 +5351,13 @@
         </is>
       </c>
       <c r="E110" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F110" s="5" t="n">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="G110" s="4" t="n">
-        <v>324</v>
+        <v>890</v>
       </c>
       <c r="H110" s="2" t="n">
         <v>1402788</v>
@@ -5398,13 +5398,13 @@
         </is>
       </c>
       <c r="E111" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F111" s="5" t="n">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="G111" s="4" t="n">
-        <v>324</v>
+        <v>890</v>
       </c>
       <c r="H111" s="2" t="n">
         <v>1402788</v>
@@ -5445,13 +5445,13 @@
         </is>
       </c>
       <c r="E112" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F112" s="5" t="n">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="G112" s="4" t="n">
-        <v>890</v>
+        <v>324</v>
       </c>
       <c r="H112" s="2" t="n">
         <v>1402788</v>
@@ -5636,10 +5636,10 @@
         <v>1</v>
       </c>
       <c r="F116" s="5" t="n">
-        <v>58</v>
+        <v>74.9</v>
       </c>
       <c r="G116" s="4" t="n">
-        <v>58</v>
+        <v>74.9</v>
       </c>
       <c r="H116" s="2" t="n">
         <v>1403644</v>
@@ -5824,10 +5824,10 @@
         <v>1</v>
       </c>
       <c r="F120" s="5" t="n">
-        <v>74.9</v>
+        <v>58</v>
       </c>
       <c r="G120" s="4" t="n">
-        <v>74.9</v>
+        <v>58</v>
       </c>
       <c r="H120" s="2" t="n">
         <v>1403644</v>
@@ -6153,10 +6153,10 @@
         <v>0.2</v>
       </c>
       <c r="F127" s="5" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G127" s="4" t="n">
-        <v>5.6</v>
+        <v>5</v>
       </c>
       <c r="H127" s="2" t="n">
         <v>1403680</v>
@@ -6200,10 +6200,10 @@
         <v>0.2</v>
       </c>
       <c r="F128" s="5" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G128" s="4" t="n">
-        <v>5</v>
+        <v>5.6</v>
       </c>
       <c r="H128" s="2" t="n">
         <v>1403680</v>
@@ -6291,13 +6291,13 @@
         </is>
       </c>
       <c r="E130" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F130" s="5" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G130" s="4" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="H130" s="2" t="n">
         <v>1403680</v>
@@ -6338,13 +6338,13 @@
         </is>
       </c>
       <c r="E131" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F131" s="5" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="G131" s="4" t="n">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="H131" s="2" t="n">
         <v>1403680</v>
@@ -6388,10 +6388,10 @@
         <v>10</v>
       </c>
       <c r="F132" s="5" t="n">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="G132" s="4" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="H132" s="2" t="n">
         <v>1403680</v>
@@ -6432,13 +6432,13 @@
         </is>
       </c>
       <c r="E133" s="4" t="n">
-        <v>1.5</v>
+        <v>10</v>
       </c>
       <c r="F133" s="5" t="n">
-        <v>16</v>
+        <v>3.5</v>
       </c>
       <c r="G133" s="4" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="H133" s="2" t="n">
         <v>1403680</v>
@@ -6479,13 +6479,13 @@
         </is>
       </c>
       <c r="E134" s="4" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="F134" s="5" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="G134" s="4" t="n">
-        <v>4.5</v>
+        <v>5.25</v>
       </c>
       <c r="H134" s="2" t="n">
         <v>1403681</v>
@@ -6529,10 +6529,10 @@
         <v>0.3</v>
       </c>
       <c r="F135" s="5" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="G135" s="4" t="n">
-        <v>30</v>
+        <v>4.5</v>
       </c>
       <c r="H135" s="2" t="n">
         <v>1403681</v>
@@ -6576,10 +6576,10 @@
         <v>0.3</v>
       </c>
       <c r="F136" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="G136" s="4" t="n">
         <v>30</v>
-      </c>
-      <c r="G136" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="H136" s="2" t="n">
         <v>1403681</v>
@@ -6620,13 +6620,13 @@
         </is>
       </c>
       <c r="E137" s="4" t="n">
-        <v>10</v>
+        <v>0.3</v>
       </c>
       <c r="F137" s="5" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G137" s="4" t="n">
-        <v>250</v>
+        <v>9</v>
       </c>
       <c r="H137" s="2" t="n">
         <v>1403681</v>
@@ -6667,13 +6667,13 @@
         </is>
       </c>
       <c r="E138" s="4" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="F138" s="5" t="n">
-        <v>2.22</v>
+        <v>25</v>
       </c>
       <c r="G138" s="4" t="n">
-        <v>222</v>
+        <v>250</v>
       </c>
       <c r="H138" s="2" t="n">
         <v>1403681</v>
@@ -6714,13 +6714,13 @@
         </is>
       </c>
       <c r="E139" s="4" t="n">
-        <v>0.15</v>
+        <v>100</v>
       </c>
       <c r="F139" s="5" t="n">
-        <v>35</v>
+        <v>2.22</v>
       </c>
       <c r="G139" s="4" t="n">
-        <v>5.25</v>
+        <v>222</v>
       </c>
       <c r="H139" s="2" t="n">
         <v>1403681</v>
@@ -10051,13 +10051,13 @@
         </is>
       </c>
       <c r="E210" s="4" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="F210" s="5" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="G210" s="4" t="n">
-        <v>2450</v>
+        <v>840</v>
       </c>
       <c r="H210" s="2" t="n">
         <v>1409782</v>
@@ -10098,13 +10098,13 @@
         </is>
       </c>
       <c r="E211" s="4" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="F211" s="5" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="G211" s="4" t="n">
-        <v>840</v>
+        <v>2450</v>
       </c>
       <c r="H211" s="2" t="n">
         <v>1409782</v>
@@ -10427,13 +10427,13 @@
         </is>
       </c>
       <c r="E218" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F218" s="5" t="n">
         <v>14.9</v>
       </c>
       <c r="G218" s="4" t="n">
-        <v>29.8</v>
+        <v>59.6</v>
       </c>
       <c r="H218" s="2" t="n">
         <v>1410100</v>
@@ -10474,13 +10474,13 @@
         </is>
       </c>
       <c r="E219" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F219" s="5" t="n">
         <v>14.9</v>
       </c>
       <c r="G219" s="4" t="n">
-        <v>59.6</v>
+        <v>29.8</v>
       </c>
       <c r="H219" s="2" t="n">
         <v>1410100</v>
@@ -10521,13 +10521,13 @@
         </is>
       </c>
       <c r="E220" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F220" s="5" t="n">
-        <v>59.9</v>
+        <v>12</v>
       </c>
       <c r="G220" s="4" t="n">
-        <v>59.9</v>
+        <v>24</v>
       </c>
       <c r="H220" s="2" t="n">
         <v>1410100</v>
@@ -10568,13 +10568,13 @@
         </is>
       </c>
       <c r="E221" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F221" s="5" t="n">
-        <v>12</v>
+        <v>59.9</v>
       </c>
       <c r="G221" s="4" t="n">
-        <v>24</v>
+        <v>59.9</v>
       </c>
       <c r="H221" s="2" t="n">
         <v>1410100</v>
@@ -12028,10 +12028,10 @@
         <v>25</v>
       </c>
       <c r="F252" s="5" t="n">
-        <v>0.462</v>
+        <v>0.4701</v>
       </c>
       <c r="G252" s="4" t="n">
-        <v>11.55</v>
+        <v>11.75</v>
       </c>
       <c r="H252" s="2" t="n">
         <v>1415875</v>
@@ -12072,13 +12072,13 @@
         </is>
       </c>
       <c r="E253" s="4" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F253" s="5" t="n">
-        <v>0.4701</v>
+        <v>0.4265</v>
       </c>
       <c r="G253" s="4" t="n">
-        <v>11.75</v>
+        <v>21.33</v>
       </c>
       <c r="H253" s="2" t="n">
         <v>1415875</v>
@@ -12119,13 +12119,13 @@
         </is>
       </c>
       <c r="E254" s="4" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="F254" s="5" t="n">
-        <v>0.4265</v>
+        <v>0.5692</v>
       </c>
       <c r="G254" s="4" t="n">
-        <v>21.33</v>
+        <v>14.23</v>
       </c>
       <c r="H254" s="2" t="n">
         <v>1415875</v>
@@ -12169,10 +12169,10 @@
         <v>25</v>
       </c>
       <c r="F255" s="5" t="n">
-        <v>0.5692</v>
+        <v>0.4265</v>
       </c>
       <c r="G255" s="4" t="n">
-        <v>14.23</v>
+        <v>10.66</v>
       </c>
       <c r="H255" s="2" t="n">
         <v>1415875</v>
@@ -12216,10 +12216,10 @@
         <v>25</v>
       </c>
       <c r="F256" s="5" t="n">
-        <v>0.4265</v>
+        <v>0.462</v>
       </c>
       <c r="G256" s="4" t="n">
-        <v>10.66</v>
+        <v>11.55</v>
       </c>
       <c r="H256" s="2" t="n">
         <v>1415875</v>
@@ -12448,13 +12448,13 @@
         </is>
       </c>
       <c r="E261" s="4" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F261" s="5" t="n">
-        <v>0.17</v>
+        <v>1.33</v>
       </c>
       <c r="G261" s="4" t="n">
-        <v>17</v>
+        <v>66.5</v>
       </c>
       <c r="H261" s="2" t="n">
         <v>1415895</v>
@@ -12495,13 +12495,13 @@
         </is>
       </c>
       <c r="E262" s="4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F262" s="5" t="n">
-        <v>1.33</v>
+        <v>0.17</v>
       </c>
       <c r="G262" s="4" t="n">
-        <v>66.5</v>
+        <v>17</v>
       </c>
       <c r="H262" s="2" t="n">
         <v>1415895</v>
@@ -12542,13 +12542,13 @@
         </is>
       </c>
       <c r="E263" s="4" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="F263" s="5" t="n">
-        <v>9</v>
+        <v>1.33</v>
       </c>
       <c r="G263" s="4" t="n">
-        <v>18</v>
+        <v>66.5</v>
       </c>
       <c r="H263" s="2" t="n">
         <v>1415895</v>
@@ -12589,13 +12589,13 @@
         </is>
       </c>
       <c r="E264" s="4" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="F264" s="5" t="n">
-        <v>1.33</v>
+        <v>15</v>
       </c>
       <c r="G264" s="4" t="n">
-        <v>66.5</v>
+        <v>15</v>
       </c>
       <c r="H264" s="2" t="n">
         <v>1415895</v>
@@ -12636,13 +12636,13 @@
         </is>
       </c>
       <c r="E265" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F265" s="5" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G265" s="4" t="n">
-        <v>15</v>
+        <v>65</v>
       </c>
       <c r="H265" s="2" t="n">
         <v>1415895</v>
@@ -12683,13 +12683,13 @@
         </is>
       </c>
       <c r="E266" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F266" s="5" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G266" s="4" t="n">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="H266" s="2" t="n">
         <v>1415895</v>
@@ -15271,10 +15271,10 @@
         <v>1</v>
       </c>
       <c r="F321" s="5" t="n">
-        <v>44.9</v>
+        <v>32</v>
       </c>
       <c r="G321" s="4" t="n">
-        <v>44.9</v>
+        <v>32</v>
       </c>
       <c r="H321" s="2" t="n">
         <v>1429506</v>
@@ -15318,10 +15318,10 @@
         <v>1</v>
       </c>
       <c r="F322" s="5" t="n">
-        <v>32</v>
+        <v>44.9</v>
       </c>
       <c r="G322" s="4" t="n">
-        <v>32</v>
+        <v>44.9</v>
       </c>
       <c r="H322" s="2" t="n">
         <v>1429506</v>
@@ -15503,13 +15503,13 @@
         </is>
       </c>
       <c r="E326" s="4" t="n">
-        <v>40</v>
+        <v>9</v>
       </c>
       <c r="F326" s="5" t="n">
-        <v>16</v>
+        <v>189</v>
       </c>
       <c r="G326" s="4" t="n">
-        <v>640</v>
+        <v>1701</v>
       </c>
       <c r="H326" s="2" t="n">
         <v>1429513</v>
@@ -15553,10 +15553,10 @@
         <v>9</v>
       </c>
       <c r="F327" s="5" t="n">
-        <v>189</v>
+        <v>130</v>
       </c>
       <c r="G327" s="4" t="n">
-        <v>1701</v>
+        <v>1170</v>
       </c>
       <c r="H327" s="2" t="n">
         <v>1429513</v>
@@ -15597,13 +15597,13 @@
         </is>
       </c>
       <c r="E328" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F328" s="5" t="n">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="G328" s="4" t="n">
-        <v>1170</v>
+        <v>115</v>
       </c>
       <c r="H328" s="2" t="n">
         <v>1429513</v>
@@ -15644,13 +15644,13 @@
         </is>
       </c>
       <c r="E329" s="4" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F329" s="5" t="n">
-        <v>115</v>
+        <v>22</v>
       </c>
       <c r="G329" s="4" t="n">
-        <v>115</v>
+        <v>176</v>
       </c>
       <c r="H329" s="2" t="n">
         <v>1429513</v>
@@ -15691,13 +15691,13 @@
         </is>
       </c>
       <c r="E330" s="4" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="F330" s="5" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="G330" s="4" t="n">
-        <v>176</v>
+        <v>640</v>
       </c>
       <c r="H330" s="2" t="n">
         <v>1429513</v>
@@ -18088,13 +18088,13 @@
         </is>
       </c>
       <c r="E381" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F381" s="5" t="n">
-        <v>3.6</v>
+        <v>30.25</v>
       </c>
       <c r="G381" s="4" t="n">
-        <v>14.4</v>
+        <v>30.25</v>
       </c>
       <c r="H381" s="2" t="n">
         <v>1437076</v>
@@ -18511,13 +18511,13 @@
         </is>
       </c>
       <c r="E390" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F390" s="5" t="n">
-        <v>30.25</v>
+        <v>3.6</v>
       </c>
       <c r="G390" s="4" t="n">
-        <v>30.25</v>
+        <v>14.4</v>
       </c>
       <c r="H390" s="2" t="n">
         <v>1437076</v>
@@ -25984,13 +25984,13 @@
         </is>
       </c>
       <c r="E549" s="4" t="n">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="F549" s="5" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G549" s="4" t="n">
-        <v>27</v>
+        <v>12.8</v>
       </c>
       <c r="H549" s="2" t="n">
         <v>1480786</v>
@@ -26034,10 +26034,10 @@
         <v>1</v>
       </c>
       <c r="F550" s="5" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G550" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="H550" s="2" t="n">
         <v>1480786</v>
@@ -26081,10 +26081,10 @@
         <v>2</v>
       </c>
       <c r="F551" s="5" t="n">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G551" s="4" t="n">
-        <v>28</v>
+        <v>80</v>
       </c>
       <c r="H551" s="2" t="n">
         <v>1480786</v>
@@ -26125,13 +26125,13 @@
         </is>
       </c>
       <c r="E552" s="4" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="F552" s="5" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G552" s="4" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H552" s="2" t="n">
         <v>1480786</v>
@@ -26172,13 +26172,13 @@
         </is>
       </c>
       <c r="E553" s="4" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F553" s="5" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G553" s="4" t="n">
-        <v>12.8</v>
+        <v>15</v>
       </c>
       <c r="H553" s="2" t="n">
         <v>1480786</v>
@@ -26219,13 +26219,13 @@
         </is>
       </c>
       <c r="E554" s="4" t="n">
-        <v>0.25</v>
+        <v>2</v>
       </c>
       <c r="F554" s="5" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G554" s="4" t="n">
-        <v>6.25</v>
+        <v>28</v>
       </c>
       <c r="H554" s="2" t="n">
         <v>1480786</v>
@@ -26266,13 +26266,13 @@
         </is>
       </c>
       <c r="E555" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F555" s="5" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G555" s="4" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="H555" s="2" t="n">
         <v>1480786</v>
@@ -26313,13 +26313,13 @@
         </is>
       </c>
       <c r="E556" s="4" t="n">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="F556" s="5" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="G556" s="4" t="n">
-        <v>80</v>
+        <v>6.25</v>
       </c>
       <c r="H556" s="2" t="n">
         <v>1480786</v>
@@ -26454,13 +26454,13 @@
         </is>
       </c>
       <c r="E559" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F559" s="5" t="n">
-        <v>14.06</v>
+        <v>2.95</v>
       </c>
       <c r="G559" s="4" t="n">
-        <v>14.06</v>
+        <v>5.9</v>
       </c>
       <c r="H559" s="2" t="n">
         <v>1480796</v>
@@ -26501,13 +26501,13 @@
         </is>
       </c>
       <c r="E560" s="4" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="F560" s="5" t="n">
-        <v>2.95</v>
+        <v>4.45</v>
       </c>
       <c r="G560" s="4" t="n">
-        <v>5.9</v>
+        <v>178</v>
       </c>
       <c r="H560" s="2" t="n">
         <v>1480796</v>
@@ -26595,13 +26595,13 @@
         </is>
       </c>
       <c r="E562" s="4" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="F562" s="5" t="n">
-        <v>4.45</v>
+        <v>14.06</v>
       </c>
       <c r="G562" s="4" t="n">
-        <v>178</v>
+        <v>14.06</v>
       </c>
       <c r="H562" s="2" t="n">
         <v>1480796</v>
@@ -26927,10 +26927,10 @@
         <v>1</v>
       </c>
       <c r="F569" s="5" t="n">
-        <v>6.08</v>
+        <v>5.83</v>
       </c>
       <c r="G569" s="4" t="n">
-        <v>6.08</v>
+        <v>5.83</v>
       </c>
       <c r="H569" s="2" t="n">
         <v>1482331</v>
@@ -26974,10 +26974,10 @@
         <v>1</v>
       </c>
       <c r="F570" s="5" t="n">
-        <v>8.23</v>
+        <v>5.74</v>
       </c>
       <c r="G570" s="4" t="n">
-        <v>8.23</v>
+        <v>5.74</v>
       </c>
       <c r="H570" s="2" t="n">
         <v>1482331</v>
@@ -27021,10 +27021,10 @@
         <v>1</v>
       </c>
       <c r="F571" s="5" t="n">
-        <v>5.74</v>
+        <v>31.33</v>
       </c>
       <c r="G571" s="4" t="n">
-        <v>5.74</v>
+        <v>31.33</v>
       </c>
       <c r="H571" s="2" t="n">
         <v>1482331</v>
@@ -27068,10 +27068,10 @@
         <v>1</v>
       </c>
       <c r="F572" s="5" t="n">
-        <v>5.83</v>
+        <v>6.08</v>
       </c>
       <c r="G572" s="4" t="n">
-        <v>5.83</v>
+        <v>6.08</v>
       </c>
       <c r="H572" s="2" t="n">
         <v>1482331</v>
@@ -27115,10 +27115,10 @@
         <v>1</v>
       </c>
       <c r="F573" s="5" t="n">
-        <v>6.16</v>
+        <v>8.23</v>
       </c>
       <c r="G573" s="4" t="n">
-        <v>6.16</v>
+        <v>8.23</v>
       </c>
       <c r="H573" s="2" t="n">
         <v>1482331</v>
@@ -27303,10 +27303,10 @@
         <v>1</v>
       </c>
       <c r="F577" s="5" t="n">
-        <v>31.33</v>
+        <v>6.16</v>
       </c>
       <c r="G577" s="4" t="n">
-        <v>31.33</v>
+        <v>6.16</v>
       </c>
       <c r="H577" s="2" t="n">
         <v>1482331</v>
@@ -27397,10 +27397,10 @@
         <v>1</v>
       </c>
       <c r="F579" s="5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G579" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H579" s="2" t="n">
         <v>1482337</v>
@@ -27441,13 +27441,13 @@
         </is>
       </c>
       <c r="E580" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F580" s="5" t="n">
-        <v>9</v>
+        <v>2.6</v>
       </c>
       <c r="G580" s="4" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H580" s="2" t="n">
         <v>1482337</v>
@@ -27535,13 +27535,13 @@
         </is>
       </c>
       <c r="E582" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F582" s="5" t="n">
         <v>2.6</v>
       </c>
       <c r="G582" s="4" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="H582" s="2" t="n">
         <v>1482337</v>
@@ -27582,13 +27582,13 @@
         </is>
       </c>
       <c r="E583" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F583" s="5" t="n">
-        <v>2.6</v>
+        <v>7</v>
       </c>
       <c r="G583" s="4" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="H583" s="2" t="n">
         <v>1482337</v>
@@ -30734,10 +30734,10 @@
         <v>200</v>
       </c>
       <c r="F650" s="5" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="G650" s="4" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="H650" s="2" t="n">
         <v>1498122</v>
@@ -30781,10 +30781,10 @@
         <v>200</v>
       </c>
       <c r="F651" s="5" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="G651" s="4" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="H651" s="2" t="n">
         <v>1498122</v>
@@ -31063,10 +31063,10 @@
         <v>1</v>
       </c>
       <c r="F657" s="5" t="n">
-        <v>14.08</v>
+        <v>21.8</v>
       </c>
       <c r="G657" s="4" t="n">
-        <v>14.08</v>
+        <v>21.8</v>
       </c>
       <c r="H657" s="2" t="n">
         <v>1499773</v>
@@ -31110,10 +31110,10 @@
         <v>1</v>
       </c>
       <c r="F658" s="5" t="n">
-        <v>21.8</v>
+        <v>14.08</v>
       </c>
       <c r="G658" s="4" t="n">
-        <v>21.8</v>
+        <v>14.08</v>
       </c>
       <c r="H658" s="2" t="n">
         <v>1499773</v>
@@ -31721,10 +31721,10 @@
         <v>2</v>
       </c>
       <c r="F671" s="5" t="n">
-        <v>0.9</v>
+        <v>30</v>
       </c>
       <c r="G671" s="4" t="n">
-        <v>1.8</v>
+        <v>60</v>
       </c>
       <c r="H671" s="2" t="n">
         <v>1503029</v>
@@ -31765,13 +31765,13 @@
         </is>
       </c>
       <c r="E672" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F672" s="5" t="n">
-        <v>30.63</v>
+        <v>0.9</v>
       </c>
       <c r="G672" s="4" t="n">
-        <v>30.63</v>
+        <v>1.8</v>
       </c>
       <c r="H672" s="2" t="n">
         <v>1503029</v>
@@ -31812,13 +31812,13 @@
         </is>
       </c>
       <c r="E673" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F673" s="5" t="n">
-        <v>5.39</v>
+        <v>2.03</v>
       </c>
       <c r="G673" s="4" t="n">
-        <v>5.39</v>
+        <v>4.06</v>
       </c>
       <c r="H673" s="2" t="n">
         <v>1503029</v>
@@ -31859,13 +31859,13 @@
         </is>
       </c>
       <c r="E674" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F674" s="5" t="n">
-        <v>2.03</v>
+        <v>5.39</v>
       </c>
       <c r="G674" s="4" t="n">
-        <v>4.06</v>
+        <v>5.39</v>
       </c>
       <c r="H674" s="2" t="n">
         <v>1503029</v>
@@ -31909,10 +31909,10 @@
         <v>2</v>
       </c>
       <c r="F675" s="5" t="n">
-        <v>30</v>
+        <v>1.01</v>
       </c>
       <c r="G675" s="4" t="n">
-        <v>60</v>
+        <v>2.02</v>
       </c>
       <c r="H675" s="2" t="n">
         <v>1503029</v>
@@ -31953,13 +31953,13 @@
         </is>
       </c>
       <c r="E676" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F676" s="5" t="n">
-        <v>1.01</v>
+        <v>30.63</v>
       </c>
       <c r="G676" s="4" t="n">
-        <v>2.02</v>
+        <v>30.63</v>
       </c>
       <c r="H676" s="2" t="n">
         <v>1503029</v>
@@ -32379,10 +32379,10 @@
         <v>1</v>
       </c>
       <c r="F685" s="5" t="n">
-        <v>4.18</v>
+        <v>13.6</v>
       </c>
       <c r="G685" s="4" t="n">
-        <v>4.18</v>
+        <v>13.6</v>
       </c>
       <c r="H685" s="2" t="n">
         <v>1503440</v>
@@ -32426,10 +32426,10 @@
         <v>1</v>
       </c>
       <c r="F686" s="5" t="n">
-        <v>14.02</v>
+        <v>4.18</v>
       </c>
       <c r="G686" s="4" t="n">
-        <v>14.02</v>
+        <v>4.18</v>
       </c>
       <c r="H686" s="2" t="n">
         <v>1503440</v>
@@ -32473,10 +32473,10 @@
         <v>1</v>
       </c>
       <c r="F687" s="5" t="n">
-        <v>13.6</v>
+        <v>14.02</v>
       </c>
       <c r="G687" s="4" t="n">
-        <v>13.6</v>
+        <v>14.02</v>
       </c>
       <c r="H687" s="2" t="n">
         <v>1503440</v>
@@ -33222,13 +33222,13 @@
         </is>
       </c>
       <c r="E703" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F703" s="5" t="n">
-        <v>27.65</v>
+        <v>2.29</v>
       </c>
       <c r="G703" s="4" t="n">
-        <v>27.65</v>
+        <v>4.58</v>
       </c>
       <c r="H703" s="2" t="n">
         <v>1512391</v>
@@ -33272,10 +33272,10 @@
         <v>2</v>
       </c>
       <c r="F704" s="5" t="n">
-        <v>2.88</v>
+        <v>2.38</v>
       </c>
       <c r="G704" s="4" t="n">
-        <v>5.76</v>
+        <v>4.76</v>
       </c>
       <c r="H704" s="2" t="n">
         <v>1512391</v>
@@ -33316,13 +33316,13 @@
         </is>
       </c>
       <c r="E705" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F705" s="5" t="n">
-        <v>2.38</v>
+        <v>27.65</v>
       </c>
       <c r="G705" s="4" t="n">
-        <v>4.76</v>
+        <v>27.65</v>
       </c>
       <c r="H705" s="2" t="n">
         <v>1512391</v>
@@ -33363,13 +33363,13 @@
         </is>
       </c>
       <c r="E706" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F706" s="5" t="n">
-        <v>15.25</v>
+        <v>2.88</v>
       </c>
       <c r="G706" s="4" t="n">
-        <v>15.25</v>
+        <v>5.76</v>
       </c>
       <c r="H706" s="2" t="n">
         <v>1512391</v>
@@ -33413,10 +33413,10 @@
         <v>1</v>
       </c>
       <c r="F707" s="5" t="n">
-        <v>10.3</v>
+        <v>12.25</v>
       </c>
       <c r="G707" s="4" t="n">
-        <v>10.3</v>
+        <v>12.25</v>
       </c>
       <c r="H707" s="2" t="n">
         <v>1512391</v>
@@ -33460,10 +33460,10 @@
         <v>1</v>
       </c>
       <c r="F708" s="5" t="n">
-        <v>12.25</v>
+        <v>10.3</v>
       </c>
       <c r="G708" s="4" t="n">
-        <v>12.25</v>
+        <v>10.3</v>
       </c>
       <c r="H708" s="2" t="n">
         <v>1512391</v>
@@ -33504,13 +33504,13 @@
         </is>
       </c>
       <c r="E709" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F709" s="5" t="n">
-        <v>2.29</v>
+        <v>15.25</v>
       </c>
       <c r="G709" s="4" t="n">
-        <v>4.58</v>
+        <v>15.25</v>
       </c>
       <c r="H709" s="2" t="n">
         <v>1512391</v>
@@ -33598,13 +33598,13 @@
         </is>
       </c>
       <c r="E711" s="4" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="F711" s="5" t="n">
-        <v>0.22</v>
+        <v>0.3</v>
       </c>
       <c r="G711" s="4" t="n">
-        <v>22</v>
+        <v>4.5</v>
       </c>
       <c r="H711" s="2" t="n">
         <v>1512750</v>
@@ -33645,13 +33645,13 @@
         </is>
       </c>
       <c r="E712" s="4" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="F712" s="5" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="G712" s="4" t="n">
-        <v>15</v>
+        <v>2.55</v>
       </c>
       <c r="H712" s="2" t="n">
         <v>1512750</v>
@@ -33739,13 +33739,13 @@
         </is>
       </c>
       <c r="E714" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F714" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G714" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="F714" s="5" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="G714" s="4" t="n">
-        <v>2.55</v>
       </c>
       <c r="H714" s="2" t="n">
         <v>1512750</v>
@@ -33789,10 +33789,10 @@
         <v>15</v>
       </c>
       <c r="F715" s="5" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="G715" s="4" t="n">
-        <v>4.5</v>
+        <v>12</v>
       </c>
       <c r="H715" s="2" t="n">
         <v>1512750</v>
@@ -33833,13 +33833,13 @@
         </is>
       </c>
       <c r="E716" s="4" t="n">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="F716" s="5" t="n">
-        <v>0.8</v>
+        <v>0.22</v>
       </c>
       <c r="G716" s="4" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="H716" s="2" t="n">
         <v>1512750</v>
@@ -34021,13 +34021,13 @@
         </is>
       </c>
       <c r="E720" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F720" s="5" t="n">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="G720" s="4" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="H720" s="2" t="n">
         <v>1513521</v>
@@ -34068,13 +34068,13 @@
         </is>
       </c>
       <c r="E721" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F721" s="5" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="G721" s="4" t="n">
-        <v>35</v>
+        <v>170</v>
       </c>
       <c r="H721" s="2" t="n">
         <v>1513521</v>
@@ -34165,10 +34165,10 @@
         <v>1</v>
       </c>
       <c r="F723" s="5" t="n">
-        <v>197.5</v>
+        <v>192.5</v>
       </c>
       <c r="G723" s="4" t="n">
-        <v>197.5</v>
+        <v>192.5</v>
       </c>
       <c r="H723" s="2" t="n">
         <v>1513541</v>
@@ -34212,10 +34212,10 @@
         <v>1</v>
       </c>
       <c r="F724" s="5" t="n">
-        <v>192.5</v>
+        <v>197.5</v>
       </c>
       <c r="G724" s="4" t="n">
-        <v>192.5</v>
+        <v>197.5</v>
       </c>
       <c r="H724" s="2" t="n">
         <v>1513541</v>
@@ -34259,10 +34259,10 @@
         <v>1</v>
       </c>
       <c r="F725" s="5" t="n">
-        <v>157.85</v>
+        <v>170.39</v>
       </c>
       <c r="G725" s="4" t="n">
-        <v>157.85</v>
+        <v>170.39</v>
       </c>
       <c r="H725" s="2" t="n">
         <v>1513749</v>
@@ -34306,10 +34306,10 @@
         <v>1</v>
       </c>
       <c r="F726" s="5" t="n">
-        <v>170.39</v>
+        <v>157.85</v>
       </c>
       <c r="G726" s="4" t="n">
-        <v>170.39</v>
+        <v>157.85</v>
       </c>
       <c r="H726" s="2" t="n">
         <v>1513749</v>
@@ -34444,13 +34444,13 @@
         </is>
       </c>
       <c r="E729" s="4" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="F729" s="5" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="G729" s="4" t="n">
-        <v>2000</v>
+        <v>750</v>
       </c>
       <c r="H729" s="2" t="n">
         <v>1513779</v>
@@ -34491,13 +34491,13 @@
         </is>
       </c>
       <c r="E730" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F730" s="5" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="G730" s="4" t="n">
-        <v>1000</v>
+        <v>750</v>
       </c>
       <c r="H730" s="2" t="n">
         <v>1513779</v>
@@ -34538,13 +34538,13 @@
         </is>
       </c>
       <c r="E731" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F731" s="5" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G731" s="4" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="H731" s="2" t="n">
         <v>1513779</v>
@@ -34585,13 +34585,13 @@
         </is>
       </c>
       <c r="E732" s="4" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="F732" s="5" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G732" s="4" t="n">
-        <v>750</v>
+        <v>2000</v>
       </c>
       <c r="H732" s="2" t="n">
         <v>1513779</v>
@@ -34679,13 +34679,13 @@
         </is>
       </c>
       <c r="E734" s="4" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F734" s="5" t="n">
-        <v>5.57</v>
+        <v>4.05</v>
       </c>
       <c r="G734" s="4" t="n">
-        <v>66.84</v>
+        <v>4.05</v>
       </c>
       <c r="H734" s="2" t="n">
         <v>1513837</v>
@@ -34726,13 +34726,13 @@
         </is>
       </c>
       <c r="E735" s="4" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F735" s="5" t="n">
-        <v>4.05</v>
+        <v>5.57</v>
       </c>
       <c r="G735" s="4" t="n">
-        <v>4.05</v>
+        <v>66.84</v>
       </c>
       <c r="H735" s="2" t="n">
         <v>1513837</v>
@@ -37170,13 +37170,13 @@
         </is>
       </c>
       <c r="E787" s="4" t="n">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="F787" s="5" t="n">
-        <v>127.6</v>
+        <v>54.3</v>
       </c>
       <c r="G787" s="4" t="n">
-        <v>1786.4</v>
+        <v>3746.7</v>
       </c>
       <c r="H787" s="2" t="n">
         <v>1522616</v>
@@ -37217,13 +37217,13 @@
         </is>
       </c>
       <c r="E788" s="4" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="F788" s="5" t="n">
-        <v>153.6</v>
+        <v>139.6</v>
       </c>
       <c r="G788" s="4" t="n">
-        <v>2457.6</v>
+        <v>279.2</v>
       </c>
       <c r="H788" s="2" t="n">
         <v>1522616</v>
@@ -37264,13 +37264,13 @@
         </is>
       </c>
       <c r="E789" s="4" t="n">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="F789" s="5" t="n">
-        <v>54.3</v>
+        <v>127.6</v>
       </c>
       <c r="G789" s="4" t="n">
-        <v>3746.7</v>
+        <v>1786.4</v>
       </c>
       <c r="H789" s="2" t="n">
         <v>1522616</v>
@@ -37311,13 +37311,13 @@
         </is>
       </c>
       <c r="E790" s="4" t="n">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="F790" s="5" t="n">
-        <v>139.6</v>
+        <v>127.6</v>
       </c>
       <c r="G790" s="4" t="n">
-        <v>279.2</v>
+        <v>4593.6</v>
       </c>
       <c r="H790" s="2" t="n">
         <v>1522616</v>
@@ -37358,13 +37358,13 @@
         </is>
       </c>
       <c r="E791" s="4" t="n">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="F791" s="5" t="n">
-        <v>127.6</v>
+        <v>153.6</v>
       </c>
       <c r="G791" s="4" t="n">
-        <v>4593.6</v>
+        <v>2457.6</v>
       </c>
       <c r="H791" s="2" t="n">
         <v>1522616</v>
@@ -38580,13 +38580,13 @@
         </is>
       </c>
       <c r="E817" s="4" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F817" s="5" t="n">
-        <v>3.89</v>
+        <v>9.59</v>
       </c>
       <c r="G817" s="4" t="n">
-        <v>58.35</v>
+        <v>9.59</v>
       </c>
       <c r="H817" s="2" t="n">
         <v>1526079</v>
@@ -38627,13 +38627,13 @@
         </is>
       </c>
       <c r="E818" s="4" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F818" s="5" t="n">
-        <v>9.59</v>
+        <v>3.89</v>
       </c>
       <c r="G818" s="4" t="n">
-        <v>9.59</v>
+        <v>58.35</v>
       </c>
       <c r="H818" s="2" t="n">
         <v>1526079</v>
@@ -38721,13 +38721,13 @@
         </is>
       </c>
       <c r="E820" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F820" s="5" t="n">
-        <v>8.99</v>
+        <v>17.5</v>
       </c>
       <c r="G820" s="4" t="n">
-        <v>17.98</v>
+        <v>17.5</v>
       </c>
       <c r="H820" s="2" t="n">
         <v>1526335</v>
@@ -38768,13 +38768,13 @@
         </is>
       </c>
       <c r="E821" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F821" s="5" t="n">
-        <v>17.5</v>
+        <v>8.99</v>
       </c>
       <c r="G821" s="4" t="n">
-        <v>17.5</v>
+        <v>17.98</v>
       </c>
       <c r="H821" s="2" t="n">
         <v>1526335</v>
@@ -40087,10 +40087,10 @@
         <v>1</v>
       </c>
       <c r="F849" s="5" t="n">
-        <v>180.4</v>
+        <v>306.68</v>
       </c>
       <c r="G849" s="4" t="n">
-        <v>180.4</v>
+        <v>306.68</v>
       </c>
       <c r="H849" s="2" t="n">
         <v>1530930</v>
@@ -40134,10 +40134,10 @@
         <v>1</v>
       </c>
       <c r="F850" s="5" t="n">
-        <v>306.68</v>
+        <v>180.4</v>
       </c>
       <c r="G850" s="4" t="n">
-        <v>306.68</v>
+        <v>180.4</v>
       </c>
       <c r="H850" s="2" t="n">
         <v>1530930</v>
@@ -40322,10 +40322,10 @@
         <v>1.5</v>
       </c>
       <c r="F854" s="5" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G854" s="4" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H854" s="2" t="n">
         <v>1532084</v>
@@ -40416,10 +40416,10 @@
         <v>1</v>
       </c>
       <c r="F856" s="5" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G856" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H856" s="2" t="n">
         <v>1532084</v>
@@ -40460,13 +40460,13 @@
         </is>
       </c>
       <c r="E857" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F857" s="5" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G857" s="4" t="n">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="H857" s="2" t="n">
         <v>1532084</v>
@@ -40507,13 +40507,13 @@
         </is>
       </c>
       <c r="E858" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F858" s="5" t="n">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="G858" s="4" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="H858" s="2" t="n">
         <v>1532084</v>
@@ -40554,13 +40554,13 @@
         </is>
       </c>
       <c r="E859" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F859" s="5" t="n">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="G859" s="4" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="H859" s="2" t="n">
         <v>1532084</v>
@@ -40601,13 +40601,13 @@
         </is>
       </c>
       <c r="E860" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F860" s="5" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G860" s="4" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="H860" s="2" t="n">
         <v>1532084</v>
@@ -43139,13 +43139,13 @@
         </is>
       </c>
       <c r="E914" s="4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F914" s="5" t="n">
-        <v>0.25</v>
+        <v>53</v>
       </c>
       <c r="G914" s="4" t="n">
-        <v>2</v>
+        <v>53</v>
       </c>
       <c r="H914" s="2" t="n">
         <v>1539898</v>
@@ -43280,13 +43280,13 @@
         </is>
       </c>
       <c r="E917" s="4" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F917" s="5" t="n">
-        <v>53</v>
+        <v>0.25</v>
       </c>
       <c r="G917" s="4" t="n">
-        <v>53</v>
+        <v>2</v>
       </c>
       <c r="H917" s="2" t="n">
         <v>1539898</v>
@@ -43847,10 +43847,10 @@
         <v>0.28</v>
       </c>
       <c r="F929" s="5" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="G929" s="4" t="n">
-        <v>28</v>
+        <v>4.2</v>
       </c>
       <c r="H929" s="2" t="n">
         <v>1546014</v>
@@ -43891,13 +43891,13 @@
         </is>
       </c>
       <c r="E930" s="4" t="n">
-        <v>0.1</v>
+        <v>0.28</v>
       </c>
       <c r="F930" s="5" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="G930" s="4" t="n">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="H930" s="2" t="n">
         <v>1546014</v>
@@ -43938,13 +43938,13 @@
         </is>
       </c>
       <c r="E931" s="4" t="n">
-        <v>0.28</v>
+        <v>0.16</v>
       </c>
       <c r="F931" s="5" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="G931" s="4" t="n">
-        <v>8.4</v>
+        <v>5.6</v>
       </c>
       <c r="H931" s="2" t="n">
         <v>1546014</v>
@@ -43985,13 +43985,13 @@
         </is>
       </c>
       <c r="E932" s="4" t="n">
-        <v>1</v>
+        <v>0.04</v>
       </c>
       <c r="F932" s="5" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="G932" s="4" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="H932" s="2" t="n">
         <v>1546014</v>
@@ -44032,13 +44032,13 @@
         </is>
       </c>
       <c r="E933" s="4" t="n">
-        <v>0.28</v>
+        <v>1</v>
       </c>
       <c r="F933" s="5" t="n">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="G933" s="4" t="n">
-        <v>4.2</v>
+        <v>70</v>
       </c>
       <c r="H933" s="2" t="n">
         <v>1546014</v>
@@ -44079,13 +44079,13 @@
         </is>
       </c>
       <c r="E934" s="4" t="n">
-        <v>0.28</v>
+        <v>0.1</v>
       </c>
       <c r="F934" s="5" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="G934" s="4" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="H934" s="2" t="n">
         <v>1546014</v>
@@ -44126,13 +44126,13 @@
         </is>
       </c>
       <c r="E935" s="4" t="n">
-        <v>0.16</v>
+        <v>0.28</v>
       </c>
       <c r="F935" s="5" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G935" s="4" t="n">
-        <v>5.6</v>
+        <v>8.4</v>
       </c>
       <c r="H935" s="2" t="n">
         <v>1546014</v>
@@ -44173,13 +44173,13 @@
         </is>
       </c>
       <c r="E936" s="4" t="n">
-        <v>0.04</v>
+        <v>0.28</v>
       </c>
       <c r="F936" s="5" t="n">
         <v>100</v>
       </c>
       <c r="G936" s="4" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="H936" s="2" t="n">
         <v>1546014</v>
@@ -44364,10 +44364,10 @@
         <v>1</v>
       </c>
       <c r="F940" s="5" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="G940" s="4" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="H940" s="2" t="n">
         <v>1547044</v>
@@ -44599,10 +44599,10 @@
         <v>1</v>
       </c>
       <c r="F945" s="5" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="G945" s="4" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="H945" s="2" t="n">
         <v>1547044</v>
@@ -49531,13 +49531,13 @@
         </is>
       </c>
       <c r="E1050" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1050" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G1050" s="4" t="n">
-        <v>14</v>
+        <v>7.5</v>
       </c>
       <c r="H1050" s="2" t="n">
         <v>1565694</v>
@@ -49578,13 +49578,13 @@
         </is>
       </c>
       <c r="E1051" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1051" s="5" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G1051" s="4" t="n">
-        <v>7.5</v>
+        <v>22</v>
       </c>
       <c r="H1051" s="2" t="n">
         <v>1565694</v>
@@ -49625,13 +49625,13 @@
         </is>
       </c>
       <c r="E1052" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1052" s="5" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G1052" s="4" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H1052" s="2" t="n">
         <v>1565694</v>
@@ -49675,10 +49675,10 @@
         <v>100</v>
       </c>
       <c r="F1053" s="5" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="G1053" s="4" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H1053" s="2" t="n">
         <v>1565694</v>
@@ -50095,13 +50095,13 @@
         </is>
       </c>
       <c r="E1062" s="4" t="n">
-        <v>0.11</v>
+        <v>1</v>
       </c>
       <c r="F1062" s="5" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G1062" s="4" t="n">
-        <v>2.75</v>
+        <v>14</v>
       </c>
       <c r="H1062" s="2" t="n">
         <v>1565694</v>
@@ -50142,13 +50142,13 @@
         </is>
       </c>
       <c r="E1063" s="4" t="n">
-        <v>5</v>
+        <v>0.11</v>
       </c>
       <c r="F1063" s="5" t="n">
-        <v>0.3</v>
+        <v>25</v>
       </c>
       <c r="G1063" s="4" t="n">
-        <v>1.5</v>
+        <v>2.75</v>
       </c>
       <c r="H1063" s="2" t="n">
         <v>1565694</v>
@@ -50377,13 +50377,13 @@
         </is>
       </c>
       <c r="E1068" s="4" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="F1068" s="5" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="G1068" s="4" t="n">
-        <v>25</v>
+        <v>1.5</v>
       </c>
       <c r="H1068" s="2" t="n">
         <v>1565694</v>
@@ -50424,13 +50424,13 @@
         </is>
       </c>
       <c r="E1069" s="4" t="n">
-        <v>0.5</v>
+        <v>100</v>
       </c>
       <c r="F1069" s="5" t="n">
-        <v>20</v>
+        <v>0.22</v>
       </c>
       <c r="G1069" s="4" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="H1069" s="2" t="n">
         <v>1565694</v>
@@ -50847,13 +50847,13 @@
         </is>
       </c>
       <c r="E1078" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F1078" s="5" t="n">
-        <v>24.96</v>
+        <v>9</v>
       </c>
       <c r="G1078" s="4" t="n">
-        <v>74.88</v>
+        <v>18</v>
       </c>
       <c r="H1078" s="2" t="n">
         <v>1570182</v>
@@ -50894,13 +50894,13 @@
         </is>
       </c>
       <c r="E1079" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F1079" s="5" t="n">
-        <v>9.712</v>
+        <v>24.96</v>
       </c>
       <c r="G1079" s="4" t="n">
-        <v>9.71</v>
+        <v>74.88</v>
       </c>
       <c r="H1079" s="2" t="n">
         <v>1570182</v>
@@ -50941,13 +50941,13 @@
         </is>
       </c>
       <c r="E1080" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1080" s="5" t="n">
-        <v>10.4</v>
+        <v>5.8</v>
       </c>
       <c r="G1080" s="4" t="n">
-        <v>10.4</v>
+        <v>11.6</v>
       </c>
       <c r="H1080" s="2" t="n">
         <v>1570182</v>
@@ -50988,13 +50988,13 @@
         </is>
       </c>
       <c r="E1081" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F1081" s="5" t="n">
-        <v>6.624</v>
+        <v>5.12</v>
       </c>
       <c r="G1081" s="4" t="n">
-        <v>6.62</v>
+        <v>20.48</v>
       </c>
       <c r="H1081" s="2" t="n">
         <v>1570182</v>
@@ -51035,13 +51035,13 @@
         </is>
       </c>
       <c r="E1082" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F1082" s="5" t="n">
-        <v>5.12</v>
+        <v>9.712</v>
       </c>
       <c r="G1082" s="4" t="n">
-        <v>20.48</v>
+        <v>9.71</v>
       </c>
       <c r="H1082" s="2" t="n">
         <v>1570182</v>
@@ -51085,10 +51085,10 @@
         <v>1</v>
       </c>
       <c r="F1083" s="5" t="n">
-        <v>12</v>
+        <v>10.4</v>
       </c>
       <c r="G1083" s="4" t="n">
-        <v>12</v>
+        <v>10.4</v>
       </c>
       <c r="H1083" s="2" t="n">
         <v>1570182</v>
@@ -51129,13 +51129,13 @@
         </is>
       </c>
       <c r="E1084" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1084" s="5" t="n">
-        <v>18.66</v>
+        <v>6.624</v>
       </c>
       <c r="G1084" s="4" t="n">
-        <v>37.32</v>
+        <v>6.62</v>
       </c>
       <c r="H1084" s="2" t="n">
         <v>1570182</v>
@@ -51223,13 +51223,13 @@
         </is>
       </c>
       <c r="E1086" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1086" s="5" t="n">
         <v>9</v>
       </c>
       <c r="G1086" s="4" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="H1086" s="2" t="n">
         <v>1570182</v>
@@ -51270,13 +51270,13 @@
         </is>
       </c>
       <c r="E1087" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1087" s="5" t="n">
-        <v>5.8</v>
+        <v>12</v>
       </c>
       <c r="G1087" s="4" t="n">
-        <v>11.6</v>
+        <v>12</v>
       </c>
       <c r="H1087" s="2" t="n">
         <v>1570182</v>
@@ -51317,13 +51317,13 @@
         </is>
       </c>
       <c r="E1088" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1088" s="5" t="n">
-        <v>9</v>
+        <v>18.66</v>
       </c>
       <c r="G1088" s="4" t="n">
-        <v>9</v>
+        <v>37.32</v>
       </c>
       <c r="H1088" s="2" t="n">
         <v>1570182</v>
@@ -51411,13 +51411,13 @@
         </is>
       </c>
       <c r="E1090" s="4" t="n">
-        <v>3</v>
+        <v>0.15</v>
       </c>
       <c r="F1090" s="5" t="n">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="G1090" s="4" t="n">
-        <v>12</v>
+        <v>6.75</v>
       </c>
       <c r="H1090" s="2" t="n">
         <v>1570192</v>
@@ -51458,13 +51458,13 @@
         </is>
       </c>
       <c r="E1091" s="4" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="F1091" s="5" t="n">
-        <v>7</v>
+        <v>90</v>
       </c>
       <c r="G1091" s="4" t="n">
-        <v>2.1</v>
+        <v>13.5</v>
       </c>
       <c r="H1091" s="2" t="n">
         <v>1570192</v>
@@ -51508,10 +51508,10 @@
         <v>0.3</v>
       </c>
       <c r="F1092" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G1092" s="4" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="H1092" s="2" t="n">
         <v>1570192</v>
@@ -51552,13 +51552,13 @@
         </is>
       </c>
       <c r="E1093" s="4" t="n">
-        <v>0.15</v>
+        <v>3</v>
       </c>
       <c r="F1093" s="5" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="G1093" s="4" t="n">
-        <v>13.5</v>
+        <v>12</v>
       </c>
       <c r="H1093" s="2" t="n">
         <v>1570192</v>
@@ -51599,13 +51599,13 @@
         </is>
       </c>
       <c r="E1094" s="4" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
       <c r="F1094" s="5" t="n">
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="G1094" s="4" t="n">
-        <v>6.75</v>
+        <v>60</v>
       </c>
       <c r="H1094" s="2" t="n">
         <v>1570192</v>
@@ -51646,13 +51646,13 @@
         </is>
       </c>
       <c r="E1095" s="4" t="n">
-        <v>0.15</v>
+        <v>1</v>
       </c>
       <c r="F1095" s="5" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G1095" s="4" t="n">
-        <v>4.8</v>
+        <v>30</v>
       </c>
       <c r="H1095" s="2" t="n">
         <v>1570192</v>
@@ -51693,13 +51693,13 @@
         </is>
       </c>
       <c r="E1096" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1096" s="5" t="n">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="G1096" s="4" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H1096" s="2" t="n">
         <v>1570192</v>
@@ -51740,13 +51740,13 @@
         </is>
       </c>
       <c r="E1097" s="4" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
       <c r="F1097" s="5" t="n">
         <v>45</v>
       </c>
       <c r="G1097" s="4" t="n">
-        <v>6.75</v>
+        <v>22.5</v>
       </c>
       <c r="H1097" s="2" t="n">
         <v>1570192</v>
@@ -51787,13 +51787,13 @@
         </is>
       </c>
       <c r="E1098" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="F1098" s="5" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="G1098" s="4" t="n">
-        <v>30</v>
+        <v>1.8</v>
       </c>
       <c r="H1098" s="2" t="n">
         <v>1570192</v>
@@ -51834,13 +51834,13 @@
         </is>
       </c>
       <c r="E1099" s="4" t="n">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="F1099" s="5" t="n">
-        <v>30</v>
+        <v>350</v>
       </c>
       <c r="G1099" s="4" t="n">
-        <v>30</v>
+        <v>3.5</v>
       </c>
       <c r="H1099" s="2" t="n">
         <v>1570192</v>
@@ -51881,13 +51881,13 @@
         </is>
       </c>
       <c r="E1100" s="4" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="F1100" s="5" t="n">
-        <v>45</v>
+        <v>170</v>
       </c>
       <c r="G1100" s="4" t="n">
-        <v>22.5</v>
+        <v>42.5</v>
       </c>
       <c r="H1100" s="2" t="n">
         <v>1570192</v>
@@ -51928,13 +51928,13 @@
         </is>
       </c>
       <c r="E1101" s="4" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="F1101" s="5" t="n">
-        <v>170</v>
+        <v>60</v>
       </c>
       <c r="G1101" s="4" t="n">
-        <v>42.5</v>
+        <v>30</v>
       </c>
       <c r="H1101" s="2" t="n">
         <v>1570192</v>
@@ -51975,13 +51975,13 @@
         </is>
       </c>
       <c r="E1102" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1102" s="5" t="n">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="G1102" s="4" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="H1102" s="2" t="n">
         <v>1570192</v>
@@ -52022,13 +52022,13 @@
         </is>
       </c>
       <c r="E1103" s="4" t="n">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="F1103" s="5" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="G1103" s="4" t="n">
-        <v>22</v>
+        <v>4.8</v>
       </c>
       <c r="H1103" s="2" t="n">
         <v>1570192</v>
@@ -52069,13 +52069,13 @@
         </is>
       </c>
       <c r="E1104" s="4" t="n">
-        <v>0.01</v>
+        <v>0.15</v>
       </c>
       <c r="F1104" s="5" t="n">
-        <v>350</v>
+        <v>45</v>
       </c>
       <c r="G1104" s="4" t="n">
-        <v>3.5</v>
+        <v>6.75</v>
       </c>
       <c r="H1104" s="2" t="n">
         <v>1570192</v>
@@ -52589,10 +52589,10 @@
         <v>1</v>
       </c>
       <c r="F1115" s="5" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G1115" s="4" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H1115" s="2" t="n">
         <v>1573232</v>
@@ -52636,10 +52636,10 @@
         <v>1</v>
       </c>
       <c r="F1116" s="5" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="G1116" s="4" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H1116" s="2" t="n">
         <v>1573232</v>
@@ -53247,10 +53247,10 @@
         <v>1</v>
       </c>
       <c r="F1129" s="5" t="n">
-        <v>13.9</v>
+        <v>7.9</v>
       </c>
       <c r="G1129" s="4" t="n">
-        <v>13.9</v>
+        <v>7.9</v>
       </c>
       <c r="H1129" s="2" t="n">
         <v>1575575</v>
@@ -53294,10 +53294,10 @@
         <v>1</v>
       </c>
       <c r="F1130" s="5" t="n">
-        <v>7.9</v>
+        <v>4.3</v>
       </c>
       <c r="G1130" s="4" t="n">
-        <v>7.9</v>
+        <v>4.3</v>
       </c>
       <c r="H1130" s="2" t="n">
         <v>1575575</v>
@@ -53435,10 +53435,10 @@
         <v>1</v>
       </c>
       <c r="F1133" s="5" t="n">
-        <v>1.4</v>
+        <v>13.9</v>
       </c>
       <c r="G1133" s="4" t="n">
-        <v>1.4</v>
+        <v>13.9</v>
       </c>
       <c r="H1133" s="2" t="n">
         <v>1575575</v>
@@ -53482,10 +53482,10 @@
         <v>1</v>
       </c>
       <c r="F1134" s="5" t="n">
-        <v>4.3</v>
+        <v>1.4</v>
       </c>
       <c r="G1134" s="4" t="n">
-        <v>4.3</v>
+        <v>1.4</v>
       </c>
       <c r="H1134" s="2" t="n">
         <v>1575575</v>
@@ -57803,10 +57803,10 @@
         </is>
       </c>
       <c r="E1226" s="4" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="F1226" s="5" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="G1226" s="4" t="n">
         <v>15</v>
@@ -57850,13 +57850,13 @@
         </is>
       </c>
       <c r="E1227" s="4" t="n">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="F1227" s="5" t="n">
-        <v>22</v>
+        <v>190</v>
       </c>
       <c r="G1227" s="4" t="n">
-        <v>22</v>
+        <v>28.5</v>
       </c>
       <c r="H1227" s="2" t="n">
         <v>1589380</v>
@@ -57897,13 +57897,13 @@
         </is>
       </c>
       <c r="E1228" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F1228" s="5" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="G1228" s="4" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="H1228" s="2" t="n">
         <v>1589380</v>
@@ -57944,10 +57944,10 @@
         </is>
       </c>
       <c r="E1229" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F1229" s="5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G1229" s="4" t="n">
         <v>15</v>
@@ -57991,13 +57991,13 @@
         </is>
       </c>
       <c r="E1230" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1230" s="5" t="n">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="G1230" s="4" t="n">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="H1230" s="2" t="n">
         <v>1589380</v>
@@ -58038,13 +58038,13 @@
         </is>
       </c>
       <c r="E1231" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1231" s="5" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="G1231" s="4" t="n">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="H1231" s="2" t="n">
         <v>1589380</v>
@@ -58088,10 +58088,10 @@
         <v>0.5</v>
       </c>
       <c r="F1232" s="5" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="G1232" s="4" t="n">
-        <v>12.5</v>
+        <v>9</v>
       </c>
       <c r="H1232" s="2" t="n">
         <v>1589380</v>
@@ -58132,13 +58132,13 @@
         </is>
       </c>
       <c r="E1233" s="4" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="F1233" s="5" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="G1233" s="4" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="H1233" s="2" t="n">
         <v>1589380</v>
@@ -58179,13 +58179,13 @@
         </is>
       </c>
       <c r="E1234" s="4" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="F1234" s="5" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="G1234" s="4" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="H1234" s="2" t="n">
         <v>1589380</v>
@@ -58229,10 +58229,10 @@
         <v>0.5</v>
       </c>
       <c r="F1235" s="5" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G1235" s="4" t="n">
-        <v>9</v>
+        <v>12.5</v>
       </c>
       <c r="H1235" s="2" t="n">
         <v>1589380</v>
@@ -58273,13 +58273,13 @@
         </is>
       </c>
       <c r="E1236" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1236" s="5" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="G1236" s="4" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="H1236" s="2" t="n">
         <v>1589380</v>
@@ -58320,13 +58320,13 @@
         </is>
       </c>
       <c r="E1237" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1237" s="5" t="n">
-        <v>120</v>
+        <v>20</v>
       </c>
       <c r="G1237" s="4" t="n">
-        <v>120</v>
+        <v>10</v>
       </c>
       <c r="H1237" s="2" t="n">
         <v>1589380</v>
@@ -58367,13 +58367,13 @@
         </is>
       </c>
       <c r="E1238" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1238" s="5" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G1238" s="4" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H1238" s="2" t="n">
         <v>1589380</v>
@@ -58414,13 +58414,13 @@
         </is>
       </c>
       <c r="E1239" s="4" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F1239" s="5" t="n">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="G1239" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H1239" s="2" t="n">
         <v>1589380</v>
@@ -58461,13 +58461,13 @@
         </is>
       </c>
       <c r="E1240" s="4" t="n">
-        <v>0.15</v>
+        <v>1.5</v>
       </c>
       <c r="F1240" s="5" t="n">
-        <v>190</v>
+        <v>6</v>
       </c>
       <c r="G1240" s="4" t="n">
-        <v>28.5</v>
+        <v>9</v>
       </c>
       <c r="H1240" s="2" t="n">
         <v>1589380</v>
@@ -58508,10 +58508,10 @@
         </is>
       </c>
       <c r="E1241" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F1241" s="5" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G1241" s="4" t="n">
         <v>15</v>
@@ -59683,13 +59683,13 @@
         </is>
       </c>
       <c r="E1266" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F1266" s="5" t="n">
-        <v>2.66</v>
+        <v>1.29</v>
       </c>
       <c r="G1266" s="4" t="n">
-        <v>15.96</v>
+        <v>5.16</v>
       </c>
       <c r="H1266" s="2" t="n">
         <v>1591999</v>
@@ -59730,13 +59730,13 @@
         </is>
       </c>
       <c r="E1267" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F1267" s="5" t="n">
-        <v>1.29</v>
+        <v>14.23</v>
       </c>
       <c r="G1267" s="4" t="n">
-        <v>5.16</v>
+        <v>14.23</v>
       </c>
       <c r="H1267" s="2" t="n">
         <v>1591999</v>
@@ -59777,13 +59777,13 @@
         </is>
       </c>
       <c r="E1268" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F1268" s="5" t="n">
-        <v>13.17</v>
+        <v>2.66</v>
       </c>
       <c r="G1268" s="4" t="n">
-        <v>26.34</v>
+        <v>15.96</v>
       </c>
       <c r="H1268" s="2" t="n">
         <v>1591999</v>
@@ -59824,13 +59824,13 @@
         </is>
       </c>
       <c r="E1269" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1269" s="5" t="n">
-        <v>14.23</v>
+        <v>3.25</v>
       </c>
       <c r="G1269" s="4" t="n">
-        <v>14.23</v>
+        <v>6.5</v>
       </c>
       <c r="H1269" s="2" t="n">
         <v>1591999</v>
@@ -59871,13 +59871,13 @@
         </is>
       </c>
       <c r="E1270" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1270" s="5" t="n">
-        <v>3.25</v>
+        <v>215.83</v>
       </c>
       <c r="G1270" s="4" t="n">
-        <v>6.5</v>
+        <v>215.83</v>
       </c>
       <c r="H1270" s="2" t="n">
         <v>1591999</v>
@@ -59921,10 +59921,10 @@
         <v>1</v>
       </c>
       <c r="F1271" s="5" t="n">
-        <v>215.83</v>
+        <v>29.93</v>
       </c>
       <c r="G1271" s="4" t="n">
-        <v>215.83</v>
+        <v>29.93</v>
       </c>
       <c r="H1271" s="2" t="n">
         <v>1591999</v>
@@ -59965,13 +59965,13 @@
         </is>
       </c>
       <c r="E1272" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1272" s="5" t="n">
-        <v>238.35</v>
+        <v>13.17</v>
       </c>
       <c r="G1272" s="4" t="n">
-        <v>238.35</v>
+        <v>26.34</v>
       </c>
       <c r="H1272" s="2" t="n">
         <v>1591999</v>
@@ -60015,10 +60015,10 @@
         <v>1</v>
       </c>
       <c r="F1273" s="5" t="n">
-        <v>41.71</v>
+        <v>238.35</v>
       </c>
       <c r="G1273" s="4" t="n">
-        <v>41.71</v>
+        <v>238.35</v>
       </c>
       <c r="H1273" s="2" t="n">
         <v>1591999</v>
@@ -60059,13 +60059,13 @@
         </is>
       </c>
       <c r="E1274" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1274" s="5" t="n">
-        <v>25.21</v>
+        <v>41.71</v>
       </c>
       <c r="G1274" s="4" t="n">
-        <v>50.42</v>
+        <v>41.71</v>
       </c>
       <c r="H1274" s="2" t="n">
         <v>1591999</v>
@@ -60106,13 +60106,13 @@
         </is>
       </c>
       <c r="E1275" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1275" s="5" t="n">
-        <v>29.93</v>
+        <v>25.21</v>
       </c>
       <c r="G1275" s="4" t="n">
-        <v>29.93</v>
+        <v>50.42</v>
       </c>
       <c r="H1275" s="2" t="n">
         <v>1591999</v>
@@ -60435,13 +60435,13 @@
         </is>
       </c>
       <c r="E1282" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1282" s="5" t="n">
-        <v>28.5</v>
+        <v>10.5</v>
       </c>
       <c r="G1282" s="4" t="n">
-        <v>57</v>
+        <v>10.5</v>
       </c>
       <c r="H1282" s="2" t="n">
         <v>1592652</v>
@@ -60482,13 +60482,13 @@
         </is>
       </c>
       <c r="E1283" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1283" s="5" t="n">
-        <v>10.5</v>
+        <v>28.5</v>
       </c>
       <c r="G1283" s="4" t="n">
-        <v>10.5</v>
+        <v>57</v>
       </c>
       <c r="H1283" s="2" t="n">
         <v>1592652</v>
@@ -61845,13 +61845,13 @@
         </is>
       </c>
       <c r="E1312" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1312" s="5" t="n">
-        <v>1.17</v>
+        <v>4.7</v>
       </c>
       <c r="G1312" s="4" t="n">
-        <v>2.34</v>
+        <v>4.7</v>
       </c>
       <c r="H1312" s="2" t="n">
         <v>1595677</v>
@@ -61895,10 +61895,10 @@
         <v>1</v>
       </c>
       <c r="F1313" s="5" t="n">
-        <v>1.62</v>
+        <v>3.09</v>
       </c>
       <c r="G1313" s="4" t="n">
-        <v>1.62</v>
+        <v>3.09</v>
       </c>
       <c r="H1313" s="2" t="n">
         <v>1595677</v>
@@ -61942,10 +61942,10 @@
         <v>1</v>
       </c>
       <c r="F1314" s="5" t="n">
-        <v>4.7</v>
+        <v>1.62</v>
       </c>
       <c r="G1314" s="4" t="n">
-        <v>4.7</v>
+        <v>1.62</v>
       </c>
       <c r="H1314" s="2" t="n">
         <v>1595677</v>
@@ -61986,13 +61986,13 @@
         </is>
       </c>
       <c r="E1315" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1315" s="5" t="n">
-        <v>3.09</v>
+        <v>1.17</v>
       </c>
       <c r="G1315" s="4" t="n">
-        <v>3.09</v>
+        <v>2.34</v>
       </c>
       <c r="H1315" s="2" t="n">
         <v>1595677</v>
@@ -67535,10 +67535,10 @@
         <v>0.2</v>
       </c>
       <c r="F1433" s="5" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="G1433" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H1433" s="2" t="n">
         <v>1607187</v>
@@ -67579,13 +67579,13 @@
         </is>
       </c>
       <c r="E1434" s="4" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="F1434" s="5" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="G1434" s="4" t="n">
-        <v>8</v>
+        <v>72</v>
       </c>
       <c r="H1434" s="2" t="n">
         <v>1607187</v>
@@ -67626,13 +67626,13 @@
         </is>
       </c>
       <c r="E1435" s="4" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="F1435" s="5" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="G1435" s="4" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H1435" s="2" t="n">
         <v>1607187</v>
@@ -67673,13 +67673,13 @@
         </is>
       </c>
       <c r="E1436" s="4" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F1436" s="5" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="G1436" s="4" t="n">
-        <v>6.4</v>
+        <v>30</v>
       </c>
       <c r="H1436" s="2" t="n">
         <v>1607187</v>
@@ -67720,13 +67720,13 @@
         </is>
       </c>
       <c r="E1437" s="4" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="F1437" s="5" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="G1437" s="4" t="n">
-        <v>5</v>
+        <v>6.4</v>
       </c>
       <c r="H1437" s="2" t="n">
         <v>1607187</v>
@@ -67770,10 +67770,10 @@
         <v>0.2</v>
       </c>
       <c r="F1438" s="5" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="G1438" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H1438" s="2" t="n">
         <v>1607187</v>
@@ -67814,13 +67814,13 @@
         </is>
       </c>
       <c r="E1439" s="4" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F1439" s="5" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G1439" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H1439" s="2" t="n">
         <v>1607187</v>
@@ -67861,13 +67861,13 @@
         </is>
       </c>
       <c r="E1440" s="4" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="F1440" s="5" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G1440" s="4" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="H1440" s="2" t="n">
         <v>1607187</v>
@@ -67911,10 +67911,10 @@
         <v>0.8</v>
       </c>
       <c r="F1441" s="5" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="G1441" s="4" t="n">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="H1441" s="2" t="n">
         <v>1607187</v>
@@ -69224,13 +69224,13 @@
         </is>
       </c>
       <c r="E1469" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1469" s="5" t="n">
-        <v>42.75</v>
+        <v>25.9</v>
       </c>
       <c r="G1469" s="4" t="n">
-        <v>85.5</v>
+        <v>25.9</v>
       </c>
       <c r="H1469" s="2" t="n">
         <v>1608017</v>
@@ -69271,13 +69271,13 @@
         </is>
       </c>
       <c r="E1470" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1470" s="5" t="n">
-        <v>57.99</v>
+        <v>42.75</v>
       </c>
       <c r="G1470" s="4" t="n">
-        <v>57.99</v>
+        <v>85.5</v>
       </c>
       <c r="H1470" s="2" t="n">
         <v>1608017</v>
@@ -69321,10 +69321,10 @@
         <v>1</v>
       </c>
       <c r="F1471" s="5" t="n">
-        <v>25.9</v>
+        <v>57.99</v>
       </c>
       <c r="G1471" s="4" t="n">
-        <v>25.9</v>
+        <v>57.99</v>
       </c>
       <c r="H1471" s="2" t="n">
         <v>1608017</v>
@@ -73219,13 +73219,13 @@
         </is>
       </c>
       <c r="E1554" s="4" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="F1554" s="5" t="n">
-        <v>54.3</v>
+        <v>153.3</v>
       </c>
       <c r="G1554" s="4" t="n">
-        <v>4235.4</v>
+        <v>1533</v>
       </c>
       <c r="H1554" s="2" t="n">
         <v>1614539</v>
@@ -73266,13 +73266,13 @@
         </is>
       </c>
       <c r="E1555" s="4" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="F1555" s="5" t="n">
-        <v>65.2</v>
+        <v>54.3</v>
       </c>
       <c r="G1555" s="4" t="n">
-        <v>2216.8</v>
+        <v>4235.4</v>
       </c>
       <c r="H1555" s="2" t="n">
         <v>1614539</v>
@@ -73313,13 +73313,13 @@
         </is>
       </c>
       <c r="E1556" s="4" t="n">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F1556" s="5" t="n">
-        <v>153.3</v>
+        <v>127.6</v>
       </c>
       <c r="G1556" s="4" t="n">
-        <v>1533</v>
+        <v>3572.8</v>
       </c>
       <c r="H1556" s="2" t="n">
         <v>1614539</v>
@@ -73360,13 +73360,13 @@
         </is>
       </c>
       <c r="E1557" s="4" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F1557" s="5" t="n">
-        <v>127.6</v>
+        <v>65.2</v>
       </c>
       <c r="G1557" s="4" t="n">
-        <v>3572.8</v>
+        <v>2216.8</v>
       </c>
       <c r="H1557" s="2" t="n">
         <v>1614539</v>
@@ -75193,13 +75193,13 @@
         </is>
       </c>
       <c r="E1596" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F1596" s="5" t="n">
-        <v>37.9538</v>
+        <v>41.1167</v>
       </c>
       <c r="G1596" s="4" t="n">
-        <v>151.82</v>
+        <v>82.23</v>
       </c>
       <c r="H1596" s="2" t="n">
         <v>1616755</v>
@@ -75334,13 +75334,13 @@
         </is>
       </c>
       <c r="E1599" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F1599" s="5" t="n">
-        <v>41.1167</v>
+        <v>37.9538</v>
       </c>
       <c r="G1599" s="4" t="n">
-        <v>82.23</v>
+        <v>151.82</v>
       </c>
       <c r="H1599" s="2" t="n">
         <v>1616755</v>
@@ -76932,13 +76932,13 @@
         </is>
       </c>
       <c r="E1633" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F1633" s="5" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G1633" s="4" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H1633" s="2" t="n">
         <v>1619290</v>
@@ -76979,13 +76979,13 @@
         </is>
       </c>
       <c r="E1634" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F1634" s="5" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G1634" s="4" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="H1634" s="2" t="n">
         <v>1619290</v>
@@ -77073,13 +77073,13 @@
         </is>
       </c>
       <c r="E1636" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F1636" s="5" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G1636" s="4" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H1636" s="2" t="n">
         <v>1619290</v>
@@ -77123,10 +77123,10 @@
         <v>1</v>
       </c>
       <c r="F1637" s="5" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="G1637" s="4" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="H1637" s="2" t="n">
         <v>1619290</v>
@@ -77167,13 +77167,13 @@
         </is>
       </c>
       <c r="E1638" s="4" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="F1638" s="5" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G1638" s="4" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="H1638" s="2" t="n">
         <v>1619290</v>
@@ -77214,13 +77214,13 @@
         </is>
       </c>
       <c r="E1639" s="4" t="n">
-        <v>1</v>
+        <v>0.26</v>
       </c>
       <c r="F1639" s="5" t="n">
-        <v>16</v>
+        <v>350</v>
       </c>
       <c r="G1639" s="4" t="n">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="H1639" s="2" t="n">
         <v>1619290</v>
@@ -77261,13 +77261,13 @@
         </is>
       </c>
       <c r="E1640" s="4" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="F1640" s="5" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G1640" s="4" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="H1640" s="2" t="n">
         <v>1619290</v>
@@ -77308,13 +77308,13 @@
         </is>
       </c>
       <c r="E1641" s="4" t="n">
-        <v>0.26</v>
+        <v>0.5</v>
       </c>
       <c r="F1641" s="5" t="n">
-        <v>350</v>
+        <v>8</v>
       </c>
       <c r="G1641" s="4" t="n">
-        <v>91</v>
+        <v>4</v>
       </c>
       <c r="H1641" s="2" t="n">
         <v>1619290</v>
@@ -81021,13 +81021,13 @@
         </is>
       </c>
       <c r="E1720" s="4" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="F1720" s="5" t="n">
-        <v>60</v>
+        <v>500</v>
       </c>
       <c r="G1720" s="4" t="n">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="H1720" s="2" t="n">
         <v>1632122</v>
@@ -81068,13 +81068,13 @@
         </is>
       </c>
       <c r="E1721" s="4" t="n">
-        <v>0.08</v>
+        <v>4</v>
       </c>
       <c r="F1721" s="5" t="n">
-        <v>500</v>
+        <v>15</v>
       </c>
       <c r="G1721" s="4" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="H1721" s="2" t="n">
         <v>1632122</v>
@@ -81115,13 +81115,13 @@
         </is>
       </c>
       <c r="E1722" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F1722" s="5" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G1722" s="4" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H1722" s="2" t="n">
         <v>1632122</v>
@@ -81162,13 +81162,13 @@
         </is>
       </c>
       <c r="E1723" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1723" s="5" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="G1723" s="4" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="H1723" s="2" t="n">
         <v>1632122</v>
@@ -81212,10 +81212,10 @@
         <v>1</v>
       </c>
       <c r="F1724" s="5" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="G1724" s="4" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="H1724" s="2" t="n">
         <v>1632122</v>
@@ -81256,13 +81256,13 @@
         </is>
       </c>
       <c r="E1725" s="4" t="n">
-        <v>1</v>
+        <v>0.04</v>
       </c>
       <c r="F1725" s="5" t="n">
-        <v>22</v>
+        <v>140</v>
       </c>
       <c r="G1725" s="4" t="n">
-        <v>22</v>
+        <v>5.6</v>
       </c>
       <c r="H1725" s="2" t="n">
         <v>1632122</v>
@@ -81306,10 +81306,10 @@
         <v>0.04</v>
       </c>
       <c r="F1726" s="5" t="n">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="G1726" s="4" t="n">
-        <v>5.6</v>
+        <v>4.4</v>
       </c>
       <c r="H1726" s="2" t="n">
         <v>1632122</v>
@@ -81350,13 +81350,13 @@
         </is>
       </c>
       <c r="E1727" s="4" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="F1727" s="5" t="n">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="G1727" s="4" t="n">
-        <v>4.4</v>
+        <v>6</v>
       </c>
       <c r="H1727" s="2" t="n">
         <v>1632122</v>
@@ -81515,6 +81515,53 @@
         <v>43060</v>
       </c>
       <c r="K1730" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1731" customHeight="1" ht="15">
+      <c r="A1731" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1731" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1731" s="2" t="n">
+        <v>37526</v>
+      </c>
+      <c r="D1731" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">DISCO-GUIAS</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1731" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1731" s="5" t="n">
+        <v>44.78</v>
+      </c>
+      <c r="G1731" s="4" t="n">
+        <v>2239</v>
+      </c>
+      <c r="H1731" s="2" t="n">
+        <v>1635065</v>
+      </c>
+      <c r="I1731" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">08/10/2026 17:04:18</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1731" s="2" t="n">
+        <v>8134</v>
+      </c>
+      <c r="K1731" s="2" t="n">
         <v>165</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Relatório de compras 12/10/2026 22:01
</commit_message>
<xml_diff>
--- a/data/relatorio.xlsx
+++ b/data/relatorio.xlsx
@@ -3001,13 +3001,13 @@
         </is>
       </c>
       <c r="E60" s="4" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>0.09</v>
+        <v>3.32</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>4.5</v>
+        <v>99.6</v>
       </c>
       <c r="H60" s="2" t="n">
         <v>1401617</v>
@@ -3518,13 +3518,13 @@
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="F71" s="5" t="n">
-        <v>3.32</v>
+        <v>30.25</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>99.6</v>
+        <v>30.25</v>
       </c>
       <c r="H71" s="2" t="n">
         <v>1401617</v>
@@ -3568,10 +3568,10 @@
         <v>1</v>
       </c>
       <c r="F72" s="5" t="n">
-        <v>30.25</v>
+        <v>238.92</v>
       </c>
       <c r="G72" s="4" t="n">
-        <v>30.25</v>
+        <v>238.92</v>
       </c>
       <c r="H72" s="2" t="n">
         <v>1401617</v>
@@ -3612,13 +3612,13 @@
         </is>
       </c>
       <c r="E73" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F73" s="5" t="n">
-        <v>238.92</v>
+        <v>0.96</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>238.92</v>
+        <v>4.8</v>
       </c>
       <c r="H73" s="2" t="n">
         <v>1401617</v>
@@ -3659,13 +3659,13 @@
         </is>
       </c>
       <c r="E74" s="4" t="n">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>0.96</v>
+        <v>0.09</v>
       </c>
       <c r="G74" s="4" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="H74" s="2" t="n">
         <v>1401617</v>
@@ -4367,10 +4367,10 @@
         <v>1</v>
       </c>
       <c r="F89" s="5" t="n">
-        <v>200</v>
+        <v>78</v>
       </c>
       <c r="G89" s="4" t="n">
-        <v>200</v>
+        <v>78</v>
       </c>
       <c r="H89" s="2" t="n">
         <v>1402331</v>
@@ -4461,10 +4461,10 @@
         <v>1</v>
       </c>
       <c r="F91" s="5" t="n">
-        <v>78</v>
+        <v>200</v>
       </c>
       <c r="G91" s="4" t="n">
-        <v>78</v>
+        <v>200</v>
       </c>
       <c r="H91" s="2" t="n">
         <v>1402331</v>
@@ -4881,13 +4881,13 @@
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F100" s="5" t="n">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="G100" s="4" t="n">
-        <v>13.2</v>
+        <v>3</v>
       </c>
       <c r="H100" s="2" t="n">
         <v>1402783</v>
@@ -4975,13 +4975,13 @@
         </is>
       </c>
       <c r="E102" s="4" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F102" s="5" t="n">
-        <v>0.1</v>
+        <v>0.22</v>
       </c>
       <c r="G102" s="4" t="n">
-        <v>3</v>
+        <v>13.2</v>
       </c>
       <c r="H102" s="2" t="n">
         <v>1402783</v>
@@ -5636,10 +5636,10 @@
         <v>1</v>
       </c>
       <c r="F116" s="5" t="n">
-        <v>33.9</v>
+        <v>12.9</v>
       </c>
       <c r="G116" s="4" t="n">
-        <v>33.9</v>
+        <v>12.9</v>
       </c>
       <c r="H116" s="2" t="n">
         <v>1403644</v>
@@ -5683,10 +5683,10 @@
         <v>1</v>
       </c>
       <c r="F117" s="5" t="n">
-        <v>74.9</v>
+        <v>10.5</v>
       </c>
       <c r="G117" s="4" t="n">
-        <v>74.9</v>
+        <v>10.5</v>
       </c>
       <c r="H117" s="2" t="n">
         <v>1403644</v>
@@ -5727,13 +5727,13 @@
         </is>
       </c>
       <c r="E118" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F118" s="5" t="n">
-        <v>19.9</v>
+        <v>33.9</v>
       </c>
       <c r="G118" s="4" t="n">
-        <v>39.8</v>
+        <v>33.9</v>
       </c>
       <c r="H118" s="2" t="n">
         <v>1403644</v>
@@ -5774,13 +5774,13 @@
         </is>
       </c>
       <c r="E119" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F119" s="5" t="n">
-        <v>10.5</v>
+        <v>19.9</v>
       </c>
       <c r="G119" s="4" t="n">
-        <v>10.5</v>
+        <v>39.8</v>
       </c>
       <c r="H119" s="2" t="n">
         <v>1403644</v>
@@ -5871,10 +5871,10 @@
         <v>1</v>
       </c>
       <c r="F121" s="5" t="n">
-        <v>12.9</v>
+        <v>74.9</v>
       </c>
       <c r="G121" s="4" t="n">
-        <v>12.9</v>
+        <v>74.9</v>
       </c>
       <c r="H121" s="2" t="n">
         <v>1403644</v>
@@ -6291,13 +6291,13 @@
         </is>
       </c>
       <c r="E130" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F130" s="5" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="G130" s="4" t="n">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="H130" s="2" t="n">
         <v>1403680</v>
@@ -6338,13 +6338,13 @@
         </is>
       </c>
       <c r="E131" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F131" s="5" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G131" s="4" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="H131" s="2" t="n">
         <v>1403680</v>
@@ -6388,10 +6388,10 @@
         <v>10</v>
       </c>
       <c r="F132" s="5" t="n">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="G132" s="4" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="H132" s="2" t="n">
         <v>1403680</v>
@@ -6432,13 +6432,13 @@
         </is>
       </c>
       <c r="E133" s="4" t="n">
-        <v>1.5</v>
+        <v>10</v>
       </c>
       <c r="F133" s="5" t="n">
-        <v>16</v>
+        <v>3.5</v>
       </c>
       <c r="G133" s="4" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="H133" s="2" t="n">
         <v>1403680</v>
@@ -6526,13 +6526,13 @@
         </is>
       </c>
       <c r="E135" s="4" t="n">
-        <v>0.3</v>
+        <v>10</v>
       </c>
       <c r="F135" s="5" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="G135" s="4" t="n">
-        <v>30</v>
+        <v>250</v>
       </c>
       <c r="H135" s="2" t="n">
         <v>1403681</v>
@@ -6573,13 +6573,13 @@
         </is>
       </c>
       <c r="E136" s="4" t="n">
-        <v>0.3</v>
+        <v>100</v>
       </c>
       <c r="F136" s="5" t="n">
-        <v>15</v>
+        <v>2.22</v>
       </c>
       <c r="G136" s="4" t="n">
-        <v>4.5</v>
+        <v>222</v>
       </c>
       <c r="H136" s="2" t="n">
         <v>1403681</v>
@@ -6620,13 +6620,13 @@
         </is>
       </c>
       <c r="E137" s="4" t="n">
-        <v>10</v>
+        <v>0.15</v>
       </c>
       <c r="F137" s="5" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G137" s="4" t="n">
-        <v>250</v>
+        <v>5.25</v>
       </c>
       <c r="H137" s="2" t="n">
         <v>1403681</v>
@@ -6667,13 +6667,13 @@
         </is>
       </c>
       <c r="E138" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F138" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="F138" s="5" t="n">
-        <v>2.22</v>
-      </c>
       <c r="G138" s="4" t="n">
-        <v>222</v>
+        <v>30</v>
       </c>
       <c r="H138" s="2" t="n">
         <v>1403681</v>
@@ -6714,13 +6714,13 @@
         </is>
       </c>
       <c r="E139" s="4" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="F139" s="5" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="G139" s="4" t="n">
-        <v>5.25</v>
+        <v>4.5</v>
       </c>
       <c r="H139" s="2" t="n">
         <v>1403681</v>
@@ -7325,13 +7325,13 @@
         </is>
       </c>
       <c r="E152" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F152" s="5" t="n">
-        <v>124.5</v>
+        <v>25.9</v>
       </c>
       <c r="G152" s="4" t="n">
-        <v>249</v>
+        <v>25.9</v>
       </c>
       <c r="H152" s="2" t="n">
         <v>1405612</v>
@@ -7419,13 +7419,13 @@
         </is>
       </c>
       <c r="E154" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F154" s="5" t="n">
-        <v>25.9</v>
+        <v>124.5</v>
       </c>
       <c r="G154" s="4" t="n">
-        <v>25.9</v>
+        <v>249</v>
       </c>
       <c r="H154" s="2" t="n">
         <v>1405612</v>
@@ -8033,10 +8033,10 @@
         <v>1</v>
       </c>
       <c r="F167" s="5" t="n">
-        <v>18.91</v>
+        <v>19.32</v>
       </c>
       <c r="G167" s="4" t="n">
-        <v>18.91</v>
+        <v>19.32</v>
       </c>
       <c r="H167" s="2" t="n">
         <v>1405673</v>
@@ -8080,10 +8080,10 @@
         <v>1</v>
       </c>
       <c r="F168" s="5" t="n">
-        <v>19.32</v>
+        <v>18.91</v>
       </c>
       <c r="G168" s="4" t="n">
-        <v>19.32</v>
+        <v>18.91</v>
       </c>
       <c r="H168" s="2" t="n">
         <v>1405673</v>
@@ -10051,13 +10051,13 @@
         </is>
       </c>
       <c r="E210" s="4" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="F210" s="5" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="G210" s="4" t="n">
-        <v>840</v>
+        <v>2450</v>
       </c>
       <c r="H210" s="2" t="n">
         <v>1409782</v>
@@ -10098,13 +10098,13 @@
         </is>
       </c>
       <c r="E211" s="4" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="F211" s="5" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="G211" s="4" t="n">
-        <v>2450</v>
+        <v>840</v>
       </c>
       <c r="H211" s="2" t="n">
         <v>1409782</v>
@@ -10521,13 +10521,13 @@
         </is>
       </c>
       <c r="E220" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F220" s="5" t="n">
-        <v>12</v>
+        <v>59.9</v>
       </c>
       <c r="G220" s="4" t="n">
-        <v>24</v>
+        <v>59.9</v>
       </c>
       <c r="H220" s="2" t="n">
         <v>1410100</v>
@@ -10568,13 +10568,13 @@
         </is>
       </c>
       <c r="E221" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F221" s="5" t="n">
-        <v>59.9</v>
+        <v>12</v>
       </c>
       <c r="G221" s="4" t="n">
-        <v>59.9</v>
+        <v>24</v>
       </c>
       <c r="H221" s="2" t="n">
         <v>1410100</v>
@@ -15503,13 +15503,13 @@
         </is>
       </c>
       <c r="E326" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F326" s="5" t="n">
-        <v>189</v>
+        <v>115</v>
       </c>
       <c r="G326" s="4" t="n">
-        <v>1701</v>
+        <v>115</v>
       </c>
       <c r="H326" s="2" t="n">
         <v>1429513</v>
@@ -15644,13 +15644,13 @@
         </is>
       </c>
       <c r="E329" s="4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F329" s="5" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="G329" s="4" t="n">
-        <v>115</v>
+        <v>1170</v>
       </c>
       <c r="H329" s="2" t="n">
         <v>1429513</v>
@@ -15694,10 +15694,10 @@
         <v>9</v>
       </c>
       <c r="F330" s="5" t="n">
-        <v>130</v>
+        <v>189</v>
       </c>
       <c r="G330" s="4" t="n">
-        <v>1170</v>
+        <v>1701</v>
       </c>
       <c r="H330" s="2" t="n">
         <v>1429513</v>
@@ -15788,10 +15788,10 @@
         <v>20</v>
       </c>
       <c r="F332" s="5" t="n">
-        <v>3.27</v>
+        <v>22.55</v>
       </c>
       <c r="G332" s="4" t="n">
-        <v>65.4</v>
+        <v>451</v>
       </c>
       <c r="H332" s="2" t="n">
         <v>1429513</v>
@@ -15835,10 +15835,10 @@
         <v>20</v>
       </c>
       <c r="F333" s="5" t="n">
-        <v>22.55</v>
+        <v>3.27</v>
       </c>
       <c r="G333" s="4" t="n">
-        <v>451</v>
+        <v>65.4</v>
       </c>
       <c r="H333" s="2" t="n">
         <v>1429513</v>
@@ -16020,13 +16020,13 @@
         </is>
       </c>
       <c r="E337" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F337" s="5" t="n">
-        <v>1.21</v>
+        <v>39</v>
       </c>
       <c r="G337" s="4" t="n">
-        <v>12.1</v>
+        <v>234</v>
       </c>
       <c r="H337" s="2" t="n">
         <v>1431621</v>
@@ -16067,13 +16067,13 @@
         </is>
       </c>
       <c r="E338" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F338" s="5" t="n">
-        <v>17.32</v>
+        <v>39</v>
       </c>
       <c r="G338" s="4" t="n">
-        <v>69.28</v>
+        <v>234</v>
       </c>
       <c r="H338" s="2" t="n">
         <v>1431621</v>
@@ -16161,13 +16161,13 @@
         </is>
       </c>
       <c r="E340" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F340" s="5" t="n">
-        <v>39</v>
+        <v>17.32</v>
       </c>
       <c r="G340" s="4" t="n">
-        <v>234</v>
+        <v>69.28</v>
       </c>
       <c r="H340" s="2" t="n">
         <v>1431621</v>
@@ -16208,13 +16208,13 @@
         </is>
       </c>
       <c r="E341" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F341" s="5" t="n">
-        <v>39</v>
+        <v>1.21</v>
       </c>
       <c r="G341" s="4" t="n">
-        <v>234</v>
+        <v>12.1</v>
       </c>
       <c r="H341" s="2" t="n">
         <v>1431621</v>
@@ -16302,13 +16302,13 @@
         </is>
       </c>
       <c r="E343" s="4" t="n">
-        <v>2.7</v>
+        <v>1</v>
       </c>
       <c r="F343" s="5" t="n">
-        <v>80</v>
+        <v>1900</v>
       </c>
       <c r="G343" s="4" t="n">
-        <v>216</v>
+        <v>1900</v>
       </c>
       <c r="H343" s="2" t="n">
         <v>1431836</v>
@@ -16349,13 +16349,13 @@
         </is>
       </c>
       <c r="E344" s="4" t="n">
-        <v>1</v>
+        <v>2.7</v>
       </c>
       <c r="F344" s="5" t="n">
-        <v>1900</v>
+        <v>80</v>
       </c>
       <c r="G344" s="4" t="n">
-        <v>1900</v>
+        <v>216</v>
       </c>
       <c r="H344" s="2" t="n">
         <v>1431836</v>
@@ -16772,13 +16772,13 @@
         </is>
       </c>
       <c r="E353" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F353" s="5" t="n">
-        <v>28.9</v>
+        <v>3.45</v>
       </c>
       <c r="G353" s="4" t="n">
-        <v>115.6</v>
+        <v>6.9</v>
       </c>
       <c r="H353" s="2" t="n">
         <v>1432029</v>
@@ -16866,13 +16866,13 @@
         </is>
       </c>
       <c r="E355" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F355" s="5" t="n">
-        <v>3.45</v>
+        <v>28.9</v>
       </c>
       <c r="G355" s="4" t="n">
-        <v>6.9</v>
+        <v>115.6</v>
       </c>
       <c r="H355" s="2" t="n">
         <v>1432029</v>
@@ -17900,13 +17900,13 @@
         </is>
       </c>
       <c r="E377" s="4" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F377" s="5" t="n">
-        <v>2.53</v>
+        <v>6.63</v>
       </c>
       <c r="G377" s="4" t="n">
-        <v>253</v>
+        <v>6.63</v>
       </c>
       <c r="H377" s="2" t="n">
         <v>1437076</v>
@@ -18420,10 +18420,10 @@
         <v>100</v>
       </c>
       <c r="F388" s="5" t="n">
-        <v>4.16</v>
+        <v>2.53</v>
       </c>
       <c r="G388" s="4" t="n">
-        <v>416</v>
+        <v>253</v>
       </c>
       <c r="H388" s="2" t="n">
         <v>1437076</v>
@@ -18464,13 +18464,13 @@
         </is>
       </c>
       <c r="E389" s="4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F389" s="5" t="n">
-        <v>6.28</v>
+        <v>4.16</v>
       </c>
       <c r="G389" s="4" t="n">
-        <v>314</v>
+        <v>416</v>
       </c>
       <c r="H389" s="2" t="n">
         <v>1437076</v>
@@ -18511,13 +18511,13 @@
         </is>
       </c>
       <c r="E390" s="4" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F390" s="5" t="n">
-        <v>6.63</v>
+        <v>6.28</v>
       </c>
       <c r="G390" s="4" t="n">
-        <v>6.63</v>
+        <v>314</v>
       </c>
       <c r="H390" s="2" t="n">
         <v>1437076</v>
@@ -19639,13 +19639,13 @@
         </is>
       </c>
       <c r="E414" s="4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F414" s="5" t="n">
-        <v>0.22</v>
+        <v>0.3</v>
       </c>
       <c r="G414" s="4" t="n">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="H414" s="2" t="n">
         <v>1442011</v>
@@ -19689,10 +19689,10 @@
         <v>50</v>
       </c>
       <c r="F415" s="5" t="n">
-        <v>2</v>
+        <v>0.49</v>
       </c>
       <c r="G415" s="4" t="n">
-        <v>100</v>
+        <v>24.5</v>
       </c>
       <c r="H415" s="2" t="n">
         <v>1442011</v>
@@ -19733,13 +19733,13 @@
         </is>
       </c>
       <c r="E416" s="4" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F416" s="5" t="n">
-        <v>0.3</v>
+        <v>0.22</v>
       </c>
       <c r="G416" s="4" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="H416" s="2" t="n">
         <v>1442011</v>
@@ -19780,13 +19780,13 @@
         </is>
       </c>
       <c r="E417" s="4" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="F417" s="5" t="n">
-        <v>0.49</v>
+        <v>0.37</v>
       </c>
       <c r="G417" s="4" t="n">
-        <v>24.5</v>
+        <v>9.25</v>
       </c>
       <c r="H417" s="2" t="n">
         <v>1442011</v>
@@ -19827,13 +19827,13 @@
         </is>
       </c>
       <c r="E418" s="4" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F418" s="5" t="n">
-        <v>0.37</v>
+        <v>2</v>
       </c>
       <c r="G418" s="4" t="n">
-        <v>9.25</v>
+        <v>100</v>
       </c>
       <c r="H418" s="2" t="n">
         <v>1442011</v>
@@ -19924,10 +19924,10 @@
         <v>1</v>
       </c>
       <c r="F420" s="5" t="n">
-        <v>32.64</v>
+        <v>95.88</v>
       </c>
       <c r="G420" s="4" t="n">
-        <v>32.64</v>
+        <v>95.88</v>
       </c>
       <c r="H420" s="2" t="n">
         <v>1442024</v>
@@ -20018,10 +20018,10 @@
         <v>1</v>
       </c>
       <c r="F422" s="5" t="n">
-        <v>95.88</v>
+        <v>32.64</v>
       </c>
       <c r="G422" s="4" t="n">
-        <v>95.88</v>
+        <v>32.64</v>
       </c>
       <c r="H422" s="2" t="n">
         <v>1442024</v>
@@ -20065,10 +20065,10 @@
         <v>1</v>
       </c>
       <c r="F423" s="5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G423" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H423" s="2" t="n">
         <v>1442618</v>
@@ -20112,10 +20112,10 @@
         <v>1</v>
       </c>
       <c r="F424" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G424" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H424" s="2" t="n">
         <v>1442618</v>
@@ -20347,10 +20347,10 @@
         <v>0.1</v>
       </c>
       <c r="F429" s="5" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G429" s="4" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="H429" s="2" t="n">
         <v>1442618</v>
@@ -20391,13 +20391,13 @@
         </is>
       </c>
       <c r="E430" s="4" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="F430" s="5" t="n">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="G430" s="4" t="n">
-        <v>2.5</v>
+        <v>7.2</v>
       </c>
       <c r="H430" s="2" t="n">
         <v>1442618</v>
@@ -20438,13 +20438,13 @@
         </is>
       </c>
       <c r="E431" s="4" t="n">
-        <v>0.04</v>
+        <v>0.2</v>
       </c>
       <c r="F431" s="5" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="G431" s="4" t="n">
-        <v>2.4</v>
+        <v>6</v>
       </c>
       <c r="H431" s="2" t="n">
         <v>1442618</v>
@@ -20488,10 +20488,10 @@
         <v>0.08</v>
       </c>
       <c r="F432" s="5" t="n">
-        <v>90</v>
+        <v>35</v>
       </c>
       <c r="G432" s="4" t="n">
-        <v>7.2</v>
+        <v>2.8</v>
       </c>
       <c r="H432" s="2" t="n">
         <v>1442618</v>
@@ -20532,13 +20532,13 @@
         </is>
       </c>
       <c r="E433" s="4" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="F433" s="5" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="G433" s="4" t="n">
-        <v>5.4</v>
+        <v>1.6</v>
       </c>
       <c r="H433" s="2" t="n">
         <v>1442618</v>
@@ -20579,13 +20579,13 @@
         </is>
       </c>
       <c r="E434" s="4" t="n">
-        <v>0.25</v>
+        <v>0.08</v>
       </c>
       <c r="F434" s="5" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G434" s="4" t="n">
-        <v>2.5</v>
+        <v>0.48</v>
       </c>
       <c r="H434" s="2" t="n">
         <v>1442618</v>
@@ -20626,13 +20626,13 @@
         </is>
       </c>
       <c r="E435" s="4" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="F435" s="5" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="G435" s="4" t="n">
-        <v>5.6</v>
+        <v>1.8</v>
       </c>
       <c r="H435" s="2" t="n">
         <v>1442618</v>
@@ -20673,13 +20673,13 @@
         </is>
       </c>
       <c r="E436" s="4" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="F436" s="5" t="n">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="G436" s="4" t="n">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="H436" s="2" t="n">
         <v>1442618</v>
@@ -20720,13 +20720,13 @@
         </is>
       </c>
       <c r="E437" s="4" t="n">
-        <v>0.2</v>
+        <v>0.08</v>
       </c>
       <c r="F437" s="5" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="G437" s="4" t="n">
-        <v>6</v>
+        <v>5.6</v>
       </c>
       <c r="H437" s="2" t="n">
         <v>1442618</v>
@@ -20770,10 +20770,10 @@
         <v>0.08</v>
       </c>
       <c r="F438" s="5" t="n">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="G438" s="4" t="n">
-        <v>2.8</v>
+        <v>5.6</v>
       </c>
       <c r="H438" s="2" t="n">
         <v>1442618</v>
@@ -20814,13 +20814,13 @@
         </is>
       </c>
       <c r="E439" s="4" t="n">
-        <v>0.08</v>
+        <v>0.25</v>
       </c>
       <c r="F439" s="5" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G439" s="4" t="n">
-        <v>1.6</v>
+        <v>2.5</v>
       </c>
       <c r="H439" s="2" t="n">
         <v>1442618</v>
@@ -20861,13 +20861,13 @@
         </is>
       </c>
       <c r="E440" s="4" t="n">
-        <v>0.08</v>
+        <v>0.25</v>
       </c>
       <c r="F440" s="5" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="G440" s="4" t="n">
-        <v>0.48</v>
+        <v>5.5</v>
       </c>
       <c r="H440" s="2" t="n">
         <v>1442618</v>
@@ -20911,10 +20911,10 @@
         <v>0.06</v>
       </c>
       <c r="F441" s="5" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="G441" s="4" t="n">
-        <v>1.8</v>
+        <v>5.4</v>
       </c>
       <c r="H441" s="2" t="n">
         <v>1442618</v>
@@ -20955,13 +20955,13 @@
         </is>
       </c>
       <c r="E442" s="4" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="F442" s="5" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="G442" s="4" t="n">
-        <v>8</v>
+        <v>2.4</v>
       </c>
       <c r="H442" s="2" t="n">
         <v>1442618</v>
@@ -21002,13 +21002,13 @@
         </is>
       </c>
       <c r="E443" s="4" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="F443" s="5" t="n">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="G443" s="4" t="n">
-        <v>5.6</v>
+        <v>1.5</v>
       </c>
       <c r="H443" s="2" t="n">
         <v>1442618</v>
@@ -21472,13 +21472,13 @@
         </is>
       </c>
       <c r="E453" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F453" s="5" t="n">
-        <v>3.45</v>
+        <v>5.1</v>
       </c>
       <c r="G453" s="4" t="n">
-        <v>17.25</v>
+        <v>10.2</v>
       </c>
       <c r="H453" s="2" t="n">
         <v>1445805</v>
@@ -21519,13 +21519,13 @@
         </is>
       </c>
       <c r="E454" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F454" s="5" t="n">
-        <v>5.1</v>
+        <v>3.45</v>
       </c>
       <c r="G454" s="4" t="n">
-        <v>10.2</v>
+        <v>17.25</v>
       </c>
       <c r="H454" s="2" t="n">
         <v>1445805</v>
@@ -28619,10 +28619,10 @@
         <v>1</v>
       </c>
       <c r="F605" s="5" t="n">
-        <v>195</v>
+        <v>230</v>
       </c>
       <c r="G605" s="4" t="n">
-        <v>195</v>
+        <v>230</v>
       </c>
       <c r="H605" s="2" t="n">
         <v>1490619</v>
@@ -28666,10 +28666,10 @@
         <v>1</v>
       </c>
       <c r="F606" s="5" t="n">
-        <v>30</v>
+        <v>195</v>
       </c>
       <c r="G606" s="4" t="n">
-        <v>30</v>
+        <v>195</v>
       </c>
       <c r="H606" s="2" t="n">
         <v>1490619</v>
@@ -28713,10 +28713,10 @@
         <v>1</v>
       </c>
       <c r="F607" s="5" t="n">
-        <v>230</v>
+        <v>165</v>
       </c>
       <c r="G607" s="4" t="n">
-        <v>230</v>
+        <v>165</v>
       </c>
       <c r="H607" s="2" t="n">
         <v>1490619</v>
@@ -28760,10 +28760,10 @@
         <v>1</v>
       </c>
       <c r="F608" s="5" t="n">
-        <v>165</v>
+        <v>30</v>
       </c>
       <c r="G608" s="4" t="n">
-        <v>165</v>
+        <v>30</v>
       </c>
       <c r="H608" s="2" t="n">
         <v>1490619</v>
@@ -28898,13 +28898,13 @@
         </is>
       </c>
       <c r="E611" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F611" s="5" t="n">
-        <v>0.86</v>
+        <v>41.71</v>
       </c>
       <c r="G611" s="4" t="n">
-        <v>8.6</v>
+        <v>83.42</v>
       </c>
       <c r="H611" s="2" t="n">
         <v>1490652</v>
@@ -28948,10 +28948,10 @@
         <v>10</v>
       </c>
       <c r="F612" s="5" t="n">
-        <v>0.48</v>
+        <v>0.86</v>
       </c>
       <c r="G612" s="4" t="n">
-        <v>4.8</v>
+        <v>8.6</v>
       </c>
       <c r="H612" s="2" t="n">
         <v>1490652</v>
@@ -28992,13 +28992,13 @@
         </is>
       </c>
       <c r="E613" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F613" s="5" t="n">
-        <v>6.6</v>
+        <v>17.52</v>
       </c>
       <c r="G613" s="4" t="n">
-        <v>19.8</v>
+        <v>70.08</v>
       </c>
       <c r="H613" s="2" t="n">
         <v>1490652</v>
@@ -29039,13 +29039,13 @@
         </is>
       </c>
       <c r="E614" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F614" s="5" t="n">
-        <v>17.52</v>
+        <v>6.6</v>
       </c>
       <c r="G614" s="4" t="n">
-        <v>70.08</v>
+        <v>19.8</v>
       </c>
       <c r="H614" s="2" t="n">
         <v>1490652</v>
@@ -29086,13 +29086,13 @@
         </is>
       </c>
       <c r="E615" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F615" s="5" t="n">
-        <v>41.71</v>
+        <v>55.99</v>
       </c>
       <c r="G615" s="4" t="n">
-        <v>83.42</v>
+        <v>167.97</v>
       </c>
       <c r="H615" s="2" t="n">
         <v>1490652</v>
@@ -29133,13 +29133,13 @@
         </is>
       </c>
       <c r="E616" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F616" s="5" t="n">
-        <v>55.99</v>
+        <v>0.48</v>
       </c>
       <c r="G616" s="4" t="n">
-        <v>167.97</v>
+        <v>4.8</v>
       </c>
       <c r="H616" s="2" t="n">
         <v>1490652</v>
@@ -29180,13 +29180,13 @@
         </is>
       </c>
       <c r="E617" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F617" s="5" t="n">
-        <v>34.82</v>
+        <v>2.84</v>
       </c>
       <c r="G617" s="4" t="n">
-        <v>34.82</v>
+        <v>28.4</v>
       </c>
       <c r="H617" s="2" t="n">
         <v>1490652</v>
@@ -29227,13 +29227,13 @@
         </is>
       </c>
       <c r="E618" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F618" s="5" t="n">
-        <v>2.84</v>
+        <v>34.82</v>
       </c>
       <c r="G618" s="4" t="n">
-        <v>28.4</v>
+        <v>34.82</v>
       </c>
       <c r="H618" s="2" t="n">
         <v>1490652</v>
@@ -30308,13 +30308,13 @@
         </is>
       </c>
       <c r="E641" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F641" s="5" t="n">
-        <v>23.95</v>
+        <v>1</v>
       </c>
       <c r="G641" s="4" t="n">
-        <v>23.95</v>
+        <v>10</v>
       </c>
       <c r="H641" s="2" t="n">
         <v>1497640</v>
@@ -30449,13 +30449,13 @@
         </is>
       </c>
       <c r="E644" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F644" s="5" t="n">
-        <v>1</v>
+        <v>178.5</v>
       </c>
       <c r="G644" s="4" t="n">
-        <v>10</v>
+        <v>357</v>
       </c>
       <c r="H644" s="2" t="n">
         <v>1497640</v>
@@ -30496,13 +30496,13 @@
         </is>
       </c>
       <c r="E645" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F645" s="5" t="n">
-        <v>178.5</v>
+        <v>23.95</v>
       </c>
       <c r="G645" s="4" t="n">
-        <v>357</v>
+        <v>23.95</v>
       </c>
       <c r="H645" s="2" t="n">
         <v>1497640</v>
@@ -31721,10 +31721,10 @@
         <v>2</v>
       </c>
       <c r="F671" s="5" t="n">
-        <v>2.03</v>
+        <v>30</v>
       </c>
       <c r="G671" s="4" t="n">
-        <v>4.06</v>
+        <v>60</v>
       </c>
       <c r="H671" s="2" t="n">
         <v>1503029</v>
@@ -31765,13 +31765,13 @@
         </is>
       </c>
       <c r="E672" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F672" s="5" t="n">
-        <v>30</v>
+        <v>30.63</v>
       </c>
       <c r="G672" s="4" t="n">
-        <v>60</v>
+        <v>30.63</v>
       </c>
       <c r="H672" s="2" t="n">
         <v>1503029</v>
@@ -31906,13 +31906,13 @@
         </is>
       </c>
       <c r="E675" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F675" s="5" t="n">
-        <v>5.39</v>
+        <v>2.03</v>
       </c>
       <c r="G675" s="4" t="n">
-        <v>5.39</v>
+        <v>4.06</v>
       </c>
       <c r="H675" s="2" t="n">
         <v>1503029</v>
@@ -31956,10 +31956,10 @@
         <v>1</v>
       </c>
       <c r="F676" s="5" t="n">
-        <v>30.63</v>
+        <v>5.39</v>
       </c>
       <c r="G676" s="4" t="n">
-        <v>30.63</v>
+        <v>5.39</v>
       </c>
       <c r="H676" s="2" t="n">
         <v>1503029</v>
@@ -32426,10 +32426,10 @@
         <v>1</v>
       </c>
       <c r="F686" s="5" t="n">
-        <v>4.18</v>
+        <v>14.02</v>
       </c>
       <c r="G686" s="4" t="n">
-        <v>4.18</v>
+        <v>14.02</v>
       </c>
       <c r="H686" s="2" t="n">
         <v>1503440</v>
@@ -32473,10 +32473,10 @@
         <v>1</v>
       </c>
       <c r="F687" s="5" t="n">
-        <v>14.02</v>
+        <v>4.18</v>
       </c>
       <c r="G687" s="4" t="n">
-        <v>14.02</v>
+        <v>4.18</v>
       </c>
       <c r="H687" s="2" t="n">
         <v>1503440</v>
@@ -32708,10 +32708,10 @@
         <v>1</v>
       </c>
       <c r="F692" s="5" t="n">
-        <v>13.3</v>
+        <v>30.65</v>
       </c>
       <c r="G692" s="4" t="n">
-        <v>13.3</v>
+        <v>30.65</v>
       </c>
       <c r="H692" s="2" t="n">
         <v>1504946</v>
@@ -32755,10 +32755,10 @@
         <v>1</v>
       </c>
       <c r="F693" s="5" t="n">
-        <v>30.65</v>
+        <v>13.3</v>
       </c>
       <c r="G693" s="4" t="n">
-        <v>30.65</v>
+        <v>13.3</v>
       </c>
       <c r="H693" s="2" t="n">
         <v>1504946</v>
@@ -33222,13 +33222,13 @@
         </is>
       </c>
       <c r="E703" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F703" s="5" t="n">
-        <v>10.3</v>
+        <v>2.88</v>
       </c>
       <c r="G703" s="4" t="n">
-        <v>10.3</v>
+        <v>5.76</v>
       </c>
       <c r="H703" s="2" t="n">
         <v>1512391</v>
@@ -33269,13 +33269,13 @@
         </is>
       </c>
       <c r="E704" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F704" s="5" t="n">
-        <v>15.25</v>
+        <v>2.29</v>
       </c>
       <c r="G704" s="4" t="n">
-        <v>15.25</v>
+        <v>4.58</v>
       </c>
       <c r="H704" s="2" t="n">
         <v>1512391</v>
@@ -33363,13 +33363,13 @@
         </is>
       </c>
       <c r="E706" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F706" s="5" t="n">
-        <v>2.29</v>
+        <v>15.25</v>
       </c>
       <c r="G706" s="4" t="n">
-        <v>4.58</v>
+        <v>15.25</v>
       </c>
       <c r="H706" s="2" t="n">
         <v>1512391</v>
@@ -33410,13 +33410,13 @@
         </is>
       </c>
       <c r="E707" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F707" s="5" t="n">
-        <v>2.88</v>
+        <v>10.3</v>
       </c>
       <c r="G707" s="4" t="n">
-        <v>5.76</v>
+        <v>10.3</v>
       </c>
       <c r="H707" s="2" t="n">
         <v>1512391</v>
@@ -33460,10 +33460,10 @@
         <v>1</v>
       </c>
       <c r="F708" s="5" t="n">
-        <v>27.65</v>
+        <v>12.25</v>
       </c>
       <c r="G708" s="4" t="n">
-        <v>27.65</v>
+        <v>12.25</v>
       </c>
       <c r="H708" s="2" t="n">
         <v>1512391</v>
@@ -33507,10 +33507,10 @@
         <v>1</v>
       </c>
       <c r="F709" s="5" t="n">
-        <v>12.25</v>
+        <v>27.65</v>
       </c>
       <c r="G709" s="4" t="n">
-        <v>12.25</v>
+        <v>27.65</v>
       </c>
       <c r="H709" s="2" t="n">
         <v>1512391</v>
@@ -33598,13 +33598,13 @@
         </is>
       </c>
       <c r="E711" s="4" t="n">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="F711" s="5" t="n">
-        <v>0.17</v>
+        <v>0.22</v>
       </c>
       <c r="G711" s="4" t="n">
-        <v>2.55</v>
+        <v>22</v>
       </c>
       <c r="H711" s="2" t="n">
         <v>1512750</v>
@@ -33645,13 +33645,13 @@
         </is>
       </c>
       <c r="E712" s="4" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F712" s="5" t="n">
-        <v>0.15</v>
+        <v>0.22</v>
       </c>
       <c r="G712" s="4" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="H712" s="2" t="n">
         <v>1512750</v>
@@ -33739,13 +33739,13 @@
         </is>
       </c>
       <c r="E714" s="4" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="F714" s="5" t="n">
-        <v>0.22</v>
+        <v>0.15</v>
       </c>
       <c r="G714" s="4" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="H714" s="2" t="n">
         <v>1512750</v>
@@ -33786,13 +33786,13 @@
         </is>
       </c>
       <c r="E715" s="4" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="F715" s="5" t="n">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="G715" s="4" t="n">
-        <v>22</v>
+        <v>2.55</v>
       </c>
       <c r="H715" s="2" t="n">
         <v>1512750</v>
@@ -33836,10 +33836,10 @@
         <v>15</v>
       </c>
       <c r="F716" s="5" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="G716" s="4" t="n">
-        <v>12</v>
+        <v>4.5</v>
       </c>
       <c r="H716" s="2" t="n">
         <v>1512750</v>
@@ -33883,10 +33883,10 @@
         <v>15</v>
       </c>
       <c r="F717" s="5" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="G717" s="4" t="n">
-        <v>4.5</v>
+        <v>12</v>
       </c>
       <c r="H717" s="2" t="n">
         <v>1512750</v>
@@ -34165,10 +34165,10 @@
         <v>1</v>
       </c>
       <c r="F723" s="5" t="n">
-        <v>192.5</v>
+        <v>197.5</v>
       </c>
       <c r="G723" s="4" t="n">
-        <v>192.5</v>
+        <v>197.5</v>
       </c>
       <c r="H723" s="2" t="n">
         <v>1513541</v>
@@ -34212,10 +34212,10 @@
         <v>1</v>
       </c>
       <c r="F724" s="5" t="n">
-        <v>197.5</v>
+        <v>192.5</v>
       </c>
       <c r="G724" s="4" t="n">
-        <v>197.5</v>
+        <v>192.5</v>
       </c>
       <c r="H724" s="2" t="n">
         <v>1513541</v>
@@ -36935,13 +36935,13 @@
         </is>
       </c>
       <c r="E782" s="4" t="n">
-        <v>1.06</v>
+        <v>1.33</v>
       </c>
       <c r="F782" s="5" t="n">
-        <v>17.9621</v>
+        <v>17.9624</v>
       </c>
       <c r="G782" s="4" t="n">
-        <v>18.95</v>
+        <v>23.89</v>
       </c>
       <c r="H782" s="2" t="n">
         <v>1522565</v>
@@ -36982,13 +36982,13 @@
         </is>
       </c>
       <c r="E783" s="4" t="n">
-        <v>1.33</v>
+        <v>1.06</v>
       </c>
       <c r="F783" s="5" t="n">
-        <v>17.9624</v>
+        <v>17.9621</v>
       </c>
       <c r="G783" s="4" t="n">
-        <v>23.89</v>
+        <v>18.95</v>
       </c>
       <c r="H783" s="2" t="n">
         <v>1522565</v>
@@ -37076,13 +37076,13 @@
         </is>
       </c>
       <c r="E785" s="4" t="n">
-        <v>37</v>
+        <v>69</v>
       </c>
       <c r="F785" s="5" t="n">
         <v>54.3</v>
       </c>
       <c r="G785" s="4" t="n">
-        <v>2009.1</v>
+        <v>3746.7</v>
       </c>
       <c r="H785" s="2" t="n">
         <v>1522616</v>
@@ -37123,13 +37123,13 @@
         </is>
       </c>
       <c r="E786" s="4" t="n">
-        <v>69</v>
+        <v>2</v>
       </c>
       <c r="F786" s="5" t="n">
-        <v>54.3</v>
+        <v>139.6</v>
       </c>
       <c r="G786" s="4" t="n">
-        <v>3746.7</v>
+        <v>279.2</v>
       </c>
       <c r="H786" s="2" t="n">
         <v>1522616</v>
@@ -37170,13 +37170,13 @@
         </is>
       </c>
       <c r="E787" s="4" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F787" s="5" t="n">
-        <v>139.6</v>
+        <v>127.6</v>
       </c>
       <c r="G787" s="4" t="n">
-        <v>279.2</v>
+        <v>1786.4</v>
       </c>
       <c r="H787" s="2" t="n">
         <v>1522616</v>
@@ -37217,13 +37217,13 @@
         </is>
       </c>
       <c r="E788" s="4" t="n">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F788" s="5" t="n">
-        <v>127.6</v>
+        <v>54.3</v>
       </c>
       <c r="G788" s="4" t="n">
-        <v>1786.4</v>
+        <v>2009.1</v>
       </c>
       <c r="H788" s="2" t="n">
         <v>1522616</v>
@@ -37264,13 +37264,13 @@
         </is>
       </c>
       <c r="E789" s="4" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="F789" s="5" t="n">
-        <v>153.6</v>
+        <v>127.6</v>
       </c>
       <c r="G789" s="4" t="n">
-        <v>2457.6</v>
+        <v>4593.6</v>
       </c>
       <c r="H789" s="2" t="n">
         <v>1522616</v>
@@ -37311,13 +37311,13 @@
         </is>
       </c>
       <c r="E790" s="4" t="n">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="F790" s="5" t="n">
-        <v>127.6</v>
+        <v>9.1</v>
       </c>
       <c r="G790" s="4" t="n">
-        <v>4593.6</v>
+        <v>127.4</v>
       </c>
       <c r="H790" s="2" t="n">
         <v>1522616</v>
@@ -37358,13 +37358,13 @@
         </is>
       </c>
       <c r="E791" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F791" s="5" t="n">
-        <v>9.1</v>
+        <v>153.6</v>
       </c>
       <c r="G791" s="4" t="n">
-        <v>127.4</v>
+        <v>2457.6</v>
       </c>
       <c r="H791" s="2" t="n">
         <v>1522616</v>
@@ -37922,13 +37922,13 @@
         </is>
       </c>
       <c r="E803" s="4" t="n">
-        <v>1</v>
+        <v>0.08</v>
       </c>
       <c r="F803" s="5" t="n">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="G803" s="4" t="n">
-        <v>36</v>
+        <v>1.44</v>
       </c>
       <c r="H803" s="2" t="n">
         <v>1524925</v>
@@ -37969,13 +37969,13 @@
         </is>
       </c>
       <c r="E804" s="4" t="n">
-        <v>1.28</v>
+        <v>1.89</v>
       </c>
       <c r="F804" s="5" t="n">
-        <v>38</v>
+        <v>150</v>
       </c>
       <c r="G804" s="4" t="n">
-        <v>48.64</v>
+        <v>283.5</v>
       </c>
       <c r="H804" s="2" t="n">
         <v>1524925</v>
@@ -38016,13 +38016,13 @@
         </is>
       </c>
       <c r="E805" s="4" t="n">
-        <v>1.89</v>
+        <v>1</v>
       </c>
       <c r="F805" s="5" t="n">
-        <v>150</v>
+        <v>36</v>
       </c>
       <c r="G805" s="4" t="n">
-        <v>283.5</v>
+        <v>36</v>
       </c>
       <c r="H805" s="2" t="n">
         <v>1524925</v>
@@ -38063,13 +38063,13 @@
         </is>
       </c>
       <c r="E806" s="4" t="n">
-        <v>0.08</v>
+        <v>1.28</v>
       </c>
       <c r="F806" s="5" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="G806" s="4" t="n">
-        <v>1.44</v>
+        <v>48.64</v>
       </c>
       <c r="H806" s="2" t="n">
         <v>1524925</v>
@@ -38580,13 +38580,13 @@
         </is>
       </c>
       <c r="E817" s="4" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F817" s="5" t="n">
-        <v>3.89</v>
+        <v>9.59</v>
       </c>
       <c r="G817" s="4" t="n">
-        <v>58.35</v>
+        <v>9.59</v>
       </c>
       <c r="H817" s="2" t="n">
         <v>1526079</v>
@@ -38627,13 +38627,13 @@
         </is>
       </c>
       <c r="E818" s="4" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F818" s="5" t="n">
-        <v>9.59</v>
+        <v>3.89</v>
       </c>
       <c r="G818" s="4" t="n">
-        <v>9.59</v>
+        <v>58.35</v>
       </c>
       <c r="H818" s="2" t="n">
         <v>1526079</v>
@@ -38674,13 +38674,13 @@
         </is>
       </c>
       <c r="E819" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F819" s="5" t="n">
-        <v>8.9</v>
+        <v>17.5</v>
       </c>
       <c r="G819" s="4" t="n">
-        <v>62.3</v>
+        <v>17.5</v>
       </c>
       <c r="H819" s="2" t="n">
         <v>1526335</v>
@@ -38721,13 +38721,13 @@
         </is>
       </c>
       <c r="E820" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F820" s="5" t="n">
-        <v>17.5</v>
+        <v>8.9</v>
       </c>
       <c r="G820" s="4" t="n">
-        <v>17.5</v>
+        <v>62.3</v>
       </c>
       <c r="H820" s="2" t="n">
         <v>1526335</v>
@@ -40322,10 +40322,10 @@
         <v>1.5</v>
       </c>
       <c r="F854" s="5" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G854" s="4" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H854" s="2" t="n">
         <v>1532084</v>
@@ -40366,13 +40366,13 @@
         </is>
       </c>
       <c r="E855" s="4" t="n">
-        <v>1.5</v>
+        <v>0.1</v>
       </c>
       <c r="F855" s="5" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="G855" s="4" t="n">
-        <v>24</v>
+        <v>2.5</v>
       </c>
       <c r="H855" s="2" t="n">
         <v>1532084</v>
@@ -40416,10 +40416,10 @@
         <v>1</v>
       </c>
       <c r="F856" s="5" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G856" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H856" s="2" t="n">
         <v>1532084</v>
@@ -40460,13 +40460,13 @@
         </is>
       </c>
       <c r="E857" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F857" s="5" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G857" s="4" t="n">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="H857" s="2" t="n">
         <v>1532084</v>
@@ -40507,13 +40507,13 @@
         </is>
       </c>
       <c r="E858" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F858" s="5" t="n">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="G858" s="4" t="n">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="H858" s="2" t="n">
         <v>1532084</v>
@@ -40554,13 +40554,13 @@
         </is>
       </c>
       <c r="E859" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F859" s="5" t="n">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="G859" s="4" t="n">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="H859" s="2" t="n">
         <v>1532084</v>
@@ -40601,13 +40601,13 @@
         </is>
       </c>
       <c r="E860" s="4" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="F860" s="5" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="G860" s="4" t="n">
-        <v>2.5</v>
+        <v>18</v>
       </c>
       <c r="H860" s="2" t="n">
         <v>1532084</v>
@@ -40883,13 +40883,13 @@
         </is>
       </c>
       <c r="E866" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F866" s="5" t="n">
-        <v>4.9</v>
+        <v>39.9</v>
       </c>
       <c r="G866" s="4" t="n">
-        <v>29.4</v>
+        <v>39.9</v>
       </c>
       <c r="H866" s="2" t="n">
         <v>1533181</v>
@@ -40930,13 +40930,13 @@
         </is>
       </c>
       <c r="E867" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F867" s="5" t="n">
-        <v>6.9</v>
+        <v>18.9</v>
       </c>
       <c r="G867" s="4" t="n">
-        <v>13.8</v>
+        <v>18.9</v>
       </c>
       <c r="H867" s="2" t="n">
         <v>1533181</v>
@@ -40977,13 +40977,13 @@
         </is>
       </c>
       <c r="E868" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F868" s="5" t="n">
-        <v>39.9</v>
+        <v>4.9</v>
       </c>
       <c r="G868" s="4" t="n">
-        <v>39.9</v>
+        <v>29.4</v>
       </c>
       <c r="H868" s="2" t="n">
         <v>1533181</v>
@@ -41024,13 +41024,13 @@
         </is>
       </c>
       <c r="E869" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F869" s="5" t="n">
-        <v>18.9</v>
+        <v>6.9</v>
       </c>
       <c r="G869" s="4" t="n">
-        <v>18.9</v>
+        <v>13.8</v>
       </c>
       <c r="H869" s="2" t="n">
         <v>1533181</v>
@@ -41776,13 +41776,13 @@
         </is>
       </c>
       <c r="E885" s="4" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="F885" s="5" t="n">
-        <v>0.19</v>
+        <v>0.6</v>
       </c>
       <c r="G885" s="4" t="n">
-        <v>5.32</v>
+        <v>2.4</v>
       </c>
       <c r="H885" s="2" t="n">
         <v>1539898</v>
@@ -41823,13 +41823,13 @@
         </is>
       </c>
       <c r="E886" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F886" s="5" t="n">
-        <v>0.22</v>
+        <v>0.6</v>
       </c>
       <c r="G886" s="4" t="n">
-        <v>1.32</v>
+        <v>2.4</v>
       </c>
       <c r="H886" s="2" t="n">
         <v>1539898</v>
@@ -41870,13 +41870,13 @@
         </is>
       </c>
       <c r="E887" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F887" s="5" t="n">
-        <v>0.15</v>
+        <v>0.8</v>
       </c>
       <c r="G887" s="4" t="n">
-        <v>1.8</v>
+        <v>8</v>
       </c>
       <c r="H887" s="2" t="n">
         <v>1539898</v>
@@ -41917,13 +41917,13 @@
         </is>
       </c>
       <c r="E888" s="4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F888" s="5" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="G888" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H888" s="2" t="n">
         <v>1539898</v>
@@ -41964,13 +41964,13 @@
         </is>
       </c>
       <c r="E889" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F889" s="5" t="n">
-        <v>53</v>
+        <v>2.3</v>
       </c>
       <c r="G889" s="4" t="n">
-        <v>53</v>
+        <v>13.8</v>
       </c>
       <c r="H889" s="2" t="n">
         <v>1539898</v>
@@ -42011,13 +42011,13 @@
         </is>
       </c>
       <c r="E890" s="4" t="n">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="F890" s="5" t="n">
-        <v>0.11</v>
+        <v>0.66</v>
       </c>
       <c r="G890" s="4" t="n">
-        <v>0.66</v>
+        <v>66</v>
       </c>
       <c r="H890" s="2" t="n">
         <v>1539898</v>
@@ -42058,13 +42058,13 @@
         </is>
       </c>
       <c r="E891" s="4" t="n">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="F891" s="5" t="n">
-        <v>0.3</v>
+        <v>0.52</v>
       </c>
       <c r="G891" s="4" t="n">
-        <v>30</v>
+        <v>4.16</v>
       </c>
       <c r="H891" s="2" t="n">
         <v>1539898</v>
@@ -42105,13 +42105,13 @@
         </is>
       </c>
       <c r="E892" s="4" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="F892" s="5" t="n">
-        <v>0.29</v>
+        <v>0.58</v>
       </c>
       <c r="G892" s="4" t="n">
-        <v>4.06</v>
+        <v>2.32</v>
       </c>
       <c r="H892" s="2" t="n">
         <v>1539898</v>
@@ -42152,13 +42152,13 @@
         </is>
       </c>
       <c r="E893" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F893" s="5" t="n">
-        <v>0.6</v>
+        <v>0.81</v>
       </c>
       <c r="G893" s="4" t="n">
-        <v>2.4</v>
+        <v>1.62</v>
       </c>
       <c r="H893" s="2" t="n">
         <v>1539898</v>
@@ -42202,10 +42202,10 @@
         <v>4</v>
       </c>
       <c r="F894" s="5" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="G894" s="4" t="n">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="H894" s="2" t="n">
         <v>1539898</v>
@@ -42246,13 +42246,13 @@
         </is>
       </c>
       <c r="E895" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F895" s="5" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="G895" s="4" t="n">
-        <v>8</v>
+        <v>2.4</v>
       </c>
       <c r="H895" s="2" t="n">
         <v>1539898</v>
@@ -42293,13 +42293,13 @@
         </is>
       </c>
       <c r="E896" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F896" s="5" t="n">
-        <v>1</v>
+        <v>1.32</v>
       </c>
       <c r="G896" s="4" t="n">
-        <v>12</v>
+        <v>5.28</v>
       </c>
       <c r="H896" s="2" t="n">
         <v>1539898</v>
@@ -42340,13 +42340,13 @@
         </is>
       </c>
       <c r="E897" s="4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F897" s="5" t="n">
-        <v>2.3</v>
+        <v>0.45</v>
       </c>
       <c r="G897" s="4" t="n">
-        <v>13.8</v>
+        <v>5.4</v>
       </c>
       <c r="H897" s="2" t="n">
         <v>1539898</v>
@@ -42390,10 +42390,10 @@
         <v>100</v>
       </c>
       <c r="F898" s="5" t="n">
-        <v>0.66</v>
+        <v>0.11</v>
       </c>
       <c r="G898" s="4" t="n">
-        <v>66</v>
+        <v>11</v>
       </c>
       <c r="H898" s="2" t="n">
         <v>1539898</v>
@@ -42434,13 +42434,13 @@
         </is>
       </c>
       <c r="E899" s="4" t="n">
-        <v>8</v>
+        <v>100</v>
       </c>
       <c r="F899" s="5" t="n">
-        <v>0.52</v>
+        <v>0.12</v>
       </c>
       <c r="G899" s="4" t="n">
-        <v>4.16</v>
+        <v>12</v>
       </c>
       <c r="H899" s="2" t="n">
         <v>1539898</v>
@@ -42481,13 +42481,13 @@
         </is>
       </c>
       <c r="E900" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F900" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G900" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="F900" s="5" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="G900" s="4" t="n">
-        <v>2.32</v>
       </c>
       <c r="H900" s="2" t="n">
         <v>1539898</v>
@@ -42528,13 +42528,13 @@
         </is>
       </c>
       <c r="E901" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F901" s="5" t="n">
-        <v>0.81</v>
+        <v>0.42</v>
       </c>
       <c r="G901" s="4" t="n">
-        <v>1.62</v>
+        <v>2.52</v>
       </c>
       <c r="H901" s="2" t="n">
         <v>1539898</v>
@@ -42575,13 +42575,13 @@
         </is>
       </c>
       <c r="E902" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F902" s="5" t="n">
-        <v>0.7</v>
+        <v>0.33</v>
       </c>
       <c r="G902" s="4" t="n">
-        <v>2.8</v>
+        <v>1.98</v>
       </c>
       <c r="H902" s="2" t="n">
         <v>1539898</v>
@@ -42622,13 +42622,13 @@
         </is>
       </c>
       <c r="E903" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F903" s="5" t="n">
-        <v>1.2</v>
+        <v>0.21</v>
       </c>
       <c r="G903" s="4" t="n">
-        <v>2.4</v>
+        <v>2.52</v>
       </c>
       <c r="H903" s="2" t="n">
         <v>1539898</v>
@@ -42669,13 +42669,13 @@
         </is>
       </c>
       <c r="E904" s="4" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="F904" s="5" t="n">
-        <v>1.32</v>
+        <v>0.29</v>
       </c>
       <c r="G904" s="4" t="n">
-        <v>5.28</v>
+        <v>4.06</v>
       </c>
       <c r="H904" s="2" t="n">
         <v>1539898</v>
@@ -42716,13 +42716,13 @@
         </is>
       </c>
       <c r="E905" s="4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F905" s="5" t="n">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="G905" s="4" t="n">
-        <v>5.4</v>
+        <v>2.1</v>
       </c>
       <c r="H905" s="2" t="n">
         <v>1539898</v>
@@ -42763,13 +42763,13 @@
         </is>
       </c>
       <c r="E906" s="4" t="n">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="F906" s="5" t="n">
-        <v>0.11</v>
+        <v>0.48</v>
       </c>
       <c r="G906" s="4" t="n">
-        <v>11</v>
+        <v>1.92</v>
       </c>
       <c r="H906" s="2" t="n">
         <v>1539898</v>
@@ -42810,13 +42810,13 @@
         </is>
       </c>
       <c r="E907" s="4" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="F907" s="5" t="n">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="G907" s="4" t="n">
-        <v>12</v>
+        <v>4.8</v>
       </c>
       <c r="H907" s="2" t="n">
         <v>1539898</v>
@@ -42857,13 +42857,13 @@
         </is>
       </c>
       <c r="E908" s="4" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F908" s="5" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="G908" s="4" t="n">
-        <v>4</v>
+        <v>5.32</v>
       </c>
       <c r="H908" s="2" t="n">
         <v>1539898</v>
@@ -42904,13 +42904,13 @@
         </is>
       </c>
       <c r="E909" s="4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F909" s="5" t="n">
-        <v>0.42</v>
+        <v>0.08</v>
       </c>
       <c r="G909" s="4" t="n">
-        <v>2.52</v>
+        <v>0.96</v>
       </c>
       <c r="H909" s="2" t="n">
         <v>1539898</v>
@@ -42951,13 +42951,13 @@
         </is>
       </c>
       <c r="E910" s="4" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F910" s="5" t="n">
-        <v>0.3</v>
+        <v>0.17</v>
       </c>
       <c r="G910" s="4" t="n">
-        <v>3</v>
+        <v>5.1</v>
       </c>
       <c r="H910" s="2" t="n">
         <v>1539898</v>
@@ -43001,10 +43001,10 @@
         <v>6</v>
       </c>
       <c r="F911" s="5" t="n">
-        <v>0.33</v>
+        <v>0.22</v>
       </c>
       <c r="G911" s="4" t="n">
-        <v>1.98</v>
+        <v>1.32</v>
       </c>
       <c r="H911" s="2" t="n">
         <v>1539898</v>
@@ -43048,10 +43048,10 @@
         <v>12</v>
       </c>
       <c r="F912" s="5" t="n">
-        <v>0.21</v>
+        <v>0.15</v>
       </c>
       <c r="G912" s="4" t="n">
-        <v>2.52</v>
+        <v>1.8</v>
       </c>
       <c r="H912" s="2" t="n">
         <v>1539898</v>
@@ -43092,13 +43092,13 @@
         </is>
       </c>
       <c r="E913" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F913" s="5" t="n">
-        <v>0.35</v>
+        <v>0.25</v>
       </c>
       <c r="G913" s="4" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="H913" s="2" t="n">
         <v>1539898</v>
@@ -43139,13 +43139,13 @@
         </is>
       </c>
       <c r="E914" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F914" s="5" t="n">
-        <v>0.48</v>
+        <v>53</v>
       </c>
       <c r="G914" s="4" t="n">
-        <v>1.92</v>
+        <v>53</v>
       </c>
       <c r="H914" s="2" t="n">
         <v>1539898</v>
@@ -43186,13 +43186,13 @@
         </is>
       </c>
       <c r="E915" s="4" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="F915" s="5" t="n">
-        <v>0.2</v>
+        <v>0.11</v>
       </c>
       <c r="G915" s="4" t="n">
-        <v>4.8</v>
+        <v>0.66</v>
       </c>
       <c r="H915" s="2" t="n">
         <v>1539898</v>
@@ -43233,13 +43233,13 @@
         </is>
       </c>
       <c r="E916" s="4" t="n">
-        <v>12</v>
+        <v>100</v>
       </c>
       <c r="F916" s="5" t="n">
-        <v>0.08</v>
+        <v>0.3</v>
       </c>
       <c r="G916" s="4" t="n">
-        <v>0.96</v>
+        <v>30</v>
       </c>
       <c r="H916" s="2" t="n">
         <v>1539898</v>
@@ -43280,13 +43280,13 @@
         </is>
       </c>
       <c r="E917" s="4" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F917" s="5" t="n">
-        <v>0.17</v>
+        <v>0.3</v>
       </c>
       <c r="G917" s="4" t="n">
-        <v>5.1</v>
+        <v>3</v>
       </c>
       <c r="H917" s="2" t="n">
         <v>1539898</v>
@@ -43891,13 +43891,13 @@
         </is>
       </c>
       <c r="E930" s="4" t="n">
-        <v>0.28</v>
+        <v>1</v>
       </c>
       <c r="F930" s="5" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="G930" s="4" t="n">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="H930" s="2" t="n">
         <v>1546014</v>
@@ -43938,13 +43938,13 @@
         </is>
       </c>
       <c r="E931" s="4" t="n">
-        <v>0.28</v>
+        <v>0.1</v>
       </c>
       <c r="F931" s="5" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="G931" s="4" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="H931" s="2" t="n">
         <v>1546014</v>
@@ -43985,13 +43985,13 @@
         </is>
       </c>
       <c r="E932" s="4" t="n">
-        <v>0.16</v>
+        <v>0.04</v>
       </c>
       <c r="F932" s="5" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="G932" s="4" t="n">
-        <v>5.6</v>
+        <v>4</v>
       </c>
       <c r="H932" s="2" t="n">
         <v>1546014</v>
@@ -44032,13 +44032,13 @@
         </is>
       </c>
       <c r="E933" s="4" t="n">
-        <v>0.04</v>
+        <v>0.28</v>
       </c>
       <c r="F933" s="5" t="n">
         <v>100</v>
       </c>
       <c r="G933" s="4" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="H933" s="2" t="n">
         <v>1546014</v>
@@ -44079,13 +44079,13 @@
         </is>
       </c>
       <c r="E934" s="4" t="n">
-        <v>1</v>
+        <v>0.28</v>
       </c>
       <c r="F934" s="5" t="n">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="G934" s="4" t="n">
-        <v>70</v>
+        <v>4.2</v>
       </c>
       <c r="H934" s="2" t="n">
         <v>1546014</v>
@@ -44126,13 +44126,13 @@
         </is>
       </c>
       <c r="E935" s="4" t="n">
-        <v>0.1</v>
+        <v>0.28</v>
       </c>
       <c r="F935" s="5" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="G935" s="4" t="n">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="H935" s="2" t="n">
         <v>1546014</v>
@@ -44173,13 +44173,13 @@
         </is>
       </c>
       <c r="E936" s="4" t="n">
-        <v>0.28</v>
+        <v>0.16</v>
       </c>
       <c r="F936" s="5" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="G936" s="4" t="n">
-        <v>4.2</v>
+        <v>5.6</v>
       </c>
       <c r="H936" s="2" t="n">
         <v>1546014</v>
@@ -44317,10 +44317,10 @@
         <v>1</v>
       </c>
       <c r="F939" s="5" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="G939" s="4" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="H939" s="2" t="n">
         <v>1547044</v>
@@ -44364,10 +44364,10 @@
         <v>1</v>
       </c>
       <c r="F940" s="5" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="G940" s="4" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="H940" s="2" t="n">
         <v>1547044</v>
@@ -44411,10 +44411,10 @@
         <v>1</v>
       </c>
       <c r="F941" s="5" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="G941" s="4" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="H941" s="2" t="n">
         <v>1547044</v>
@@ -44505,10 +44505,10 @@
         <v>1</v>
       </c>
       <c r="F943" s="5" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="G943" s="4" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="H943" s="2" t="n">
         <v>1547044</v>
@@ -44552,10 +44552,10 @@
         <v>1</v>
       </c>
       <c r="F944" s="5" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="G944" s="4" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="H944" s="2" t="n">
         <v>1547044</v>
@@ -44599,10 +44599,10 @@
         <v>1</v>
       </c>
       <c r="F945" s="5" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="G945" s="4" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="H945" s="2" t="n">
         <v>1547044</v>
@@ -45257,10 +45257,10 @@
         <v>1</v>
       </c>
       <c r="F959" s="5" t="n">
-        <v>33.5</v>
+        <v>12.5</v>
       </c>
       <c r="G959" s="4" t="n">
-        <v>33.5</v>
+        <v>12.5</v>
       </c>
       <c r="H959" s="2" t="n">
         <v>1549629</v>
@@ -45301,13 +45301,13 @@
         </is>
       </c>
       <c r="E960" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F960" s="5" t="n">
-        <v>1.35</v>
+        <v>33.5</v>
       </c>
       <c r="G960" s="4" t="n">
-        <v>4.05</v>
+        <v>33.5</v>
       </c>
       <c r="H960" s="2" t="n">
         <v>1549629</v>
@@ -45348,13 +45348,13 @@
         </is>
       </c>
       <c r="E961" s="4" t="n">
-        <v>5</v>
+        <v>0.2</v>
       </c>
       <c r="F961" s="5" t="n">
-        <v>6.1</v>
+        <v>20</v>
       </c>
       <c r="G961" s="4" t="n">
-        <v>30.5</v>
+        <v>4</v>
       </c>
       <c r="H961" s="2" t="n">
         <v>1549629</v>
@@ -45395,13 +45395,13 @@
         </is>
       </c>
       <c r="E962" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F962" s="5" t="n">
-        <v>12.5</v>
+        <v>1.35</v>
       </c>
       <c r="G962" s="4" t="n">
-        <v>12.5</v>
+        <v>4.05</v>
       </c>
       <c r="H962" s="2" t="n">
         <v>1549629</v>
@@ -45442,13 +45442,13 @@
         </is>
       </c>
       <c r="E963" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F963" s="5" t="n">
-        <v>2</v>
+        <v>1.35</v>
       </c>
       <c r="G963" s="4" t="n">
-        <v>20</v>
+        <v>4.05</v>
       </c>
       <c r="H963" s="2" t="n">
         <v>1549629</v>
@@ -45489,13 +45489,13 @@
         </is>
       </c>
       <c r="E964" s="4" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="F964" s="5" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G964" s="4" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="H964" s="2" t="n">
         <v>1549629</v>
@@ -45536,13 +45536,13 @@
         </is>
       </c>
       <c r="E965" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F965" s="5" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="G965" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H965" s="2" t="n">
         <v>1549629</v>
@@ -45583,13 +45583,13 @@
         </is>
       </c>
       <c r="E966" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F966" s="5" t="n">
-        <v>1.35</v>
+        <v>6.1</v>
       </c>
       <c r="G966" s="4" t="n">
-        <v>4.05</v>
+        <v>30.5</v>
       </c>
       <c r="H966" s="2" t="n">
         <v>1549629</v>
@@ -46996,10 +46996,10 @@
         <v>1</v>
       </c>
       <c r="F996" s="5" t="n">
-        <v>225.72</v>
+        <v>112.86</v>
       </c>
       <c r="G996" s="4" t="n">
-        <v>225.72</v>
+        <v>112.86</v>
       </c>
       <c r="H996" s="2" t="n">
         <v>1555387</v>
@@ -47043,10 +47043,10 @@
         <v>1</v>
       </c>
       <c r="F997" s="5" t="n">
-        <v>112.86</v>
+        <v>225.72</v>
       </c>
       <c r="G997" s="4" t="n">
-        <v>112.86</v>
+        <v>225.72</v>
       </c>
       <c r="H997" s="2" t="n">
         <v>1555387</v>
@@ -47228,13 +47228,13 @@
         </is>
       </c>
       <c r="E1001" s="4" t="n">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="F1001" s="5" t="n">
-        <v>25.6</v>
+        <v>0.6</v>
       </c>
       <c r="G1001" s="4" t="n">
-        <v>25.6</v>
+        <v>300</v>
       </c>
       <c r="H1001" s="2" t="n">
         <v>1557862</v>
@@ -47275,13 +47275,13 @@
         </is>
       </c>
       <c r="E1002" s="4" t="n">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="F1002" s="5" t="n">
-        <v>0.6</v>
+        <v>25.6</v>
       </c>
       <c r="G1002" s="4" t="n">
-        <v>300</v>
+        <v>25.6</v>
       </c>
       <c r="H1002" s="2" t="n">
         <v>1557862</v>
@@ -49578,13 +49578,13 @@
         </is>
       </c>
       <c r="E1051" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1051" s="5" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G1051" s="4" t="n">
-        <v>7.5</v>
+        <v>22</v>
       </c>
       <c r="H1051" s="2" t="n">
         <v>1565694</v>
@@ -49625,13 +49625,13 @@
         </is>
       </c>
       <c r="E1052" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1052" s="5" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G1052" s="4" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H1052" s="2" t="n">
         <v>1565694</v>
@@ -49675,10 +49675,10 @@
         <v>100</v>
       </c>
       <c r="F1053" s="5" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="G1053" s="4" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H1053" s="2" t="n">
         <v>1565694</v>
@@ -50377,13 +50377,13 @@
         </is>
       </c>
       <c r="E1068" s="4" t="n">
-        <v>100</v>
+        <v>0.5</v>
       </c>
       <c r="F1068" s="5" t="n">
-        <v>0.25</v>
+        <v>15</v>
       </c>
       <c r="G1068" s="4" t="n">
-        <v>25</v>
+        <v>7.5</v>
       </c>
       <c r="H1068" s="2" t="n">
         <v>1565694</v>
@@ -50424,13 +50424,13 @@
         </is>
       </c>
       <c r="E1069" s="4" t="n">
-        <v>0.5</v>
+        <v>100</v>
       </c>
       <c r="F1069" s="5" t="n">
-        <v>20</v>
+        <v>0.22</v>
       </c>
       <c r="G1069" s="4" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="H1069" s="2" t="n">
         <v>1565694</v>
@@ -50847,13 +50847,13 @@
         </is>
       </c>
       <c r="E1078" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F1078" s="5" t="n">
-        <v>9</v>
+        <v>24.96</v>
       </c>
       <c r="G1078" s="4" t="n">
-        <v>18</v>
+        <v>74.88</v>
       </c>
       <c r="H1078" s="2" t="n">
         <v>1570182</v>
@@ -50894,13 +50894,13 @@
         </is>
       </c>
       <c r="E1079" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F1079" s="5" t="n">
-        <v>24.96</v>
+        <v>9.712</v>
       </c>
       <c r="G1079" s="4" t="n">
-        <v>74.88</v>
+        <v>9.71</v>
       </c>
       <c r="H1079" s="2" t="n">
         <v>1570182</v>
@@ -50941,13 +50941,13 @@
         </is>
       </c>
       <c r="E1080" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1080" s="5" t="n">
-        <v>5.8</v>
+        <v>10.4</v>
       </c>
       <c r="G1080" s="4" t="n">
-        <v>11.6</v>
+        <v>10.4</v>
       </c>
       <c r="H1080" s="2" t="n">
         <v>1570182</v>
@@ -50988,13 +50988,13 @@
         </is>
       </c>
       <c r="E1081" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F1081" s="5" t="n">
-        <v>5.12</v>
+        <v>6.624</v>
       </c>
       <c r="G1081" s="4" t="n">
-        <v>20.48</v>
+        <v>6.62</v>
       </c>
       <c r="H1081" s="2" t="n">
         <v>1570182</v>
@@ -51035,13 +51035,13 @@
         </is>
       </c>
       <c r="E1082" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F1082" s="5" t="n">
-        <v>9.712</v>
+        <v>5.12</v>
       </c>
       <c r="G1082" s="4" t="n">
-        <v>9.71</v>
+        <v>20.48</v>
       </c>
       <c r="H1082" s="2" t="n">
         <v>1570182</v>
@@ -51085,10 +51085,10 @@
         <v>1</v>
       </c>
       <c r="F1083" s="5" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="G1083" s="4" t="n">
-        <v>10.4</v>
+        <v>12</v>
       </c>
       <c r="H1083" s="2" t="n">
         <v>1570182</v>
@@ -51129,13 +51129,13 @@
         </is>
       </c>
       <c r="E1084" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1084" s="5" t="n">
-        <v>6.624</v>
+        <v>18.66</v>
       </c>
       <c r="G1084" s="4" t="n">
-        <v>6.62</v>
+        <v>37.32</v>
       </c>
       <c r="H1084" s="2" t="n">
         <v>1570182</v>
@@ -51223,13 +51223,13 @@
         </is>
       </c>
       <c r="E1086" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1086" s="5" t="n">
         <v>9</v>
       </c>
       <c r="G1086" s="4" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="H1086" s="2" t="n">
         <v>1570182</v>
@@ -51270,13 +51270,13 @@
         </is>
       </c>
       <c r="E1087" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1087" s="5" t="n">
-        <v>12</v>
+        <v>5.8</v>
       </c>
       <c r="G1087" s="4" t="n">
-        <v>12</v>
+        <v>11.6</v>
       </c>
       <c r="H1087" s="2" t="n">
         <v>1570182</v>
@@ -51317,13 +51317,13 @@
         </is>
       </c>
       <c r="E1088" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1088" s="5" t="n">
-        <v>18.66</v>
+        <v>9</v>
       </c>
       <c r="G1088" s="4" t="n">
-        <v>37.32</v>
+        <v>9</v>
       </c>
       <c r="H1088" s="2" t="n">
         <v>1570182</v>
@@ -51411,13 +51411,13 @@
         </is>
       </c>
       <c r="E1090" s="4" t="n">
-        <v>0.15</v>
+        <v>3</v>
       </c>
       <c r="F1090" s="5" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="G1090" s="4" t="n">
-        <v>13.5</v>
+        <v>12</v>
       </c>
       <c r="H1090" s="2" t="n">
         <v>1570192</v>
@@ -51461,10 +51461,10 @@
         <v>0.3</v>
       </c>
       <c r="F1091" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G1091" s="4" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="H1091" s="2" t="n">
         <v>1570192</v>
@@ -51508,10 +51508,10 @@
         <v>0.3</v>
       </c>
       <c r="F1092" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G1092" s="4" t="n">
-        <v>2.1</v>
+        <v>1.8</v>
       </c>
       <c r="H1092" s="2" t="n">
         <v>1570192</v>
@@ -51552,13 +51552,13 @@
         </is>
       </c>
       <c r="E1093" s="4" t="n">
-        <v>3</v>
+        <v>0.15</v>
       </c>
       <c r="F1093" s="5" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="G1093" s="4" t="n">
-        <v>12</v>
+        <v>13.5</v>
       </c>
       <c r="H1093" s="2" t="n">
         <v>1570192</v>
@@ -51602,10 +51602,10 @@
         <v>0.15</v>
       </c>
       <c r="F1094" s="5" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="G1094" s="4" t="n">
-        <v>4.8</v>
+        <v>6.75</v>
       </c>
       <c r="H1094" s="2" t="n">
         <v>1570192</v>
@@ -51646,13 +51646,13 @@
         </is>
       </c>
       <c r="E1095" s="4" t="n">
-        <v>0.5</v>
+        <v>0.15</v>
       </c>
       <c r="F1095" s="5" t="n">
-        <v>120</v>
+        <v>32</v>
       </c>
       <c r="G1095" s="4" t="n">
-        <v>60</v>
+        <v>4.8</v>
       </c>
       <c r="H1095" s="2" t="n">
         <v>1570192</v>
@@ -51693,13 +51693,13 @@
         </is>
       </c>
       <c r="E1096" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1096" s="5" t="n">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="G1096" s="4" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H1096" s="2" t="n">
         <v>1570192</v>
@@ -51740,13 +51740,13 @@
         </is>
       </c>
       <c r="E1097" s="4" t="n">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="F1097" s="5" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="G1097" s="4" t="n">
-        <v>30</v>
+        <v>6.75</v>
       </c>
       <c r="H1097" s="2" t="n">
         <v>1570192</v>
@@ -51787,13 +51787,13 @@
         </is>
       </c>
       <c r="E1098" s="4" t="n">
-        <v>0.5</v>
+        <v>0.01</v>
       </c>
       <c r="F1098" s="5" t="n">
-        <v>45</v>
+        <v>350</v>
       </c>
       <c r="G1098" s="4" t="n">
-        <v>22.5</v>
+        <v>3.5</v>
       </c>
       <c r="H1098" s="2" t="n">
         <v>1570192</v>
@@ -51834,13 +51834,13 @@
         </is>
       </c>
       <c r="E1099" s="4" t="n">
-        <v>0.01</v>
+        <v>1</v>
       </c>
       <c r="F1099" s="5" t="n">
-        <v>350</v>
+        <v>30</v>
       </c>
       <c r="G1099" s="4" t="n">
-        <v>3.5</v>
+        <v>30</v>
       </c>
       <c r="H1099" s="2" t="n">
         <v>1570192</v>
@@ -51881,13 +51881,13 @@
         </is>
       </c>
       <c r="E1100" s="4" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F1100" s="5" t="n">
-        <v>170</v>
+        <v>30</v>
       </c>
       <c r="G1100" s="4" t="n">
-        <v>42.5</v>
+        <v>30</v>
       </c>
       <c r="H1100" s="2" t="n">
         <v>1570192</v>
@@ -51931,10 +51931,10 @@
         <v>0.5</v>
       </c>
       <c r="F1101" s="5" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="G1101" s="4" t="n">
-        <v>30</v>
+        <v>22.5</v>
       </c>
       <c r="H1101" s="2" t="n">
         <v>1570192</v>
@@ -51975,13 +51975,13 @@
         </is>
       </c>
       <c r="E1102" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1102" s="5" t="n">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="G1102" s="4" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H1102" s="2" t="n">
         <v>1570192</v>
@@ -52022,13 +52022,13 @@
         </is>
       </c>
       <c r="E1103" s="4" t="n">
-        <v>0.15</v>
+        <v>1</v>
       </c>
       <c r="F1103" s="5" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="G1103" s="4" t="n">
-        <v>6.75</v>
+        <v>22</v>
       </c>
       <c r="H1103" s="2" t="n">
         <v>1570192</v>
@@ -52069,13 +52069,13 @@
         </is>
       </c>
       <c r="E1104" s="4" t="n">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
       <c r="F1104" s="5" t="n">
-        <v>45</v>
+        <v>170</v>
       </c>
       <c r="G1104" s="4" t="n">
-        <v>6.75</v>
+        <v>42.5</v>
       </c>
       <c r="H1104" s="2" t="n">
         <v>1570192</v>
@@ -52589,10 +52589,10 @@
         <v>1</v>
       </c>
       <c r="F1115" s="5" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="G1115" s="4" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H1115" s="2" t="n">
         <v>1573232</v>
@@ -52636,10 +52636,10 @@
         <v>1</v>
       </c>
       <c r="F1116" s="5" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G1116" s="4" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H1116" s="2" t="n">
         <v>1573232</v>
@@ -53200,10 +53200,10 @@
         <v>1</v>
       </c>
       <c r="F1128" s="5" t="n">
-        <v>4.3</v>
+        <v>8.9</v>
       </c>
       <c r="G1128" s="4" t="n">
-        <v>4.3</v>
+        <v>8.9</v>
       </c>
       <c r="H1128" s="2" t="n">
         <v>1575575</v>
@@ -53247,10 +53247,10 @@
         <v>1</v>
       </c>
       <c r="F1129" s="5" t="n">
-        <v>3.5</v>
+        <v>13.9</v>
       </c>
       <c r="G1129" s="4" t="n">
-        <v>3.5</v>
+        <v>13.9</v>
       </c>
       <c r="H1129" s="2" t="n">
         <v>1575575</v>
@@ -53294,10 +53294,10 @@
         <v>1</v>
       </c>
       <c r="F1130" s="5" t="n">
-        <v>3.45</v>
+        <v>7.9</v>
       </c>
       <c r="G1130" s="4" t="n">
-        <v>3.45</v>
+        <v>7.9</v>
       </c>
       <c r="H1130" s="2" t="n">
         <v>1575575</v>
@@ -53388,10 +53388,10 @@
         <v>1</v>
       </c>
       <c r="F1132" s="5" t="n">
-        <v>13.9</v>
+        <v>3.5</v>
       </c>
       <c r="G1132" s="4" t="n">
-        <v>13.9</v>
+        <v>3.5</v>
       </c>
       <c r="H1132" s="2" t="n">
         <v>1575575</v>
@@ -53435,10 +53435,10 @@
         <v>1</v>
       </c>
       <c r="F1133" s="5" t="n">
-        <v>7.9</v>
+        <v>4.3</v>
       </c>
       <c r="G1133" s="4" t="n">
-        <v>7.9</v>
+        <v>4.3</v>
       </c>
       <c r="H1133" s="2" t="n">
         <v>1575575</v>
@@ -53482,10 +53482,10 @@
         <v>1</v>
       </c>
       <c r="F1134" s="5" t="n">
-        <v>8.9</v>
+        <v>1.4</v>
       </c>
       <c r="G1134" s="4" t="n">
-        <v>8.9</v>
+        <v>1.4</v>
       </c>
       <c r="H1134" s="2" t="n">
         <v>1575575</v>
@@ -53529,10 +53529,10 @@
         <v>1</v>
       </c>
       <c r="F1135" s="5" t="n">
-        <v>1.4</v>
+        <v>3.45</v>
       </c>
       <c r="G1135" s="4" t="n">
-        <v>1.4</v>
+        <v>3.45</v>
       </c>
       <c r="H1135" s="2" t="n">
         <v>1575575</v>
@@ -53949,13 +53949,13 @@
         </is>
       </c>
       <c r="E1144" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F1144" s="5" t="n">
-        <v>6</v>
+        <v>450</v>
       </c>
       <c r="G1144" s="4" t="n">
-        <v>24</v>
+        <v>450</v>
       </c>
       <c r="H1144" s="2" t="n">
         <v>1575890</v>
@@ -53996,13 +53996,13 @@
         </is>
       </c>
       <c r="E1145" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F1145" s="5" t="n">
-        <v>450</v>
+        <v>6</v>
       </c>
       <c r="G1145" s="4" t="n">
-        <v>450</v>
+        <v>24</v>
       </c>
       <c r="H1145" s="2" t="n">
         <v>1575890</v>
@@ -56866,10 +56866,10 @@
         <v>1</v>
       </c>
       <c r="F1206" s="5" t="n">
-        <v>9.05</v>
+        <v>132.98</v>
       </c>
       <c r="G1206" s="4" t="n">
-        <v>9.05</v>
+        <v>132.98</v>
       </c>
       <c r="H1206" s="2" t="n">
         <v>1588897</v>
@@ -56913,10 +56913,10 @@
         <v>1</v>
       </c>
       <c r="F1207" s="5" t="n">
-        <v>132.98</v>
+        <v>9.05</v>
       </c>
       <c r="G1207" s="4" t="n">
-        <v>132.98</v>
+        <v>9.05</v>
       </c>
       <c r="H1207" s="2" t="n">
         <v>1588897</v>
@@ -57004,13 +57004,13 @@
         </is>
       </c>
       <c r="E1209" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1209" s="5" t="n">
-        <v>17.38</v>
+        <v>23.99</v>
       </c>
       <c r="G1209" s="4" t="n">
-        <v>34.76</v>
+        <v>23.99</v>
       </c>
       <c r="H1209" s="2" t="n">
         <v>1588909</v>
@@ -57051,13 +57051,13 @@
         </is>
       </c>
       <c r="E1210" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1210" s="5" t="n">
-        <v>23.99</v>
+        <v>17.38</v>
       </c>
       <c r="G1210" s="4" t="n">
-        <v>23.99</v>
+        <v>34.76</v>
       </c>
       <c r="H1210" s="2" t="n">
         <v>1588909</v>
@@ -57803,10 +57803,10 @@
         </is>
       </c>
       <c r="E1226" s="4" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="F1226" s="5" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="G1226" s="4" t="n">
         <v>15</v>
@@ -57853,10 +57853,10 @@
         <v>1</v>
       </c>
       <c r="F1227" s="5" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G1227" s="4" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H1227" s="2" t="n">
         <v>1589380</v>
@@ -57897,13 +57897,13 @@
         </is>
       </c>
       <c r="E1228" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F1228" s="5" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="G1228" s="4" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="H1228" s="2" t="n">
         <v>1589380</v>
@@ -57991,13 +57991,13 @@
         </is>
       </c>
       <c r="E1230" s="4" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="F1230" s="5" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="G1230" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H1230" s="2" t="n">
         <v>1589380</v>
@@ -58041,10 +58041,10 @@
         <v>1</v>
       </c>
       <c r="F1231" s="5" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="G1231" s="4" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H1231" s="2" t="n">
         <v>1589380</v>
@@ -58088,10 +58088,10 @@
         <v>0.5</v>
       </c>
       <c r="F1232" s="5" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G1232" s="4" t="n">
-        <v>15</v>
+        <v>12.5</v>
       </c>
       <c r="H1232" s="2" t="n">
         <v>1589380</v>
@@ -58132,13 +58132,13 @@
         </is>
       </c>
       <c r="E1233" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1233" s="5" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G1233" s="4" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H1233" s="2" t="n">
         <v>1589380</v>
@@ -58179,13 +58179,13 @@
         </is>
       </c>
       <c r="E1234" s="4" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="F1234" s="5" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="G1234" s="4" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="H1234" s="2" t="n">
         <v>1589380</v>
@@ -58229,10 +58229,10 @@
         <v>0.5</v>
       </c>
       <c r="F1235" s="5" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="G1235" s="4" t="n">
-        <v>12.5</v>
+        <v>9</v>
       </c>
       <c r="H1235" s="2" t="n">
         <v>1589380</v>
@@ -58273,13 +58273,13 @@
         </is>
       </c>
       <c r="E1236" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1236" s="5" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G1236" s="4" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="H1236" s="2" t="n">
         <v>1589380</v>
@@ -58320,13 +58320,13 @@
         </is>
       </c>
       <c r="E1237" s="4" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="F1237" s="5" t="n">
-        <v>16</v>
+        <v>120</v>
       </c>
       <c r="G1237" s="4" t="n">
-        <v>12</v>
+        <v>120</v>
       </c>
       <c r="H1237" s="2" t="n">
         <v>1589380</v>
@@ -58367,13 +58367,13 @@
         </is>
       </c>
       <c r="E1238" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1238" s="5" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G1238" s="4" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="H1238" s="2" t="n">
         <v>1589380</v>
@@ -58414,13 +58414,13 @@
         </is>
       </c>
       <c r="E1239" s="4" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="F1239" s="5" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="G1239" s="4" t="n">
-        <v>120</v>
+        <v>15</v>
       </c>
       <c r="H1239" s="2" t="n">
         <v>1589380</v>
@@ -58508,13 +58508,13 @@
         </is>
       </c>
       <c r="E1241" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1241" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G1241" s="4" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="H1241" s="2" t="n">
         <v>1589380</v>
@@ -58602,13 +58602,13 @@
         </is>
       </c>
       <c r="E1243" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F1243" s="5" t="n">
-        <v>12</v>
+        <v>1362.5</v>
       </c>
       <c r="G1243" s="4" t="n">
-        <v>120</v>
+        <v>1362.5</v>
       </c>
       <c r="H1243" s="2" t="n">
         <v>1589394</v>
@@ -58649,13 +58649,13 @@
         </is>
       </c>
       <c r="E1244" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F1244" s="5" t="n">
-        <v>252.5</v>
+        <v>12</v>
       </c>
       <c r="G1244" s="4" t="n">
-        <v>252.5</v>
+        <v>120</v>
       </c>
       <c r="H1244" s="2" t="n">
         <v>1589394</v>
@@ -58699,10 +58699,10 @@
         <v>1</v>
       </c>
       <c r="F1245" s="5" t="n">
-        <v>592.5</v>
+        <v>252.5</v>
       </c>
       <c r="G1245" s="4" t="n">
-        <v>592.5</v>
+        <v>252.5</v>
       </c>
       <c r="H1245" s="2" t="n">
         <v>1589394</v>
@@ -58746,10 +58746,10 @@
         <v>1</v>
       </c>
       <c r="F1246" s="5" t="n">
-        <v>507.5</v>
+        <v>592.5</v>
       </c>
       <c r="G1246" s="4" t="n">
-        <v>507.5</v>
+        <v>592.5</v>
       </c>
       <c r="H1246" s="2" t="n">
         <v>1589394</v>
@@ -58793,10 +58793,10 @@
         <v>1</v>
       </c>
       <c r="F1247" s="5" t="n">
-        <v>1362.5</v>
+        <v>507.5</v>
       </c>
       <c r="G1247" s="4" t="n">
-        <v>1362.5</v>
+        <v>507.5</v>
       </c>
       <c r="H1247" s="2" t="n">
         <v>1589394</v>
@@ -59357,10 +59357,10 @@
         <v>0.04</v>
       </c>
       <c r="F1259" s="5" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="G1259" s="4" t="n">
-        <v>0.4</v>
+        <v>3.6</v>
       </c>
       <c r="H1259" s="2" t="n">
         <v>1591938</v>
@@ -59404,10 +59404,10 @@
         <v>0.04</v>
       </c>
       <c r="F1260" s="5" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G1260" s="4" t="n">
-        <v>1.6</v>
+        <v>0.4</v>
       </c>
       <c r="H1260" s="2" t="n">
         <v>1591938</v>
@@ -59451,10 +59451,10 @@
         <v>0.04</v>
       </c>
       <c r="F1261" s="5" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="G1261" s="4" t="n">
-        <v>0.32</v>
+        <v>1.6</v>
       </c>
       <c r="H1261" s="2" t="n">
         <v>1591938</v>
@@ -59495,13 +59495,13 @@
         </is>
       </c>
       <c r="E1262" s="4" t="n">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="F1262" s="5" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G1262" s="4" t="n">
-        <v>3.6</v>
+        <v>1.6</v>
       </c>
       <c r="H1262" s="2" t="n">
         <v>1591938</v>
@@ -59545,10 +59545,10 @@
         <v>0.02</v>
       </c>
       <c r="F1263" s="5" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="G1263" s="4" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="H1263" s="2" t="n">
         <v>1591938</v>
@@ -59589,13 +59589,13 @@
         </is>
       </c>
       <c r="E1264" s="4" t="n">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="F1264" s="5" t="n">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="G1264" s="4" t="n">
-        <v>2</v>
+        <v>0.32</v>
       </c>
       <c r="H1264" s="2" t="n">
         <v>1591938</v>
@@ -59683,13 +59683,13 @@
         </is>
       </c>
       <c r="E1266" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F1266" s="5" t="n">
-        <v>2.66</v>
+        <v>1.29</v>
       </c>
       <c r="G1266" s="4" t="n">
-        <v>15.96</v>
+        <v>5.16</v>
       </c>
       <c r="H1266" s="2" t="n">
         <v>1591999</v>
@@ -59730,13 +59730,13 @@
         </is>
       </c>
       <c r="E1267" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1267" s="5" t="n">
-        <v>14.23</v>
+        <v>13.17</v>
       </c>
       <c r="G1267" s="4" t="n">
-        <v>14.23</v>
+        <v>26.34</v>
       </c>
       <c r="H1267" s="2" t="n">
         <v>1591999</v>
@@ -59777,13 +59777,13 @@
         </is>
       </c>
       <c r="E1268" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F1268" s="5" t="n">
-        <v>3.25</v>
+        <v>2.66</v>
       </c>
       <c r="G1268" s="4" t="n">
-        <v>6.5</v>
+        <v>15.96</v>
       </c>
       <c r="H1268" s="2" t="n">
         <v>1591999</v>
@@ -59824,13 +59824,13 @@
         </is>
       </c>
       <c r="E1269" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1269" s="5" t="n">
-        <v>215.83</v>
+        <v>3.25</v>
       </c>
       <c r="G1269" s="4" t="n">
-        <v>215.83</v>
+        <v>6.5</v>
       </c>
       <c r="H1269" s="2" t="n">
         <v>1591999</v>
@@ -59871,13 +59871,13 @@
         </is>
       </c>
       <c r="E1270" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F1270" s="5" t="n">
-        <v>1.29</v>
+        <v>215.83</v>
       </c>
       <c r="G1270" s="4" t="n">
-        <v>5.16</v>
+        <v>215.83</v>
       </c>
       <c r="H1270" s="2" t="n">
         <v>1591999</v>
@@ -59918,13 +59918,13 @@
         </is>
       </c>
       <c r="E1271" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1271" s="5" t="n">
-        <v>13.17</v>
+        <v>14.23</v>
       </c>
       <c r="G1271" s="4" t="n">
-        <v>26.34</v>
+        <v>14.23</v>
       </c>
       <c r="H1271" s="2" t="n">
         <v>1591999</v>
@@ -60156,10 +60156,10 @@
         <v>25</v>
       </c>
       <c r="F1276" s="5" t="n">
-        <v>0.19</v>
+        <v>0.92</v>
       </c>
       <c r="G1276" s="4" t="n">
-        <v>4.75</v>
+        <v>23</v>
       </c>
       <c r="H1276" s="2" t="n">
         <v>1591999</v>
@@ -60203,10 +60203,10 @@
         <v>25</v>
       </c>
       <c r="F1277" s="5" t="n">
-        <v>0.58</v>
+        <v>0.19</v>
       </c>
       <c r="G1277" s="4" t="n">
-        <v>14.5</v>
+        <v>4.75</v>
       </c>
       <c r="H1277" s="2" t="n">
         <v>1591999</v>
@@ -60250,10 +60250,10 @@
         <v>25</v>
       </c>
       <c r="F1278" s="5" t="n">
-        <v>0.92</v>
+        <v>0.58</v>
       </c>
       <c r="G1278" s="4" t="n">
-        <v>23</v>
+        <v>14.5</v>
       </c>
       <c r="H1278" s="2" t="n">
         <v>1591999</v>
@@ -61939,13 +61939,13 @@
         </is>
       </c>
       <c r="E1314" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1314" s="5" t="n">
-        <v>1.17</v>
+        <v>1.62</v>
       </c>
       <c r="G1314" s="4" t="n">
-        <v>2.34</v>
+        <v>1.62</v>
       </c>
       <c r="H1314" s="2" t="n">
         <v>1595677</v>
@@ -61986,13 +61986,13 @@
         </is>
       </c>
       <c r="E1315" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1315" s="5" t="n">
-        <v>1.62</v>
+        <v>1.17</v>
       </c>
       <c r="G1315" s="4" t="n">
-        <v>1.62</v>
+        <v>2.34</v>
       </c>
       <c r="H1315" s="2" t="n">
         <v>1595677</v>
@@ -67109,13 +67109,13 @@
         </is>
       </c>
       <c r="E1424" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1424" s="5" t="n">
-        <v>12.9</v>
+        <v>8.9</v>
       </c>
       <c r="G1424" s="4" t="n">
-        <v>12.9</v>
+        <v>17.8</v>
       </c>
       <c r="H1424" s="2" t="n">
         <v>1606516</v>
@@ -67438,13 +67438,13 @@
         </is>
       </c>
       <c r="E1431" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1431" s="5" t="n">
-        <v>8.9</v>
+        <v>12.9</v>
       </c>
       <c r="G1431" s="4" t="n">
-        <v>17.8</v>
+        <v>12.9</v>
       </c>
       <c r="H1431" s="2" t="n">
         <v>1606516</v>
@@ -73266,13 +73266,13 @@
         </is>
       </c>
       <c r="E1555" s="4" t="n">
-        <v>10</v>
+        <v>78</v>
       </c>
       <c r="F1555" s="5" t="n">
-        <v>153.3</v>
+        <v>54.3</v>
       </c>
       <c r="G1555" s="4" t="n">
-        <v>1533</v>
+        <v>4235.4</v>
       </c>
       <c r="H1555" s="2" t="n">
         <v>1614539</v>
@@ -73313,13 +73313,13 @@
         </is>
       </c>
       <c r="E1556" s="4" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="F1556" s="5" t="n">
-        <v>127.6</v>
+        <v>153.3</v>
       </c>
       <c r="G1556" s="4" t="n">
-        <v>3572.8</v>
+        <v>1533</v>
       </c>
       <c r="H1556" s="2" t="n">
         <v>1614539</v>
@@ -73360,13 +73360,13 @@
         </is>
       </c>
       <c r="E1557" s="4" t="n">
-        <v>78</v>
+        <v>28</v>
       </c>
       <c r="F1557" s="5" t="n">
-        <v>54.3</v>
+        <v>127.6</v>
       </c>
       <c r="G1557" s="4" t="n">
-        <v>4235.4</v>
+        <v>3572.8</v>
       </c>
       <c r="H1557" s="2" t="n">
         <v>1614539</v>
@@ -75193,13 +75193,13 @@
         </is>
       </c>
       <c r="E1596" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F1596" s="5" t="n">
-        <v>37.9538</v>
+        <v>41.1167</v>
       </c>
       <c r="G1596" s="4" t="n">
-        <v>151.82</v>
+        <v>82.23</v>
       </c>
       <c r="H1596" s="2" t="n">
         <v>1616755</v>
@@ -75334,13 +75334,13 @@
         </is>
       </c>
       <c r="E1599" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F1599" s="5" t="n">
-        <v>41.1167</v>
+        <v>37.9538</v>
       </c>
       <c r="G1599" s="4" t="n">
-        <v>82.23</v>
+        <v>151.82</v>
       </c>
       <c r="H1599" s="2" t="n">
         <v>1616755</v>
@@ -78060,13 +78060,13 @@
         </is>
       </c>
       <c r="E1657" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F1657" s="5" t="n">
-        <v>38.53</v>
+        <v>1.01</v>
       </c>
       <c r="G1657" s="4" t="n">
-        <v>38.53</v>
+        <v>3.03</v>
       </c>
       <c r="H1657" s="2" t="n">
         <v>1620592</v>
@@ -78110,10 +78110,10 @@
         <v>1</v>
       </c>
       <c r="F1658" s="5" t="n">
-        <v>103.85</v>
+        <v>38.53</v>
       </c>
       <c r="G1658" s="4" t="n">
-        <v>103.85</v>
+        <v>38.53</v>
       </c>
       <c r="H1658" s="2" t="n">
         <v>1620592</v>
@@ -78154,13 +78154,13 @@
         </is>
       </c>
       <c r="E1659" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F1659" s="5" t="n">
-        <v>1.01</v>
+        <v>103.85</v>
       </c>
       <c r="G1659" s="4" t="n">
-        <v>3.03</v>
+        <v>103.85</v>
       </c>
       <c r="H1659" s="2" t="n">
         <v>1620592</v>
@@ -81021,13 +81021,13 @@
         </is>
       </c>
       <c r="E1720" s="4" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="F1720" s="5" t="n">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="G1720" s="4" t="n">
-        <v>6</v>
+        <v>4.4</v>
       </c>
       <c r="H1720" s="2" t="n">
         <v>1632122</v>
@@ -81068,13 +81068,13 @@
         </is>
       </c>
       <c r="E1721" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F1721" s="5" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G1721" s="4" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H1721" s="2" t="n">
         <v>1632122</v>
@@ -81118,10 +81118,10 @@
         <v>0.04</v>
       </c>
       <c r="F1722" s="5" t="n">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="G1722" s="4" t="n">
-        <v>4.4</v>
+        <v>5.6</v>
       </c>
       <c r="H1722" s="2" t="n">
         <v>1632122</v>
@@ -81209,13 +81209,13 @@
         </is>
       </c>
       <c r="E1724" s="4" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="F1724" s="5" t="n">
-        <v>500</v>
+        <v>60</v>
       </c>
       <c r="G1724" s="4" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="H1724" s="2" t="n">
         <v>1632122</v>
@@ -81256,13 +81256,13 @@
         </is>
       </c>
       <c r="E1725" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1725" s="5" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="G1725" s="4" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="H1725" s="2" t="n">
         <v>1632122</v>
@@ -81303,13 +81303,13 @@
         </is>
       </c>
       <c r="E1726" s="4" t="n">
-        <v>4</v>
+        <v>0.08</v>
       </c>
       <c r="F1726" s="5" t="n">
-        <v>15</v>
+        <v>500</v>
       </c>
       <c r="G1726" s="4" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="H1726" s="2" t="n">
         <v>1632122</v>
@@ -81350,13 +81350,13 @@
         </is>
       </c>
       <c r="E1727" s="4" t="n">
-        <v>0.04</v>
+        <v>1</v>
       </c>
       <c r="F1727" s="5" t="n">
-        <v>140</v>
+        <v>16</v>
       </c>
       <c r="G1727" s="4" t="n">
-        <v>5.6</v>
+        <v>16</v>
       </c>
       <c r="H1727" s="2" t="n">
         <v>1632122</v>

</xml_diff>

<commit_message>
Relatório de compras 15/10/2026 22:01
</commit_message>
<xml_diff>
--- a/data/relatorio.xlsx
+++ b/data/relatorio.xlsx
@@ -322,13 +322,13 @@
         </is>
       </c>
       <c r="E3" s="4" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.63</v>
+        <v>23.36</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>7.56</v>
+        <v>70.08</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>1397499</v>
@@ -369,13 +369,13 @@
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>33.44</v>
+        <v>0.63</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>33.44</v>
+        <v>7.56</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>1397499</v>
@@ -416,13 +416,13 @@
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.78</v>
+        <v>29.744</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>9.36</v>
+        <v>89.23</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>1397499</v>
@@ -510,13 +510,13 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>23.36</v>
+        <v>4.675</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>70.08</v>
+        <v>9.35</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>1397499</v>
@@ -557,13 +557,13 @@
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>28.768</v>
+        <v>23.36</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>28.76</v>
+        <v>70.08</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>1397499</v>
@@ -604,13 +604,13 @@
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>23.36</v>
+        <v>28.768</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>70.08</v>
+        <v>28.76</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>1397499</v>
@@ -654,10 +654,10 @@
         <v>1</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>4.5</v>
+        <v>33.44</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>4.5</v>
+        <v>33.44</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>1397499</v>
@@ -698,13 +698,13 @@
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>4.675</v>
+        <v>0.78</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>9.35</v>
+        <v>9.36</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>1397499</v>
@@ -745,13 +745,13 @@
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>29.744</v>
+        <v>4.5</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>89.23</v>
+        <v>4.5</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>1397499</v>
@@ -839,13 +839,13 @@
         </is>
       </c>
       <c r="E14" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G14" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>1397500</v>
@@ -886,13 +886,13 @@
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.74</v>
+        <v>0.4</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>29.6</v>
+        <v>4</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>1397500</v>
@@ -933,13 +933,13 @@
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.59</v>
+        <v>0.74</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>118</v>
+        <v>29.6</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>1397500</v>
@@ -980,13 +980,13 @@
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.63</v>
+        <v>0.59</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1.26</v>
+        <v>118</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>1397500</v>
@@ -1074,13 +1074,13 @@
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.1</v>
+        <v>0.63</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>10</v>
+        <v>1.26</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>1397500</v>
@@ -1309,13 +1309,13 @@
         </is>
       </c>
       <c r="E24" s="4" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="H24" s="2" t="n">
         <v>1398186</v>
@@ -1403,13 +1403,13 @@
         </is>
       </c>
       <c r="E26" s="4" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>40</v>
+        <v>110</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="H26" s="2" t="n">
         <v>1398186</v>
@@ -1641,10 +1641,10 @@
         <v>1</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>9.3</v>
+        <v>59.9</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>9.3</v>
+        <v>59.9</v>
       </c>
       <c r="H31" s="2" t="n">
         <v>1398686</v>
@@ -1688,10 +1688,10 @@
         <v>1</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>9.3</v>
+        <v>18.5</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>9.3</v>
+        <v>18.5</v>
       </c>
       <c r="H32" s="2" t="n">
         <v>1398686</v>
@@ -1782,10 +1782,10 @@
         <v>1</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>18.5</v>
+        <v>9.3</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>18.5</v>
+        <v>9.3</v>
       </c>
       <c r="H34" s="2" t="n">
         <v>1398686</v>
@@ -1829,10 +1829,10 @@
         <v>1</v>
       </c>
       <c r="F35" s="5" t="n">
-        <v>59.9</v>
+        <v>9.3</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>59.9</v>
+        <v>9.3</v>
       </c>
       <c r="H35" s="2" t="n">
         <v>1398686</v>
@@ -2249,13 +2249,13 @@
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>0.6</v>
+        <v>1.65</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>36</v>
+        <v>90.75</v>
       </c>
       <c r="H44" s="2" t="n">
         <v>1400747</v>
@@ -2296,13 +2296,13 @@
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>1.65</v>
+        <v>2.4</v>
       </c>
       <c r="F45" s="5" t="n">
         <v>55</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>90.75</v>
+        <v>132</v>
       </c>
       <c r="H45" s="2" t="n">
         <v>1400747</v>
@@ -2343,13 +2343,13 @@
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>2.4</v>
+        <v>0.6</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>132</v>
+        <v>36</v>
       </c>
       <c r="H46" s="2" t="n">
         <v>1400747</v>
@@ -3001,13 +3001,13 @@
         </is>
       </c>
       <c r="E60" s="4" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>30.25</v>
+        <v>3.32</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>30.25</v>
+        <v>99.6</v>
       </c>
       <c r="H60" s="2" t="n">
         <v>1401617</v>
@@ -3518,13 +3518,13 @@
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="F71" s="5" t="n">
-        <v>3.32</v>
+        <v>30.25</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>99.6</v>
+        <v>30.25</v>
       </c>
       <c r="H71" s="2" t="n">
         <v>1401617</v>
@@ -4414,10 +4414,10 @@
         <v>1</v>
       </c>
       <c r="F90" s="5" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="G90" s="4" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="H90" s="2" t="n">
         <v>1402331</v>
@@ -4461,10 +4461,10 @@
         <v>1</v>
       </c>
       <c r="F91" s="5" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="G91" s="4" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="H91" s="2" t="n">
         <v>1402331</v>
@@ -5072,10 +5072,10 @@
         <v>30</v>
       </c>
       <c r="F104" s="5" t="n">
-        <v>0.1</v>
+        <v>0.42</v>
       </c>
       <c r="G104" s="4" t="n">
-        <v>3</v>
+        <v>12.6</v>
       </c>
       <c r="H104" s="2" t="n">
         <v>1402783</v>
@@ -5166,10 +5166,10 @@
         <v>30</v>
       </c>
       <c r="F106" s="5" t="n">
-        <v>0.42</v>
+        <v>0.1</v>
       </c>
       <c r="G106" s="4" t="n">
-        <v>12.6</v>
+        <v>3</v>
       </c>
       <c r="H106" s="2" t="n">
         <v>1402783</v>
@@ -6479,13 +6479,13 @@
         </is>
       </c>
       <c r="E134" s="4" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="F134" s="5" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="G134" s="4" t="n">
-        <v>5.25</v>
+        <v>30</v>
       </c>
       <c r="H134" s="2" t="n">
         <v>1403681</v>
@@ -6620,13 +6620,13 @@
         </is>
       </c>
       <c r="E137" s="4" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="F137" s="5" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="G137" s="4" t="n">
-        <v>4.5</v>
+        <v>5.25</v>
       </c>
       <c r="H137" s="2" t="n">
         <v>1403681</v>
@@ -6670,10 +6670,10 @@
         <v>0.3</v>
       </c>
       <c r="F138" s="5" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="G138" s="4" t="n">
-        <v>30</v>
+        <v>4.5</v>
       </c>
       <c r="H138" s="2" t="n">
         <v>1403681</v>
@@ -7278,13 +7278,13 @@
         </is>
       </c>
       <c r="E151" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F151" s="5" t="n">
-        <v>25.9</v>
+        <v>27.5</v>
       </c>
       <c r="G151" s="4" t="n">
-        <v>25.9</v>
+        <v>192.5</v>
       </c>
       <c r="H151" s="2" t="n">
         <v>1405612</v>
@@ -7325,13 +7325,13 @@
         </is>
       </c>
       <c r="E152" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F152" s="5" t="n">
-        <v>124.5</v>
+        <v>25.9</v>
       </c>
       <c r="G152" s="4" t="n">
-        <v>249</v>
+        <v>25.9</v>
       </c>
       <c r="H152" s="2" t="n">
         <v>1405612</v>
@@ -7372,13 +7372,13 @@
         </is>
       </c>
       <c r="E153" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F153" s="5" t="n">
-        <v>55.2</v>
+        <v>42</v>
       </c>
       <c r="G153" s="4" t="n">
-        <v>55.2</v>
+        <v>168</v>
       </c>
       <c r="H153" s="2" t="n">
         <v>1405612</v>
@@ -7419,13 +7419,13 @@
         </is>
       </c>
       <c r="E154" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F154" s="5" t="n">
-        <v>42</v>
+        <v>55.2</v>
       </c>
       <c r="G154" s="4" t="n">
-        <v>168</v>
+        <v>55.2</v>
       </c>
       <c r="H154" s="2" t="n">
         <v>1405612</v>
@@ -7466,13 +7466,13 @@
         </is>
       </c>
       <c r="E155" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F155" s="5" t="n">
-        <v>8.5</v>
+        <v>38</v>
       </c>
       <c r="G155" s="4" t="n">
-        <v>51</v>
+        <v>266</v>
       </c>
       <c r="H155" s="2" t="n">
         <v>1405612</v>
@@ -7513,13 +7513,13 @@
         </is>
       </c>
       <c r="E156" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F156" s="5" t="n">
-        <v>27.5</v>
+        <v>8.5</v>
       </c>
       <c r="G156" s="4" t="n">
-        <v>192.5</v>
+        <v>51</v>
       </c>
       <c r="H156" s="2" t="n">
         <v>1405612</v>
@@ -7560,13 +7560,13 @@
         </is>
       </c>
       <c r="E157" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F157" s="5" t="n">
-        <v>38</v>
+        <v>124.5</v>
       </c>
       <c r="G157" s="4" t="n">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="H157" s="2" t="n">
         <v>1405612</v>
@@ -7607,13 +7607,13 @@
         </is>
       </c>
       <c r="E158" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F158" s="5" t="n">
-        <v>2.11</v>
+        <v>19.32</v>
       </c>
       <c r="G158" s="4" t="n">
-        <v>10.55</v>
+        <v>19.32</v>
       </c>
       <c r="H158" s="2" t="n">
         <v>1405673</v>
@@ -7842,13 +7842,13 @@
         </is>
       </c>
       <c r="E163" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F163" s="5" t="n">
-        <v>17.43</v>
+        <v>2.11</v>
       </c>
       <c r="G163" s="4" t="n">
-        <v>17.43</v>
+        <v>10.55</v>
       </c>
       <c r="H163" s="2" t="n">
         <v>1405673</v>
@@ -7986,10 +7986,10 @@
         <v>1</v>
       </c>
       <c r="F166" s="5" t="n">
-        <v>19.32</v>
+        <v>17.43</v>
       </c>
       <c r="G166" s="4" t="n">
-        <v>19.32</v>
+        <v>17.43</v>
       </c>
       <c r="H166" s="2" t="n">
         <v>1405673</v>
@@ -8033,10 +8033,10 @@
         <v>1</v>
       </c>
       <c r="F167" s="5" t="n">
-        <v>18.91</v>
+        <v>19.32</v>
       </c>
       <c r="G167" s="4" t="n">
-        <v>18.91</v>
+        <v>19.32</v>
       </c>
       <c r="H167" s="2" t="n">
         <v>1405673</v>
@@ -8080,10 +8080,10 @@
         <v>1</v>
       </c>
       <c r="F168" s="5" t="n">
-        <v>19.32</v>
+        <v>18.91</v>
       </c>
       <c r="G168" s="4" t="n">
-        <v>19.32</v>
+        <v>18.91</v>
       </c>
       <c r="H168" s="2" t="n">
         <v>1405673</v>
@@ -8644,10 +8644,10 @@
         <v>1</v>
       </c>
       <c r="F180" s="5" t="n">
-        <v>5870</v>
+        <v>4287</v>
       </c>
       <c r="G180" s="4" t="n">
-        <v>5870</v>
+        <v>4287</v>
       </c>
       <c r="H180" s="2" t="n">
         <v>1406248</v>
@@ -8691,10 +8691,10 @@
         <v>1</v>
       </c>
       <c r="F181" s="5" t="n">
-        <v>550</v>
+        <v>5870</v>
       </c>
       <c r="G181" s="4" t="n">
-        <v>550</v>
+        <v>5870</v>
       </c>
       <c r="H181" s="2" t="n">
         <v>1406248</v>
@@ -8738,10 +8738,10 @@
         <v>1</v>
       </c>
       <c r="F182" s="5" t="n">
-        <v>4287</v>
+        <v>550</v>
       </c>
       <c r="G182" s="4" t="n">
-        <v>4287</v>
+        <v>550</v>
       </c>
       <c r="H182" s="2" t="n">
         <v>1406248</v>
@@ -10051,13 +10051,13 @@
         </is>
       </c>
       <c r="E210" s="4" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="F210" s="5" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="G210" s="4" t="n">
-        <v>840</v>
+        <v>2450</v>
       </c>
       <c r="H210" s="2" t="n">
         <v>1409782</v>
@@ -10098,13 +10098,13 @@
         </is>
       </c>
       <c r="E211" s="4" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="F211" s="5" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="G211" s="4" t="n">
-        <v>2450</v>
+        <v>840</v>
       </c>
       <c r="H211" s="2" t="n">
         <v>1409782</v>
@@ -10427,13 +10427,13 @@
         </is>
       </c>
       <c r="E218" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F218" s="5" t="n">
         <v>14.9</v>
       </c>
       <c r="G218" s="4" t="n">
-        <v>59.6</v>
+        <v>29.8</v>
       </c>
       <c r="H218" s="2" t="n">
         <v>1410100</v>
@@ -10474,13 +10474,13 @@
         </is>
       </c>
       <c r="E219" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F219" s="5" t="n">
         <v>14.9</v>
       </c>
       <c r="G219" s="4" t="n">
-        <v>29.8</v>
+        <v>59.6</v>
       </c>
       <c r="H219" s="2" t="n">
         <v>1410100</v>
@@ -10521,13 +10521,13 @@
         </is>
       </c>
       <c r="E220" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F220" s="5" t="n">
-        <v>12</v>
+        <v>59.9</v>
       </c>
       <c r="G220" s="4" t="n">
-        <v>24</v>
+        <v>59.9</v>
       </c>
       <c r="H220" s="2" t="n">
         <v>1410100</v>
@@ -10568,13 +10568,13 @@
         </is>
       </c>
       <c r="E221" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F221" s="5" t="n">
-        <v>59.9</v>
+        <v>12</v>
       </c>
       <c r="G221" s="4" t="n">
-        <v>59.9</v>
+        <v>24</v>
       </c>
       <c r="H221" s="2" t="n">
         <v>1410100</v>
@@ -10947,10 +10947,10 @@
         <v>2</v>
       </c>
       <c r="F229" s="5" t="n">
-        <v>593.505</v>
+        <v>2374.03</v>
       </c>
       <c r="G229" s="4" t="n">
-        <v>1187.01</v>
+        <v>4748.06</v>
       </c>
       <c r="H229" s="2" t="n">
         <v>1410106</v>
@@ -11041,10 +11041,10 @@
         <v>2</v>
       </c>
       <c r="F231" s="5" t="n">
-        <v>2374.03</v>
+        <v>593.505</v>
       </c>
       <c r="G231" s="4" t="n">
-        <v>4748.06</v>
+        <v>1187.01</v>
       </c>
       <c r="H231" s="2" t="n">
         <v>1410106</v>
@@ -15503,13 +15503,13 @@
         </is>
       </c>
       <c r="E326" s="4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F326" s="5" t="n">
-        <v>115</v>
+        <v>189</v>
       </c>
       <c r="G326" s="4" t="n">
-        <v>115</v>
+        <v>1701</v>
       </c>
       <c r="H326" s="2" t="n">
         <v>1429513</v>
@@ -15550,13 +15550,13 @@
         </is>
       </c>
       <c r="E327" s="4" t="n">
-        <v>40</v>
+        <v>9</v>
       </c>
       <c r="F327" s="5" t="n">
-        <v>16</v>
+        <v>130</v>
       </c>
       <c r="G327" s="4" t="n">
-        <v>640</v>
+        <v>1170</v>
       </c>
       <c r="H327" s="2" t="n">
         <v>1429513</v>
@@ -15597,13 +15597,13 @@
         </is>
       </c>
       <c r="E328" s="4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F328" s="5" t="n">
-        <v>22</v>
+        <v>115</v>
       </c>
       <c r="G328" s="4" t="n">
-        <v>176</v>
+        <v>115</v>
       </c>
       <c r="H328" s="2" t="n">
         <v>1429513</v>
@@ -15644,13 +15644,13 @@
         </is>
       </c>
       <c r="E329" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F329" s="5" t="n">
-        <v>130</v>
+        <v>22</v>
       </c>
       <c r="G329" s="4" t="n">
-        <v>1170</v>
+        <v>176</v>
       </c>
       <c r="H329" s="2" t="n">
         <v>1429513</v>
@@ -15691,13 +15691,13 @@
         </is>
       </c>
       <c r="E330" s="4" t="n">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="F330" s="5" t="n">
-        <v>189</v>
+        <v>16</v>
       </c>
       <c r="G330" s="4" t="n">
-        <v>1701</v>
+        <v>640</v>
       </c>
       <c r="H330" s="2" t="n">
         <v>1429513</v>
@@ -15788,10 +15788,10 @@
         <v>20</v>
       </c>
       <c r="F332" s="5" t="n">
-        <v>22.55</v>
+        <v>3.27</v>
       </c>
       <c r="G332" s="4" t="n">
-        <v>451</v>
+        <v>65.4</v>
       </c>
       <c r="H332" s="2" t="n">
         <v>1429513</v>
@@ -15835,10 +15835,10 @@
         <v>20</v>
       </c>
       <c r="F333" s="5" t="n">
-        <v>3.27</v>
+        <v>22.55</v>
       </c>
       <c r="G333" s="4" t="n">
-        <v>65.4</v>
+        <v>451</v>
       </c>
       <c r="H333" s="2" t="n">
         <v>1429513</v>
@@ -16020,13 +16020,13 @@
         </is>
       </c>
       <c r="E337" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F337" s="5" t="n">
-        <v>39</v>
+        <v>17.32</v>
       </c>
       <c r="G337" s="4" t="n">
-        <v>234</v>
+        <v>69.28</v>
       </c>
       <c r="H337" s="2" t="n">
         <v>1431621</v>
@@ -16161,13 +16161,13 @@
         </is>
       </c>
       <c r="E340" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F340" s="5" t="n">
-        <v>17.32</v>
+        <v>39</v>
       </c>
       <c r="G340" s="4" t="n">
-        <v>69.28</v>
+        <v>234</v>
       </c>
       <c r="H340" s="2" t="n">
         <v>1431621</v>
@@ -16302,13 +16302,13 @@
         </is>
       </c>
       <c r="E343" s="4" t="n">
-        <v>1</v>
+        <v>2.7</v>
       </c>
       <c r="F343" s="5" t="n">
-        <v>1900</v>
+        <v>80</v>
       </c>
       <c r="G343" s="4" t="n">
-        <v>1900</v>
+        <v>216</v>
       </c>
       <c r="H343" s="2" t="n">
         <v>1431836</v>
@@ -16349,13 +16349,13 @@
         </is>
       </c>
       <c r="E344" s="4" t="n">
-        <v>2.7</v>
+        <v>1</v>
       </c>
       <c r="F344" s="5" t="n">
-        <v>80</v>
+        <v>1900</v>
       </c>
       <c r="G344" s="4" t="n">
-        <v>216</v>
+        <v>1900</v>
       </c>
       <c r="H344" s="2" t="n">
         <v>1431836</v>
@@ -16772,13 +16772,13 @@
         </is>
       </c>
       <c r="E353" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F353" s="5" t="n">
-        <v>28.9</v>
+        <v>3.45</v>
       </c>
       <c r="G353" s="4" t="n">
-        <v>115.6</v>
+        <v>6.9</v>
       </c>
       <c r="H353" s="2" t="n">
         <v>1432029</v>
@@ -16866,13 +16866,13 @@
         </is>
       </c>
       <c r="E355" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F355" s="5" t="n">
-        <v>3.45</v>
+        <v>28.9</v>
       </c>
       <c r="G355" s="4" t="n">
-        <v>6.9</v>
+        <v>115.6</v>
       </c>
       <c r="H355" s="2" t="n">
         <v>1432029</v>
@@ -16916,10 +16916,10 @@
         <v>15</v>
       </c>
       <c r="F356" s="5" t="n">
-        <v>1.5</v>
+        <v>3.99</v>
       </c>
       <c r="G356" s="4" t="n">
-        <v>22.5</v>
+        <v>59.85</v>
       </c>
       <c r="H356" s="2" t="n">
         <v>1432046</v>
@@ -16963,10 +16963,10 @@
         <v>15</v>
       </c>
       <c r="F357" s="5" t="n">
-        <v>3.99</v>
+        <v>1.5</v>
       </c>
       <c r="G357" s="4" t="n">
-        <v>59.85</v>
+        <v>22.5</v>
       </c>
       <c r="H357" s="2" t="n">
         <v>1432046</v>
@@ -17900,13 +17900,13 @@
         </is>
       </c>
       <c r="E377" s="4" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="F377" s="5" t="n">
-        <v>6.28</v>
+        <v>5.28</v>
       </c>
       <c r="G377" s="4" t="n">
-        <v>314</v>
+        <v>5.28</v>
       </c>
       <c r="H377" s="2" t="n">
         <v>1437076</v>
@@ -17947,13 +17947,13 @@
         </is>
       </c>
       <c r="E378" s="4" t="n">
-        <v>2</v>
+        <v>80</v>
       </c>
       <c r="F378" s="5" t="n">
-        <v>2.95</v>
+        <v>0.63</v>
       </c>
       <c r="G378" s="4" t="n">
-        <v>5.9</v>
+        <v>50.4</v>
       </c>
       <c r="H378" s="2" t="n">
         <v>1437076</v>
@@ -17994,13 +17994,13 @@
         </is>
       </c>
       <c r="E379" s="4" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="F379" s="5" t="n">
-        <v>1.95</v>
+        <v>4.12</v>
       </c>
       <c r="G379" s="4" t="n">
-        <v>58.5</v>
+        <v>8.24</v>
       </c>
       <c r="H379" s="2" t="n">
         <v>1437076</v>
@@ -18044,10 +18044,10 @@
         <v>1</v>
       </c>
       <c r="F380" s="5" t="n">
-        <v>5.28</v>
+        <v>5.62</v>
       </c>
       <c r="G380" s="4" t="n">
-        <v>5.28</v>
+        <v>5.62</v>
       </c>
       <c r="H380" s="2" t="n">
         <v>1437076</v>
@@ -18088,13 +18088,13 @@
         </is>
       </c>
       <c r="E381" s="4" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F381" s="5" t="n">
-        <v>0.63</v>
+        <v>2.53</v>
       </c>
       <c r="G381" s="4" t="n">
-        <v>50.4</v>
+        <v>253</v>
       </c>
       <c r="H381" s="2" t="n">
         <v>1437076</v>
@@ -18135,13 +18135,13 @@
         </is>
       </c>
       <c r="E382" s="4" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F382" s="5" t="n">
-        <v>4.12</v>
+        <v>1.29</v>
       </c>
       <c r="G382" s="4" t="n">
-        <v>8.24</v>
+        <v>12.9</v>
       </c>
       <c r="H382" s="2" t="n">
         <v>1437076</v>
@@ -18182,13 +18182,13 @@
         </is>
       </c>
       <c r="E383" s="4" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F383" s="5" t="n">
-        <v>5.62</v>
+        <v>2.53</v>
       </c>
       <c r="G383" s="4" t="n">
-        <v>5.62</v>
+        <v>253</v>
       </c>
       <c r="H383" s="2" t="n">
         <v>1437076</v>
@@ -18229,13 +18229,13 @@
         </is>
       </c>
       <c r="E384" s="4" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="F384" s="5" t="n">
-        <v>27.7</v>
+        <v>2.53</v>
       </c>
       <c r="G384" s="4" t="n">
-        <v>55.4</v>
+        <v>253</v>
       </c>
       <c r="H384" s="2" t="n">
         <v>1437076</v>
@@ -18276,13 +18276,13 @@
         </is>
       </c>
       <c r="E385" s="4" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="F385" s="5" t="n">
-        <v>8.81</v>
+        <v>4.16</v>
       </c>
       <c r="G385" s="4" t="n">
-        <v>17.62</v>
+        <v>416</v>
       </c>
       <c r="H385" s="2" t="n">
         <v>1437076</v>
@@ -18323,13 +18323,13 @@
         </is>
       </c>
       <c r="E386" s="4" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="F386" s="5" t="n">
-        <v>1.29</v>
+        <v>6.28</v>
       </c>
       <c r="G386" s="4" t="n">
-        <v>12.9</v>
+        <v>314</v>
       </c>
       <c r="H386" s="2" t="n">
         <v>1437076</v>
@@ -18370,13 +18370,13 @@
         </is>
       </c>
       <c r="E387" s="4" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F387" s="5" t="n">
-        <v>2.53</v>
+        <v>6.63</v>
       </c>
       <c r="G387" s="4" t="n">
-        <v>253</v>
+        <v>6.63</v>
       </c>
       <c r="H387" s="2" t="n">
         <v>1437076</v>
@@ -18417,13 +18417,13 @@
         </is>
       </c>
       <c r="E388" s="4" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="F388" s="5" t="n">
-        <v>2.53</v>
+        <v>8.81</v>
       </c>
       <c r="G388" s="4" t="n">
-        <v>253</v>
+        <v>17.62</v>
       </c>
       <c r="H388" s="2" t="n">
         <v>1437076</v>
@@ -18464,13 +18464,13 @@
         </is>
       </c>
       <c r="E389" s="4" t="n">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="F389" s="5" t="n">
-        <v>2.53</v>
+        <v>3.6</v>
       </c>
       <c r="G389" s="4" t="n">
-        <v>253</v>
+        <v>14.4</v>
       </c>
       <c r="H389" s="2" t="n">
         <v>1437076</v>
@@ -18511,13 +18511,13 @@
         </is>
       </c>
       <c r="E390" s="4" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F390" s="5" t="n">
-        <v>4.16</v>
+        <v>30.25</v>
       </c>
       <c r="G390" s="4" t="n">
-        <v>416</v>
+        <v>30.25</v>
       </c>
       <c r="H390" s="2" t="n">
         <v>1437076</v>
@@ -18558,13 +18558,13 @@
         </is>
       </c>
       <c r="E391" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F391" s="5" t="n">
-        <v>6.63</v>
+        <v>30.25</v>
       </c>
       <c r="G391" s="4" t="n">
-        <v>6.63</v>
+        <v>90.75</v>
       </c>
       <c r="H391" s="2" t="n">
         <v>1437076</v>
@@ -18605,13 +18605,13 @@
         </is>
       </c>
       <c r="E392" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F392" s="5" t="n">
-        <v>3.6</v>
+        <v>15.27</v>
       </c>
       <c r="G392" s="4" t="n">
-        <v>14.4</v>
+        <v>30.54</v>
       </c>
       <c r="H392" s="2" t="n">
         <v>1437076</v>
@@ -18652,13 +18652,13 @@
         </is>
       </c>
       <c r="E393" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F393" s="5" t="n">
-        <v>30.25</v>
+        <v>27.7</v>
       </c>
       <c r="G393" s="4" t="n">
-        <v>30.25</v>
+        <v>55.4</v>
       </c>
       <c r="H393" s="2" t="n">
         <v>1437076</v>
@@ -18699,13 +18699,13 @@
         </is>
       </c>
       <c r="E394" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F394" s="5" t="n">
-        <v>30.25</v>
+        <v>2.95</v>
       </c>
       <c r="G394" s="4" t="n">
-        <v>90.75</v>
+        <v>5.9</v>
       </c>
       <c r="H394" s="2" t="n">
         <v>1437076</v>
@@ -18746,13 +18746,13 @@
         </is>
       </c>
       <c r="E395" s="4" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="F395" s="5" t="n">
-        <v>15.27</v>
+        <v>1.95</v>
       </c>
       <c r="G395" s="4" t="n">
-        <v>30.54</v>
+        <v>58.5</v>
       </c>
       <c r="H395" s="2" t="n">
         <v>1437076</v>
@@ -18796,10 +18796,10 @@
         <v>80</v>
       </c>
       <c r="F396" s="5" t="n">
-        <v>0.86</v>
+        <v>0.19</v>
       </c>
       <c r="G396" s="4" t="n">
-        <v>68.8</v>
+        <v>15.2</v>
       </c>
       <c r="H396" s="2" t="n">
         <v>1437076</v>
@@ -18843,10 +18843,10 @@
         <v>80</v>
       </c>
       <c r="F397" s="5" t="n">
-        <v>0.19</v>
+        <v>0.86</v>
       </c>
       <c r="G397" s="4" t="n">
-        <v>15.2</v>
+        <v>68.8</v>
       </c>
       <c r="H397" s="2" t="n">
         <v>1437076</v>
@@ -19028,13 +19028,13 @@
         </is>
       </c>
       <c r="E401" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F401" s="5" t="n">
-        <v>8.5</v>
+        <v>6.75</v>
       </c>
       <c r="G401" s="4" t="n">
-        <v>25.5</v>
+        <v>27</v>
       </c>
       <c r="H401" s="2" t="n">
         <v>1437082</v>
@@ -19075,13 +19075,13 @@
         </is>
       </c>
       <c r="E402" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F402" s="5" t="n">
-        <v>6.75</v>
+        <v>8.5</v>
       </c>
       <c r="G402" s="4" t="n">
-        <v>27</v>
+        <v>25.5</v>
       </c>
       <c r="H402" s="2" t="n">
         <v>1437082</v>
@@ -25984,13 +25984,13 @@
         </is>
       </c>
       <c r="E549" s="4" t="n">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="F549" s="5" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="G549" s="4" t="n">
-        <v>80</v>
+        <v>6.25</v>
       </c>
       <c r="H549" s="2" t="n">
         <v>1480786</v>
@@ -26078,13 +26078,13 @@
         </is>
       </c>
       <c r="E551" s="4" t="n">
-        <v>0.25</v>
+        <v>0.8</v>
       </c>
       <c r="F551" s="5" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="G551" s="4" t="n">
-        <v>6.25</v>
+        <v>12.8</v>
       </c>
       <c r="H551" s="2" t="n">
         <v>1480786</v>
@@ -26125,13 +26125,13 @@
         </is>
       </c>
       <c r="E552" s="4" t="n">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="F552" s="5" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G552" s="4" t="n">
-        <v>12.8</v>
+        <v>27</v>
       </c>
       <c r="H552" s="2" t="n">
         <v>1480786</v>
@@ -26172,13 +26172,13 @@
         </is>
       </c>
       <c r="E553" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F553" s="5" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G553" s="4" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="H553" s="2" t="n">
         <v>1480786</v>
@@ -26219,13 +26219,13 @@
         </is>
       </c>
       <c r="E554" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F554" s="5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G554" s="4" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H554" s="2" t="n">
         <v>1480786</v>
@@ -26269,10 +26269,10 @@
         <v>2</v>
       </c>
       <c r="F555" s="5" t="n">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G555" s="4" t="n">
-        <v>28</v>
+        <v>80</v>
       </c>
       <c r="H555" s="2" t="n">
         <v>1480786</v>
@@ -26360,13 +26360,13 @@
         </is>
       </c>
       <c r="E557" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F557" s="5" t="n">
-        <v>8.81</v>
+        <v>0.33</v>
       </c>
       <c r="G557" s="4" t="n">
-        <v>17.62</v>
+        <v>2.64</v>
       </c>
       <c r="H557" s="2" t="n">
         <v>1480796</v>
@@ -26407,13 +26407,13 @@
         </is>
       </c>
       <c r="E558" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F558" s="5" t="n">
-        <v>0.33</v>
+        <v>8.81</v>
       </c>
       <c r="G558" s="4" t="n">
-        <v>2.64</v>
+        <v>17.62</v>
       </c>
       <c r="H558" s="2" t="n">
         <v>1480796</v>
@@ -26454,13 +26454,13 @@
         </is>
       </c>
       <c r="E559" s="4" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="F559" s="5" t="n">
-        <v>1.89</v>
+        <v>2.95</v>
       </c>
       <c r="G559" s="4" t="n">
-        <v>37.8</v>
+        <v>5.9</v>
       </c>
       <c r="H559" s="2" t="n">
         <v>1480796</v>
@@ -26548,13 +26548,13 @@
         </is>
       </c>
       <c r="E561" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F561" s="5" t="n">
-        <v>2.95</v>
+        <v>14.06</v>
       </c>
       <c r="G561" s="4" t="n">
-        <v>5.9</v>
+        <v>14.06</v>
       </c>
       <c r="H561" s="2" t="n">
         <v>1480796</v>
@@ -26595,13 +26595,13 @@
         </is>
       </c>
       <c r="E562" s="4" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F562" s="5" t="n">
-        <v>14.06</v>
+        <v>1.89</v>
       </c>
       <c r="G562" s="4" t="n">
-        <v>14.06</v>
+        <v>37.8</v>
       </c>
       <c r="H562" s="2" t="n">
         <v>1480796</v>
@@ -26927,10 +26927,10 @@
         <v>1</v>
       </c>
       <c r="F569" s="5" t="n">
-        <v>6.08</v>
+        <v>5.83</v>
       </c>
       <c r="G569" s="4" t="n">
-        <v>6.08</v>
+        <v>5.83</v>
       </c>
       <c r="H569" s="2" t="n">
         <v>1482331</v>
@@ -26974,10 +26974,10 @@
         <v>1</v>
       </c>
       <c r="F570" s="5" t="n">
-        <v>8.23</v>
+        <v>5.74</v>
       </c>
       <c r="G570" s="4" t="n">
-        <v>8.23</v>
+        <v>5.74</v>
       </c>
       <c r="H570" s="2" t="n">
         <v>1482331</v>
@@ -27021,10 +27021,10 @@
         <v>1</v>
       </c>
       <c r="F571" s="5" t="n">
-        <v>5.74</v>
+        <v>31.33</v>
       </c>
       <c r="G571" s="4" t="n">
-        <v>5.74</v>
+        <v>31.33</v>
       </c>
       <c r="H571" s="2" t="n">
         <v>1482331</v>
@@ -27068,10 +27068,10 @@
         <v>1</v>
       </c>
       <c r="F572" s="5" t="n">
-        <v>5.83</v>
+        <v>6.08</v>
       </c>
       <c r="G572" s="4" t="n">
-        <v>5.83</v>
+        <v>6.08</v>
       </c>
       <c r="H572" s="2" t="n">
         <v>1482331</v>
@@ -27115,10 +27115,10 @@
         <v>1</v>
       </c>
       <c r="F573" s="5" t="n">
-        <v>6.16</v>
+        <v>8.23</v>
       </c>
       <c r="G573" s="4" t="n">
-        <v>6.16</v>
+        <v>8.23</v>
       </c>
       <c r="H573" s="2" t="n">
         <v>1482331</v>
@@ -27303,10 +27303,10 @@
         <v>1</v>
       </c>
       <c r="F577" s="5" t="n">
-        <v>31.33</v>
+        <v>6.16</v>
       </c>
       <c r="G577" s="4" t="n">
-        <v>31.33</v>
+        <v>6.16</v>
       </c>
       <c r="H577" s="2" t="n">
         <v>1482331</v>
@@ -27397,10 +27397,10 @@
         <v>1</v>
       </c>
       <c r="F579" s="5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G579" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H579" s="2" t="n">
         <v>1482337</v>
@@ -27441,13 +27441,13 @@
         </is>
       </c>
       <c r="E580" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F580" s="5" t="n">
-        <v>9</v>
+        <v>2.6</v>
       </c>
       <c r="G580" s="4" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H580" s="2" t="n">
         <v>1482337</v>
@@ -27535,13 +27535,13 @@
         </is>
       </c>
       <c r="E582" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F582" s="5" t="n">
         <v>2.6</v>
       </c>
       <c r="G582" s="4" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="H582" s="2" t="n">
         <v>1482337</v>
@@ -27582,13 +27582,13 @@
         </is>
       </c>
       <c r="E583" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F583" s="5" t="n">
-        <v>2.6</v>
+        <v>7</v>
       </c>
       <c r="G583" s="4" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="H583" s="2" t="n">
         <v>1482337</v>
@@ -28851,13 +28851,13 @@
         </is>
       </c>
       <c r="E610" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F610" s="5" t="n">
-        <v>17.52</v>
+        <v>6.6</v>
       </c>
       <c r="G610" s="4" t="n">
-        <v>70.08</v>
+        <v>19.8</v>
       </c>
       <c r="H610" s="2" t="n">
         <v>1490652</v>
@@ -28901,10 +28901,10 @@
         <v>3</v>
       </c>
       <c r="F611" s="5" t="n">
-        <v>6.6</v>
+        <v>55.99</v>
       </c>
       <c r="G611" s="4" t="n">
-        <v>19.8</v>
+        <v>167.97</v>
       </c>
       <c r="H611" s="2" t="n">
         <v>1490652</v>
@@ -28945,13 +28945,13 @@
         </is>
       </c>
       <c r="E612" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F612" s="5" t="n">
-        <v>55.99</v>
+        <v>0.48</v>
       </c>
       <c r="G612" s="4" t="n">
-        <v>167.97</v>
+        <v>4.8</v>
       </c>
       <c r="H612" s="2" t="n">
         <v>1490652</v>
@@ -28995,10 +28995,10 @@
         <v>10</v>
       </c>
       <c r="F613" s="5" t="n">
-        <v>0.48</v>
+        <v>0.86</v>
       </c>
       <c r="G613" s="4" t="n">
-        <v>4.8</v>
+        <v>8.6</v>
       </c>
       <c r="H613" s="2" t="n">
         <v>1490652</v>
@@ -29039,13 +29039,13 @@
         </is>
       </c>
       <c r="E614" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F614" s="5" t="n">
-        <v>41.71</v>
+        <v>17.52</v>
       </c>
       <c r="G614" s="4" t="n">
-        <v>83.42</v>
+        <v>70.08</v>
       </c>
       <c r="H614" s="2" t="n">
         <v>1490652</v>
@@ -29086,13 +29086,13 @@
         </is>
       </c>
       <c r="E615" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F615" s="5" t="n">
-        <v>49.9</v>
+        <v>41.71</v>
       </c>
       <c r="G615" s="4" t="n">
-        <v>49.9</v>
+        <v>83.42</v>
       </c>
       <c r="H615" s="2" t="n">
         <v>1490652</v>
@@ -29133,13 +29133,13 @@
         </is>
       </c>
       <c r="E616" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F616" s="5" t="n">
-        <v>0.86</v>
+        <v>49.9</v>
       </c>
       <c r="G616" s="4" t="n">
-        <v>8.6</v>
+        <v>49.9</v>
       </c>
       <c r="H616" s="2" t="n">
         <v>1490652</v>
@@ -30449,13 +30449,13 @@
         </is>
       </c>
       <c r="E644" s="4" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F644" s="5" t="n">
-        <v>178.5</v>
+        <v>1</v>
       </c>
       <c r="G644" s="4" t="n">
-        <v>357</v>
+        <v>10</v>
       </c>
       <c r="H644" s="2" t="n">
         <v>1497640</v>
@@ -30496,13 +30496,13 @@
         </is>
       </c>
       <c r="E645" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F645" s="5" t="n">
-        <v>1</v>
+        <v>178.5</v>
       </c>
       <c r="G645" s="4" t="n">
-        <v>10</v>
+        <v>357</v>
       </c>
       <c r="H645" s="2" t="n">
         <v>1497640</v>
@@ -30734,10 +30734,10 @@
         <v>200</v>
       </c>
       <c r="F650" s="5" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="G650" s="4" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="H650" s="2" t="n">
         <v>1498122</v>
@@ -30781,10 +30781,10 @@
         <v>200</v>
       </c>
       <c r="F651" s="5" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="G651" s="4" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="H651" s="2" t="n">
         <v>1498122</v>
@@ -31721,10 +31721,10 @@
         <v>2</v>
       </c>
       <c r="F671" s="5" t="n">
-        <v>2.03</v>
+        <v>1.01</v>
       </c>
       <c r="G671" s="4" t="n">
-        <v>4.06</v>
+        <v>2.02</v>
       </c>
       <c r="H671" s="2" t="n">
         <v>1503029</v>
@@ -31765,13 +31765,13 @@
         </is>
       </c>
       <c r="E672" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F672" s="5" t="n">
-        <v>30</v>
+        <v>30.63</v>
       </c>
       <c r="G672" s="4" t="n">
-        <v>60</v>
+        <v>30.63</v>
       </c>
       <c r="H672" s="2" t="n">
         <v>1503029</v>
@@ -31862,10 +31862,10 @@
         <v>2</v>
       </c>
       <c r="F674" s="5" t="n">
-        <v>1.01</v>
+        <v>30</v>
       </c>
       <c r="G674" s="4" t="n">
-        <v>2.02</v>
+        <v>60</v>
       </c>
       <c r="H674" s="2" t="n">
         <v>1503029</v>
@@ -31906,13 +31906,13 @@
         </is>
       </c>
       <c r="E675" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F675" s="5" t="n">
-        <v>5.39</v>
+        <v>2.03</v>
       </c>
       <c r="G675" s="4" t="n">
-        <v>5.39</v>
+        <v>4.06</v>
       </c>
       <c r="H675" s="2" t="n">
         <v>1503029</v>
@@ -31956,10 +31956,10 @@
         <v>1</v>
       </c>
       <c r="F676" s="5" t="n">
-        <v>30.63</v>
+        <v>5.39</v>
       </c>
       <c r="G676" s="4" t="n">
-        <v>30.63</v>
+        <v>5.39</v>
       </c>
       <c r="H676" s="2" t="n">
         <v>1503029</v>
@@ -32379,10 +32379,10 @@
         <v>1</v>
       </c>
       <c r="F685" s="5" t="n">
-        <v>4.18</v>
+        <v>14.02</v>
       </c>
       <c r="G685" s="4" t="n">
-        <v>4.18</v>
+        <v>14.02</v>
       </c>
       <c r="H685" s="2" t="n">
         <v>1503440</v>
@@ -32426,10 +32426,10 @@
         <v>1</v>
       </c>
       <c r="F686" s="5" t="n">
-        <v>13.6</v>
+        <v>4.18</v>
       </c>
       <c r="G686" s="4" t="n">
-        <v>13.6</v>
+        <v>4.18</v>
       </c>
       <c r="H686" s="2" t="n">
         <v>1503440</v>
@@ -32473,10 +32473,10 @@
         <v>1</v>
       </c>
       <c r="F687" s="5" t="n">
-        <v>14.02</v>
+        <v>13.6</v>
       </c>
       <c r="G687" s="4" t="n">
-        <v>14.02</v>
+        <v>13.6</v>
       </c>
       <c r="H687" s="2" t="n">
         <v>1503440</v>
@@ -33225,10 +33225,10 @@
         <v>2</v>
       </c>
       <c r="F703" s="5" t="n">
-        <v>2.29</v>
+        <v>2.38</v>
       </c>
       <c r="G703" s="4" t="n">
-        <v>4.58</v>
+        <v>4.76</v>
       </c>
       <c r="H703" s="2" t="n">
         <v>1512391</v>
@@ -33272,10 +33272,10 @@
         <v>2</v>
       </c>
       <c r="F704" s="5" t="n">
-        <v>2.38</v>
+        <v>2.88</v>
       </c>
       <c r="G704" s="4" t="n">
-        <v>4.76</v>
+        <v>5.76</v>
       </c>
       <c r="H704" s="2" t="n">
         <v>1512391</v>
@@ -33319,10 +33319,10 @@
         <v>1</v>
       </c>
       <c r="F705" s="5" t="n">
-        <v>15.25</v>
+        <v>27.65</v>
       </c>
       <c r="G705" s="4" t="n">
-        <v>15.25</v>
+        <v>27.65</v>
       </c>
       <c r="H705" s="2" t="n">
         <v>1512391</v>
@@ -33366,10 +33366,10 @@
         <v>1</v>
       </c>
       <c r="F706" s="5" t="n">
-        <v>10.3</v>
+        <v>15.25</v>
       </c>
       <c r="G706" s="4" t="n">
-        <v>10.3</v>
+        <v>15.25</v>
       </c>
       <c r="H706" s="2" t="n">
         <v>1512391</v>
@@ -33413,10 +33413,10 @@
         <v>1</v>
       </c>
       <c r="F707" s="5" t="n">
-        <v>12.25</v>
+        <v>10.3</v>
       </c>
       <c r="G707" s="4" t="n">
-        <v>12.25</v>
+        <v>10.3</v>
       </c>
       <c r="H707" s="2" t="n">
         <v>1512391</v>
@@ -33460,10 +33460,10 @@
         <v>1</v>
       </c>
       <c r="F708" s="5" t="n">
-        <v>27.65</v>
+        <v>12.25</v>
       </c>
       <c r="G708" s="4" t="n">
-        <v>27.65</v>
+        <v>12.25</v>
       </c>
       <c r="H708" s="2" t="n">
         <v>1512391</v>
@@ -33507,10 +33507,10 @@
         <v>2</v>
       </c>
       <c r="F709" s="5" t="n">
-        <v>2.88</v>
+        <v>2.29</v>
       </c>
       <c r="G709" s="4" t="n">
-        <v>5.76</v>
+        <v>4.58</v>
       </c>
       <c r="H709" s="2" t="n">
         <v>1512391</v>
@@ -33739,13 +33739,13 @@
         </is>
       </c>
       <c r="E714" s="4" t="n">
-        <v>300</v>
+        <v>15</v>
       </c>
       <c r="F714" s="5" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="G714" s="4" t="n">
-        <v>45</v>
+        <v>2.55</v>
       </c>
       <c r="H714" s="2" t="n">
         <v>1512750</v>
@@ -33789,10 +33789,10 @@
         <v>15</v>
       </c>
       <c r="F715" s="5" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="G715" s="4" t="n">
-        <v>12</v>
+        <v>4.5</v>
       </c>
       <c r="H715" s="2" t="n">
         <v>1512750</v>
@@ -33836,10 +33836,10 @@
         <v>15</v>
       </c>
       <c r="F716" s="5" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="G716" s="4" t="n">
-        <v>4.5</v>
+        <v>12</v>
       </c>
       <c r="H716" s="2" t="n">
         <v>1512750</v>
@@ -33880,13 +33880,13 @@
         </is>
       </c>
       <c r="E717" s="4" t="n">
-        <v>15</v>
+        <v>300</v>
       </c>
       <c r="F717" s="5" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="G717" s="4" t="n">
-        <v>2.55</v>
+        <v>45</v>
       </c>
       <c r="H717" s="2" t="n">
         <v>1512750</v>
@@ -33974,13 +33974,13 @@
         </is>
       </c>
       <c r="E719" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F719" s="5" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G719" s="4" t="n">
-        <v>170</v>
+        <v>25</v>
       </c>
       <c r="H719" s="2" t="n">
         <v>1513521</v>
@@ -34024,10 +34024,10 @@
         <v>1</v>
       </c>
       <c r="F720" s="5" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G720" s="4" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H720" s="2" t="n">
         <v>1513521</v>
@@ -34068,13 +34068,13 @@
         </is>
       </c>
       <c r="E721" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F721" s="5" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="G721" s="4" t="n">
-        <v>35</v>
+        <v>170</v>
       </c>
       <c r="H721" s="2" t="n">
         <v>1513521</v>
@@ -34491,13 +34491,13 @@
         </is>
       </c>
       <c r="E730" s="4" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F730" s="5" t="n">
         <v>100</v>
       </c>
       <c r="G730" s="4" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="H730" s="2" t="n">
         <v>1513779</v>
@@ -34538,13 +34538,13 @@
         </is>
       </c>
       <c r="E731" s="4" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="F731" s="5" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G731" s="4" t="n">
-        <v>750</v>
+        <v>2000</v>
       </c>
       <c r="H731" s="2" t="n">
         <v>1513779</v>
@@ -34585,13 +34585,13 @@
         </is>
       </c>
       <c r="E732" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F732" s="5" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="G732" s="4" t="n">
-        <v>1000</v>
+        <v>750</v>
       </c>
       <c r="H732" s="2" t="n">
         <v>1513779</v>
@@ -36935,13 +36935,13 @@
         </is>
       </c>
       <c r="E782" s="4" t="n">
-        <v>1.06</v>
+        <v>1.33</v>
       </c>
       <c r="F782" s="5" t="n">
-        <v>17.9621</v>
+        <v>17.9624</v>
       </c>
       <c r="G782" s="4" t="n">
-        <v>18.95</v>
+        <v>23.89</v>
       </c>
       <c r="H782" s="2" t="n">
         <v>1522565</v>
@@ -36982,13 +36982,13 @@
         </is>
       </c>
       <c r="E783" s="4" t="n">
-        <v>1.33</v>
+        <v>1.06</v>
       </c>
       <c r="F783" s="5" t="n">
-        <v>17.9624</v>
+        <v>17.9621</v>
       </c>
       <c r="G783" s="4" t="n">
-        <v>23.89</v>
+        <v>18.95</v>
       </c>
       <c r="H783" s="2" t="n">
         <v>1522565</v>
@@ -37217,13 +37217,13 @@
         </is>
       </c>
       <c r="E788" s="4" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="F788" s="5" t="n">
-        <v>127.6</v>
+        <v>139.6</v>
       </c>
       <c r="G788" s="4" t="n">
-        <v>1786.4</v>
+        <v>279.2</v>
       </c>
       <c r="H788" s="2" t="n">
         <v>1522616</v>
@@ -37358,13 +37358,13 @@
         </is>
       </c>
       <c r="E791" s="4" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F791" s="5" t="n">
-        <v>139.6</v>
+        <v>127.6</v>
       </c>
       <c r="G791" s="4" t="n">
-        <v>279.2</v>
+        <v>1786.4</v>
       </c>
       <c r="H791" s="2" t="n">
         <v>1522616</v>
@@ -41776,13 +41776,13 @@
         </is>
       </c>
       <c r="E885" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F885" s="5" t="n">
-        <v>0.11</v>
+        <v>53</v>
       </c>
       <c r="G885" s="4" t="n">
-        <v>0.66</v>
+        <v>53</v>
       </c>
       <c r="H885" s="2" t="n">
         <v>1539898</v>
@@ -43233,13 +43233,13 @@
         </is>
       </c>
       <c r="E916" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F916" s="5" t="n">
-        <v>53</v>
+        <v>0.11</v>
       </c>
       <c r="G916" s="4" t="n">
-        <v>53</v>
+        <v>0.66</v>
       </c>
       <c r="H916" s="2" t="n">
         <v>1539898</v>
@@ -49813,13 +49813,13 @@
         </is>
       </c>
       <c r="E1056" s="4" t="n">
-        <v>100</v>
+        <v>0.5</v>
       </c>
       <c r="F1056" s="5" t="n">
-        <v>0.22</v>
+        <v>20</v>
       </c>
       <c r="G1056" s="4" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H1056" s="2" t="n">
         <v>1565694</v>
@@ -49863,10 +49863,10 @@
         <v>100</v>
       </c>
       <c r="F1057" s="5" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="G1057" s="4" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H1057" s="2" t="n">
         <v>1565694</v>
@@ -50051,10 +50051,10 @@
         <v>1</v>
       </c>
       <c r="F1061" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G1061" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H1061" s="2" t="n">
         <v>1565694</v>
@@ -50095,13 +50095,13 @@
         </is>
       </c>
       <c r="E1062" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1062" s="5" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G1062" s="4" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="H1062" s="2" t="n">
         <v>1565694</v>
@@ -50142,13 +50142,13 @@
         </is>
       </c>
       <c r="E1063" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1063" s="5" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G1063" s="4" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="H1063" s="2" t="n">
         <v>1565694</v>
@@ -50424,13 +50424,13 @@
         </is>
       </c>
       <c r="E1069" s="4" t="n">
-        <v>0.5</v>
+        <v>100</v>
       </c>
       <c r="F1069" s="5" t="n">
-        <v>20</v>
+        <v>0.25</v>
       </c>
       <c r="G1069" s="4" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H1069" s="2" t="n">
         <v>1565694</v>
@@ -59683,13 +59683,13 @@
         </is>
       </c>
       <c r="E1266" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F1266" s="5" t="n">
-        <v>2.66</v>
+        <v>1.29</v>
       </c>
       <c r="G1266" s="4" t="n">
-        <v>15.96</v>
+        <v>5.16</v>
       </c>
       <c r="H1266" s="2" t="n">
         <v>1591999</v>
@@ -59730,13 +59730,13 @@
         </is>
       </c>
       <c r="E1267" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F1267" s="5" t="n">
-        <v>1.29</v>
+        <v>3.25</v>
       </c>
       <c r="G1267" s="4" t="n">
-        <v>5.16</v>
+        <v>6.5</v>
       </c>
       <c r="H1267" s="2" t="n">
         <v>1591999</v>
@@ -59777,13 +59777,13 @@
         </is>
       </c>
       <c r="E1268" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F1268" s="5" t="n">
-        <v>13.17</v>
+        <v>2.66</v>
       </c>
       <c r="G1268" s="4" t="n">
-        <v>26.34</v>
+        <v>15.96</v>
       </c>
       <c r="H1268" s="2" t="n">
         <v>1591999</v>
@@ -59871,13 +59871,13 @@
         </is>
       </c>
       <c r="E1270" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1270" s="5" t="n">
-        <v>3.25</v>
+        <v>215.83</v>
       </c>
       <c r="G1270" s="4" t="n">
-        <v>6.5</v>
+        <v>215.83</v>
       </c>
       <c r="H1270" s="2" t="n">
         <v>1591999</v>
@@ -59921,10 +59921,10 @@
         <v>1</v>
       </c>
       <c r="F1271" s="5" t="n">
-        <v>215.83</v>
+        <v>29.93</v>
       </c>
       <c r="G1271" s="4" t="n">
-        <v>215.83</v>
+        <v>29.93</v>
       </c>
       <c r="H1271" s="2" t="n">
         <v>1591999</v>
@@ -59965,13 +59965,13 @@
         </is>
       </c>
       <c r="E1272" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1272" s="5" t="n">
-        <v>238.35</v>
+        <v>13.17</v>
       </c>
       <c r="G1272" s="4" t="n">
-        <v>238.35</v>
+        <v>26.34</v>
       </c>
       <c r="H1272" s="2" t="n">
         <v>1591999</v>
@@ -60015,10 +60015,10 @@
         <v>1</v>
       </c>
       <c r="F1273" s="5" t="n">
-        <v>41.71</v>
+        <v>238.35</v>
       </c>
       <c r="G1273" s="4" t="n">
-        <v>41.71</v>
+        <v>238.35</v>
       </c>
       <c r="H1273" s="2" t="n">
         <v>1591999</v>
@@ -60059,13 +60059,13 @@
         </is>
       </c>
       <c r="E1274" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1274" s="5" t="n">
-        <v>25.21</v>
+        <v>41.71</v>
       </c>
       <c r="G1274" s="4" t="n">
-        <v>50.42</v>
+        <v>41.71</v>
       </c>
       <c r="H1274" s="2" t="n">
         <v>1591999</v>
@@ -60106,13 +60106,13 @@
         </is>
       </c>
       <c r="E1275" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1275" s="5" t="n">
-        <v>29.93</v>
+        <v>25.21</v>
       </c>
       <c r="G1275" s="4" t="n">
-        <v>29.93</v>
+        <v>50.42</v>
       </c>
       <c r="H1275" s="2" t="n">
         <v>1591999</v>
@@ -63349,13 +63349,13 @@
         </is>
       </c>
       <c r="E1344" s="4" t="n">
-        <v>1</v>
+        <v>0.39</v>
       </c>
       <c r="F1344" s="5" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G1344" s="4" t="n">
-        <v>18</v>
+        <v>9.75</v>
       </c>
       <c r="H1344" s="2" t="n">
         <v>1600774</v>
@@ -63396,13 +63396,13 @@
         </is>
       </c>
       <c r="E1345" s="4" t="n">
-        <v>0.4</v>
+        <v>100</v>
       </c>
       <c r="F1345" s="5" t="n">
-        <v>28</v>
+        <v>0.75</v>
       </c>
       <c r="G1345" s="4" t="n">
-        <v>11.2</v>
+        <v>75</v>
       </c>
       <c r="H1345" s="2" t="n">
         <v>1600774</v>
@@ -63443,13 +63443,13 @@
         </is>
       </c>
       <c r="E1346" s="4" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F1346" s="5" t="n">
-        <v>0.75</v>
+        <v>16</v>
       </c>
       <c r="G1346" s="4" t="n">
-        <v>75</v>
+        <v>16</v>
       </c>
       <c r="H1346" s="2" t="n">
         <v>1600774</v>
@@ -63493,10 +63493,10 @@
         <v>1</v>
       </c>
       <c r="F1347" s="5" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G1347" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H1347" s="2" t="n">
         <v>1600774</v>
@@ -63725,13 +63725,13 @@
         </is>
       </c>
       <c r="E1352" s="4" t="n">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="F1352" s="5" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G1352" s="4" t="n">
-        <v>9.75</v>
+        <v>11.2</v>
       </c>
       <c r="H1352" s="2" t="n">
         <v>1600774</v>
@@ -65746,13 +65746,13 @@
         </is>
       </c>
       <c r="E1395" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1395" s="5" t="n">
-        <v>65.2</v>
+        <v>54.3</v>
       </c>
       <c r="G1395" s="4" t="n">
-        <v>260.8</v>
+        <v>325.8</v>
       </c>
       <c r="H1395" s="2" t="n">
         <v>1603907</v>
@@ -65793,13 +65793,13 @@
         </is>
       </c>
       <c r="E1396" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F1396" s="5" t="n">
         <v>65.2</v>
       </c>
       <c r="G1396" s="4" t="n">
-        <v>130.4</v>
+        <v>260.8</v>
       </c>
       <c r="H1396" s="2" t="n">
         <v>1603907</v>
@@ -65840,13 +65840,13 @@
         </is>
       </c>
       <c r="E1397" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F1397" s="5" t="n">
-        <v>54.3</v>
+        <v>65.2</v>
       </c>
       <c r="G1397" s="4" t="n">
-        <v>325.8</v>
+        <v>130.4</v>
       </c>
       <c r="H1397" s="2" t="n">
         <v>1603907</v>
@@ -66921,13 +66921,13 @@
         </is>
       </c>
       <c r="E1420" s="4" t="n">
-        <v>1.63</v>
+        <v>7.26</v>
       </c>
       <c r="F1420" s="5" t="n">
-        <v>112</v>
+        <v>144</v>
       </c>
       <c r="G1420" s="4" t="n">
-        <v>182.56</v>
+        <v>1045.44</v>
       </c>
       <c r="H1420" s="2" t="n">
         <v>1606285</v>
@@ -66968,13 +66968,13 @@
         </is>
       </c>
       <c r="E1421" s="4" t="n">
-        <v>7.26</v>
+        <v>1.63</v>
       </c>
       <c r="F1421" s="5" t="n">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="G1421" s="4" t="n">
-        <v>1045.44</v>
+        <v>182.56</v>
       </c>
       <c r="H1421" s="2" t="n">
         <v>1606285</v>
@@ -67062,13 +67062,13 @@
         </is>
       </c>
       <c r="E1423" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1423" s="5" t="n">
-        <v>21.9</v>
+        <v>8.9</v>
       </c>
       <c r="G1423" s="4" t="n">
-        <v>21.9</v>
+        <v>17.8</v>
       </c>
       <c r="H1423" s="2" t="n">
         <v>1606516</v>
@@ -67109,13 +67109,13 @@
         </is>
       </c>
       <c r="E1424" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F1424" s="5" t="n">
-        <v>5.9</v>
+        <v>12.9</v>
       </c>
       <c r="G1424" s="4" t="n">
-        <v>59</v>
+        <v>12.9</v>
       </c>
       <c r="H1424" s="2" t="n">
         <v>1606516</v>
@@ -67156,13 +67156,13 @@
         </is>
       </c>
       <c r="E1425" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F1425" s="5" t="n">
-        <v>43.9</v>
+        <v>1</v>
       </c>
       <c r="G1425" s="4" t="n">
-        <v>43.9</v>
+        <v>5</v>
       </c>
       <c r="H1425" s="2" t="n">
         <v>1606516</v>
@@ -67206,10 +67206,10 @@
         <v>1</v>
       </c>
       <c r="F1426" s="5" t="n">
-        <v>43.9</v>
+        <v>4.75</v>
       </c>
       <c r="G1426" s="4" t="n">
-        <v>43.9</v>
+        <v>4.75</v>
       </c>
       <c r="H1426" s="2" t="n">
         <v>1606516</v>
@@ -67297,13 +67297,13 @@
         </is>
       </c>
       <c r="E1428" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1428" s="5" t="n">
-        <v>8.9</v>
+        <v>43.9</v>
       </c>
       <c r="G1428" s="4" t="n">
-        <v>17.8</v>
+        <v>43.9</v>
       </c>
       <c r="H1428" s="2" t="n">
         <v>1606516</v>
@@ -67347,10 +67347,10 @@
         <v>1</v>
       </c>
       <c r="F1429" s="5" t="n">
-        <v>12.9</v>
+        <v>21.9</v>
       </c>
       <c r="G1429" s="4" t="n">
-        <v>12.9</v>
+        <v>21.9</v>
       </c>
       <c r="H1429" s="2" t="n">
         <v>1606516</v>
@@ -67391,13 +67391,13 @@
         </is>
       </c>
       <c r="E1430" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F1430" s="5" t="n">
-        <v>1</v>
+        <v>5.9</v>
       </c>
       <c r="G1430" s="4" t="n">
-        <v>5</v>
+        <v>59</v>
       </c>
       <c r="H1430" s="2" t="n">
         <v>1606516</v>
@@ -67441,10 +67441,10 @@
         <v>1</v>
       </c>
       <c r="F1431" s="5" t="n">
-        <v>4.75</v>
+        <v>43.9</v>
       </c>
       <c r="G1431" s="4" t="n">
-        <v>4.75</v>
+        <v>43.9</v>
       </c>
       <c r="H1431" s="2" t="n">
         <v>1606516</v>
@@ -67579,13 +67579,13 @@
         </is>
       </c>
       <c r="E1434" s="4" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="F1434" s="5" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="G1434" s="4" t="n">
-        <v>8</v>
+        <v>72</v>
       </c>
       <c r="H1434" s="2" t="n">
         <v>1607187</v>
@@ -67626,13 +67626,13 @@
         </is>
       </c>
       <c r="E1435" s="4" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="F1435" s="5" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="G1435" s="4" t="n">
-        <v>72</v>
+        <v>8</v>
       </c>
       <c r="H1435" s="2" t="n">
         <v>1607187</v>
@@ -69650,10 +69650,10 @@
         <v>1</v>
       </c>
       <c r="F1478" s="5" t="n">
-        <v>6.8</v>
+        <v>5.253</v>
       </c>
       <c r="G1478" s="4" t="n">
-        <v>6.8</v>
+        <v>5.25</v>
       </c>
       <c r="H1478" s="2" t="n">
         <v>1608374</v>
@@ -69697,10 +69697,10 @@
         <v>1</v>
       </c>
       <c r="F1479" s="5" t="n">
-        <v>43.428</v>
+        <v>6.8</v>
       </c>
       <c r="G1479" s="4" t="n">
-        <v>43.42</v>
+        <v>6.8</v>
       </c>
       <c r="H1479" s="2" t="n">
         <v>1608374</v>
@@ -69744,10 +69744,10 @@
         <v>1</v>
       </c>
       <c r="F1480" s="5" t="n">
-        <v>5.253</v>
+        <v>43.428</v>
       </c>
       <c r="G1480" s="4" t="n">
-        <v>5.25</v>
+        <v>43.42</v>
       </c>
       <c r="H1480" s="2" t="n">
         <v>1608374</v>
@@ -70308,10 +70308,10 @@
         <v>1</v>
       </c>
       <c r="F1492" s="5" t="n">
-        <v>5.5</v>
+        <v>169.9</v>
       </c>
       <c r="G1492" s="4" t="n">
-        <v>5.5</v>
+        <v>169.9</v>
       </c>
       <c r="H1492" s="2" t="n">
         <v>1608875</v>
@@ -70355,10 +70355,10 @@
         <v>1</v>
       </c>
       <c r="F1493" s="5" t="n">
-        <v>169.9</v>
+        <v>5.5</v>
       </c>
       <c r="G1493" s="4" t="n">
-        <v>169.9</v>
+        <v>5.5</v>
       </c>
       <c r="H1493" s="2" t="n">
         <v>1608875</v>
@@ -71013,10 +71013,10 @@
         <v>1</v>
       </c>
       <c r="F1507" s="5" t="n">
-        <v>3.64</v>
+        <v>3.75</v>
       </c>
       <c r="G1507" s="4" t="n">
-        <v>3.64</v>
+        <v>3.75</v>
       </c>
       <c r="H1507" s="2" t="n">
         <v>1610784</v>
@@ -71107,10 +71107,10 @@
         <v>1</v>
       </c>
       <c r="F1509" s="5" t="n">
-        <v>3.75</v>
+        <v>3.64</v>
       </c>
       <c r="G1509" s="4" t="n">
-        <v>3.75</v>
+        <v>3.64</v>
       </c>
       <c r="H1509" s="2" t="n">
         <v>1610784</v>
@@ -73266,13 +73266,13 @@
         </is>
       </c>
       <c r="E1555" s="4" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="F1555" s="5" t="n">
-        <v>65.2</v>
+        <v>54.3</v>
       </c>
       <c r="G1555" s="4" t="n">
-        <v>2216.8</v>
+        <v>4235.4</v>
       </c>
       <c r="H1555" s="2" t="n">
         <v>1614539</v>
@@ -73360,13 +73360,13 @@
         </is>
       </c>
       <c r="E1557" s="4" t="n">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="F1557" s="5" t="n">
-        <v>54.3</v>
+        <v>65.2</v>
       </c>
       <c r="G1557" s="4" t="n">
-        <v>4235.4</v>
+        <v>2216.8</v>
       </c>
       <c r="H1557" s="2" t="n">
         <v>1614539</v>
@@ -75710,13 +75710,13 @@
         </is>
       </c>
       <c r="E1607" s="4" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="F1607" s="5" t="n">
-        <v>24.67</v>
+        <v>37.9538</v>
       </c>
       <c r="G1607" s="4" t="n">
-        <v>1233.5</v>
+        <v>2580.86</v>
       </c>
       <c r="H1607" s="2" t="n">
         <v>1617955</v>
@@ -75757,13 +75757,13 @@
         </is>
       </c>
       <c r="E1608" s="4" t="n">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="F1608" s="5" t="n">
-        <v>37.9538</v>
+        <v>24.67</v>
       </c>
       <c r="G1608" s="4" t="n">
-        <v>2580.86</v>
+        <v>1233.5</v>
       </c>
       <c r="H1608" s="2" t="n">
         <v>1617955</v>
@@ -76932,13 +76932,13 @@
         </is>
       </c>
       <c r="E1633" s="4" t="n">
-        <v>0.26</v>
+        <v>1.5</v>
       </c>
       <c r="F1633" s="5" t="n">
-        <v>350</v>
+        <v>22</v>
       </c>
       <c r="G1633" s="4" t="n">
-        <v>91</v>
+        <v>33</v>
       </c>
       <c r="H1633" s="2" t="n">
         <v>1619290</v>
@@ -76982,10 +76982,10 @@
         <v>1.5</v>
       </c>
       <c r="F1634" s="5" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="G1634" s="4" t="n">
-        <v>33</v>
+        <v>22.5</v>
       </c>
       <c r="H1634" s="2" t="n">
         <v>1619290</v>
@@ -77029,10 +77029,10 @@
         <v>1.5</v>
       </c>
       <c r="F1635" s="5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G1635" s="4" t="n">
-        <v>22.5</v>
+        <v>21</v>
       </c>
       <c r="H1635" s="2" t="n">
         <v>1619290</v>
@@ -77073,13 +77073,13 @@
         </is>
       </c>
       <c r="E1636" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F1636" s="5" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G1636" s="4" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H1636" s="2" t="n">
         <v>1619290</v>
@@ -77120,13 +77120,13 @@
         </is>
       </c>
       <c r="E1637" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1637" s="5" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="G1637" s="4" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="H1637" s="2" t="n">
         <v>1619290</v>
@@ -77170,10 +77170,10 @@
         <v>1</v>
       </c>
       <c r="F1638" s="5" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G1638" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H1638" s="2" t="n">
         <v>1619290</v>
@@ -77214,13 +77214,13 @@
         </is>
       </c>
       <c r="E1639" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1639" s="5" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G1639" s="4" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H1639" s="2" t="n">
         <v>1619290</v>
@@ -77261,13 +77261,13 @@
         </is>
       </c>
       <c r="E1640" s="4" t="n">
-        <v>2</v>
+        <v>0.26</v>
       </c>
       <c r="F1640" s="5" t="n">
-        <v>14</v>
+        <v>350</v>
       </c>
       <c r="G1640" s="4" t="n">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="H1640" s="2" t="n">
         <v>1619290</v>
@@ -77308,13 +77308,13 @@
         </is>
       </c>
       <c r="E1641" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1641" s="5" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G1641" s="4" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="H1641" s="2" t="n">
         <v>1619290</v>
@@ -77872,13 +77872,13 @@
         </is>
       </c>
       <c r="E1653" s="4" t="n">
-        <v>1.65</v>
+        <v>3.1</v>
       </c>
       <c r="F1653" s="5" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="G1653" s="4" t="n">
-        <v>115.5</v>
+        <v>186</v>
       </c>
       <c r="H1653" s="2" t="n">
         <v>1619783</v>
@@ -77919,13 +77919,13 @@
         </is>
       </c>
       <c r="E1654" s="4" t="n">
-        <v>3.1</v>
+        <v>1.65</v>
       </c>
       <c r="F1654" s="5" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G1654" s="4" t="n">
-        <v>186</v>
+        <v>115.5</v>
       </c>
       <c r="H1654" s="2" t="n">
         <v>1619783</v>
@@ -80081,13 +80081,13 @@
         </is>
       </c>
       <c r="E1700" s="4" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="F1700" s="5" t="n">
-        <v>2.9</v>
+        <v>0.22</v>
       </c>
       <c r="G1700" s="4" t="n">
-        <v>14.5</v>
+        <v>22</v>
       </c>
       <c r="H1700" s="2" t="n">
         <v>1630277</v>
@@ -80131,10 +80131,10 @@
         <v>100</v>
       </c>
       <c r="F1701" s="5" t="n">
-        <v>1.35</v>
+        <v>0.15</v>
       </c>
       <c r="G1701" s="4" t="n">
-        <v>135</v>
+        <v>15</v>
       </c>
       <c r="H1701" s="2" t="n">
         <v>1630277</v>
@@ -80178,10 +80178,10 @@
         <v>100</v>
       </c>
       <c r="F1702" s="5" t="n">
-        <v>0.22</v>
+        <v>1.35</v>
       </c>
       <c r="G1702" s="4" t="n">
-        <v>22</v>
+        <v>135</v>
       </c>
       <c r="H1702" s="2" t="n">
         <v>1630277</v>
@@ -80222,13 +80222,13 @@
         </is>
       </c>
       <c r="E1703" s="4" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="F1703" s="5" t="n">
-        <v>0.15</v>
+        <v>2.9</v>
       </c>
       <c r="G1703" s="4" t="n">
-        <v>15</v>
+        <v>14.5</v>
       </c>
       <c r="H1703" s="2" t="n">
         <v>1630277</v>
@@ -81021,13 +81021,13 @@
         </is>
       </c>
       <c r="E1720" s="4" t="n">
-        <v>0.04</v>
+        <v>1</v>
       </c>
       <c r="F1720" s="5" t="n">
-        <v>110</v>
+        <v>22</v>
       </c>
       <c r="G1720" s="4" t="n">
-        <v>4.4</v>
+        <v>22</v>
       </c>
       <c r="H1720" s="2" t="n">
         <v>1632122</v>
@@ -81068,13 +81068,13 @@
         </is>
       </c>
       <c r="E1721" s="4" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="F1721" s="5" t="n">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="G1721" s="4" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="H1721" s="2" t="n">
         <v>1632122</v>
@@ -81115,13 +81115,13 @@
         </is>
       </c>
       <c r="E1722" s="4" t="n">
-        <v>0.08</v>
+        <v>2</v>
       </c>
       <c r="F1722" s="5" t="n">
-        <v>500</v>
+        <v>25</v>
       </c>
       <c r="G1722" s="4" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H1722" s="2" t="n">
         <v>1632122</v>
@@ -81209,13 +81209,13 @@
         </is>
       </c>
       <c r="E1724" s="4" t="n">
-        <v>1</v>
+        <v>0.08</v>
       </c>
       <c r="F1724" s="5" t="n">
-        <v>16</v>
+        <v>500</v>
       </c>
       <c r="G1724" s="4" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="H1724" s="2" t="n">
         <v>1632122</v>
@@ -81256,13 +81256,13 @@
         </is>
       </c>
       <c r="E1725" s="4" t="n">
-        <v>2</v>
+        <v>0.04</v>
       </c>
       <c r="F1725" s="5" t="n">
-        <v>25</v>
+        <v>110</v>
       </c>
       <c r="G1725" s="4" t="n">
-        <v>50</v>
+        <v>4.4</v>
       </c>
       <c r="H1725" s="2" t="n">
         <v>1632122</v>
@@ -81303,13 +81303,13 @@
         </is>
       </c>
       <c r="E1726" s="4" t="n">
-        <v>1</v>
+        <v>0.04</v>
       </c>
       <c r="F1726" s="5" t="n">
-        <v>22</v>
+        <v>140</v>
       </c>
       <c r="G1726" s="4" t="n">
-        <v>22</v>
+        <v>5.6</v>
       </c>
       <c r="H1726" s="2" t="n">
         <v>1632122</v>
@@ -81350,13 +81350,13 @@
         </is>
       </c>
       <c r="E1727" s="4" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="F1727" s="5" t="n">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="G1727" s="4" t="n">
-        <v>5.6</v>
+        <v>6</v>
       </c>
       <c r="H1727" s="2" t="n">
         <v>1632122</v>
@@ -82126,6 +82126,382 @@
         <v>2368</v>
       </c>
       <c r="K1743" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1744" customHeight="1" ht="15">
+      <c r="A1744" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1744" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1744" s="2" t="n">
+        <v>13388</v>
+      </c>
+      <c r="D1744" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">LUVA-NITRILO</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1744" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1744" s="5" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="G1744" s="4" t="n">
+        <v>179.5</v>
+      </c>
+      <c r="H1744" s="2" t="n">
+        <v>1638982</v>
+      </c>
+      <c r="I1744" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">15/10/2026 09:44:02</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1744" s="2" t="n">
+        <v>1695</v>
+      </c>
+      <c r="K1744" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1745" customHeight="1" ht="15">
+      <c r="A1745" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1745" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1745" s="2" t="n">
+        <v>15039</v>
+      </c>
+      <c r="D1745" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_USE</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1745" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1745" s="5" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G1745" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="H1745" s="2" t="n">
+        <v>1639137</v>
+      </c>
+      <c r="I1745" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">15/10/2026 11:37:56</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1745" s="2" t="n">
+        <v>2318</v>
+      </c>
+      <c r="K1745" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1746" customHeight="1" ht="15">
+      <c r="A1746" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1746" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1746" s="2" t="n">
+        <v>13169</v>
+      </c>
+      <c r="D1746" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">BOBINA-PAPEL</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1746" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1746" s="5" t="n">
+        <v>33.68</v>
+      </c>
+      <c r="G1746" s="4" t="n">
+        <v>336.8</v>
+      </c>
+      <c r="H1746" s="2" t="n">
+        <v>1639159</v>
+      </c>
+      <c r="I1746" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">15/10/2026 12:09:19</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1746" s="2" t="n">
+        <v>36364</v>
+      </c>
+      <c r="K1746" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1747" customHeight="1" ht="15">
+      <c r="A1747" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1747" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1747" s="2" t="n">
+        <v>13195</v>
+      </c>
+      <c r="D1747" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">SABONETE-LIQ</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1747" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1747" s="5" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="G1747" s="4" t="n">
+        <v>37.14</v>
+      </c>
+      <c r="H1747" s="2" t="n">
+        <v>1639159</v>
+      </c>
+      <c r="I1747" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">15/10/2026 12:09:19</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1747" s="2" t="n">
+        <v>36364</v>
+      </c>
+      <c r="K1747" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1748" customHeight="1" ht="15">
+      <c r="A1748" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1748" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1748" s="2" t="n">
+        <v>13956</v>
+      </c>
+      <c r="D1748" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">ALCOOL-LIQ</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1748" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1748" s="5" t="n">
+        <v>29.36</v>
+      </c>
+      <c r="G1748" s="4" t="n">
+        <v>88.08</v>
+      </c>
+      <c r="H1748" s="2" t="n">
+        <v>1639159</v>
+      </c>
+      <c r="I1748" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">15/10/2026 12:09:19</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1748" s="2" t="n">
+        <v>36364</v>
+      </c>
+      <c r="K1748" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1749" customHeight="1" ht="15">
+      <c r="A1749" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1749" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1749" s="2" t="n">
+        <v>31085</v>
+      </c>
+      <c r="D1749" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">COLA-AZUL</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1749" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F1749" s="5" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="G1749" s="4" t="n">
+        <v>1138</v>
+      </c>
+      <c r="H1749" s="2" t="n">
+        <v>1639202</v>
+      </c>
+      <c r="I1749" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">15/10/2026 13:52:37</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1749" s="2" t="n">
+        <v>923</v>
+      </c>
+      <c r="K1749" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1750" customHeight="1" ht="15">
+      <c r="A1750" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1750" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1750" s="2" t="n">
+        <v>37988</v>
+      </c>
+      <c r="D1750" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">THINNER-5L</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1750" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1750" s="5" t="n">
+        <v>96.8</v>
+      </c>
+      <c r="G1750" s="4" t="n">
+        <v>193.6</v>
+      </c>
+      <c r="H1750" s="2" t="n">
+        <v>1639202</v>
+      </c>
+      <c r="I1750" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">15/10/2026 13:52:37</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1750" s="2" t="n">
+        <v>923</v>
+      </c>
+      <c r="K1750" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1751" customHeight="1" ht="15">
+      <c r="A1751" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1751" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1751" s="2" t="n">
+        <v>26328</v>
+      </c>
+      <c r="D1751" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">CAIXA-F</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1751" s="4" t="n">
+        <v>862</v>
+      </c>
+      <c r="F1751" s="5" t="n">
+        <v>6.529</v>
+      </c>
+      <c r="G1751" s="4" t="n">
+        <v>5628</v>
+      </c>
+      <c r="H1751" s="2" t="n">
+        <v>1639207</v>
+      </c>
+      <c r="I1751" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">15/10/2026 14:00:43</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1751" s="2" t="n">
+        <v>11205</v>
+      </c>
+      <c r="K1751" s="2" t="n">
         <v>165</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Relatório de compras 19/10/2026 22:01
</commit_message>
<xml_diff>
--- a/data/relatorio.xlsx
+++ b/data/relatorio.xlsx
@@ -369,13 +369,13 @@
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>29.744</v>
+        <v>3.5</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>89.23</v>
+        <v>3.5</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>1397499</v>
@@ -419,10 +419,10 @@
         <v>1</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>1397499</v>
@@ -463,13 +463,13 @@
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>4.5</v>
+        <v>4.675</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>4.5</v>
+        <v>9.35</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>1397499</v>
@@ -510,13 +510,13 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>4.675</v>
+        <v>33.44</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>9.35</v>
+        <v>33.44</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>1397499</v>
@@ -607,10 +607,10 @@
         <v>3</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>23.36</v>
+        <v>29.744</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>70.08</v>
+        <v>89.23</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>1397499</v>
@@ -651,13 +651,13 @@
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>33.44</v>
+        <v>23.36</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>33.44</v>
+        <v>70.08</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>1397499</v>
@@ -3004,10 +3004,10 @@
         <v>1</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>1.59</v>
+        <v>30.25</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>1.59</v>
+        <v>30.25</v>
       </c>
       <c r="H60" s="2" t="n">
         <v>1401617</v>
@@ -3098,10 +3098,10 @@
         <v>1</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>19.94</v>
+        <v>1.59</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>19.94</v>
+        <v>1.59</v>
       </c>
       <c r="H62" s="2" t="n">
         <v>1401617</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="E64" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>1.33</v>
+        <v>19.94</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>6.65</v>
+        <v>19.94</v>
       </c>
       <c r="H64" s="2" t="n">
         <v>1401617</v>
@@ -3333,10 +3333,10 @@
         <v>5</v>
       </c>
       <c r="F67" s="5" t="n">
-        <v>1.39</v>
+        <v>1.33</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>6.95</v>
+        <v>6.65</v>
       </c>
       <c r="H67" s="2" t="n">
         <v>1401617</v>
@@ -3377,13 +3377,13 @@
         </is>
       </c>
       <c r="E68" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F68" s="5" t="n">
-        <v>28.82</v>
+        <v>1.39</v>
       </c>
       <c r="G68" s="4" t="n">
-        <v>28.82</v>
+        <v>6.95</v>
       </c>
       <c r="H68" s="2" t="n">
         <v>1401617</v>
@@ -3424,13 +3424,13 @@
         </is>
       </c>
       <c r="E69" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F69" s="5" t="n">
-        <v>23.65</v>
+        <v>28.82</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>47.3</v>
+        <v>28.82</v>
       </c>
       <c r="H69" s="2" t="n">
         <v>1401617</v>
@@ -3471,13 +3471,13 @@
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="F70" s="5" t="n">
-        <v>3.32</v>
+        <v>23.65</v>
       </c>
       <c r="G70" s="4" t="n">
-        <v>99.6</v>
+        <v>47.3</v>
       </c>
       <c r="H70" s="2" t="n">
         <v>1401617</v>
@@ -3518,13 +3518,13 @@
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="F71" s="5" t="n">
-        <v>30.25</v>
+        <v>3.32</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>30.25</v>
+        <v>99.6</v>
       </c>
       <c r="H71" s="2" t="n">
         <v>1401617</v>
@@ -4881,13 +4881,13 @@
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>30</v>
+        <v>200</v>
       </c>
       <c r="F100" s="5" t="n">
-        <v>0.6</v>
+        <v>0.17</v>
       </c>
       <c r="G100" s="4" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="H100" s="2" t="n">
         <v>1402783</v>
@@ -4928,13 +4928,13 @@
         </is>
       </c>
       <c r="E101" s="4" t="n">
-        <v>268</v>
+        <v>60</v>
       </c>
       <c r="F101" s="5" t="n">
         <v>0.22</v>
       </c>
       <c r="G101" s="4" t="n">
-        <v>58.96</v>
+        <v>13.2</v>
       </c>
       <c r="H101" s="2" t="n">
         <v>1402783</v>
@@ -4975,13 +4975,13 @@
         </is>
       </c>
       <c r="E102" s="4" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F102" s="5" t="n">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="G102" s="4" t="n">
-        <v>13.2</v>
+        <v>3</v>
       </c>
       <c r="H102" s="2" t="n">
         <v>1402783</v>
@@ -5025,10 +5025,10 @@
         <v>30</v>
       </c>
       <c r="F103" s="5" t="n">
-        <v>0.1</v>
+        <v>0.42</v>
       </c>
       <c r="G103" s="4" t="n">
-        <v>3</v>
+        <v>12.6</v>
       </c>
       <c r="H103" s="2" t="n">
         <v>1402783</v>
@@ -5072,10 +5072,10 @@
         <v>30</v>
       </c>
       <c r="F104" s="5" t="n">
-        <v>0.42</v>
+        <v>0.12</v>
       </c>
       <c r="G104" s="4" t="n">
-        <v>12.6</v>
+        <v>3.6</v>
       </c>
       <c r="H104" s="2" t="n">
         <v>1402783</v>
@@ -5119,10 +5119,10 @@
         <v>30</v>
       </c>
       <c r="F105" s="5" t="n">
-        <v>0.12</v>
+        <v>1.85</v>
       </c>
       <c r="G105" s="4" t="n">
-        <v>3.6</v>
+        <v>55.5</v>
       </c>
       <c r="H105" s="2" t="n">
         <v>1402783</v>
@@ -5163,13 +5163,13 @@
         </is>
       </c>
       <c r="E106" s="4" t="n">
-        <v>200</v>
+        <v>268</v>
       </c>
       <c r="F106" s="5" t="n">
-        <v>0.17</v>
+        <v>0.22</v>
       </c>
       <c r="G106" s="4" t="n">
-        <v>34</v>
+        <v>58.96</v>
       </c>
       <c r="H106" s="2" t="n">
         <v>1402783</v>
@@ -5213,10 +5213,10 @@
         <v>30</v>
       </c>
       <c r="F107" s="5" t="n">
-        <v>1.85</v>
+        <v>0.6</v>
       </c>
       <c r="G107" s="4" t="n">
-        <v>55.5</v>
+        <v>18</v>
       </c>
       <c r="H107" s="2" t="n">
         <v>1402783</v>
@@ -5351,13 +5351,13 @@
         </is>
       </c>
       <c r="E110" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F110" s="5" t="n">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="G110" s="4" t="n">
-        <v>890</v>
+        <v>324</v>
       </c>
       <c r="H110" s="2" t="n">
         <v>1402788</v>
@@ -5445,13 +5445,13 @@
         </is>
       </c>
       <c r="E112" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F112" s="5" t="n">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="G112" s="4" t="n">
-        <v>324</v>
+        <v>890</v>
       </c>
       <c r="H112" s="2" t="n">
         <v>1402788</v>
@@ -5636,10 +5636,10 @@
         <v>1</v>
       </c>
       <c r="F116" s="5" t="n">
-        <v>33.9</v>
+        <v>74.9</v>
       </c>
       <c r="G116" s="4" t="n">
-        <v>33.9</v>
+        <v>74.9</v>
       </c>
       <c r="H116" s="2" t="n">
         <v>1403644</v>
@@ -5683,10 +5683,10 @@
         <v>1</v>
       </c>
       <c r="F117" s="5" t="n">
-        <v>74.9</v>
+        <v>58</v>
       </c>
       <c r="G117" s="4" t="n">
-        <v>74.9</v>
+        <v>58</v>
       </c>
       <c r="H117" s="2" t="n">
         <v>1403644</v>
@@ -5730,10 +5730,10 @@
         <v>1</v>
       </c>
       <c r="F118" s="5" t="n">
-        <v>58</v>
+        <v>12.9</v>
       </c>
       <c r="G118" s="4" t="n">
-        <v>58</v>
+        <v>12.9</v>
       </c>
       <c r="H118" s="2" t="n">
         <v>1403644</v>
@@ -5777,10 +5777,10 @@
         <v>1</v>
       </c>
       <c r="F119" s="5" t="n">
-        <v>12.9</v>
+        <v>10.5</v>
       </c>
       <c r="G119" s="4" t="n">
-        <v>12.9</v>
+        <v>10.5</v>
       </c>
       <c r="H119" s="2" t="n">
         <v>1403644</v>
@@ -5824,10 +5824,10 @@
         <v>1</v>
       </c>
       <c r="F120" s="5" t="n">
-        <v>10.5</v>
+        <v>33.9</v>
       </c>
       <c r="G120" s="4" t="n">
-        <v>10.5</v>
+        <v>33.9</v>
       </c>
       <c r="H120" s="2" t="n">
         <v>1403644</v>
@@ -6103,13 +6103,13 @@
         </is>
       </c>
       <c r="E126" s="4" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="F126" s="5" t="n">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="G126" s="4" t="n">
-        <v>3.75</v>
+        <v>5</v>
       </c>
       <c r="H126" s="2" t="n">
         <v>1403680</v>
@@ -6150,13 +6150,13 @@
         </is>
       </c>
       <c r="E127" s="4" t="n">
-        <v>0.2</v>
+        <v>3</v>
       </c>
       <c r="F127" s="5" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="G127" s="4" t="n">
-        <v>5.6</v>
+        <v>45</v>
       </c>
       <c r="H127" s="2" t="n">
         <v>1403680</v>
@@ -6197,13 +6197,13 @@
         </is>
       </c>
       <c r="E128" s="4" t="n">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="F128" s="5" t="n">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="G128" s="4" t="n">
-        <v>5</v>
+        <v>3.75</v>
       </c>
       <c r="H128" s="2" t="n">
         <v>1403680</v>
@@ -6244,13 +6244,13 @@
         </is>
       </c>
       <c r="E129" s="4" t="n">
-        <v>1.5</v>
+        <v>0.2</v>
       </c>
       <c r="F129" s="5" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="G129" s="4" t="n">
-        <v>24</v>
+        <v>5.6</v>
       </c>
       <c r="H129" s="2" t="n">
         <v>1403680</v>
@@ -6291,13 +6291,13 @@
         </is>
       </c>
       <c r="E130" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F130" s="5" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="G130" s="4" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="H130" s="2" t="n">
         <v>1403680</v>
@@ -6338,13 +6338,13 @@
         </is>
       </c>
       <c r="E131" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F131" s="5" t="n">
-        <v>14</v>
+        <v>3.5</v>
       </c>
       <c r="G131" s="4" t="n">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="H131" s="2" t="n">
         <v>1403680</v>
@@ -6385,13 +6385,13 @@
         </is>
       </c>
       <c r="E132" s="4" t="n">
-        <v>10</v>
+        <v>1.5</v>
       </c>
       <c r="F132" s="5" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G132" s="4" t="n">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="H132" s="2" t="n">
         <v>1403680</v>
@@ -6432,13 +6432,13 @@
         </is>
       </c>
       <c r="E133" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F133" s="5" t="n">
-        <v>3.5</v>
+        <v>14</v>
       </c>
       <c r="G133" s="4" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="H133" s="2" t="n">
         <v>1403680</v>
@@ -6482,10 +6482,10 @@
         <v>0.3</v>
       </c>
       <c r="F134" s="5" t="n">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="G134" s="4" t="n">
-        <v>4.5</v>
+        <v>30</v>
       </c>
       <c r="H134" s="2" t="n">
         <v>1403681</v>
@@ -6526,13 +6526,13 @@
         </is>
       </c>
       <c r="E135" s="4" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="F135" s="5" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G135" s="4" t="n">
-        <v>5.25</v>
+        <v>9</v>
       </c>
       <c r="H135" s="2" t="n">
         <v>1403681</v>
@@ -6573,13 +6573,13 @@
         </is>
       </c>
       <c r="E136" s="4" t="n">
-        <v>0.3</v>
+        <v>10</v>
       </c>
       <c r="F136" s="5" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="G136" s="4" t="n">
-        <v>30</v>
+        <v>250</v>
       </c>
       <c r="H136" s="2" t="n">
         <v>1403681</v>
@@ -6620,13 +6620,13 @@
         </is>
       </c>
       <c r="E137" s="4" t="n">
-        <v>0.3</v>
+        <v>100</v>
       </c>
       <c r="F137" s="5" t="n">
-        <v>30</v>
+        <v>2.22</v>
       </c>
       <c r="G137" s="4" t="n">
-        <v>9</v>
+        <v>222</v>
       </c>
       <c r="H137" s="2" t="n">
         <v>1403681</v>
@@ -6667,13 +6667,13 @@
         </is>
       </c>
       <c r="E138" s="4" t="n">
-        <v>10</v>
+        <v>0.3</v>
       </c>
       <c r="F138" s="5" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G138" s="4" t="n">
-        <v>250</v>
+        <v>4.5</v>
       </c>
       <c r="H138" s="2" t="n">
         <v>1403681</v>
@@ -6714,13 +6714,13 @@
         </is>
       </c>
       <c r="E139" s="4" t="n">
-        <v>100</v>
+        <v>0.15</v>
       </c>
       <c r="F139" s="5" t="n">
-        <v>2.22</v>
+        <v>35</v>
       </c>
       <c r="G139" s="4" t="n">
-        <v>222</v>
+        <v>5.25</v>
       </c>
       <c r="H139" s="2" t="n">
         <v>1403681</v>
@@ -7328,10 +7328,10 @@
         <v>1</v>
       </c>
       <c r="F152" s="5" t="n">
-        <v>55.2</v>
+        <v>25.9</v>
       </c>
       <c r="G152" s="4" t="n">
-        <v>55.2</v>
+        <v>25.9</v>
       </c>
       <c r="H152" s="2" t="n">
         <v>1405612</v>
@@ -7419,13 +7419,13 @@
         </is>
       </c>
       <c r="E154" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F154" s="5" t="n">
-        <v>25.9</v>
+        <v>124.5</v>
       </c>
       <c r="G154" s="4" t="n">
-        <v>25.9</v>
+        <v>249</v>
       </c>
       <c r="H154" s="2" t="n">
         <v>1405612</v>
@@ -7466,13 +7466,13 @@
         </is>
       </c>
       <c r="E155" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F155" s="5" t="n">
-        <v>38</v>
+        <v>8.5</v>
       </c>
       <c r="G155" s="4" t="n">
-        <v>266</v>
+        <v>51</v>
       </c>
       <c r="H155" s="2" t="n">
         <v>1405612</v>
@@ -7513,13 +7513,13 @@
         </is>
       </c>
       <c r="E156" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F156" s="5" t="n">
-        <v>8.5</v>
+        <v>55.2</v>
       </c>
       <c r="G156" s="4" t="n">
-        <v>51</v>
+        <v>55.2</v>
       </c>
       <c r="H156" s="2" t="n">
         <v>1405612</v>
@@ -7560,13 +7560,13 @@
         </is>
       </c>
       <c r="E157" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F157" s="5" t="n">
-        <v>124.5</v>
+        <v>38</v>
       </c>
       <c r="G157" s="4" t="n">
-        <v>249</v>
+        <v>266</v>
       </c>
       <c r="H157" s="2" t="n">
         <v>1405612</v>
@@ -7704,10 +7704,10 @@
         <v>1</v>
       </c>
       <c r="F160" s="5" t="n">
-        <v>17.43</v>
+        <v>18.91</v>
       </c>
       <c r="G160" s="4" t="n">
-        <v>17.43</v>
+        <v>18.91</v>
       </c>
       <c r="H160" s="2" t="n">
         <v>1405673</v>
@@ -7748,13 +7748,13 @@
         </is>
       </c>
       <c r="E161" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F161" s="5" t="n">
-        <v>18.91</v>
+        <v>13.17</v>
       </c>
       <c r="G161" s="4" t="n">
-        <v>18.91</v>
+        <v>26.34</v>
       </c>
       <c r="H161" s="2" t="n">
         <v>1405673</v>
@@ -7795,13 +7795,13 @@
         </is>
       </c>
       <c r="E162" s="4" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="F162" s="5" t="n">
-        <v>13.17</v>
+        <v>0.54</v>
       </c>
       <c r="G162" s="4" t="n">
-        <v>26.34</v>
+        <v>10.8</v>
       </c>
       <c r="H162" s="2" t="n">
         <v>1405673</v>
@@ -7986,10 +7986,10 @@
         <v>1</v>
       </c>
       <c r="F166" s="5" t="n">
-        <v>19.32</v>
+        <v>17.43</v>
       </c>
       <c r="G166" s="4" t="n">
-        <v>19.32</v>
+        <v>17.43</v>
       </c>
       <c r="H166" s="2" t="n">
         <v>1405673</v>
@@ -8077,13 +8077,13 @@
         </is>
       </c>
       <c r="E168" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F168" s="5" t="n">
-        <v>5.67</v>
+        <v>19.32</v>
       </c>
       <c r="G168" s="4" t="n">
-        <v>28.35</v>
+        <v>19.32</v>
       </c>
       <c r="H168" s="2" t="n">
         <v>1405673</v>
@@ -8124,13 +8124,13 @@
         </is>
       </c>
       <c r="E169" s="4" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="F169" s="5" t="n">
-        <v>0.54</v>
+        <v>5.67</v>
       </c>
       <c r="G169" s="4" t="n">
-        <v>10.8</v>
+        <v>28.35</v>
       </c>
       <c r="H169" s="2" t="n">
         <v>1405673</v>
@@ -10051,13 +10051,13 @@
         </is>
       </c>
       <c r="E210" s="4" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="F210" s="5" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="G210" s="4" t="n">
-        <v>840</v>
+        <v>2450</v>
       </c>
       <c r="H210" s="2" t="n">
         <v>1409782</v>
@@ -10098,13 +10098,13 @@
         </is>
       </c>
       <c r="E211" s="4" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="F211" s="5" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="G211" s="4" t="n">
-        <v>2450</v>
+        <v>840</v>
       </c>
       <c r="H211" s="2" t="n">
         <v>1409782</v>
@@ -10427,13 +10427,13 @@
         </is>
       </c>
       <c r="E218" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F218" s="5" t="n">
         <v>14.9</v>
       </c>
       <c r="G218" s="4" t="n">
-        <v>59.6</v>
+        <v>29.8</v>
       </c>
       <c r="H218" s="2" t="n">
         <v>1410100</v>
@@ -10474,13 +10474,13 @@
         </is>
       </c>
       <c r="E219" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F219" s="5" t="n">
         <v>14.9</v>
       </c>
       <c r="G219" s="4" t="n">
-        <v>29.8</v>
+        <v>59.6</v>
       </c>
       <c r="H219" s="2" t="n">
         <v>1410100</v>
@@ -10521,13 +10521,13 @@
         </is>
       </c>
       <c r="E220" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F220" s="5" t="n">
-        <v>12</v>
+        <v>59.9</v>
       </c>
       <c r="G220" s="4" t="n">
-        <v>24</v>
+        <v>59.9</v>
       </c>
       <c r="H220" s="2" t="n">
         <v>1410100</v>
@@ -10568,13 +10568,13 @@
         </is>
       </c>
       <c r="E221" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F221" s="5" t="n">
-        <v>59.9</v>
+        <v>12</v>
       </c>
       <c r="G221" s="4" t="n">
-        <v>59.9</v>
+        <v>24</v>
       </c>
       <c r="H221" s="2" t="n">
         <v>1410100</v>
@@ -12028,10 +12028,10 @@
         <v>25</v>
       </c>
       <c r="F252" s="5" t="n">
-        <v>0.462</v>
+        <v>0.4701</v>
       </c>
       <c r="G252" s="4" t="n">
-        <v>11.55</v>
+        <v>11.75</v>
       </c>
       <c r="H252" s="2" t="n">
         <v>1415875</v>
@@ -12072,13 +12072,13 @@
         </is>
       </c>
       <c r="E253" s="4" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F253" s="5" t="n">
-        <v>0.4701</v>
+        <v>0.4265</v>
       </c>
       <c r="G253" s="4" t="n">
-        <v>11.75</v>
+        <v>21.33</v>
       </c>
       <c r="H253" s="2" t="n">
         <v>1415875</v>
@@ -12119,13 +12119,13 @@
         </is>
       </c>
       <c r="E254" s="4" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="F254" s="5" t="n">
-        <v>0.4265</v>
+        <v>0.5692</v>
       </c>
       <c r="G254" s="4" t="n">
-        <v>21.33</v>
+        <v>14.23</v>
       </c>
       <c r="H254" s="2" t="n">
         <v>1415875</v>
@@ -12169,10 +12169,10 @@
         <v>25</v>
       </c>
       <c r="F255" s="5" t="n">
-        <v>0.5692</v>
+        <v>0.4265</v>
       </c>
       <c r="G255" s="4" t="n">
-        <v>14.23</v>
+        <v>10.66</v>
       </c>
       <c r="H255" s="2" t="n">
         <v>1415875</v>
@@ -12216,10 +12216,10 @@
         <v>25</v>
       </c>
       <c r="F256" s="5" t="n">
-        <v>0.4265</v>
+        <v>0.462</v>
       </c>
       <c r="G256" s="4" t="n">
-        <v>10.66</v>
+        <v>11.55</v>
       </c>
       <c r="H256" s="2" t="n">
         <v>1415875</v>
@@ -15271,10 +15271,10 @@
         <v>1</v>
       </c>
       <c r="F321" s="5" t="n">
-        <v>44.9</v>
+        <v>32</v>
       </c>
       <c r="G321" s="4" t="n">
-        <v>44.9</v>
+        <v>32</v>
       </c>
       <c r="H321" s="2" t="n">
         <v>1429506</v>
@@ -15318,10 +15318,10 @@
         <v>1</v>
       </c>
       <c r="F322" s="5" t="n">
-        <v>32</v>
+        <v>44.9</v>
       </c>
       <c r="G322" s="4" t="n">
-        <v>32</v>
+        <v>44.9</v>
       </c>
       <c r="H322" s="2" t="n">
         <v>1429506</v>
@@ -17900,13 +17900,13 @@
         </is>
       </c>
       <c r="E377" s="4" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F377" s="5" t="n">
-        <v>6.63</v>
+        <v>6.28</v>
       </c>
       <c r="G377" s="4" t="n">
-        <v>6.63</v>
+        <v>314</v>
       </c>
       <c r="H377" s="2" t="n">
         <v>1437076</v>
@@ -18276,13 +18276,13 @@
         </is>
       </c>
       <c r="E385" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F385" s="5" t="n">
-        <v>1.29</v>
+        <v>15.27</v>
       </c>
       <c r="G385" s="4" t="n">
-        <v>12.9</v>
+        <v>30.54</v>
       </c>
       <c r="H385" s="2" t="n">
         <v>1437076</v>
@@ -18323,13 +18323,13 @@
         </is>
       </c>
       <c r="E386" s="4" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="F386" s="5" t="n">
-        <v>2.53</v>
+        <v>1.29</v>
       </c>
       <c r="G386" s="4" t="n">
-        <v>253</v>
+        <v>12.9</v>
       </c>
       <c r="H386" s="2" t="n">
         <v>1437076</v>
@@ -18467,10 +18467,10 @@
         <v>100</v>
       </c>
       <c r="F389" s="5" t="n">
-        <v>4.16</v>
+        <v>2.53</v>
       </c>
       <c r="G389" s="4" t="n">
-        <v>416</v>
+        <v>253</v>
       </c>
       <c r="H389" s="2" t="n">
         <v>1437076</v>
@@ -18511,13 +18511,13 @@
         </is>
       </c>
       <c r="E390" s="4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F390" s="5" t="n">
-        <v>6.28</v>
+        <v>4.16</v>
       </c>
       <c r="G390" s="4" t="n">
-        <v>314</v>
+        <v>416</v>
       </c>
       <c r="H390" s="2" t="n">
         <v>1437076</v>
@@ -18558,13 +18558,13 @@
         </is>
       </c>
       <c r="E391" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F391" s="5" t="n">
-        <v>8.81</v>
+        <v>6.63</v>
       </c>
       <c r="G391" s="4" t="n">
-        <v>17.62</v>
+        <v>6.63</v>
       </c>
       <c r="H391" s="2" t="n">
         <v>1437076</v>
@@ -18605,13 +18605,13 @@
         </is>
       </c>
       <c r="E392" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F392" s="5" t="n">
-        <v>3.6</v>
+        <v>8.81</v>
       </c>
       <c r="G392" s="4" t="n">
-        <v>14.4</v>
+        <v>17.62</v>
       </c>
       <c r="H392" s="2" t="n">
         <v>1437076</v>
@@ -18652,13 +18652,13 @@
         </is>
       </c>
       <c r="E393" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F393" s="5" t="n">
-        <v>30.25</v>
+        <v>3.6</v>
       </c>
       <c r="G393" s="4" t="n">
-        <v>30.25</v>
+        <v>14.4</v>
       </c>
       <c r="H393" s="2" t="n">
         <v>1437076</v>
@@ -18699,13 +18699,13 @@
         </is>
       </c>
       <c r="E394" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F394" s="5" t="n">
         <v>30.25</v>
       </c>
       <c r="G394" s="4" t="n">
-        <v>90.75</v>
+        <v>30.25</v>
       </c>
       <c r="H394" s="2" t="n">
         <v>1437076</v>
@@ -18746,13 +18746,13 @@
         </is>
       </c>
       <c r="E395" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F395" s="5" t="n">
-        <v>15.27</v>
+        <v>30.25</v>
       </c>
       <c r="G395" s="4" t="n">
-        <v>30.54</v>
+        <v>90.75</v>
       </c>
       <c r="H395" s="2" t="n">
         <v>1437076</v>
@@ -20297,13 +20297,13 @@
         </is>
       </c>
       <c r="E428" s="4" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="F428" s="5" t="n">
-        <v>200</v>
+        <v>25</v>
       </c>
       <c r="G428" s="4" t="n">
-        <v>10</v>
+        <v>2.5</v>
       </c>
       <c r="H428" s="2" t="n">
         <v>1442618</v>
@@ -20347,10 +20347,10 @@
         <v>0.1</v>
       </c>
       <c r="F429" s="5" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G429" s="4" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="H429" s="2" t="n">
         <v>1442618</v>
@@ -20391,13 +20391,13 @@
         </is>
       </c>
       <c r="E430" s="4" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="F430" s="5" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="G430" s="4" t="n">
-        <v>1.5</v>
+        <v>2.4</v>
       </c>
       <c r="H430" s="2" t="n">
         <v>1442618</v>
@@ -20438,13 +20438,13 @@
         </is>
       </c>
       <c r="E431" s="4" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="F431" s="5" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="G431" s="4" t="n">
-        <v>2.4</v>
+        <v>7.2</v>
       </c>
       <c r="H431" s="2" t="n">
         <v>1442618</v>
@@ -20485,13 +20485,13 @@
         </is>
       </c>
       <c r="E432" s="4" t="n">
-        <v>0.06</v>
+        <v>0.25</v>
       </c>
       <c r="F432" s="5" t="n">
-        <v>90</v>
+        <v>22</v>
       </c>
       <c r="G432" s="4" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="H432" s="2" t="n">
         <v>1442618</v>
@@ -20532,13 +20532,13 @@
         </is>
       </c>
       <c r="E433" s="4" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="F433" s="5" t="n">
         <v>90</v>
       </c>
       <c r="G433" s="4" t="n">
-        <v>7.2</v>
+        <v>5.4</v>
       </c>
       <c r="H433" s="2" t="n">
         <v>1442618</v>
@@ -20582,10 +20582,10 @@
         <v>0.25</v>
       </c>
       <c r="F434" s="5" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="G434" s="4" t="n">
-        <v>5.5</v>
+        <v>2.5</v>
       </c>
       <c r="H434" s="2" t="n">
         <v>1442618</v>
@@ -20626,13 +20626,13 @@
         </is>
       </c>
       <c r="E435" s="4" t="n">
-        <v>0.25</v>
+        <v>0.08</v>
       </c>
       <c r="F435" s="5" t="n">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="G435" s="4" t="n">
-        <v>2.5</v>
+        <v>5.6</v>
       </c>
       <c r="H435" s="2" t="n">
         <v>1442618</v>
@@ -20720,13 +20720,13 @@
         </is>
       </c>
       <c r="E437" s="4" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="F437" s="5" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="G437" s="4" t="n">
-        <v>5.6</v>
+        <v>8</v>
       </c>
       <c r="H437" s="2" t="n">
         <v>1442618</v>
@@ -20767,13 +20767,13 @@
         </is>
       </c>
       <c r="E438" s="4" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="F438" s="5" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="G438" s="4" t="n">
-        <v>8</v>
+        <v>1.8</v>
       </c>
       <c r="H438" s="2" t="n">
         <v>1442618</v>
@@ -20814,13 +20814,13 @@
         </is>
       </c>
       <c r="E439" s="4" t="n">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="F439" s="5" t="n">
-        <v>30</v>
+        <v>200</v>
       </c>
       <c r="G439" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H439" s="2" t="n">
         <v>1442618</v>
@@ -20861,13 +20861,13 @@
         </is>
       </c>
       <c r="E440" s="4" t="n">
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
       <c r="F440" s="5" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G440" s="4" t="n">
-        <v>2.8</v>
+        <v>6</v>
       </c>
       <c r="H440" s="2" t="n">
         <v>1442618</v>
@@ -20911,10 +20911,10 @@
         <v>0.08</v>
       </c>
       <c r="F441" s="5" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="G441" s="4" t="n">
-        <v>1.6</v>
+        <v>2.8</v>
       </c>
       <c r="H441" s="2" t="n">
         <v>1442618</v>
@@ -20958,10 +20958,10 @@
         <v>0.08</v>
       </c>
       <c r="F442" s="5" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="G442" s="4" t="n">
-        <v>0.48</v>
+        <v>1.6</v>
       </c>
       <c r="H442" s="2" t="n">
         <v>1442618</v>
@@ -21002,13 +21002,13 @@
         </is>
       </c>
       <c r="E443" s="4" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="F443" s="5" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="G443" s="4" t="n">
-        <v>1.8</v>
+        <v>0.48</v>
       </c>
       <c r="H443" s="2" t="n">
         <v>1442618</v>
@@ -26219,13 +26219,13 @@
         </is>
       </c>
       <c r="E554" s="4" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="F554" s="5" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="G554" s="4" t="n">
-        <v>12</v>
+        <v>6.25</v>
       </c>
       <c r="H554" s="2" t="n">
         <v>1480786</v>
@@ -26266,13 +26266,13 @@
         </is>
       </c>
       <c r="E555" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F555" s="5" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="G555" s="4" t="n">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="H555" s="2" t="n">
         <v>1480786</v>
@@ -26313,13 +26313,13 @@
         </is>
       </c>
       <c r="E556" s="4" t="n">
-        <v>0.25</v>
+        <v>2</v>
       </c>
       <c r="F556" s="5" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="G556" s="4" t="n">
-        <v>6.25</v>
+        <v>80</v>
       </c>
       <c r="H556" s="2" t="n">
         <v>1480786</v>
@@ -26454,13 +26454,13 @@
         </is>
       </c>
       <c r="E559" s="4" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F559" s="5" t="n">
-        <v>1.89</v>
+        <v>14.06</v>
       </c>
       <c r="G559" s="4" t="n">
-        <v>37.8</v>
+        <v>14.06</v>
       </c>
       <c r="H559" s="2" t="n">
         <v>1480796</v>
@@ -26501,13 +26501,13 @@
         </is>
       </c>
       <c r="E560" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F560" s="5" t="n">
-        <v>14.06</v>
+        <v>2.95</v>
       </c>
       <c r="G560" s="4" t="n">
-        <v>14.06</v>
+        <v>5.9</v>
       </c>
       <c r="H560" s="2" t="n">
         <v>1480796</v>
@@ -26548,13 +26548,13 @@
         </is>
       </c>
       <c r="E561" s="4" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F561" s="5" t="n">
-        <v>4.45</v>
+        <v>1.89</v>
       </c>
       <c r="G561" s="4" t="n">
-        <v>178</v>
+        <v>37.8</v>
       </c>
       <c r="H561" s="2" t="n">
         <v>1480796</v>
@@ -26595,13 +26595,13 @@
         </is>
       </c>
       <c r="E562" s="4" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="F562" s="5" t="n">
-        <v>2.95</v>
+        <v>4.45</v>
       </c>
       <c r="G562" s="4" t="n">
-        <v>5.9</v>
+        <v>178</v>
       </c>
       <c r="H562" s="2" t="n">
         <v>1480796</v>
@@ -28619,10 +28619,10 @@
         <v>1</v>
       </c>
       <c r="F605" s="5" t="n">
-        <v>195</v>
+        <v>30</v>
       </c>
       <c r="G605" s="4" t="n">
-        <v>195</v>
+        <v>30</v>
       </c>
       <c r="H605" s="2" t="n">
         <v>1490619</v>
@@ -28666,10 +28666,10 @@
         <v>1</v>
       </c>
       <c r="F606" s="5" t="n">
-        <v>230</v>
+        <v>165</v>
       </c>
       <c r="G606" s="4" t="n">
-        <v>230</v>
+        <v>165</v>
       </c>
       <c r="H606" s="2" t="n">
         <v>1490619</v>
@@ -28713,10 +28713,10 @@
         <v>1</v>
       </c>
       <c r="F607" s="5" t="n">
-        <v>165</v>
+        <v>230</v>
       </c>
       <c r="G607" s="4" t="n">
-        <v>165</v>
+        <v>230</v>
       </c>
       <c r="H607" s="2" t="n">
         <v>1490619</v>
@@ -28760,10 +28760,10 @@
         <v>1</v>
       </c>
       <c r="F608" s="5" t="n">
-        <v>30</v>
+        <v>195</v>
       </c>
       <c r="G608" s="4" t="n">
-        <v>30</v>
+        <v>195</v>
       </c>
       <c r="H608" s="2" t="n">
         <v>1490619</v>
@@ -28851,13 +28851,13 @@
         </is>
       </c>
       <c r="E610" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F610" s="5" t="n">
-        <v>6.6</v>
+        <v>41.71</v>
       </c>
       <c r="G610" s="4" t="n">
-        <v>19.8</v>
+        <v>83.42</v>
       </c>
       <c r="H610" s="2" t="n">
         <v>1490652</v>
@@ -28898,13 +28898,13 @@
         </is>
       </c>
       <c r="E611" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F611" s="5" t="n">
-        <v>55.99</v>
+        <v>49.9</v>
       </c>
       <c r="G611" s="4" t="n">
-        <v>167.97</v>
+        <v>49.9</v>
       </c>
       <c r="H611" s="2" t="n">
         <v>1490652</v>
@@ -28992,13 +28992,13 @@
         </is>
       </c>
       <c r="E613" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F613" s="5" t="n">
-        <v>0.86</v>
+        <v>55.99</v>
       </c>
       <c r="G613" s="4" t="n">
-        <v>8.6</v>
+        <v>167.97</v>
       </c>
       <c r="H613" s="2" t="n">
         <v>1490652</v>
@@ -29039,13 +29039,13 @@
         </is>
       </c>
       <c r="E614" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F614" s="5" t="n">
-        <v>17.52</v>
+        <v>6.6</v>
       </c>
       <c r="G614" s="4" t="n">
-        <v>70.08</v>
+        <v>19.8</v>
       </c>
       <c r="H614" s="2" t="n">
         <v>1490652</v>
@@ -29086,13 +29086,13 @@
         </is>
       </c>
       <c r="E615" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F615" s="5" t="n">
-        <v>41.71</v>
+        <v>17.52</v>
       </c>
       <c r="G615" s="4" t="n">
-        <v>83.42</v>
+        <v>70.08</v>
       </c>
       <c r="H615" s="2" t="n">
         <v>1490652</v>
@@ -29133,13 +29133,13 @@
         </is>
       </c>
       <c r="E616" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F616" s="5" t="n">
-        <v>49.9</v>
+        <v>0.86</v>
       </c>
       <c r="G616" s="4" t="n">
-        <v>49.9</v>
+        <v>8.6</v>
       </c>
       <c r="H616" s="2" t="n">
         <v>1490652</v>
@@ -30734,10 +30734,10 @@
         <v>200</v>
       </c>
       <c r="F650" s="5" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="G650" s="4" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="H650" s="2" t="n">
         <v>1498122</v>
@@ -30781,10 +30781,10 @@
         <v>200</v>
       </c>
       <c r="F651" s="5" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="G651" s="4" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="H651" s="2" t="n">
         <v>1498122</v>
@@ -31721,10 +31721,10 @@
         <v>2</v>
       </c>
       <c r="F671" s="5" t="n">
-        <v>2.03</v>
+        <v>0.9</v>
       </c>
       <c r="G671" s="4" t="n">
-        <v>4.06</v>
+        <v>1.8</v>
       </c>
       <c r="H671" s="2" t="n">
         <v>1503029</v>
@@ -31765,13 +31765,13 @@
         </is>
       </c>
       <c r="E672" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F672" s="5" t="n">
-        <v>30</v>
+        <v>30.63</v>
       </c>
       <c r="G672" s="4" t="n">
-        <v>60</v>
+        <v>30.63</v>
       </c>
       <c r="H672" s="2" t="n">
         <v>1503029</v>
@@ -31812,13 +31812,13 @@
         </is>
       </c>
       <c r="E673" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F673" s="5" t="n">
-        <v>0.9</v>
+        <v>5.39</v>
       </c>
       <c r="G673" s="4" t="n">
-        <v>1.8</v>
+        <v>5.39</v>
       </c>
       <c r="H673" s="2" t="n">
         <v>1503029</v>
@@ -31862,10 +31862,10 @@
         <v>2</v>
       </c>
       <c r="F674" s="5" t="n">
-        <v>1.01</v>
+        <v>2.03</v>
       </c>
       <c r="G674" s="4" t="n">
-        <v>2.02</v>
+        <v>4.06</v>
       </c>
       <c r="H674" s="2" t="n">
         <v>1503029</v>
@@ -31906,13 +31906,13 @@
         </is>
       </c>
       <c r="E675" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F675" s="5" t="n">
-        <v>5.39</v>
+        <v>30</v>
       </c>
       <c r="G675" s="4" t="n">
-        <v>5.39</v>
+        <v>60</v>
       </c>
       <c r="H675" s="2" t="n">
         <v>1503029</v>
@@ -31953,13 +31953,13 @@
         </is>
       </c>
       <c r="E676" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F676" s="5" t="n">
-        <v>30.63</v>
+        <v>1.01</v>
       </c>
       <c r="G676" s="4" t="n">
-        <v>30.63</v>
+        <v>2.02</v>
       </c>
       <c r="H676" s="2" t="n">
         <v>1503029</v>
@@ -32379,10 +32379,10 @@
         <v>1</v>
       </c>
       <c r="F685" s="5" t="n">
-        <v>14.02</v>
+        <v>13.6</v>
       </c>
       <c r="G685" s="4" t="n">
-        <v>14.02</v>
+        <v>13.6</v>
       </c>
       <c r="H685" s="2" t="n">
         <v>1503440</v>
@@ -32473,10 +32473,10 @@
         <v>1</v>
       </c>
       <c r="F687" s="5" t="n">
-        <v>13.6</v>
+        <v>14.02</v>
       </c>
       <c r="G687" s="4" t="n">
-        <v>13.6</v>
+        <v>14.02</v>
       </c>
       <c r="H687" s="2" t="n">
         <v>1503440</v>
@@ -33272,10 +33272,10 @@
         <v>2</v>
       </c>
       <c r="F704" s="5" t="n">
-        <v>2.88</v>
+        <v>2.29</v>
       </c>
       <c r="G704" s="4" t="n">
-        <v>5.76</v>
+        <v>4.58</v>
       </c>
       <c r="H704" s="2" t="n">
         <v>1512391</v>
@@ -33319,10 +33319,10 @@
         <v>2</v>
       </c>
       <c r="F705" s="5" t="n">
-        <v>2.29</v>
+        <v>2.38</v>
       </c>
       <c r="G705" s="4" t="n">
-        <v>4.58</v>
+        <v>4.76</v>
       </c>
       <c r="H705" s="2" t="n">
         <v>1512391</v>
@@ -33363,13 +33363,13 @@
         </is>
       </c>
       <c r="E706" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F706" s="5" t="n">
-        <v>2.38</v>
+        <v>15.25</v>
       </c>
       <c r="G706" s="4" t="n">
-        <v>4.76</v>
+        <v>15.25</v>
       </c>
       <c r="H706" s="2" t="n">
         <v>1512391</v>
@@ -33413,10 +33413,10 @@
         <v>1</v>
       </c>
       <c r="F707" s="5" t="n">
-        <v>15.25</v>
+        <v>10.3</v>
       </c>
       <c r="G707" s="4" t="n">
-        <v>15.25</v>
+        <v>10.3</v>
       </c>
       <c r="H707" s="2" t="n">
         <v>1512391</v>
@@ -33460,10 +33460,10 @@
         <v>1</v>
       </c>
       <c r="F708" s="5" t="n">
-        <v>10.3</v>
+        <v>12.25</v>
       </c>
       <c r="G708" s="4" t="n">
-        <v>10.3</v>
+        <v>12.25</v>
       </c>
       <c r="H708" s="2" t="n">
         <v>1512391</v>
@@ -33504,13 +33504,13 @@
         </is>
       </c>
       <c r="E709" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F709" s="5" t="n">
-        <v>12.25</v>
+        <v>2.88</v>
       </c>
       <c r="G709" s="4" t="n">
-        <v>12.25</v>
+        <v>5.76</v>
       </c>
       <c r="H709" s="2" t="n">
         <v>1512391</v>
@@ -33598,13 +33598,13 @@
         </is>
       </c>
       <c r="E711" s="4" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="F711" s="5" t="n">
-        <v>0.22</v>
+        <v>0.8</v>
       </c>
       <c r="G711" s="4" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="H711" s="2" t="n">
         <v>1512750</v>
@@ -33648,10 +33648,10 @@
         <v>100</v>
       </c>
       <c r="F712" s="5" t="n">
-        <v>0.15</v>
+        <v>0.22</v>
       </c>
       <c r="G712" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H712" s="2" t="n">
         <v>1512750</v>
@@ -33692,13 +33692,13 @@
         </is>
       </c>
       <c r="E713" s="4" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F713" s="5" t="n">
-        <v>0.15</v>
+        <v>0.22</v>
       </c>
       <c r="G713" s="4" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="H713" s="2" t="n">
         <v>1512750</v>
@@ -33739,13 +33739,13 @@
         </is>
       </c>
       <c r="E714" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F714" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G714" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="F714" s="5" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="G714" s="4" t="n">
-        <v>2.55</v>
       </c>
       <c r="H714" s="2" t="n">
         <v>1512750</v>
@@ -33786,13 +33786,13 @@
         </is>
       </c>
       <c r="E715" s="4" t="n">
-        <v>15</v>
+        <v>300</v>
       </c>
       <c r="F715" s="5" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="G715" s="4" t="n">
-        <v>4.5</v>
+        <v>45</v>
       </c>
       <c r="H715" s="2" t="n">
         <v>1512750</v>
@@ -33836,10 +33836,10 @@
         <v>15</v>
       </c>
       <c r="F716" s="5" t="n">
-        <v>0.8</v>
+        <v>0.17</v>
       </c>
       <c r="G716" s="4" t="n">
-        <v>12</v>
+        <v>2.55</v>
       </c>
       <c r="H716" s="2" t="n">
         <v>1512750</v>
@@ -33880,13 +33880,13 @@
         </is>
       </c>
       <c r="E717" s="4" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="F717" s="5" t="n">
-        <v>0.22</v>
+        <v>0.3</v>
       </c>
       <c r="G717" s="4" t="n">
-        <v>22</v>
+        <v>4.5</v>
       </c>
       <c r="H717" s="2" t="n">
         <v>1512750</v>
@@ -34259,10 +34259,10 @@
         <v>1</v>
       </c>
       <c r="F725" s="5" t="n">
-        <v>170.39</v>
+        <v>157.85</v>
       </c>
       <c r="G725" s="4" t="n">
-        <v>170.39</v>
+        <v>157.85</v>
       </c>
       <c r="H725" s="2" t="n">
         <v>1513749</v>
@@ -34306,10 +34306,10 @@
         <v>1</v>
       </c>
       <c r="F726" s="5" t="n">
-        <v>157.85</v>
+        <v>170.39</v>
       </c>
       <c r="G726" s="4" t="n">
-        <v>157.85</v>
+        <v>170.39</v>
       </c>
       <c r="H726" s="2" t="n">
         <v>1513749</v>
@@ -35478,13 +35478,13 @@
         </is>
       </c>
       <c r="E751" s="4" t="n">
-        <v>0.04</v>
+        <v>4</v>
       </c>
       <c r="F751" s="5" t="n">
-        <v>60</v>
+        <v>95</v>
       </c>
       <c r="G751" s="4" t="n">
-        <v>2.4</v>
+        <v>380</v>
       </c>
       <c r="H751" s="2" t="n">
         <v>1517956</v>
@@ -35619,13 +35619,13 @@
         </is>
       </c>
       <c r="E754" s="4" t="n">
-        <v>4</v>
+        <v>0.04</v>
       </c>
       <c r="F754" s="5" t="n">
-        <v>95</v>
+        <v>25</v>
       </c>
       <c r="G754" s="4" t="n">
-        <v>380</v>
+        <v>1</v>
       </c>
       <c r="H754" s="2" t="n">
         <v>1517956</v>
@@ -35669,10 +35669,10 @@
         <v>0.04</v>
       </c>
       <c r="F755" s="5" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="G755" s="4" t="n">
-        <v>1.4</v>
+        <v>2.4</v>
       </c>
       <c r="H755" s="2" t="n">
         <v>1517956</v>
@@ -35713,13 +35713,13 @@
         </is>
       </c>
       <c r="E756" s="4" t="n">
-        <v>4</v>
+        <v>0.04</v>
       </c>
       <c r="F756" s="5" t="n">
-        <v>0.75</v>
+        <v>35</v>
       </c>
       <c r="G756" s="4" t="n">
-        <v>3</v>
+        <v>1.4</v>
       </c>
       <c r="H756" s="2" t="n">
         <v>1517956</v>
@@ -35760,13 +35760,13 @@
         </is>
       </c>
       <c r="E757" s="4" t="n">
-        <v>0.04</v>
+        <v>4</v>
       </c>
       <c r="F757" s="5" t="n">
-        <v>25</v>
+        <v>0.75</v>
       </c>
       <c r="G757" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H757" s="2" t="n">
         <v>1517956</v>
@@ -37076,13 +37076,13 @@
         </is>
       </c>
       <c r="E785" s="4" t="n">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="F785" s="5" t="n">
-        <v>54.3</v>
+        <v>9.1</v>
       </c>
       <c r="G785" s="4" t="n">
-        <v>2009.1</v>
+        <v>127.4</v>
       </c>
       <c r="H785" s="2" t="n">
         <v>1522616</v>
@@ -37123,13 +37123,13 @@
         </is>
       </c>
       <c r="E786" s="4" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="F786" s="5" t="n">
-        <v>153.6</v>
+        <v>54.3</v>
       </c>
       <c r="G786" s="4" t="n">
-        <v>2457.6</v>
+        <v>2009.1</v>
       </c>
       <c r="H786" s="2" t="n">
         <v>1522616</v>
@@ -37217,13 +37217,13 @@
         </is>
       </c>
       <c r="E788" s="4" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="F788" s="5" t="n">
-        <v>139.6</v>
+        <v>153.6</v>
       </c>
       <c r="G788" s="4" t="n">
-        <v>279.2</v>
+        <v>2457.6</v>
       </c>
       <c r="H788" s="2" t="n">
         <v>1522616</v>
@@ -37264,13 +37264,13 @@
         </is>
       </c>
       <c r="E789" s="4" t="n">
-        <v>36</v>
+        <v>69</v>
       </c>
       <c r="F789" s="5" t="n">
-        <v>127.6</v>
+        <v>54.3</v>
       </c>
       <c r="G789" s="4" t="n">
-        <v>4593.6</v>
+        <v>3746.7</v>
       </c>
       <c r="H789" s="2" t="n">
         <v>1522616</v>
@@ -37311,13 +37311,13 @@
         </is>
       </c>
       <c r="E790" s="4" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="F790" s="5" t="n">
-        <v>9.1</v>
+        <v>139.6</v>
       </c>
       <c r="G790" s="4" t="n">
-        <v>127.4</v>
+        <v>279.2</v>
       </c>
       <c r="H790" s="2" t="n">
         <v>1522616</v>
@@ -37358,13 +37358,13 @@
         </is>
       </c>
       <c r="E791" s="4" t="n">
-        <v>69</v>
+        <v>36</v>
       </c>
       <c r="F791" s="5" t="n">
-        <v>54.3</v>
+        <v>127.6</v>
       </c>
       <c r="G791" s="4" t="n">
-        <v>3746.7</v>
+        <v>4593.6</v>
       </c>
       <c r="H791" s="2" t="n">
         <v>1522616</v>
@@ -37922,13 +37922,13 @@
         </is>
       </c>
       <c r="E803" s="4" t="n">
-        <v>1.28</v>
+        <v>1</v>
       </c>
       <c r="F803" s="5" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G803" s="4" t="n">
-        <v>48.64</v>
+        <v>36</v>
       </c>
       <c r="H803" s="2" t="n">
         <v>1524925</v>
@@ -37969,13 +37969,13 @@
         </is>
       </c>
       <c r="E804" s="4" t="n">
-        <v>1.89</v>
+        <v>0.08</v>
       </c>
       <c r="F804" s="5" t="n">
-        <v>150</v>
+        <v>18</v>
       </c>
       <c r="G804" s="4" t="n">
-        <v>283.5</v>
+        <v>1.44</v>
       </c>
       <c r="H804" s="2" t="n">
         <v>1524925</v>
@@ -38016,13 +38016,13 @@
         </is>
       </c>
       <c r="E805" s="4" t="n">
-        <v>0.08</v>
+        <v>1.89</v>
       </c>
       <c r="F805" s="5" t="n">
-        <v>18</v>
+        <v>150</v>
       </c>
       <c r="G805" s="4" t="n">
-        <v>1.44</v>
+        <v>283.5</v>
       </c>
       <c r="H805" s="2" t="n">
         <v>1524925</v>
@@ -38063,13 +38063,13 @@
         </is>
       </c>
       <c r="E806" s="4" t="n">
-        <v>1</v>
+        <v>1.28</v>
       </c>
       <c r="F806" s="5" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G806" s="4" t="n">
-        <v>36</v>
+        <v>48.64</v>
       </c>
       <c r="H806" s="2" t="n">
         <v>1524925</v>
@@ -38580,13 +38580,13 @@
         </is>
       </c>
       <c r="E817" s="4" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F817" s="5" t="n">
-        <v>9.59</v>
+        <v>3.89</v>
       </c>
       <c r="G817" s="4" t="n">
-        <v>9.59</v>
+        <v>58.35</v>
       </c>
       <c r="H817" s="2" t="n">
         <v>1526079</v>
@@ -38627,13 +38627,13 @@
         </is>
       </c>
       <c r="E818" s="4" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F818" s="5" t="n">
-        <v>3.89</v>
+        <v>9.59</v>
       </c>
       <c r="G818" s="4" t="n">
-        <v>58.35</v>
+        <v>9.59</v>
       </c>
       <c r="H818" s="2" t="n">
         <v>1526079</v>
@@ -40087,10 +40087,10 @@
         <v>1</v>
       </c>
       <c r="F849" s="5" t="n">
-        <v>306.68</v>
+        <v>180.4</v>
       </c>
       <c r="G849" s="4" t="n">
-        <v>306.68</v>
+        <v>180.4</v>
       </c>
       <c r="H849" s="2" t="n">
         <v>1530930</v>
@@ -40134,10 +40134,10 @@
         <v>1</v>
       </c>
       <c r="F850" s="5" t="n">
-        <v>180.4</v>
+        <v>306.68</v>
       </c>
       <c r="G850" s="4" t="n">
-        <v>180.4</v>
+        <v>306.68</v>
       </c>
       <c r="H850" s="2" t="n">
         <v>1530930</v>
@@ -40413,13 +40413,13 @@
         </is>
       </c>
       <c r="E856" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F856" s="5" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G856" s="4" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="H856" s="2" t="n">
         <v>1532084</v>
@@ -40463,10 +40463,10 @@
         <v>1</v>
       </c>
       <c r="F857" s="5" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="G857" s="4" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="H857" s="2" t="n">
         <v>1532084</v>
@@ -40507,13 +40507,13 @@
         </is>
       </c>
       <c r="E858" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F858" s="5" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G858" s="4" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="H858" s="2" t="n">
         <v>1532084</v>
@@ -40557,10 +40557,10 @@
         <v>1</v>
       </c>
       <c r="F859" s="5" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="G859" s="4" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="H859" s="2" t="n">
         <v>1532084</v>
@@ -40604,10 +40604,10 @@
         <v>1.5</v>
       </c>
       <c r="F860" s="5" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="G860" s="4" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="H860" s="2" t="n">
         <v>1532084</v>
@@ -41823,13 +41823,13 @@
         </is>
       </c>
       <c r="E886" s="4" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F886" s="5" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="G886" s="4" t="n">
-        <v>8</v>
+        <v>2.4</v>
       </c>
       <c r="H886" s="2" t="n">
         <v>1539898</v>
@@ -41870,13 +41870,13 @@
         </is>
       </c>
       <c r="E887" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F887" s="5" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G887" s="4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H887" s="2" t="n">
         <v>1539898</v>
@@ -41917,13 +41917,13 @@
         </is>
       </c>
       <c r="E888" s="4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F888" s="5" t="n">
-        <v>2.3</v>
+        <v>1</v>
       </c>
       <c r="G888" s="4" t="n">
-        <v>13.8</v>
+        <v>12</v>
       </c>
       <c r="H888" s="2" t="n">
         <v>1539898</v>
@@ -41964,13 +41964,13 @@
         </is>
       </c>
       <c r="E889" s="4" t="n">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="F889" s="5" t="n">
-        <v>0.66</v>
+        <v>2.3</v>
       </c>
       <c r="G889" s="4" t="n">
-        <v>66</v>
+        <v>13.8</v>
       </c>
       <c r="H889" s="2" t="n">
         <v>1539898</v>
@@ -42011,13 +42011,13 @@
         </is>
       </c>
       <c r="E890" s="4" t="n">
-        <v>8</v>
+        <v>100</v>
       </c>
       <c r="F890" s="5" t="n">
-        <v>0.52</v>
+        <v>0.66</v>
       </c>
       <c r="G890" s="4" t="n">
-        <v>4.16</v>
+        <v>66</v>
       </c>
       <c r="H890" s="2" t="n">
         <v>1539898</v>
@@ -42058,13 +42058,13 @@
         </is>
       </c>
       <c r="E891" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F891" s="5" t="n">
-        <v>0.58</v>
+        <v>0.52</v>
       </c>
       <c r="G891" s="4" t="n">
-        <v>2.32</v>
+        <v>4.16</v>
       </c>
       <c r="H891" s="2" t="n">
         <v>1539898</v>
@@ -42105,13 +42105,13 @@
         </is>
       </c>
       <c r="E892" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F892" s="5" t="n">
-        <v>0.81</v>
+        <v>0.58</v>
       </c>
       <c r="G892" s="4" t="n">
-        <v>1.62</v>
+        <v>2.32</v>
       </c>
       <c r="H892" s="2" t="n">
         <v>1539898</v>
@@ -42152,13 +42152,13 @@
         </is>
       </c>
       <c r="E893" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F893" s="5" t="n">
-        <v>0.7</v>
+        <v>0.81</v>
       </c>
       <c r="G893" s="4" t="n">
-        <v>2.8</v>
+        <v>1.62</v>
       </c>
       <c r="H893" s="2" t="n">
         <v>1539898</v>
@@ -42199,13 +42199,13 @@
         </is>
       </c>
       <c r="E894" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F894" s="5" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="G894" s="4" t="n">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="H894" s="2" t="n">
         <v>1539898</v>
@@ -42246,13 +42246,13 @@
         </is>
       </c>
       <c r="E895" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F895" s="5" t="n">
-        <v>1.32</v>
+        <v>1.2</v>
       </c>
       <c r="G895" s="4" t="n">
-        <v>5.28</v>
+        <v>2.4</v>
       </c>
       <c r="H895" s="2" t="n">
         <v>1539898</v>
@@ -42293,13 +42293,13 @@
         </is>
       </c>
       <c r="E896" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F896" s="5" t="n">
-        <v>0.45</v>
+        <v>1.32</v>
       </c>
       <c r="G896" s="4" t="n">
-        <v>5.4</v>
+        <v>5.28</v>
       </c>
       <c r="H896" s="2" t="n">
         <v>1539898</v>
@@ -42340,13 +42340,13 @@
         </is>
       </c>
       <c r="E897" s="4" t="n">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="F897" s="5" t="n">
-        <v>0.11</v>
+        <v>0.45</v>
       </c>
       <c r="G897" s="4" t="n">
-        <v>11</v>
+        <v>5.4</v>
       </c>
       <c r="H897" s="2" t="n">
         <v>1539898</v>
@@ -42390,10 +42390,10 @@
         <v>100</v>
       </c>
       <c r="F898" s="5" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="G898" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H898" s="2" t="n">
         <v>1539898</v>
@@ -42434,13 +42434,13 @@
         </is>
       </c>
       <c r="E899" s="4" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="F899" s="5" t="n">
-        <v>0.2</v>
+        <v>0.12</v>
       </c>
       <c r="G899" s="4" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H899" s="2" t="n">
         <v>1539898</v>
@@ -42481,13 +42481,13 @@
         </is>
       </c>
       <c r="E900" s="4" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="F900" s="5" t="n">
-        <v>0.42</v>
+        <v>0.2</v>
       </c>
       <c r="G900" s="4" t="n">
-        <v>2.52</v>
+        <v>4</v>
       </c>
       <c r="H900" s="2" t="n">
         <v>1539898</v>
@@ -42528,13 +42528,13 @@
         </is>
       </c>
       <c r="E901" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F901" s="5" t="n">
-        <v>0.3</v>
+        <v>0.42</v>
       </c>
       <c r="G901" s="4" t="n">
-        <v>3</v>
+        <v>2.52</v>
       </c>
       <c r="H901" s="2" t="n">
         <v>1539898</v>
@@ -42575,13 +42575,13 @@
         </is>
       </c>
       <c r="E902" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F902" s="5" t="n">
-        <v>0.33</v>
+        <v>0.3</v>
       </c>
       <c r="G902" s="4" t="n">
-        <v>1.98</v>
+        <v>3</v>
       </c>
       <c r="H902" s="2" t="n">
         <v>1539898</v>
@@ -42622,13 +42622,13 @@
         </is>
       </c>
       <c r="E903" s="4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F903" s="5" t="n">
-        <v>0.21</v>
+        <v>0.33</v>
       </c>
       <c r="G903" s="4" t="n">
-        <v>2.52</v>
+        <v>1.98</v>
       </c>
       <c r="H903" s="2" t="n">
         <v>1539898</v>
@@ -42669,13 +42669,13 @@
         </is>
       </c>
       <c r="E904" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F904" s="5" t="n">
-        <v>0.29</v>
+        <v>0.21</v>
       </c>
       <c r="G904" s="4" t="n">
-        <v>4.06</v>
+        <v>2.52</v>
       </c>
       <c r="H904" s="2" t="n">
         <v>1539898</v>
@@ -42716,13 +42716,13 @@
         </is>
       </c>
       <c r="E905" s="4" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="F905" s="5" t="n">
-        <v>0.35</v>
+        <v>0.29</v>
       </c>
       <c r="G905" s="4" t="n">
-        <v>2.1</v>
+        <v>4.06</v>
       </c>
       <c r="H905" s="2" t="n">
         <v>1539898</v>
@@ -42763,13 +42763,13 @@
         </is>
       </c>
       <c r="E906" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F906" s="5" t="n">
-        <v>0.48</v>
+        <v>0.35</v>
       </c>
       <c r="G906" s="4" t="n">
-        <v>1.92</v>
+        <v>2.1</v>
       </c>
       <c r="H906" s="2" t="n">
         <v>1539898</v>
@@ -42810,13 +42810,13 @@
         </is>
       </c>
       <c r="E907" s="4" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="F907" s="5" t="n">
-        <v>0.2</v>
+        <v>0.48</v>
       </c>
       <c r="G907" s="4" t="n">
-        <v>4.8</v>
+        <v>1.92</v>
       </c>
       <c r="H907" s="2" t="n">
         <v>1539898</v>
@@ -42857,13 +42857,13 @@
         </is>
       </c>
       <c r="E908" s="4" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F908" s="5" t="n">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="G908" s="4" t="n">
-        <v>5.32</v>
+        <v>4.8</v>
       </c>
       <c r="H908" s="2" t="n">
         <v>1539898</v>
@@ -42904,13 +42904,13 @@
         </is>
       </c>
       <c r="E909" s="4" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F909" s="5" t="n">
-        <v>0.08</v>
+        <v>0.19</v>
       </c>
       <c r="G909" s="4" t="n">
-        <v>0.96</v>
+        <v>5.32</v>
       </c>
       <c r="H909" s="2" t="n">
         <v>1539898</v>
@@ -42951,13 +42951,13 @@
         </is>
       </c>
       <c r="E910" s="4" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F910" s="5" t="n">
-        <v>0.17</v>
+        <v>0.08</v>
       </c>
       <c r="G910" s="4" t="n">
-        <v>5.1</v>
+        <v>0.96</v>
       </c>
       <c r="H910" s="2" t="n">
         <v>1539898</v>
@@ -42998,13 +42998,13 @@
         </is>
       </c>
       <c r="E911" s="4" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="F911" s="5" t="n">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="G911" s="4" t="n">
-        <v>1.32</v>
+        <v>5.1</v>
       </c>
       <c r="H911" s="2" t="n">
         <v>1539898</v>
@@ -43045,13 +43045,13 @@
         </is>
       </c>
       <c r="E912" s="4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F912" s="5" t="n">
-        <v>0.15</v>
+        <v>0.22</v>
       </c>
       <c r="G912" s="4" t="n">
-        <v>1.8</v>
+        <v>1.32</v>
       </c>
       <c r="H912" s="2" t="n">
         <v>1539898</v>
@@ -43092,13 +43092,13 @@
         </is>
       </c>
       <c r="E913" s="4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F913" s="5" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="G913" s="4" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="H913" s="2" t="n">
         <v>1539898</v>
@@ -43280,13 +43280,13 @@
         </is>
       </c>
       <c r="E917" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F917" s="5" t="n">
-        <v>0.6</v>
+        <v>0.25</v>
       </c>
       <c r="G917" s="4" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="H917" s="2" t="n">
         <v>1539898</v>
@@ -44364,10 +44364,10 @@
         <v>1</v>
       </c>
       <c r="F940" s="5" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="G940" s="4" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="H940" s="2" t="n">
         <v>1547044</v>
@@ -44411,10 +44411,10 @@
         <v>1</v>
       </c>
       <c r="F941" s="5" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="G941" s="4" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="H941" s="2" t="n">
         <v>1547044</v>
@@ -44505,10 +44505,10 @@
         <v>1</v>
       </c>
       <c r="F943" s="5" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="G943" s="4" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="H943" s="2" t="n">
         <v>1547044</v>
@@ -44599,10 +44599,10 @@
         <v>1</v>
       </c>
       <c r="F945" s="5" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="G945" s="4" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="H945" s="2" t="n">
         <v>1547044</v>
@@ -48500,10 +48500,10 @@
         <v>3</v>
       </c>
       <c r="F1028" s="5" t="n">
-        <v>21.9</v>
+        <v>25.9</v>
       </c>
       <c r="G1028" s="4" t="n">
-        <v>65.7</v>
+        <v>77.7</v>
       </c>
       <c r="H1028" s="2" t="n">
         <v>1561933</v>
@@ -48544,13 +48544,13 @@
         </is>
       </c>
       <c r="E1029" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F1029" s="5" t="n">
-        <v>31.9</v>
+        <v>21.9</v>
       </c>
       <c r="G1029" s="4" t="n">
-        <v>31.9</v>
+        <v>65.7</v>
       </c>
       <c r="H1029" s="2" t="n">
         <v>1561933</v>
@@ -48591,13 +48591,13 @@
         </is>
       </c>
       <c r="E1030" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F1030" s="5" t="n">
-        <v>25.9</v>
+        <v>31.9</v>
       </c>
       <c r="G1030" s="4" t="n">
-        <v>77.7</v>
+        <v>31.9</v>
       </c>
       <c r="H1030" s="2" t="n">
         <v>1561933</v>
@@ -49531,13 +49531,13 @@
         </is>
       </c>
       <c r="E1050" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1050" s="5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G1050" s="4" t="n">
-        <v>7.5</v>
+        <v>14</v>
       </c>
       <c r="H1050" s="2" t="n">
         <v>1565694</v>
@@ -49578,13 +49578,13 @@
         </is>
       </c>
       <c r="E1051" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1051" s="5" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="G1051" s="4" t="n">
-        <v>22</v>
+        <v>7.5</v>
       </c>
       <c r="H1051" s="2" t="n">
         <v>1565694</v>
@@ -49625,13 +49625,13 @@
         </is>
       </c>
       <c r="E1052" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1052" s="5" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G1052" s="4" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="H1052" s="2" t="n">
         <v>1565694</v>
@@ -49675,10 +49675,10 @@
         <v>100</v>
       </c>
       <c r="F1053" s="5" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="G1053" s="4" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H1053" s="2" t="n">
         <v>1565694</v>
@@ -50095,13 +50095,13 @@
         </is>
       </c>
       <c r="E1062" s="4" t="n">
-        <v>1</v>
+        <v>0.11</v>
       </c>
       <c r="F1062" s="5" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G1062" s="4" t="n">
-        <v>14</v>
+        <v>2.75</v>
       </c>
       <c r="H1062" s="2" t="n">
         <v>1565694</v>
@@ -50142,13 +50142,13 @@
         </is>
       </c>
       <c r="E1063" s="4" t="n">
-        <v>0.11</v>
+        <v>5</v>
       </c>
       <c r="F1063" s="5" t="n">
-        <v>25</v>
+        <v>0.3</v>
       </c>
       <c r="G1063" s="4" t="n">
-        <v>2.75</v>
+        <v>1.5</v>
       </c>
       <c r="H1063" s="2" t="n">
         <v>1565694</v>
@@ -50189,13 +50189,13 @@
         </is>
       </c>
       <c r="E1064" s="4" t="n">
-        <v>5</v>
+        <v>0.16</v>
       </c>
       <c r="F1064" s="5" t="n">
-        <v>0.3</v>
+        <v>20</v>
       </c>
       <c r="G1064" s="4" t="n">
-        <v>1.5</v>
+        <v>3.2</v>
       </c>
       <c r="H1064" s="2" t="n">
         <v>1565694</v>
@@ -50236,13 +50236,13 @@
         </is>
       </c>
       <c r="E1065" s="4" t="n">
-        <v>0.16</v>
+        <v>1</v>
       </c>
       <c r="F1065" s="5" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G1065" s="4" t="n">
-        <v>3.2</v>
+        <v>25</v>
       </c>
       <c r="H1065" s="2" t="n">
         <v>1565694</v>
@@ -50283,13 +50283,13 @@
         </is>
       </c>
       <c r="E1066" s="4" t="n">
-        <v>1</v>
+        <v>0.16</v>
       </c>
       <c r="F1066" s="5" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G1066" s="4" t="n">
-        <v>25</v>
+        <v>3.2</v>
       </c>
       <c r="H1066" s="2" t="n">
         <v>1565694</v>
@@ -50330,13 +50330,13 @@
         </is>
       </c>
       <c r="E1067" s="4" t="n">
-        <v>0.16</v>
+        <v>1</v>
       </c>
       <c r="F1067" s="5" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G1067" s="4" t="n">
-        <v>3.2</v>
+        <v>12</v>
       </c>
       <c r="H1067" s="2" t="n">
         <v>1565694</v>
@@ -50377,13 +50377,13 @@
         </is>
       </c>
       <c r="E1068" s="4" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F1068" s="5" t="n">
-        <v>12</v>
+        <v>0.25</v>
       </c>
       <c r="G1068" s="4" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="H1068" s="2" t="n">
         <v>1565694</v>
@@ -50424,13 +50424,13 @@
         </is>
       </c>
       <c r="E1069" s="4" t="n">
-        <v>100</v>
+        <v>0.5</v>
       </c>
       <c r="F1069" s="5" t="n">
-        <v>0.22</v>
+        <v>20</v>
       </c>
       <c r="G1069" s="4" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H1069" s="2" t="n">
         <v>1565694</v>
@@ -50847,13 +50847,13 @@
         </is>
       </c>
       <c r="E1078" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F1078" s="5" t="n">
-        <v>5.8</v>
+        <v>24.96</v>
       </c>
       <c r="G1078" s="4" t="n">
-        <v>11.6</v>
+        <v>74.88</v>
       </c>
       <c r="H1078" s="2" t="n">
         <v>1570182</v>
@@ -50894,13 +50894,13 @@
         </is>
       </c>
       <c r="E1079" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F1079" s="5" t="n">
-        <v>24.96</v>
+        <v>9.712</v>
       </c>
       <c r="G1079" s="4" t="n">
-        <v>74.88</v>
+        <v>9.71</v>
       </c>
       <c r="H1079" s="2" t="n">
         <v>1570182</v>
@@ -50941,13 +50941,13 @@
         </is>
       </c>
       <c r="E1080" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F1080" s="5" t="n">
-        <v>5.12</v>
+        <v>10.4</v>
       </c>
       <c r="G1080" s="4" t="n">
-        <v>20.48</v>
+        <v>10.4</v>
       </c>
       <c r="H1080" s="2" t="n">
         <v>1570182</v>
@@ -50988,13 +50988,13 @@
         </is>
       </c>
       <c r="E1081" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1081" s="5" t="n">
-        <v>18.66</v>
+        <v>6.624</v>
       </c>
       <c r="G1081" s="4" t="n">
-        <v>37.32</v>
+        <v>6.62</v>
       </c>
       <c r="H1081" s="2" t="n">
         <v>1570182</v>
@@ -51035,13 +51035,13 @@
         </is>
       </c>
       <c r="E1082" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F1082" s="5" t="n">
-        <v>10.4</v>
+        <v>5.12</v>
       </c>
       <c r="G1082" s="4" t="n">
-        <v>10.4</v>
+        <v>20.48</v>
       </c>
       <c r="H1082" s="2" t="n">
         <v>1570182</v>
@@ -51085,10 +51085,10 @@
         <v>1</v>
       </c>
       <c r="F1083" s="5" t="n">
-        <v>6.624</v>
+        <v>12</v>
       </c>
       <c r="G1083" s="4" t="n">
-        <v>6.62</v>
+        <v>12</v>
       </c>
       <c r="H1083" s="2" t="n">
         <v>1570182</v>
@@ -51129,13 +51129,13 @@
         </is>
       </c>
       <c r="E1084" s="4" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="F1084" s="5" t="n">
-        <v>0.87</v>
+        <v>18.66</v>
       </c>
       <c r="G1084" s="4" t="n">
-        <v>17.4</v>
+        <v>37.32</v>
       </c>
       <c r="H1084" s="2" t="n">
         <v>1570182</v>
@@ -51176,13 +51176,13 @@
         </is>
       </c>
       <c r="E1085" s="4" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F1085" s="5" t="n">
-        <v>9</v>
+        <v>0.87</v>
       </c>
       <c r="G1085" s="4" t="n">
-        <v>9</v>
+        <v>17.4</v>
       </c>
       <c r="H1085" s="2" t="n">
         <v>1570182</v>
@@ -51223,13 +51223,13 @@
         </is>
       </c>
       <c r="E1086" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1086" s="5" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G1086" s="4" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H1086" s="2" t="n">
         <v>1570182</v>
@@ -51273,10 +51273,10 @@
         <v>2</v>
       </c>
       <c r="F1087" s="5" t="n">
-        <v>9</v>
+        <v>5.8</v>
       </c>
       <c r="G1087" s="4" t="n">
-        <v>18</v>
+        <v>11.6</v>
       </c>
       <c r="H1087" s="2" t="n">
         <v>1570182</v>
@@ -51320,10 +51320,10 @@
         <v>1</v>
       </c>
       <c r="F1088" s="5" t="n">
-        <v>9.712</v>
+        <v>9</v>
       </c>
       <c r="G1088" s="4" t="n">
-        <v>9.71</v>
+        <v>9</v>
       </c>
       <c r="H1088" s="2" t="n">
         <v>1570182</v>
@@ -51411,13 +51411,13 @@
         </is>
       </c>
       <c r="E1090" s="4" t="n">
-        <v>0.15</v>
+        <v>3</v>
       </c>
       <c r="F1090" s="5" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="G1090" s="4" t="n">
-        <v>13.5</v>
+        <v>12</v>
       </c>
       <c r="H1090" s="2" t="n">
         <v>1570192</v>
@@ -51458,13 +51458,13 @@
         </is>
       </c>
       <c r="E1091" s="4" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="F1091" s="5" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="G1091" s="4" t="n">
-        <v>6.75</v>
+        <v>2.1</v>
       </c>
       <c r="H1091" s="2" t="n">
         <v>1570192</v>
@@ -51508,10 +51508,10 @@
         <v>0.3</v>
       </c>
       <c r="F1092" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G1092" s="4" t="n">
-        <v>2.1</v>
+        <v>1.8</v>
       </c>
       <c r="H1092" s="2" t="n">
         <v>1570192</v>
@@ -51552,13 +51552,13 @@
         </is>
       </c>
       <c r="E1093" s="4" t="n">
-        <v>3</v>
+        <v>0.15</v>
       </c>
       <c r="F1093" s="5" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="G1093" s="4" t="n">
-        <v>12</v>
+        <v>13.5</v>
       </c>
       <c r="H1093" s="2" t="n">
         <v>1570192</v>
@@ -51740,13 +51740,13 @@
         </is>
       </c>
       <c r="E1097" s="4" t="n">
-        <v>0.01</v>
+        <v>0.15</v>
       </c>
       <c r="F1097" s="5" t="n">
-        <v>350</v>
+        <v>45</v>
       </c>
       <c r="G1097" s="4" t="n">
-        <v>3.5</v>
+        <v>6.75</v>
       </c>
       <c r="H1097" s="2" t="n">
         <v>1570192</v>
@@ -51787,13 +51787,13 @@
         </is>
       </c>
       <c r="E1098" s="4" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F1098" s="5" t="n">
-        <v>170</v>
+        <v>30</v>
       </c>
       <c r="G1098" s="4" t="n">
-        <v>42.5</v>
+        <v>30</v>
       </c>
       <c r="H1098" s="2" t="n">
         <v>1570192</v>
@@ -51834,10 +51834,10 @@
         </is>
       </c>
       <c r="E1099" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1099" s="5" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="G1099" s="4" t="n">
         <v>30</v>
@@ -51881,13 +51881,13 @@
         </is>
       </c>
       <c r="E1100" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1100" s="5" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="G1100" s="4" t="n">
-        <v>22</v>
+        <v>22.5</v>
       </c>
       <c r="H1100" s="2" t="n">
         <v>1570192</v>
@@ -51928,13 +51928,13 @@
         </is>
       </c>
       <c r="E1101" s="4" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="F1101" s="5" t="n">
-        <v>30</v>
+        <v>170</v>
       </c>
       <c r="G1101" s="4" t="n">
-        <v>30</v>
+        <v>42.5</v>
       </c>
       <c r="H1101" s="2" t="n">
         <v>1570192</v>
@@ -51975,10 +51975,10 @@
         </is>
       </c>
       <c r="E1102" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1102" s="5" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="G1102" s="4" t="n">
         <v>30</v>
@@ -52022,13 +52022,13 @@
         </is>
       </c>
       <c r="E1103" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1103" s="5" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="G1103" s="4" t="n">
-        <v>22.5</v>
+        <v>22</v>
       </c>
       <c r="H1103" s="2" t="n">
         <v>1570192</v>
@@ -52069,13 +52069,13 @@
         </is>
       </c>
       <c r="E1104" s="4" t="n">
-        <v>0.3</v>
+        <v>0.01</v>
       </c>
       <c r="F1104" s="5" t="n">
-        <v>6</v>
+        <v>350</v>
       </c>
       <c r="G1104" s="4" t="n">
-        <v>1.8</v>
+        <v>3.5</v>
       </c>
       <c r="H1104" s="2" t="n">
         <v>1570192</v>
@@ -53338,13 +53338,13 @@
         </is>
       </c>
       <c r="E1131" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F1131" s="5" t="n">
-        <v>3.45</v>
+        <v>8.3</v>
       </c>
       <c r="G1131" s="4" t="n">
-        <v>3.45</v>
+        <v>49.8</v>
       </c>
       <c r="H1131" s="2" t="n">
         <v>1575575</v>
@@ -53385,13 +53385,13 @@
         </is>
       </c>
       <c r="E1132" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F1132" s="5" t="n">
-        <v>8.3</v>
+        <v>3.5</v>
       </c>
       <c r="G1132" s="4" t="n">
-        <v>49.8</v>
+        <v>3.5</v>
       </c>
       <c r="H1132" s="2" t="n">
         <v>1575575</v>
@@ -53435,10 +53435,10 @@
         <v>1</v>
       </c>
       <c r="F1133" s="5" t="n">
-        <v>3.5</v>
+        <v>1.4</v>
       </c>
       <c r="G1133" s="4" t="n">
-        <v>3.5</v>
+        <v>1.4</v>
       </c>
       <c r="H1133" s="2" t="n">
         <v>1575575</v>
@@ -53529,10 +53529,10 @@
         <v>1</v>
       </c>
       <c r="F1135" s="5" t="n">
-        <v>1.4</v>
+        <v>3.45</v>
       </c>
       <c r="G1135" s="4" t="n">
-        <v>1.4</v>
+        <v>3.45</v>
       </c>
       <c r="H1135" s="2" t="n">
         <v>1575575</v>
@@ -58229,10 +58229,10 @@
         <v>0.5</v>
       </c>
       <c r="F1235" s="5" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G1235" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H1235" s="2" t="n">
         <v>1589380</v>
@@ -58273,13 +58273,13 @@
         </is>
       </c>
       <c r="E1236" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F1236" s="5" t="n">
-        <v>14</v>
+        <v>120</v>
       </c>
       <c r="G1236" s="4" t="n">
-        <v>7</v>
+        <v>120</v>
       </c>
       <c r="H1236" s="2" t="n">
         <v>1589380</v>
@@ -58320,13 +58320,13 @@
         </is>
       </c>
       <c r="E1237" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F1237" s="5" t="n">
-        <v>120</v>
+        <v>18</v>
       </c>
       <c r="G1237" s="4" t="n">
-        <v>120</v>
+        <v>9</v>
       </c>
       <c r="H1237" s="2" t="n">
         <v>1589380</v>
@@ -58602,13 +58602,13 @@
         </is>
       </c>
       <c r="E1243" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F1243" s="5" t="n">
-        <v>1362.5</v>
+        <v>12</v>
       </c>
       <c r="G1243" s="4" t="n">
-        <v>1362.5</v>
+        <v>120</v>
       </c>
       <c r="H1243" s="2" t="n">
         <v>1589394</v>
@@ -58649,13 +58649,13 @@
         </is>
       </c>
       <c r="E1244" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F1244" s="5" t="n">
-        <v>12</v>
+        <v>252.5</v>
       </c>
       <c r="G1244" s="4" t="n">
-        <v>120</v>
+        <v>252.5</v>
       </c>
       <c r="H1244" s="2" t="n">
         <v>1589394</v>
@@ -58699,10 +58699,10 @@
         <v>1</v>
       </c>
       <c r="F1245" s="5" t="n">
-        <v>252.5</v>
+        <v>592.5</v>
       </c>
       <c r="G1245" s="4" t="n">
-        <v>252.5</v>
+        <v>592.5</v>
       </c>
       <c r="H1245" s="2" t="n">
         <v>1589394</v>
@@ -58746,10 +58746,10 @@
         <v>1</v>
       </c>
       <c r="F1246" s="5" t="n">
-        <v>592.5</v>
+        <v>507.5</v>
       </c>
       <c r="G1246" s="4" t="n">
-        <v>592.5</v>
+        <v>507.5</v>
       </c>
       <c r="H1246" s="2" t="n">
         <v>1589394</v>
@@ -58793,10 +58793,10 @@
         <v>1</v>
       </c>
       <c r="F1247" s="5" t="n">
-        <v>507.5</v>
+        <v>1362.5</v>
       </c>
       <c r="G1247" s="4" t="n">
-        <v>507.5</v>
+        <v>1362.5</v>
       </c>
       <c r="H1247" s="2" t="n">
         <v>1589394</v>
@@ -59354,13 +59354,13 @@
         </is>
       </c>
       <c r="E1259" s="4" t="n">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="F1259" s="5" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G1259" s="4" t="n">
-        <v>1.6</v>
+        <v>3.6</v>
       </c>
       <c r="H1259" s="2" t="n">
         <v>1591938</v>
@@ -59404,10 +59404,10 @@
         <v>0.04</v>
       </c>
       <c r="F1260" s="5" t="n">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="G1260" s="4" t="n">
-        <v>3.6</v>
+        <v>0.4</v>
       </c>
       <c r="H1260" s="2" t="n">
         <v>1591938</v>
@@ -59498,10 +59498,10 @@
         <v>0.02</v>
       </c>
       <c r="F1262" s="5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="G1262" s="4" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="H1262" s="2" t="n">
         <v>1591938</v>
@@ -59542,13 +59542,13 @@
         </is>
       </c>
       <c r="E1263" s="4" t="n">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="F1263" s="5" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="G1263" s="4" t="n">
-        <v>0.4</v>
+        <v>2</v>
       </c>
       <c r="H1263" s="2" t="n">
         <v>1591938</v>
@@ -59683,13 +59683,13 @@
         </is>
       </c>
       <c r="E1266" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F1266" s="5" t="n">
-        <v>2.66</v>
+        <v>1.29</v>
       </c>
       <c r="G1266" s="4" t="n">
-        <v>15.96</v>
+        <v>5.16</v>
       </c>
       <c r="H1266" s="2" t="n">
         <v>1591999</v>
@@ -59730,13 +59730,13 @@
         </is>
       </c>
       <c r="E1267" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F1267" s="5" t="n">
-        <v>1.29</v>
+        <v>13.17</v>
       </c>
       <c r="G1267" s="4" t="n">
-        <v>5.16</v>
+        <v>26.34</v>
       </c>
       <c r="H1267" s="2" t="n">
         <v>1591999</v>
@@ -59777,13 +59777,13 @@
         </is>
       </c>
       <c r="E1268" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F1268" s="5" t="n">
-        <v>13.17</v>
+        <v>2.66</v>
       </c>
       <c r="G1268" s="4" t="n">
-        <v>26.34</v>
+        <v>15.96</v>
       </c>
       <c r="H1268" s="2" t="n">
         <v>1591999</v>
@@ -59824,13 +59824,13 @@
         </is>
       </c>
       <c r="E1269" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1269" s="5" t="n">
-        <v>14.23</v>
+        <v>3.25</v>
       </c>
       <c r="G1269" s="4" t="n">
-        <v>14.23</v>
+        <v>6.5</v>
       </c>
       <c r="H1269" s="2" t="n">
         <v>1591999</v>
@@ -59871,13 +59871,13 @@
         </is>
       </c>
       <c r="E1270" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1270" s="5" t="n">
-        <v>3.25</v>
+        <v>215.83</v>
       </c>
       <c r="G1270" s="4" t="n">
-        <v>6.5</v>
+        <v>215.83</v>
       </c>
       <c r="H1270" s="2" t="n">
         <v>1591999</v>
@@ -59921,10 +59921,10 @@
         <v>1</v>
       </c>
       <c r="F1271" s="5" t="n">
-        <v>215.83</v>
+        <v>14.23</v>
       </c>
       <c r="G1271" s="4" t="n">
-        <v>215.83</v>
+        <v>14.23</v>
       </c>
       <c r="H1271" s="2" t="n">
         <v>1591999</v>
@@ -60435,13 +60435,13 @@
         </is>
       </c>
       <c r="E1282" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F1282" s="5" t="n">
-        <v>10.5</v>
+        <v>28.5</v>
       </c>
       <c r="G1282" s="4" t="n">
-        <v>10.5</v>
+        <v>57</v>
       </c>
       <c r="H1282" s="2" t="n">
         <v>1592652</v>
@@ -60482,13 +60482,13 @@
         </is>
       </c>
       <c r="E1283" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1283" s="5" t="n">
-        <v>28.5</v>
+        <v>10.5</v>
       </c>
       <c r="G1283" s="4" t="n">
-        <v>57</v>
+        <v>10.5</v>
       </c>
       <c r="H1283" s="2" t="n">
         <v>1592652</v>
@@ -61848,10 +61848,10 @@
         <v>1</v>
       </c>
       <c r="F1312" s="5" t="n">
-        <v>4.7</v>
+        <v>3.09</v>
       </c>
       <c r="G1312" s="4" t="n">
-        <v>4.7</v>
+        <v>3.09</v>
       </c>
       <c r="H1312" s="2" t="n">
         <v>1595677</v>
@@ -61895,10 +61895,10 @@
         <v>1</v>
       </c>
       <c r="F1313" s="5" t="n">
-        <v>3.09</v>
+        <v>1.62</v>
       </c>
       <c r="G1313" s="4" t="n">
-        <v>3.09</v>
+        <v>1.62</v>
       </c>
       <c r="H1313" s="2" t="n">
         <v>1595677</v>
@@ -61942,10 +61942,10 @@
         <v>1</v>
       </c>
       <c r="F1314" s="5" t="n">
-        <v>1.62</v>
+        <v>4.7</v>
       </c>
       <c r="G1314" s="4" t="n">
-        <v>1.62</v>
+        <v>4.7</v>
       </c>
       <c r="H1314" s="2" t="n">
         <v>1595677</v>
@@ -63349,13 +63349,13 @@
         </is>
       </c>
       <c r="E1344" s="4" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F1344" s="5" t="n">
-        <v>15</v>
+        <v>0.75</v>
       </c>
       <c r="G1344" s="4" t="n">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="H1344" s="2" t="n">
         <v>1600774</v>
@@ -63443,13 +63443,13 @@
         </is>
       </c>
       <c r="E1346" s="4" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F1346" s="5" t="n">
-        <v>0.75</v>
+        <v>16</v>
       </c>
       <c r="G1346" s="4" t="n">
-        <v>75</v>
+        <v>16</v>
       </c>
       <c r="H1346" s="2" t="n">
         <v>1600774</v>
@@ -63493,10 +63493,10 @@
         <v>1</v>
       </c>
       <c r="F1347" s="5" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G1347" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H1347" s="2" t="n">
         <v>1600774</v>
@@ -63537,10 +63537,10 @@
         </is>
       </c>
       <c r="E1348" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="F1348" s="5" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="G1348" s="4" t="n">
         <v>18</v>
@@ -63584,13 +63584,13 @@
         </is>
       </c>
       <c r="E1349" s="4" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="F1349" s="5" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="G1349" s="4" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="H1349" s="2" t="n">
         <v>1600774</v>
@@ -63631,13 +63631,13 @@
         </is>
       </c>
       <c r="E1350" s="4" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="F1350" s="5" t="n">
-        <v>25</v>
+        <v>80</v>
       </c>
       <c r="G1350" s="4" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="H1350" s="2" t="n">
         <v>1600774</v>
@@ -63678,13 +63678,13 @@
         </is>
       </c>
       <c r="E1351" s="4" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="F1351" s="5" t="n">
-        <v>80</v>
+        <v>15</v>
       </c>
       <c r="G1351" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H1351" s="2" t="n">
         <v>1600774</v>
@@ -65934,13 +65934,13 @@
         </is>
       </c>
       <c r="E1399" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1399" s="5" t="n">
-        <v>153.3</v>
+        <v>127.6</v>
       </c>
       <c r="G1399" s="4" t="n">
-        <v>613.2</v>
+        <v>765.6</v>
       </c>
       <c r="H1399" s="2" t="n">
         <v>1603907</v>
@@ -66075,13 +66075,13 @@
         </is>
       </c>
       <c r="E1402" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F1402" s="5" t="n">
-        <v>127.6</v>
+        <v>153.3</v>
       </c>
       <c r="G1402" s="4" t="n">
-        <v>765.6</v>
+        <v>613.2</v>
       </c>
       <c r="H1402" s="2" t="n">
         <v>1603907</v>
@@ -76932,13 +76932,13 @@
         </is>
       </c>
       <c r="E1633" s="4" t="n">
-        <v>0.26</v>
+        <v>1.5</v>
       </c>
       <c r="F1633" s="5" t="n">
-        <v>350</v>
+        <v>15</v>
       </c>
       <c r="G1633" s="4" t="n">
-        <v>91</v>
+        <v>22.5</v>
       </c>
       <c r="H1633" s="2" t="n">
         <v>1619290</v>
@@ -76982,10 +76982,10 @@
         <v>1.5</v>
       </c>
       <c r="F1634" s="5" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="G1634" s="4" t="n">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="H1634" s="2" t="n">
         <v>1619290</v>
@@ -77026,13 +77026,13 @@
         </is>
       </c>
       <c r="E1635" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F1635" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G1635" s="4" t="n">
-        <v>22.5</v>
+        <v>16</v>
       </c>
       <c r="H1635" s="2" t="n">
         <v>1619290</v>
@@ -77073,13 +77073,13 @@
         </is>
       </c>
       <c r="E1636" s="4" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="F1636" s="5" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="G1636" s="4" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="H1636" s="2" t="n">
         <v>1619290</v>
@@ -77123,10 +77123,10 @@
         <v>1</v>
       </c>
       <c r="F1637" s="5" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="G1637" s="4" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="H1637" s="2" t="n">
         <v>1619290</v>
@@ -77167,13 +77167,13 @@
         </is>
       </c>
       <c r="E1638" s="4" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="F1638" s="5" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G1638" s="4" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="H1638" s="2" t="n">
         <v>1619290</v>
@@ -77214,13 +77214,13 @@
         </is>
       </c>
       <c r="E1639" s="4" t="n">
-        <v>1</v>
+        <v>0.26</v>
       </c>
       <c r="F1639" s="5" t="n">
-        <v>16</v>
+        <v>350</v>
       </c>
       <c r="G1639" s="4" t="n">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="H1639" s="2" t="n">
         <v>1619290</v>
@@ -77261,13 +77261,13 @@
         </is>
       </c>
       <c r="E1640" s="4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F1640" s="5" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G1640" s="4" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="H1640" s="2" t="n">
         <v>1619290</v>
@@ -77308,13 +77308,13 @@
         </is>
       </c>
       <c r="E1641" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F1641" s="5" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G1641" s="4" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H1641" s="2" t="n">
         <v>1619290</v>
@@ -80131,10 +80131,10 @@
         <v>100</v>
       </c>
       <c r="F1701" s="5" t="n">
-        <v>0.22</v>
+        <v>0.15</v>
       </c>
       <c r="G1701" s="4" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H1701" s="2" t="n">
         <v>1630277</v>
@@ -80178,10 +80178,10 @@
         <v>100</v>
       </c>
       <c r="F1702" s="5" t="n">
-        <v>0.15</v>
+        <v>0.22</v>
       </c>
       <c r="G1702" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H1702" s="2" t="n">
         <v>1630277</v>
@@ -81021,13 +81021,13 @@
         </is>
       </c>
       <c r="E1720" s="4" t="n">
-        <v>1</v>
+        <v>0.04</v>
       </c>
       <c r="F1720" s="5" t="n">
-        <v>22</v>
+        <v>140</v>
       </c>
       <c r="G1720" s="4" t="n">
-        <v>22</v>
+        <v>5.6</v>
       </c>
       <c r="H1720" s="2" t="n">
         <v>1632122</v>
@@ -81068,13 +81068,13 @@
         </is>
       </c>
       <c r="E1721" s="4" t="n">
-        <v>1</v>
+        <v>0.04</v>
       </c>
       <c r="F1721" s="5" t="n">
-        <v>16</v>
+        <v>110</v>
       </c>
       <c r="G1721" s="4" t="n">
-        <v>16</v>
+        <v>4.4</v>
       </c>
       <c r="H1721" s="2" t="n">
         <v>1632122</v>
@@ -81115,13 +81115,13 @@
         </is>
       </c>
       <c r="E1722" s="4" t="n">
-        <v>2</v>
+        <v>0.1</v>
       </c>
       <c r="F1722" s="5" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="G1722" s="4" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="H1722" s="2" t="n">
         <v>1632122</v>
@@ -81162,13 +81162,13 @@
         </is>
       </c>
       <c r="E1723" s="4" t="n">
-        <v>4</v>
+        <v>0.08</v>
       </c>
       <c r="F1723" s="5" t="n">
-        <v>15</v>
+        <v>500</v>
       </c>
       <c r="G1723" s="4" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="H1723" s="2" t="n">
         <v>1632122</v>
@@ -81209,13 +81209,13 @@
         </is>
       </c>
       <c r="E1724" s="4" t="n">
-        <v>0.08</v>
+        <v>4</v>
       </c>
       <c r="F1724" s="5" t="n">
-        <v>500</v>
+        <v>15</v>
       </c>
       <c r="G1724" s="4" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="H1724" s="2" t="n">
         <v>1632122</v>
@@ -81256,13 +81256,13 @@
         </is>
       </c>
       <c r="E1725" s="4" t="n">
-        <v>0.1</v>
+        <v>2</v>
       </c>
       <c r="F1725" s="5" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="G1725" s="4" t="n">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="H1725" s="2" t="n">
         <v>1632122</v>
@@ -81303,13 +81303,13 @@
         </is>
       </c>
       <c r="E1726" s="4" t="n">
-        <v>0.04</v>
+        <v>1</v>
       </c>
       <c r="F1726" s="5" t="n">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="G1726" s="4" t="n">
-        <v>4.4</v>
+        <v>16</v>
       </c>
       <c r="H1726" s="2" t="n">
         <v>1632122</v>
@@ -81350,13 +81350,13 @@
         </is>
       </c>
       <c r="E1727" s="4" t="n">
-        <v>0.04</v>
+        <v>1</v>
       </c>
       <c r="F1727" s="5" t="n">
-        <v>140</v>
+        <v>22</v>
       </c>
       <c r="G1727" s="4" t="n">
-        <v>5.6</v>
+        <v>22</v>
       </c>
       <c r="H1727" s="2" t="n">
         <v>1632122</v>
@@ -82525,13 +82525,13 @@
         </is>
       </c>
       <c r="E1752" s="4" t="n">
-        <v>100</v>
+        <v>2000</v>
       </c>
       <c r="F1752" s="5" t="n">
-        <v>20.5</v>
+        <v>1.5725</v>
       </c>
       <c r="G1752" s="4" t="n">
-        <v>2050</v>
+        <v>3145</v>
       </c>
       <c r="H1752" s="2" t="n">
         <v>1639555</v>
@@ -82572,13 +82572,13 @@
         </is>
       </c>
       <c r="E1753" s="4" t="n">
-        <v>2000</v>
+        <v>300</v>
       </c>
       <c r="F1753" s="5" t="n">
-        <v>1.5725</v>
+        <v>0.8333</v>
       </c>
       <c r="G1753" s="4" t="n">
-        <v>3145</v>
+        <v>250</v>
       </c>
       <c r="H1753" s="2" t="n">
         <v>1639555</v>
@@ -82619,13 +82619,13 @@
         </is>
       </c>
       <c r="E1754" s="4" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F1754" s="5" t="n">
-        <v>0.8333</v>
+        <v>20.5</v>
       </c>
       <c r="G1754" s="4" t="n">
-        <v>250</v>
+        <v>2050</v>
       </c>
       <c r="H1754" s="2" t="n">
         <v>1639555</v>
@@ -82810,10 +82810,10 @@
         <v>1</v>
       </c>
       <c r="F1758" s="5" t="n">
-        <v>12.11</v>
+        <v>10.93</v>
       </c>
       <c r="G1758" s="4" t="n">
-        <v>12.11</v>
+        <v>10.93</v>
       </c>
       <c r="H1758" s="2" t="n">
         <v>1639631</v>
@@ -82857,10 +82857,10 @@
         <v>1</v>
       </c>
       <c r="F1759" s="5" t="n">
-        <v>10.93</v>
+        <v>12.11</v>
       </c>
       <c r="G1759" s="4" t="n">
-        <v>10.93</v>
+        <v>12.11</v>
       </c>
       <c r="H1759" s="2" t="n">
         <v>1639631</v>
@@ -83089,13 +83089,13 @@
         </is>
       </c>
       <c r="E1764" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F1764" s="5" t="n">
         <v>5</v>
       </c>
       <c r="G1764" s="4" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H1764" s="2" t="n">
         <v>1639777</v>
@@ -83183,13 +83183,13 @@
         </is>
       </c>
       <c r="E1766" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F1766" s="5" t="n">
         <v>5</v>
       </c>
       <c r="G1766" s="4" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H1766" s="2" t="n">
         <v>1639777</v>
@@ -83254,6 +83254,100 @@
         <v>1695</v>
       </c>
       <c r="K1767" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1768" customHeight="1" ht="15">
+      <c r="A1768" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1768" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1768" s="2" t="n">
+        <v>26653</v>
+      </c>
+      <c r="D1768" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_LIMP</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1768" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1768" s="5" t="n">
+        <v>9.9983</v>
+      </c>
+      <c r="G1768" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="H1768" s="2" t="n">
+        <v>1641552</v>
+      </c>
+      <c r="I1768" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">19/10/2026 15:40:01</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1768" s="2" t="n">
+        <v>43442</v>
+      </c>
+      <c r="K1768" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1769" customHeight="1" ht="15">
+      <c r="A1769" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1769" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1769" s="2" t="n">
+        <v>15039</v>
+      </c>
+      <c r="D1769" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_USE</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1769" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1769" s="5" t="n">
+        <v>41.99</v>
+      </c>
+      <c r="G1769" s="4" t="n">
+        <v>41.99</v>
+      </c>
+      <c r="H1769" s="2" t="n">
+        <v>1641567</v>
+      </c>
+      <c r="I1769" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">19/10/2026 16:20:50</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1769" s="2" t="n">
+        <v>43306</v>
+      </c>
+      <c r="K1769" s="2" t="n">
         <v>165</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Relatório de compras 21/10/2026 22:01
</commit_message>
<xml_diff>
--- a/data/relatorio.xlsx
+++ b/data/relatorio.xlsx
@@ -26927,10 +26927,10 @@
         <v>1</v>
       </c>
       <c r="F569" s="5" t="n">
-        <v>6.08</v>
+        <v>113.57</v>
       </c>
       <c r="G569" s="4" t="n">
-        <v>6.08</v>
+        <v>113.57</v>
       </c>
       <c r="H569" s="2" t="n">
         <v>1482331</v>
@@ -26974,10 +26974,10 @@
         <v>1</v>
       </c>
       <c r="F570" s="5" t="n">
-        <v>55.88</v>
+        <v>6.08</v>
       </c>
       <c r="G570" s="4" t="n">
-        <v>55.88</v>
+        <v>6.08</v>
       </c>
       <c r="H570" s="2" t="n">
         <v>1482331</v>
@@ -27021,10 +27021,10 @@
         <v>1</v>
       </c>
       <c r="F571" s="5" t="n">
-        <v>5.74</v>
+        <v>8.23</v>
       </c>
       <c r="G571" s="4" t="n">
-        <v>5.74</v>
+        <v>8.23</v>
       </c>
       <c r="H571" s="2" t="n">
         <v>1482331</v>
@@ -27068,10 +27068,10 @@
         <v>1</v>
       </c>
       <c r="F572" s="5" t="n">
-        <v>5.83</v>
+        <v>5.74</v>
       </c>
       <c r="G572" s="4" t="n">
-        <v>5.83</v>
+        <v>5.74</v>
       </c>
       <c r="H572" s="2" t="n">
         <v>1482331</v>
@@ -27115,10 +27115,10 @@
         <v>1</v>
       </c>
       <c r="F573" s="5" t="n">
-        <v>31.33</v>
+        <v>5.83</v>
       </c>
       <c r="G573" s="4" t="n">
-        <v>31.33</v>
+        <v>5.83</v>
       </c>
       <c r="H573" s="2" t="n">
         <v>1482331</v>
@@ -27162,10 +27162,10 @@
         <v>1</v>
       </c>
       <c r="F574" s="5" t="n">
-        <v>6.16</v>
+        <v>31.33</v>
       </c>
       <c r="G574" s="4" t="n">
-        <v>6.16</v>
+        <v>31.33</v>
       </c>
       <c r="H574" s="2" t="n">
         <v>1482331</v>
@@ -27209,10 +27209,10 @@
         <v>1</v>
       </c>
       <c r="F575" s="5" t="n">
-        <v>113.57</v>
+        <v>6.16</v>
       </c>
       <c r="G575" s="4" t="n">
-        <v>113.57</v>
+        <v>6.16</v>
       </c>
       <c r="H575" s="2" t="n">
         <v>1482331</v>
@@ -27256,10 +27256,10 @@
         <v>1</v>
       </c>
       <c r="F576" s="5" t="n">
-        <v>8.23</v>
+        <v>117.18</v>
       </c>
       <c r="G576" s="4" t="n">
-        <v>8.23</v>
+        <v>117.18</v>
       </c>
       <c r="H576" s="2" t="n">
         <v>1482331</v>
@@ -27303,10 +27303,10 @@
         <v>1</v>
       </c>
       <c r="F577" s="5" t="n">
-        <v>117.18</v>
+        <v>55.88</v>
       </c>
       <c r="G577" s="4" t="n">
-        <v>117.18</v>
+        <v>55.88</v>
       </c>
       <c r="H577" s="2" t="n">
         <v>1482331</v>
@@ -27441,13 +27441,13 @@
         </is>
       </c>
       <c r="E580" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F580" s="5" t="n">
         <v>2.6</v>
       </c>
       <c r="G580" s="4" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="H580" s="2" t="n">
         <v>1482337</v>
@@ -27488,13 +27488,13 @@
         </is>
       </c>
       <c r="E581" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F581" s="5" t="n">
-        <v>9</v>
+        <v>2.6</v>
       </c>
       <c r="G581" s="4" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H581" s="2" t="n">
         <v>1482337</v>
@@ -27538,10 +27538,10 @@
         <v>1</v>
       </c>
       <c r="F582" s="5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G582" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H582" s="2" t="n">
         <v>1482337</v>
@@ -27582,13 +27582,13 @@
         </is>
       </c>
       <c r="E583" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F583" s="5" t="n">
-        <v>2.6</v>
+        <v>7</v>
       </c>
       <c r="G583" s="4" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="H583" s="2" t="n">
         <v>1482337</v>
@@ -28619,10 +28619,10 @@
         <v>1</v>
       </c>
       <c r="F605" s="5" t="n">
-        <v>30</v>
+        <v>195</v>
       </c>
       <c r="G605" s="4" t="n">
-        <v>30</v>
+        <v>195</v>
       </c>
       <c r="H605" s="2" t="n">
         <v>1490619</v>
@@ -28666,10 +28666,10 @@
         <v>1</v>
       </c>
       <c r="F606" s="5" t="n">
-        <v>165</v>
+        <v>230</v>
       </c>
       <c r="G606" s="4" t="n">
-        <v>165</v>
+        <v>230</v>
       </c>
       <c r="H606" s="2" t="n">
         <v>1490619</v>
@@ -28713,10 +28713,10 @@
         <v>1</v>
       </c>
       <c r="F607" s="5" t="n">
-        <v>195</v>
+        <v>165</v>
       </c>
       <c r="G607" s="4" t="n">
-        <v>195</v>
+        <v>165</v>
       </c>
       <c r="H607" s="2" t="n">
         <v>1490619</v>
@@ -28760,10 +28760,10 @@
         <v>1</v>
       </c>
       <c r="F608" s="5" t="n">
-        <v>230</v>
+        <v>30</v>
       </c>
       <c r="G608" s="4" t="n">
-        <v>230</v>
+        <v>30</v>
       </c>
       <c r="H608" s="2" t="n">
         <v>1490619</v>
@@ -28851,13 +28851,13 @@
         </is>
       </c>
       <c r="E610" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F610" s="5" t="n">
-        <v>41.71</v>
+        <v>6.6</v>
       </c>
       <c r="G610" s="4" t="n">
-        <v>83.42</v>
+        <v>19.8</v>
       </c>
       <c r="H610" s="2" t="n">
         <v>1490652</v>
@@ -28898,13 +28898,13 @@
         </is>
       </c>
       <c r="E611" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F611" s="5" t="n">
-        <v>49.9</v>
+        <v>55.99</v>
       </c>
       <c r="G611" s="4" t="n">
-        <v>49.9</v>
+        <v>167.97</v>
       </c>
       <c r="H611" s="2" t="n">
         <v>1490652</v>
@@ -28992,13 +28992,13 @@
         </is>
       </c>
       <c r="E613" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F613" s="5" t="n">
-        <v>55.99</v>
+        <v>0.86</v>
       </c>
       <c r="G613" s="4" t="n">
-        <v>167.97</v>
+        <v>8.6</v>
       </c>
       <c r="H613" s="2" t="n">
         <v>1490652</v>
@@ -29039,13 +29039,13 @@
         </is>
       </c>
       <c r="E614" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F614" s="5" t="n">
-        <v>6.6</v>
+        <v>17.52</v>
       </c>
       <c r="G614" s="4" t="n">
-        <v>19.8</v>
+        <v>70.08</v>
       </c>
       <c r="H614" s="2" t="n">
         <v>1490652</v>
@@ -29086,13 +29086,13 @@
         </is>
       </c>
       <c r="E615" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F615" s="5" t="n">
-        <v>17.52</v>
+        <v>41.71</v>
       </c>
       <c r="G615" s="4" t="n">
-        <v>70.08</v>
+        <v>83.42</v>
       </c>
       <c r="H615" s="2" t="n">
         <v>1490652</v>
@@ -29133,13 +29133,13 @@
         </is>
       </c>
       <c r="E616" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F616" s="5" t="n">
-        <v>0.86</v>
+        <v>49.9</v>
       </c>
       <c r="G616" s="4" t="n">
-        <v>8.6</v>
+        <v>49.9</v>
       </c>
       <c r="H616" s="2" t="n">
         <v>1490652</v>
@@ -29415,13 +29415,13 @@
         </is>
       </c>
       <c r="E622" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F622" s="5" t="n">
-        <v>19.03</v>
+        <v>5.28</v>
       </c>
       <c r="G622" s="4" t="n">
-        <v>76.12</v>
+        <v>10.56</v>
       </c>
       <c r="H622" s="2" t="n">
         <v>1492428</v>
@@ -29462,13 +29462,13 @@
         </is>
       </c>
       <c r="E623" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F623" s="5" t="n">
-        <v>26.31</v>
+        <v>19.03</v>
       </c>
       <c r="G623" s="4" t="n">
-        <v>52.62</v>
+        <v>76.12</v>
       </c>
       <c r="H623" s="2" t="n">
         <v>1492428</v>
@@ -29512,10 +29512,10 @@
         <v>2</v>
       </c>
       <c r="F624" s="5" t="n">
-        <v>5.28</v>
+        <v>26.31</v>
       </c>
       <c r="G624" s="4" t="n">
-        <v>10.56</v>
+        <v>52.62</v>
       </c>
       <c r="H624" s="2" t="n">
         <v>1492428</v>
@@ -29556,13 +29556,13 @@
         </is>
       </c>
       <c r="E625" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F625" s="5" t="n">
-        <v>5.62</v>
+        <v>4.18</v>
       </c>
       <c r="G625" s="4" t="n">
-        <v>11.24</v>
+        <v>50.16</v>
       </c>
       <c r="H625" s="2" t="n">
         <v>1492428</v>
@@ -29603,13 +29603,13 @@
         </is>
       </c>
       <c r="E626" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F626" s="5" t="n">
-        <v>4.18</v>
+        <v>5.62</v>
       </c>
       <c r="G626" s="4" t="n">
-        <v>50.16</v>
+        <v>11.24</v>
       </c>
       <c r="H626" s="2" t="n">
         <v>1492428</v>
@@ -29885,13 +29885,13 @@
         </is>
       </c>
       <c r="E632" s="4" t="n">
-        <v>0.1</v>
+        <v>2</v>
       </c>
       <c r="F632" s="5" t="n">
-        <v>75</v>
+        <v>22</v>
       </c>
       <c r="G632" s="4" t="n">
-        <v>7.5</v>
+        <v>44</v>
       </c>
       <c r="H632" s="2" t="n">
         <v>1493814</v>
@@ -29932,13 +29932,13 @@
         </is>
       </c>
       <c r="E633" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F633" s="5" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="G633" s="4" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="H633" s="2" t="n">
         <v>1493814</v>
@@ -29979,13 +29979,13 @@
         </is>
       </c>
       <c r="E634" s="4" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="F634" s="5" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="G634" s="4" t="n">
-        <v>40</v>
+        <v>7.5</v>
       </c>
       <c r="H634" s="2" t="n">
         <v>1493814</v>
@@ -30308,13 +30308,13 @@
         </is>
       </c>
       <c r="E641" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F641" s="5" t="n">
-        <v>178.5</v>
+        <v>23.95</v>
       </c>
       <c r="G641" s="4" t="n">
-        <v>357</v>
+        <v>23.95</v>
       </c>
       <c r="H641" s="2" t="n">
         <v>1497640</v>
@@ -30496,13 +30496,13 @@
         </is>
       </c>
       <c r="E645" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F645" s="5" t="n">
-        <v>23.95</v>
+        <v>178.5</v>
       </c>
       <c r="G645" s="4" t="n">
-        <v>23.95</v>
+        <v>357</v>
       </c>
       <c r="H645" s="2" t="n">
         <v>1497640</v>
@@ -30734,10 +30734,10 @@
         <v>200</v>
       </c>
       <c r="F650" s="5" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="G650" s="4" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="H650" s="2" t="n">
         <v>1498122</v>
@@ -30781,10 +30781,10 @@
         <v>200</v>
       </c>
       <c r="F651" s="5" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="G651" s="4" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="H651" s="2" t="n">
         <v>1498122</v>
@@ -31016,10 +31016,10 @@
         <v>1</v>
       </c>
       <c r="F656" s="5" t="n">
-        <v>14.08</v>
+        <v>38.06</v>
       </c>
       <c r="G656" s="4" t="n">
-        <v>14.08</v>
+        <v>38.06</v>
       </c>
       <c r="H656" s="2" t="n">
         <v>1499773</v>
@@ -31063,10 +31063,10 @@
         <v>1</v>
       </c>
       <c r="F657" s="5" t="n">
-        <v>38.06</v>
+        <v>14.08</v>
       </c>
       <c r="G657" s="4" t="n">
-        <v>38.06</v>
+        <v>14.08</v>
       </c>
       <c r="H657" s="2" t="n">
         <v>1499773</v>
@@ -31721,10 +31721,10 @@
         <v>2</v>
       </c>
       <c r="F671" s="5" t="n">
-        <v>30</v>
+        <v>2.03</v>
       </c>
       <c r="G671" s="4" t="n">
-        <v>60</v>
+        <v>4.06</v>
       </c>
       <c r="H671" s="2" t="n">
         <v>1503029</v>
@@ -31768,10 +31768,10 @@
         <v>2</v>
       </c>
       <c r="F672" s="5" t="n">
-        <v>1.01</v>
+        <v>30</v>
       </c>
       <c r="G672" s="4" t="n">
-        <v>2.02</v>
+        <v>60</v>
       </c>
       <c r="H672" s="2" t="n">
         <v>1503029</v>
@@ -31859,13 +31859,13 @@
         </is>
       </c>
       <c r="E674" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F674" s="5" t="n">
-        <v>5.39</v>
+        <v>1.01</v>
       </c>
       <c r="G674" s="4" t="n">
-        <v>5.39</v>
+        <v>2.02</v>
       </c>
       <c r="H674" s="2" t="n">
         <v>1503029</v>
@@ -31906,13 +31906,13 @@
         </is>
       </c>
       <c r="E675" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F675" s="5" t="n">
-        <v>2.03</v>
+        <v>5.39</v>
       </c>
       <c r="G675" s="4" t="n">
-        <v>4.06</v>
+        <v>5.39</v>
       </c>
       <c r="H675" s="2" t="n">
         <v>1503029</v>
@@ -33319,10 +33319,10 @@
         <v>2</v>
       </c>
       <c r="F705" s="5" t="n">
-        <v>2.38</v>
+        <v>2.29</v>
       </c>
       <c r="G705" s="4" t="n">
-        <v>4.76</v>
+        <v>4.58</v>
       </c>
       <c r="H705" s="2" t="n">
         <v>1512391</v>
@@ -33363,13 +33363,13 @@
         </is>
       </c>
       <c r="E706" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F706" s="5" t="n">
-        <v>15.25</v>
+        <v>2.38</v>
       </c>
       <c r="G706" s="4" t="n">
-        <v>15.25</v>
+        <v>4.76</v>
       </c>
       <c r="H706" s="2" t="n">
         <v>1512391</v>
@@ -33413,10 +33413,10 @@
         <v>1</v>
       </c>
       <c r="F707" s="5" t="n">
-        <v>10.3</v>
+        <v>15.25</v>
       </c>
       <c r="G707" s="4" t="n">
-        <v>10.3</v>
+        <v>15.25</v>
       </c>
       <c r="H707" s="2" t="n">
         <v>1512391</v>
@@ -33460,10 +33460,10 @@
         <v>1</v>
       </c>
       <c r="F708" s="5" t="n">
-        <v>12.25</v>
+        <v>10.3</v>
       </c>
       <c r="G708" s="4" t="n">
-        <v>12.25</v>
+        <v>10.3</v>
       </c>
       <c r="H708" s="2" t="n">
         <v>1512391</v>
@@ -33504,13 +33504,13 @@
         </is>
       </c>
       <c r="E709" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F709" s="5" t="n">
-        <v>2.29</v>
+        <v>12.25</v>
       </c>
       <c r="G709" s="4" t="n">
-        <v>4.58</v>
+        <v>12.25</v>
       </c>
       <c r="H709" s="2" t="n">
         <v>1512391</v>
@@ -33598,13 +33598,13 @@
         </is>
       </c>
       <c r="E711" s="4" t="n">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="F711" s="5" t="n">
-        <v>0.8</v>
+        <v>0.22</v>
       </c>
       <c r="G711" s="4" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="H711" s="2" t="n">
         <v>1512750</v>
@@ -33645,13 +33645,13 @@
         </is>
       </c>
       <c r="E712" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="F712" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G712" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="F712" s="5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G712" s="4" t="n">
-        <v>4.5</v>
       </c>
       <c r="H712" s="2" t="n">
         <v>1512750</v>
@@ -33692,13 +33692,13 @@
         </is>
       </c>
       <c r="E713" s="4" t="n">
-        <v>15</v>
+        <v>300</v>
       </c>
       <c r="F713" s="5" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="G713" s="4" t="n">
-        <v>2.55</v>
+        <v>45</v>
       </c>
       <c r="H713" s="2" t="n">
         <v>1512750</v>
@@ -33739,13 +33739,13 @@
         </is>
       </c>
       <c r="E714" s="4" t="n">
-        <v>300</v>
+        <v>15</v>
       </c>
       <c r="F714" s="5" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="G714" s="4" t="n">
-        <v>45</v>
+        <v>2.55</v>
       </c>
       <c r="H714" s="2" t="n">
         <v>1512750</v>
@@ -33786,13 +33786,13 @@
         </is>
       </c>
       <c r="E715" s="4" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="F715" s="5" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="G715" s="4" t="n">
-        <v>15</v>
+        <v>4.5</v>
       </c>
       <c r="H715" s="2" t="n">
         <v>1512750</v>
@@ -33833,13 +33833,13 @@
         </is>
       </c>
       <c r="E716" s="4" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="F716" s="5" t="n">
-        <v>0.22</v>
+        <v>0.8</v>
       </c>
       <c r="G716" s="4" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="H716" s="2" t="n">
         <v>1512750</v>
@@ -33977,10 +33977,10 @@
         <v>1</v>
       </c>
       <c r="F719" s="5" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G719" s="4" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H719" s="2" t="n">
         <v>1513521</v>
@@ -34021,13 +34021,13 @@
         </is>
       </c>
       <c r="E720" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F720" s="5" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G720" s="4" t="n">
-        <v>170</v>
+        <v>25</v>
       </c>
       <c r="H720" s="2" t="n">
         <v>1513521</v>
@@ -34068,13 +34068,13 @@
         </is>
       </c>
       <c r="E721" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F721" s="5" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="G721" s="4" t="n">
-        <v>35</v>
+        <v>170</v>
       </c>
       <c r="H721" s="2" t="n">
         <v>1513521</v>
@@ -34165,10 +34165,10 @@
         <v>1</v>
       </c>
       <c r="F723" s="5" t="n">
-        <v>192.5</v>
+        <v>197.5</v>
       </c>
       <c r="G723" s="4" t="n">
-        <v>192.5</v>
+        <v>197.5</v>
       </c>
       <c r="H723" s="2" t="n">
         <v>1513541</v>
@@ -34212,10 +34212,10 @@
         <v>1</v>
       </c>
       <c r="F724" s="5" t="n">
-        <v>197.5</v>
+        <v>192.5</v>
       </c>
       <c r="G724" s="4" t="n">
-        <v>197.5</v>
+        <v>192.5</v>
       </c>
       <c r="H724" s="2" t="n">
         <v>1513541</v>
@@ -34491,13 +34491,13 @@
         </is>
       </c>
       <c r="E730" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F730" s="5" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="G730" s="4" t="n">
-        <v>1000</v>
+        <v>750</v>
       </c>
       <c r="H730" s="2" t="n">
         <v>1513779</v>
@@ -34585,13 +34585,13 @@
         </is>
       </c>
       <c r="E732" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F732" s="5" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G732" s="4" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="H732" s="2" t="n">
         <v>1513779</v>
@@ -35246,10 +35246,10 @@
         <v>1</v>
       </c>
       <c r="F746" s="5" t="n">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="G746" s="4" t="n">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="H746" s="2" t="n">
         <v>1516916</v>
@@ -35293,10 +35293,10 @@
         <v>1</v>
       </c>
       <c r="F747" s="5" t="n">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="G747" s="4" t="n">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="H747" s="2" t="n">
         <v>1516916</v>
@@ -35575,10 +35575,10 @@
         <v>0.04</v>
       </c>
       <c r="F753" s="5" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="G753" s="4" t="n">
-        <v>1.4</v>
+        <v>0.2</v>
       </c>
       <c r="H753" s="2" t="n">
         <v>1517956</v>
@@ -35619,13 +35619,13 @@
         </is>
       </c>
       <c r="E754" s="4" t="n">
-        <v>0.04</v>
+        <v>4</v>
       </c>
       <c r="F754" s="5" t="n">
-        <v>25</v>
+        <v>95</v>
       </c>
       <c r="G754" s="4" t="n">
-        <v>1</v>
+        <v>380</v>
       </c>
       <c r="H754" s="2" t="n">
         <v>1517956</v>
@@ -35669,10 +35669,10 @@
         <v>0.04</v>
       </c>
       <c r="F755" s="5" t="n">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="G755" s="4" t="n">
-        <v>0.2</v>
+        <v>1.4</v>
       </c>
       <c r="H755" s="2" t="n">
         <v>1517956</v>
@@ -35760,13 +35760,13 @@
         </is>
       </c>
       <c r="E757" s="4" t="n">
-        <v>4</v>
+        <v>0.04</v>
       </c>
       <c r="F757" s="5" t="n">
-        <v>95</v>
+        <v>25</v>
       </c>
       <c r="G757" s="4" t="n">
-        <v>380</v>
+        <v>1</v>
       </c>
       <c r="H757" s="2" t="n">
         <v>1517956</v>
@@ -36280,10 +36280,10 @@
         <v>1</v>
       </c>
       <c r="F768" s="5" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G768" s="4" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H768" s="2" t="n">
         <v>1518833</v>
@@ -36421,10 +36421,10 @@
         <v>1</v>
       </c>
       <c r="F771" s="5" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G771" s="4" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H771" s="2" t="n">
         <v>1518833</v>
@@ -36559,13 +36559,13 @@
         </is>
       </c>
       <c r="E774" s="4" t="n">
-        <v>2</v>
+        <v>0.08</v>
       </c>
       <c r="F774" s="5" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="G774" s="4" t="n">
-        <v>22</v>
+        <v>1.6</v>
       </c>
       <c r="H774" s="2" t="n">
         <v>1520281</v>
@@ -36606,13 +36606,13 @@
         </is>
       </c>
       <c r="E775" s="4" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="F775" s="5" t="n">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="G775" s="4" t="n">
-        <v>87</v>
+        <v>22</v>
       </c>
       <c r="H775" s="2" t="n">
         <v>1520281</v>
@@ -36653,13 +36653,13 @@
         </is>
       </c>
       <c r="E776" s="4" t="n">
-        <v>0.08</v>
+        <v>1.5</v>
       </c>
       <c r="F776" s="5" t="n">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="G776" s="4" t="n">
-        <v>1.6</v>
+        <v>87</v>
       </c>
       <c r="H776" s="2" t="n">
         <v>1520281</v>
@@ -37076,13 +37076,13 @@
         </is>
       </c>
       <c r="E785" s="4" t="n">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="F785" s="5" t="n">
-        <v>127.6</v>
+        <v>9.1</v>
       </c>
       <c r="G785" s="4" t="n">
-        <v>4593.6</v>
+        <v>127.4</v>
       </c>
       <c r="H785" s="2" t="n">
         <v>1522616</v>
@@ -37123,13 +37123,13 @@
         </is>
       </c>
       <c r="E786" s="4" t="n">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F786" s="5" t="n">
-        <v>9.1</v>
+        <v>54.3</v>
       </c>
       <c r="G786" s="4" t="n">
-        <v>127.4</v>
+        <v>2009.1</v>
       </c>
       <c r="H786" s="2" t="n">
         <v>1522616</v>
@@ -37170,13 +37170,13 @@
         </is>
       </c>
       <c r="E787" s="4" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F787" s="5" t="n">
-        <v>54.3</v>
+        <v>127.6</v>
       </c>
       <c r="G787" s="4" t="n">
-        <v>2009.1</v>
+        <v>4593.6</v>
       </c>
       <c r="H787" s="2" t="n">
         <v>1522616</v>
@@ -37217,13 +37217,13 @@
         </is>
       </c>
       <c r="E788" s="4" t="n">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="F788" s="5" t="n">
-        <v>54.3</v>
+        <v>127.6</v>
       </c>
       <c r="G788" s="4" t="n">
-        <v>3746.7</v>
+        <v>1786.4</v>
       </c>
       <c r="H788" s="2" t="n">
         <v>1522616</v>
@@ -37264,13 +37264,13 @@
         </is>
       </c>
       <c r="E789" s="4" t="n">
-        <v>2</v>
+        <v>69</v>
       </c>
       <c r="F789" s="5" t="n">
-        <v>139.6</v>
+        <v>54.3</v>
       </c>
       <c r="G789" s="4" t="n">
-        <v>279.2</v>
+        <v>3746.7</v>
       </c>
       <c r="H789" s="2" t="n">
         <v>1522616</v>
@@ -37311,13 +37311,13 @@
         </is>
       </c>
       <c r="E790" s="4" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="F790" s="5" t="n">
-        <v>127.6</v>
+        <v>139.6</v>
       </c>
       <c r="G790" s="4" t="n">
-        <v>1786.4</v>
+        <v>279.2</v>
       </c>
       <c r="H790" s="2" t="n">
         <v>1522616</v>
@@ -37922,13 +37922,13 @@
         </is>
       </c>
       <c r="E803" s="4" t="n">
-        <v>1.28</v>
+        <v>1</v>
       </c>
       <c r="F803" s="5" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G803" s="4" t="n">
-        <v>48.64</v>
+        <v>36</v>
       </c>
       <c r="H803" s="2" t="n">
         <v>1524925</v>
@@ -37969,13 +37969,13 @@
         </is>
       </c>
       <c r="E804" s="4" t="n">
-        <v>1</v>
+        <v>0.08</v>
       </c>
       <c r="F804" s="5" t="n">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="G804" s="4" t="n">
-        <v>36</v>
+        <v>1.44</v>
       </c>
       <c r="H804" s="2" t="n">
         <v>1524925</v>
@@ -38063,13 +38063,13 @@
         </is>
       </c>
       <c r="E806" s="4" t="n">
-        <v>0.08</v>
+        <v>1.28</v>
       </c>
       <c r="F806" s="5" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="G806" s="4" t="n">
-        <v>1.44</v>
+        <v>48.64</v>
       </c>
       <c r="H806" s="2" t="n">
         <v>1524925</v>
@@ -38580,13 +38580,13 @@
         </is>
       </c>
       <c r="E817" s="4" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F817" s="5" t="n">
-        <v>9.59</v>
+        <v>3.89</v>
       </c>
       <c r="G817" s="4" t="n">
-        <v>9.59</v>
+        <v>58.35</v>
       </c>
       <c r="H817" s="2" t="n">
         <v>1526079</v>
@@ -38627,13 +38627,13 @@
         </is>
       </c>
       <c r="E818" s="4" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F818" s="5" t="n">
-        <v>3.89</v>
+        <v>9.59</v>
       </c>
       <c r="G818" s="4" t="n">
-        <v>58.35</v>
+        <v>9.59</v>
       </c>
       <c r="H818" s="2" t="n">
         <v>1526079</v>
@@ -38674,13 +38674,13 @@
         </is>
       </c>
       <c r="E819" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F819" s="5" t="n">
-        <v>17.5</v>
+        <v>8.9</v>
       </c>
       <c r="G819" s="4" t="n">
-        <v>17.5</v>
+        <v>62.3</v>
       </c>
       <c r="H819" s="2" t="n">
         <v>1526335</v>
@@ -38721,13 +38721,13 @@
         </is>
       </c>
       <c r="E820" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F820" s="5" t="n">
-        <v>8.9</v>
+        <v>8.99</v>
       </c>
       <c r="G820" s="4" t="n">
-        <v>62.3</v>
+        <v>17.98</v>
       </c>
       <c r="H820" s="2" t="n">
         <v>1526335</v>
@@ -38768,13 +38768,13 @@
         </is>
       </c>
       <c r="E821" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F821" s="5" t="n">
-        <v>8.99</v>
+        <v>17.5</v>
       </c>
       <c r="G821" s="4" t="n">
-        <v>17.98</v>
+        <v>17.5</v>
       </c>
       <c r="H821" s="2" t="n">
         <v>1526335</v>
@@ -40087,10 +40087,10 @@
         <v>1</v>
       </c>
       <c r="F849" s="5" t="n">
-        <v>306.68</v>
+        <v>180.4</v>
       </c>
       <c r="G849" s="4" t="n">
-        <v>306.68</v>
+        <v>180.4</v>
       </c>
       <c r="H849" s="2" t="n">
         <v>1530930</v>
@@ -40134,10 +40134,10 @@
         <v>1</v>
       </c>
       <c r="F850" s="5" t="n">
-        <v>180.4</v>
+        <v>306.68</v>
       </c>
       <c r="G850" s="4" t="n">
-        <v>180.4</v>
+        <v>306.68</v>
       </c>
       <c r="H850" s="2" t="n">
         <v>1530930</v>
@@ -40886,10 +40886,10 @@
         <v>1</v>
       </c>
       <c r="F866" s="5" t="n">
-        <v>39.9</v>
+        <v>18.9</v>
       </c>
       <c r="G866" s="4" t="n">
-        <v>39.9</v>
+        <v>18.9</v>
       </c>
       <c r="H866" s="2" t="n">
         <v>1533181</v>
@@ -40930,13 +40930,13 @@
         </is>
       </c>
       <c r="E867" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F867" s="5" t="n">
-        <v>4.9</v>
+        <v>6.9</v>
       </c>
       <c r="G867" s="4" t="n">
-        <v>29.4</v>
+        <v>13.8</v>
       </c>
       <c r="H867" s="2" t="n">
         <v>1533181</v>
@@ -40977,13 +40977,13 @@
         </is>
       </c>
       <c r="E868" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F868" s="5" t="n">
-        <v>6.9</v>
+        <v>4.9</v>
       </c>
       <c r="G868" s="4" t="n">
-        <v>13.8</v>
+        <v>29.4</v>
       </c>
       <c r="H868" s="2" t="n">
         <v>1533181</v>
@@ -41027,10 +41027,10 @@
         <v>1</v>
       </c>
       <c r="F869" s="5" t="n">
-        <v>18.9</v>
+        <v>39.9</v>
       </c>
       <c r="G869" s="4" t="n">
-        <v>18.9</v>
+        <v>39.9</v>
       </c>
       <c r="H869" s="2" t="n">
         <v>1533181</v>
@@ -41776,13 +41776,13 @@
         </is>
       </c>
       <c r="E885" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F885" s="5" t="n">
-        <v>0.35</v>
+        <v>0.6</v>
       </c>
       <c r="G885" s="4" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="H885" s="2" t="n">
         <v>1539898</v>
@@ -41823,13 +41823,13 @@
         </is>
       </c>
       <c r="E886" s="4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F886" s="5" t="n">
-        <v>0.29</v>
+        <v>0.8</v>
       </c>
       <c r="G886" s="4" t="n">
-        <v>4.06</v>
+        <v>8</v>
       </c>
       <c r="H886" s="2" t="n">
         <v>1539898</v>
@@ -41873,10 +41873,10 @@
         <v>12</v>
       </c>
       <c r="F887" s="5" t="n">
-        <v>0.08</v>
+        <v>1</v>
       </c>
       <c r="G887" s="4" t="n">
-        <v>0.96</v>
+        <v>12</v>
       </c>
       <c r="H887" s="2" t="n">
         <v>1539898</v>
@@ -41917,13 +41917,13 @@
         </is>
       </c>
       <c r="E888" s="4" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="F888" s="5" t="n">
-        <v>0.17</v>
+        <v>2.3</v>
       </c>
       <c r="G888" s="4" t="n">
-        <v>5.1</v>
+        <v>13.8</v>
       </c>
       <c r="H888" s="2" t="n">
         <v>1539898</v>
@@ -41964,13 +41964,13 @@
         </is>
       </c>
       <c r="E889" s="4" t="n">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="F889" s="5" t="n">
-        <v>0.22</v>
+        <v>0.66</v>
       </c>
       <c r="G889" s="4" t="n">
-        <v>1.32</v>
+        <v>66</v>
       </c>
       <c r="H889" s="2" t="n">
         <v>1539898</v>
@@ -42011,13 +42011,13 @@
         </is>
       </c>
       <c r="E890" s="4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F890" s="5" t="n">
-        <v>0.15</v>
+        <v>0.52</v>
       </c>
       <c r="G890" s="4" t="n">
-        <v>1.8</v>
+        <v>4.16</v>
       </c>
       <c r="H890" s="2" t="n">
         <v>1539898</v>
@@ -42058,13 +42058,13 @@
         </is>
       </c>
       <c r="E891" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F891" s="5" t="n">
-        <v>0.25</v>
+        <v>0.58</v>
       </c>
       <c r="G891" s="4" t="n">
-        <v>2</v>
+        <v>2.32</v>
       </c>
       <c r="H891" s="2" t="n">
         <v>1539898</v>
@@ -42105,13 +42105,13 @@
         </is>
       </c>
       <c r="E892" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F892" s="5" t="n">
-        <v>53</v>
+        <v>0.81</v>
       </c>
       <c r="G892" s="4" t="n">
-        <v>53</v>
+        <v>1.62</v>
       </c>
       <c r="H892" s="2" t="n">
         <v>1539898</v>
@@ -42152,13 +42152,13 @@
         </is>
       </c>
       <c r="E893" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F893" s="5" t="n">
-        <v>0.11</v>
+        <v>0.7</v>
       </c>
       <c r="G893" s="4" t="n">
-        <v>0.66</v>
+        <v>2.8</v>
       </c>
       <c r="H893" s="2" t="n">
         <v>1539898</v>
@@ -42199,13 +42199,13 @@
         </is>
       </c>
       <c r="E894" s="4" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="F894" s="5" t="n">
-        <v>0.3</v>
+        <v>1.2</v>
       </c>
       <c r="G894" s="4" t="n">
-        <v>30</v>
+        <v>2.4</v>
       </c>
       <c r="H894" s="2" t="n">
         <v>1539898</v>
@@ -42246,13 +42246,13 @@
         </is>
       </c>
       <c r="E895" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F895" s="5" t="n">
-        <v>0.21</v>
+        <v>1.32</v>
       </c>
       <c r="G895" s="4" t="n">
-        <v>2.52</v>
+        <v>5.28</v>
       </c>
       <c r="H895" s="2" t="n">
         <v>1539898</v>
@@ -42293,13 +42293,13 @@
         </is>
       </c>
       <c r="E896" s="4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F896" s="5" t="n">
-        <v>0.33</v>
+        <v>0.45</v>
       </c>
       <c r="G896" s="4" t="n">
-        <v>1.98</v>
+        <v>5.4</v>
       </c>
       <c r="H896" s="2" t="n">
         <v>1539898</v>
@@ -42340,13 +42340,13 @@
         </is>
       </c>
       <c r="E897" s="4" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="F897" s="5" t="n">
-        <v>0.3</v>
+        <v>0.11</v>
       </c>
       <c r="G897" s="4" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="H897" s="2" t="n">
         <v>1539898</v>
@@ -42387,13 +42387,13 @@
         </is>
       </c>
       <c r="E898" s="4" t="n">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="F898" s="5" t="n">
-        <v>0.42</v>
+        <v>0.12</v>
       </c>
       <c r="G898" s="4" t="n">
-        <v>2.52</v>
+        <v>12</v>
       </c>
       <c r="H898" s="2" t="n">
         <v>1539898</v>
@@ -42481,13 +42481,13 @@
         </is>
       </c>
       <c r="E900" s="4" t="n">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="F900" s="5" t="n">
-        <v>0.12</v>
+        <v>0.42</v>
       </c>
       <c r="G900" s="4" t="n">
-        <v>12</v>
+        <v>2.52</v>
       </c>
       <c r="H900" s="2" t="n">
         <v>1539898</v>
@@ -42528,13 +42528,13 @@
         </is>
       </c>
       <c r="E901" s="4" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="F901" s="5" t="n">
-        <v>0.11</v>
+        <v>0.3</v>
       </c>
       <c r="G901" s="4" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="H901" s="2" t="n">
         <v>1539898</v>
@@ -42575,13 +42575,13 @@
         </is>
       </c>
       <c r="E902" s="4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F902" s="5" t="n">
-        <v>0.45</v>
+        <v>0.33</v>
       </c>
       <c r="G902" s="4" t="n">
-        <v>5.4</v>
+        <v>1.98</v>
       </c>
       <c r="H902" s="2" t="n">
         <v>1539898</v>
@@ -42622,13 +42622,13 @@
         </is>
       </c>
       <c r="E903" s="4" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F903" s="5" t="n">
-        <v>1.32</v>
+        <v>0.21</v>
       </c>
       <c r="G903" s="4" t="n">
-        <v>5.28</v>
+        <v>2.52</v>
       </c>
       <c r="H903" s="2" t="n">
         <v>1539898</v>
@@ -42669,13 +42669,13 @@
         </is>
       </c>
       <c r="E904" s="4" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F904" s="5" t="n">
-        <v>1.2</v>
+        <v>0.29</v>
       </c>
       <c r="G904" s="4" t="n">
-        <v>2.4</v>
+        <v>4.06</v>
       </c>
       <c r="H904" s="2" t="n">
         <v>1539898</v>
@@ -42716,13 +42716,13 @@
         </is>
       </c>
       <c r="E905" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F905" s="5" t="n">
-        <v>0.7</v>
+        <v>0.35</v>
       </c>
       <c r="G905" s="4" t="n">
-        <v>2.8</v>
+        <v>2.1</v>
       </c>
       <c r="H905" s="2" t="n">
         <v>1539898</v>
@@ -42763,13 +42763,13 @@
         </is>
       </c>
       <c r="E906" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F906" s="5" t="n">
-        <v>0.81</v>
+        <v>0.48</v>
       </c>
       <c r="G906" s="4" t="n">
-        <v>1.62</v>
+        <v>1.92</v>
       </c>
       <c r="H906" s="2" t="n">
         <v>1539898</v>
@@ -42810,13 +42810,13 @@
         </is>
       </c>
       <c r="E907" s="4" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="F907" s="5" t="n">
-        <v>0.58</v>
+        <v>0.2</v>
       </c>
       <c r="G907" s="4" t="n">
-        <v>2.32</v>
+        <v>4.8</v>
       </c>
       <c r="H907" s="2" t="n">
         <v>1539898</v>
@@ -42857,13 +42857,13 @@
         </is>
       </c>
       <c r="E908" s="4" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="F908" s="5" t="n">
-        <v>0.52</v>
+        <v>0.19</v>
       </c>
       <c r="G908" s="4" t="n">
-        <v>4.16</v>
+        <v>5.32</v>
       </c>
       <c r="H908" s="2" t="n">
         <v>1539898</v>
@@ -42904,13 +42904,13 @@
         </is>
       </c>
       <c r="E909" s="4" t="n">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="F909" s="5" t="n">
-        <v>0.66</v>
+        <v>0.08</v>
       </c>
       <c r="G909" s="4" t="n">
-        <v>66</v>
+        <v>0.96</v>
       </c>
       <c r="H909" s="2" t="n">
         <v>1539898</v>
@@ -42951,13 +42951,13 @@
         </is>
       </c>
       <c r="E910" s="4" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="F910" s="5" t="n">
-        <v>2.3</v>
+        <v>0.17</v>
       </c>
       <c r="G910" s="4" t="n">
-        <v>13.8</v>
+        <v>5.1</v>
       </c>
       <c r="H910" s="2" t="n">
         <v>1539898</v>
@@ -42998,13 +42998,13 @@
         </is>
       </c>
       <c r="E911" s="4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F911" s="5" t="n">
-        <v>1</v>
+        <v>0.22</v>
       </c>
       <c r="G911" s="4" t="n">
-        <v>12</v>
+        <v>1.32</v>
       </c>
       <c r="H911" s="2" t="n">
         <v>1539898</v>
@@ -43045,13 +43045,13 @@
         </is>
       </c>
       <c r="E912" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F912" s="5" t="n">
-        <v>0.8</v>
+        <v>0.15</v>
       </c>
       <c r="G912" s="4" t="n">
-        <v>8</v>
+        <v>1.8</v>
       </c>
       <c r="H912" s="2" t="n">
         <v>1539898</v>
@@ -43092,13 +43092,13 @@
         </is>
       </c>
       <c r="E913" s="4" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="F913" s="5" t="n">
-        <v>0.19</v>
+        <v>0.25</v>
       </c>
       <c r="G913" s="4" t="n">
-        <v>5.32</v>
+        <v>2</v>
       </c>
       <c r="H913" s="2" t="n">
         <v>1539898</v>
@@ -43139,13 +43139,13 @@
         </is>
       </c>
       <c r="E914" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F914" s="5" t="n">
-        <v>0.6</v>
+        <v>53</v>
       </c>
       <c r="G914" s="4" t="n">
-        <v>2.4</v>
+        <v>53</v>
       </c>
       <c r="H914" s="2" t="n">
         <v>1539898</v>
@@ -43186,13 +43186,13 @@
         </is>
       </c>
       <c r="E915" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F915" s="5" t="n">
-        <v>0.6</v>
+        <v>0.11</v>
       </c>
       <c r="G915" s="4" t="n">
-        <v>2.4</v>
+        <v>0.66</v>
       </c>
       <c r="H915" s="2" t="n">
         <v>1539898</v>
@@ -43233,13 +43233,13 @@
         </is>
       </c>
       <c r="E916" s="4" t="n">
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="F916" s="5" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="G916" s="4" t="n">
-        <v>4.8</v>
+        <v>30</v>
       </c>
       <c r="H916" s="2" t="n">
         <v>1539898</v>
@@ -43283,10 +43283,10 @@
         <v>4</v>
       </c>
       <c r="F917" s="5" t="n">
-        <v>0.48</v>
+        <v>0.6</v>
       </c>
       <c r="G917" s="4" t="n">
-        <v>1.92</v>
+        <v>2.4</v>
       </c>
       <c r="H917" s="2" t="n">
         <v>1539898</v>
@@ -43844,13 +43844,13 @@
         </is>
       </c>
       <c r="E929" s="4" t="n">
-        <v>0.04</v>
+        <v>0.28</v>
       </c>
       <c r="F929" s="5" t="n">
         <v>100</v>
       </c>
       <c r="G929" s="4" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="H929" s="2" t="n">
         <v>1546014</v>
@@ -43891,13 +43891,13 @@
         </is>
       </c>
       <c r="E930" s="4" t="n">
-        <v>0.16</v>
+        <v>0.1</v>
       </c>
       <c r="F930" s="5" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G930" s="4" t="n">
-        <v>5.6</v>
+        <v>4</v>
       </c>
       <c r="H930" s="2" t="n">
         <v>1546014</v>
@@ -43941,10 +43941,10 @@
         <v>0.28</v>
       </c>
       <c r="F931" s="5" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="G931" s="4" t="n">
-        <v>4.2</v>
+        <v>8.4</v>
       </c>
       <c r="H931" s="2" t="n">
         <v>1546014</v>
@@ -44035,10 +44035,10 @@
         <v>0.28</v>
       </c>
       <c r="F933" s="5" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="G933" s="4" t="n">
-        <v>28</v>
+        <v>4.2</v>
       </c>
       <c r="H933" s="2" t="n">
         <v>1546014</v>
@@ -44126,13 +44126,13 @@
         </is>
       </c>
       <c r="E935" s="4" t="n">
-        <v>0.1</v>
+        <v>0.16</v>
       </c>
       <c r="F935" s="5" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G935" s="4" t="n">
-        <v>4</v>
+        <v>5.6</v>
       </c>
       <c r="H935" s="2" t="n">
         <v>1546014</v>
@@ -44173,13 +44173,13 @@
         </is>
       </c>
       <c r="E936" s="4" t="n">
-        <v>0.28</v>
+        <v>0.04</v>
       </c>
       <c r="F936" s="5" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="G936" s="4" t="n">
-        <v>8.4</v>
+        <v>4</v>
       </c>
       <c r="H936" s="2" t="n">
         <v>1546014</v>
@@ -44317,10 +44317,10 @@
         <v>1</v>
       </c>
       <c r="F939" s="5" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="G939" s="4" t="n">
-        <v>157.85</v>
+        <v>171.7</v>
       </c>
       <c r="H939" s="2" t="n">
         <v>1547044</v>
@@ -44505,10 +44505,10 @@
         <v>1</v>
       </c>
       <c r="F943" s="5" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="G943" s="4" t="n">
-        <v>171.7</v>
+        <v>157.85</v>
       </c>
       <c r="H943" s="2" t="n">
         <v>1547044</v>
@@ -80131,10 +80131,10 @@
         <v>100</v>
       </c>
       <c r="F1701" s="5" t="n">
-        <v>0.22</v>
+        <v>1.35</v>
       </c>
       <c r="G1701" s="4" t="n">
-        <v>22</v>
+        <v>135</v>
       </c>
       <c r="H1701" s="2" t="n">
         <v>1630277</v>
@@ -80225,10 +80225,10 @@
         <v>100</v>
       </c>
       <c r="F1703" s="5" t="n">
-        <v>1.35</v>
+        <v>0.22</v>
       </c>
       <c r="G1703" s="4" t="n">
-        <v>135</v>
+        <v>22</v>
       </c>
       <c r="H1703" s="2" t="n">
         <v>1630277</v>
@@ -81021,13 +81021,13 @@
         </is>
       </c>
       <c r="E1720" s="4" t="n">
-        <v>2</v>
+        <v>0.1</v>
       </c>
       <c r="F1720" s="5" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="G1720" s="4" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="H1720" s="2" t="n">
         <v>1632122</v>
@@ -81068,13 +81068,13 @@
         </is>
       </c>
       <c r="E1721" s="4" t="n">
-        <v>1</v>
+        <v>0.08</v>
       </c>
       <c r="F1721" s="5" t="n">
-        <v>16</v>
+        <v>500</v>
       </c>
       <c r="G1721" s="4" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="H1721" s="2" t="n">
         <v>1632122</v>
@@ -81162,13 +81162,13 @@
         </is>
       </c>
       <c r="E1723" s="4" t="n">
-        <v>0.08</v>
+        <v>2</v>
       </c>
       <c r="F1723" s="5" t="n">
-        <v>500</v>
+        <v>25</v>
       </c>
       <c r="G1723" s="4" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H1723" s="2" t="n">
         <v>1632122</v>
@@ -81209,13 +81209,13 @@
         </is>
       </c>
       <c r="E1724" s="4" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="F1724" s="5" t="n">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="G1724" s="4" t="n">
-        <v>6</v>
+        <v>4.4</v>
       </c>
       <c r="H1724" s="2" t="n">
         <v>1632122</v>
@@ -81256,13 +81256,13 @@
         </is>
       </c>
       <c r="E1725" s="4" t="n">
-        <v>0.04</v>
+        <v>1</v>
       </c>
       <c r="F1725" s="5" t="n">
-        <v>110</v>
+        <v>22</v>
       </c>
       <c r="G1725" s="4" t="n">
-        <v>4.4</v>
+        <v>22</v>
       </c>
       <c r="H1725" s="2" t="n">
         <v>1632122</v>
@@ -81303,13 +81303,13 @@
         </is>
       </c>
       <c r="E1726" s="4" t="n">
-        <v>0.04</v>
+        <v>1</v>
       </c>
       <c r="F1726" s="5" t="n">
-        <v>140</v>
+        <v>16</v>
       </c>
       <c r="G1726" s="4" t="n">
-        <v>5.6</v>
+        <v>16</v>
       </c>
       <c r="H1726" s="2" t="n">
         <v>1632122</v>
@@ -81350,13 +81350,13 @@
         </is>
       </c>
       <c r="E1727" s="4" t="n">
-        <v>1</v>
+        <v>0.04</v>
       </c>
       <c r="F1727" s="5" t="n">
-        <v>22</v>
+        <v>140</v>
       </c>
       <c r="G1727" s="4" t="n">
-        <v>22</v>
+        <v>5.6</v>
       </c>
       <c r="H1727" s="2" t="n">
         <v>1632122</v>
@@ -82810,10 +82810,10 @@
         <v>1</v>
       </c>
       <c r="F1758" s="5" t="n">
-        <v>10.93</v>
+        <v>12.11</v>
       </c>
       <c r="G1758" s="4" t="n">
-        <v>10.93</v>
+        <v>12.11</v>
       </c>
       <c r="H1758" s="2" t="n">
         <v>1639631</v>
@@ -82857,10 +82857,10 @@
         <v>1</v>
       </c>
       <c r="F1759" s="5" t="n">
-        <v>12.11</v>
+        <v>10.93</v>
       </c>
       <c r="G1759" s="4" t="n">
-        <v>12.11</v>
+        <v>10.93</v>
       </c>
       <c r="H1759" s="2" t="n">
         <v>1639631</v>
@@ -83136,13 +83136,13 @@
         </is>
       </c>
       <c r="E1765" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F1765" s="5" t="n">
         <v>5</v>
       </c>
       <c r="G1765" s="4" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H1765" s="2" t="n">
         <v>1639777</v>
@@ -83183,13 +83183,13 @@
         </is>
       </c>
       <c r="E1766" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F1766" s="5" t="n">
         <v>5</v>
       </c>
       <c r="G1766" s="4" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H1766" s="2" t="n">
         <v>1639777</v>
@@ -83559,13 +83559,13 @@
         </is>
       </c>
       <c r="E1774" s="4" t="n">
-        <v>0.2</v>
+        <v>1.5</v>
       </c>
       <c r="F1774" s="5" t="n">
-        <v>70</v>
+        <v>18</v>
       </c>
       <c r="G1774" s="4" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="H1774" s="2" t="n">
         <v>1642001</v>
@@ -83606,13 +83606,13 @@
         </is>
       </c>
       <c r="E1775" s="4" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="F1775" s="5" t="n">
-        <v>220</v>
+        <v>18</v>
       </c>
       <c r="G1775" s="4" t="n">
-        <v>110</v>
+        <v>27</v>
       </c>
       <c r="H1775" s="2" t="n">
         <v>1642001</v>
@@ -83653,13 +83653,13 @@
         </is>
       </c>
       <c r="E1776" s="4" t="n">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
       <c r="F1776" s="5" t="n">
-        <v>40</v>
+        <v>1600</v>
       </c>
       <c r="G1776" s="4" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="H1776" s="2" t="n">
         <v>1642001</v>
@@ -83700,13 +83700,13 @@
         </is>
       </c>
       <c r="E1777" s="4" t="n">
-        <v>2</v>
+        <v>0.06</v>
       </c>
       <c r="F1777" s="5" t="n">
-        <v>14</v>
+        <v>850</v>
       </c>
       <c r="G1777" s="4" t="n">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="H1777" s="2" t="n">
         <v>1642001</v>
@@ -83747,13 +83747,13 @@
         </is>
       </c>
       <c r="E1778" s="4" t="n">
-        <v>0.02</v>
+        <v>0.2</v>
       </c>
       <c r="F1778" s="5" t="n">
-        <v>1600</v>
+        <v>70</v>
       </c>
       <c r="G1778" s="4" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="H1778" s="2" t="n">
         <v>1642001</v>
@@ -83794,13 +83794,13 @@
         </is>
       </c>
       <c r="E1779" s="4" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="F1779" s="5" t="n">
-        <v>18</v>
+        <v>220</v>
       </c>
       <c r="G1779" s="4" t="n">
-        <v>27</v>
+        <v>110</v>
       </c>
       <c r="H1779" s="2" t="n">
         <v>1642001</v>
@@ -83841,13 +83841,13 @@
         </is>
       </c>
       <c r="E1780" s="4" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="F1780" s="5" t="n">
-        <v>850</v>
+        <v>40</v>
       </c>
       <c r="G1780" s="4" t="n">
-        <v>51</v>
+        <v>4</v>
       </c>
       <c r="H1780" s="2" t="n">
         <v>1642001</v>
@@ -83888,13 +83888,13 @@
         </is>
       </c>
       <c r="E1781" s="4" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="F1781" s="5" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G1781" s="4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H1781" s="2" t="n">
         <v>1642001</v>
@@ -84054,6 +84054,1181 @@
       </c>
       <c r="K1784" s="2" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="1785" customHeight="1" ht="15">
+      <c r="A1785" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1785" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1785" s="2" t="n">
+        <v>37208</v>
+      </c>
+      <c r="D1785" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">RESMA-SULFITE</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1785" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F1785" s="5" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="G1785" s="4" t="n">
+        <v>1274.5</v>
+      </c>
+      <c r="H1785" s="2" t="n">
+        <v>1642254</v>
+      </c>
+      <c r="I1785" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 08:28:44</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1785" s="2" t="n">
+        <v>26094</v>
+      </c>
+      <c r="K1785" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1786" customHeight="1" ht="15">
+      <c r="A1786" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1786" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1786" s="2" t="n">
+        <v>15538</v>
+      </c>
+      <c r="D1786" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_ESC</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1786" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1786" s="5" t="n">
+        <v>95.6</v>
+      </c>
+      <c r="G1786" s="4" t="n">
+        <v>191.2</v>
+      </c>
+      <c r="H1786" s="2" t="n">
+        <v>1642274</v>
+      </c>
+      <c r="I1786" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 08:50:41</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1786" s="2" t="n">
+        <v>37589</v>
+      </c>
+      <c r="K1786" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1787" customHeight="1" ht="15">
+      <c r="A1787" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1787" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1787" s="2" t="n">
+        <v>39526</v>
+      </c>
+      <c r="D1787" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">INS-MGMN300-H-LF6018</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1787" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1787" s="5" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="G1787" s="4" t="n">
+        <v>234</v>
+      </c>
+      <c r="H1787" s="2" t="n">
+        <v>1642365</v>
+      </c>
+      <c r="I1787" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 10:42:38</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1787" s="2" t="n">
+        <v>12770</v>
+      </c>
+      <c r="K1787" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1788" customHeight="1" ht="15">
+      <c r="A1788" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1788" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1788" s="2" t="n">
+        <v>12839</v>
+      </c>
+      <c r="D1788" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">ESCOVA-ACO-6</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1788" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1788" s="5" t="n">
+        <v>29.39</v>
+      </c>
+      <c r="G1788" s="4" t="n">
+        <v>117.56</v>
+      </c>
+      <c r="H1788" s="2" t="n">
+        <v>1642381</v>
+      </c>
+      <c r="I1788" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 10:55:11</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1788" s="2" t="n">
+        <v>14143</v>
+      </c>
+      <c r="K1788" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1789" customHeight="1" ht="15">
+      <c r="A1789" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1789" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1789" s="2" t="n">
+        <v>31042</v>
+      </c>
+      <c r="D1789" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">COS-M16X1.5</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1789" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1789" s="5" t="n">
+        <v>531.15</v>
+      </c>
+      <c r="G1789" s="4" t="n">
+        <v>1062.3</v>
+      </c>
+      <c r="H1789" s="2" t="n">
+        <v>1642381</v>
+      </c>
+      <c r="I1789" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 10:55:11</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1789" s="2" t="n">
+        <v>14143</v>
+      </c>
+      <c r="K1789" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1790" customHeight="1" ht="15">
+      <c r="A1790" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1790" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1790" s="2" t="n">
+        <v>31086</v>
+      </c>
+      <c r="D1790" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">COLA-VERMELHA</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1790" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F1790" s="5" t="n">
+        <v>276.38</v>
+      </c>
+      <c r="G1790" s="4" t="n">
+        <v>4145.7</v>
+      </c>
+      <c r="H1790" s="2" t="n">
+        <v>1642381</v>
+      </c>
+      <c r="I1790" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 10:55:11</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1790" s="2" t="n">
+        <v>14143</v>
+      </c>
+      <c r="K1790" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1791" customHeight="1" ht="15">
+      <c r="A1791" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1791" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1791" s="2" t="n">
+        <v>37209</v>
+      </c>
+      <c r="D1791" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">VASELINA-LIQUIDA</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1791" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1791" s="5" t="n">
+        <v>13.87</v>
+      </c>
+      <c r="G1791" s="4" t="n">
+        <v>110.96</v>
+      </c>
+      <c r="H1791" s="2" t="n">
+        <v>1642381</v>
+      </c>
+      <c r="I1791" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 10:55:11</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1791" s="2" t="n">
+        <v>14143</v>
+      </c>
+      <c r="K1791" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1792" customHeight="1" ht="15">
+      <c r="A1792" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1792" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1792" s="2" t="n">
+        <v>37539</v>
+      </c>
+      <c r="D1792" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">COS-M10X1.25</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1792" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1792" s="5" t="n">
+        <v>294.43</v>
+      </c>
+      <c r="G1792" s="4" t="n">
+        <v>588.86</v>
+      </c>
+      <c r="H1792" s="2" t="n">
+        <v>1642381</v>
+      </c>
+      <c r="I1792" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 10:55:11</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1792" s="2" t="n">
+        <v>14143</v>
+      </c>
+      <c r="K1792" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1793" customHeight="1" ht="15">
+      <c r="A1793" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1793" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1793" s="2" t="n">
+        <v>37540</v>
+      </c>
+      <c r="D1793" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">COS-M12X1.25</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1793" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1793" s="5" t="n">
+        <v>356.18</v>
+      </c>
+      <c r="G1793" s="4" t="n">
+        <v>356.18</v>
+      </c>
+      <c r="H1793" s="2" t="n">
+        <v>1642381</v>
+      </c>
+      <c r="I1793" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 10:55:11</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1793" s="2" t="n">
+        <v>14143</v>
+      </c>
+      <c r="K1793" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1794" customHeight="1" ht="15">
+      <c r="A1794" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1794" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1794" s="2" t="n">
+        <v>37546</v>
+      </c>
+      <c r="D1794" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">COS-M6X1.0</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1794" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1794" s="5" t="n">
+        <v>178.11</v>
+      </c>
+      <c r="G1794" s="4" t="n">
+        <v>356.22</v>
+      </c>
+      <c r="H1794" s="2" t="n">
+        <v>1642381</v>
+      </c>
+      <c r="I1794" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 10:55:11</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1794" s="2" t="n">
+        <v>14143</v>
+      </c>
+      <c r="K1794" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1795" customHeight="1" ht="15">
+      <c r="A1795" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1795" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1795" s="2" t="n">
+        <v>37554</v>
+      </c>
+      <c r="D1795" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">MACHO-H-M10X1.5</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1795" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1795" s="5" t="n">
+        <v>128.76</v>
+      </c>
+      <c r="G1795" s="4" t="n">
+        <v>257.52</v>
+      </c>
+      <c r="H1795" s="2" t="n">
+        <v>1642381</v>
+      </c>
+      <c r="I1795" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 10:55:11</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1795" s="2" t="n">
+        <v>14143</v>
+      </c>
+      <c r="K1795" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1796" customHeight="1" ht="15">
+      <c r="A1796" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1796" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1796" s="2" t="n">
+        <v>37694</v>
+      </c>
+      <c r="D1796" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">WD40</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1796" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1796" s="5" t="n">
+        <v>30.03</v>
+      </c>
+      <c r="G1796" s="4" t="n">
+        <v>150.15</v>
+      </c>
+      <c r="H1796" s="2" t="n">
+        <v>1642381</v>
+      </c>
+      <c r="I1796" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 10:55:11</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1796" s="2" t="n">
+        <v>14143</v>
+      </c>
+      <c r="K1796" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1797" customHeight="1" ht="15">
+      <c r="A1797" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1797" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1797" s="2" t="n">
+        <v>37946</v>
+      </c>
+      <c r="D1797" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">COS-M20X1.50</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1797" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1797" s="5" t="n">
+        <v>531.15</v>
+      </c>
+      <c r="G1797" s="4" t="n">
+        <v>1593.45</v>
+      </c>
+      <c r="H1797" s="2" t="n">
+        <v>1642381</v>
+      </c>
+      <c r="I1797" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 10:55:11</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1797" s="2" t="n">
+        <v>14143</v>
+      </c>
+      <c r="K1797" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1798" customHeight="1" ht="15">
+      <c r="A1798" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1798" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1798" s="2" t="n">
+        <v>39517</v>
+      </c>
+      <c r="D1798" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">BROCA-AR-10.3</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1798" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1798" s="5" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="G1798" s="4" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="H1798" s="2" t="n">
+        <v>1642381</v>
+      </c>
+      <c r="I1798" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 10:55:11</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1798" s="2" t="n">
+        <v>14143</v>
+      </c>
+      <c r="K1798" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1799" customHeight="1" ht="15">
+      <c r="A1799" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1799" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1799" s="2" t="n">
+        <v>43934</v>
+      </c>
+      <c r="D1799" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">BROCA-AR-12</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1799" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1799" s="5" t="n">
+        <v>29.39</v>
+      </c>
+      <c r="G1799" s="4" t="n">
+        <v>29.39</v>
+      </c>
+      <c r="H1799" s="2" t="n">
+        <v>1642381</v>
+      </c>
+      <c r="I1799" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 10:55:11</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1799" s="2" t="n">
+        <v>14143</v>
+      </c>
+      <c r="K1799" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1800" customHeight="1" ht="15">
+      <c r="A1800" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1800" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1800" s="2" t="n">
+        <v>15039</v>
+      </c>
+      <c r="D1800" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_USE</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1800" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1800" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="G1800" s="4" t="n">
+        <v>350</v>
+      </c>
+      <c r="H1800" s="2" t="n">
+        <v>1642469</v>
+      </c>
+      <c r="I1800" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 12:33:25</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1800" s="2" t="n">
+        <v>2368</v>
+      </c>
+      <c r="K1800" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1801" customHeight="1" ht="15">
+      <c r="A1801" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1801" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1801" s="2" t="n">
+        <v>15538</v>
+      </c>
+      <c r="D1801" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_ESC</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1801" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1801" s="5" t="n">
+        <v>960.77</v>
+      </c>
+      <c r="G1801" s="4" t="n">
+        <v>960.77</v>
+      </c>
+      <c r="H1801" s="2" t="n">
+        <v>1642604</v>
+      </c>
+      <c r="I1801" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 15:21:16</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1801" s="2" t="n">
+        <v>43385</v>
+      </c>
+      <c r="K1801" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1802" customHeight="1" ht="15">
+      <c r="A1802" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1802" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1802" s="2" t="n">
+        <v>15538</v>
+      </c>
+      <c r="D1802" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_ESC</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1802" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1802" s="5" t="n">
+        <v>408.69</v>
+      </c>
+      <c r="G1802" s="4" t="n">
+        <v>408.69</v>
+      </c>
+      <c r="H1802" s="2" t="n">
+        <v>1642604</v>
+      </c>
+      <c r="I1802" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 15:21:16</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1802" s="2" t="n">
+        <v>43385</v>
+      </c>
+      <c r="K1802" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1803" customHeight="1" ht="15">
+      <c r="A1803" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1803" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1803" s="2" t="n">
+        <v>15538</v>
+      </c>
+      <c r="D1803" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_ESC</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1803" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1803" s="5" t="n">
+        <v>444.99</v>
+      </c>
+      <c r="G1803" s="4" t="n">
+        <v>889.98</v>
+      </c>
+      <c r="H1803" s="2" t="n">
+        <v>1642604</v>
+      </c>
+      <c r="I1803" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 15:21:16</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1803" s="2" t="n">
+        <v>43385</v>
+      </c>
+      <c r="K1803" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1804" customHeight="1" ht="15">
+      <c r="A1804" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1804" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1804" s="2" t="n">
+        <v>15538</v>
+      </c>
+      <c r="D1804" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_ESC</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1804" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1804" s="5" t="n">
+        <v>455.49</v>
+      </c>
+      <c r="G1804" s="4" t="n">
+        <v>455.49</v>
+      </c>
+      <c r="H1804" s="2" t="n">
+        <v>1642604</v>
+      </c>
+      <c r="I1804" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 15:21:16</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1804" s="2" t="n">
+        <v>43385</v>
+      </c>
+      <c r="K1804" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1805" customHeight="1" ht="15">
+      <c r="A1805" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1805" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1805" s="2" t="n">
+        <v>15538</v>
+      </c>
+      <c r="D1805" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_ESC</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1805" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1805" s="5" t="n">
+        <v>231.32</v>
+      </c>
+      <c r="G1805" s="4" t="n">
+        <v>231.32</v>
+      </c>
+      <c r="H1805" s="2" t="n">
+        <v>1642604</v>
+      </c>
+      <c r="I1805" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 15:21:16</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1805" s="2" t="n">
+        <v>43385</v>
+      </c>
+      <c r="K1805" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1806" customHeight="1" ht="15">
+      <c r="A1806" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1806" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1806" s="2" t="n">
+        <v>15538</v>
+      </c>
+      <c r="D1806" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_ESC</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1806" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1806" s="5" t="n">
+        <v>99.99</v>
+      </c>
+      <c r="G1806" s="4" t="n">
+        <v>99.99</v>
+      </c>
+      <c r="H1806" s="2" t="n">
+        <v>1642604</v>
+      </c>
+      <c r="I1806" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 15:21:16</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1806" s="2" t="n">
+        <v>43385</v>
+      </c>
+      <c r="K1806" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1807" customHeight="1" ht="15">
+      <c r="A1807" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1807" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1807" s="2" t="n">
+        <v>15538</v>
+      </c>
+      <c r="D1807" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_ESC</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1807" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1807" s="5" t="n">
+        <v>159.99</v>
+      </c>
+      <c r="G1807" s="4" t="n">
+        <v>159.99</v>
+      </c>
+      <c r="H1807" s="2" t="n">
+        <v>1642604</v>
+      </c>
+      <c r="I1807" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 15:21:16</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1807" s="2" t="n">
+        <v>43385</v>
+      </c>
+      <c r="K1807" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1808" customHeight="1" ht="15">
+      <c r="A1808" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1808" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1808" s="2" t="n">
+        <v>15538</v>
+      </c>
+      <c r="D1808" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_ESC</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1808" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1808" s="5" t="n">
+        <v>69.99</v>
+      </c>
+      <c r="G1808" s="4" t="n">
+        <v>69.99</v>
+      </c>
+      <c r="H1808" s="2" t="n">
+        <v>1642604</v>
+      </c>
+      <c r="I1808" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 15:21:16</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1808" s="2" t="n">
+        <v>43385</v>
+      </c>
+      <c r="K1808" s="2" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1809" customHeight="1" ht="15">
+      <c r="A1809" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1809" s="2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C1809" s="2" t="n">
+        <v>15538</v>
+      </c>
+      <c r="D1809" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">M1_ESC</t>
+          </r>
+        </is>
+      </c>
+      <c r="E1809" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1809" s="5" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="G1809" s="4" t="n">
+        <v>1499.99</v>
+      </c>
+      <c r="H1809" s="2" t="n">
+        <v>1642604</v>
+      </c>
+      <c r="I1809" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+       </rPr>
+            <t xml:space="preserve">21/10/2026 15:21:16</t>
+          </r>
+        </is>
+      </c>
+      <c r="J1809" s="2" t="n">
+        <v>43385</v>
+      </c>
+      <c r="K1809" s="2" t="n">
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>